<commit_message>
refactor(PA需求列表): update strategy requirement sheet with more details
1. add 4 new requirement items for strategy management
2. supplement official documentation references for most existing items
3. update description of NAT zone matching logic and QoS DSCP support status
4. add migration evaluation notes for multiple new and existing features
</commit_message>
<xml_diff>
--- a/PA替代需求列表.xlsx
+++ b/PA替代需求列表.xlsx
@@ -2785,7 +2785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.7" customWidth="1" style="101" min="1" max="1"/>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="D2" s="113" t="inlineStr">
         <is>
-          <t>PA Web界面『策略』章节定义多种策略类型，按用途各自独立配置；对应功能矩阵#2-9/33/52/122/128/129</t>
+          <t>PA Web界面『策略』章节定义多种策略类型，按用途各自独立配置（PA Web帮助p113起）；对应功能矩阵#2-9/33/52/122/128/129</t>
         </is>
       </c>
       <c r="E2" s="112" t="inlineStr">
@@ -2878,7 +2878,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="51" customHeight="1" s="101">
+    <row r="3" ht="66" customHeight="1" s="101">
       <c r="A3" s="116" t="n"/>
       <c r="B3" s="116" t="n"/>
       <c r="C3" s="113" t="inlineStr">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="D3" s="113" t="inlineStr">
         <is>
-          <t>PA支持将策略规则移动/克隆到虚拟系统或Panorama设备组（含共享位置）；天融信访问控制策略支持移动策略与克隆模板[toc450050600]</t>
+          <t>PA支持将策略规则移动/克隆到虚拟系统或Panorama设备组（含共享位置，PA Web帮助p115）；天融信访问控制策略支持移动策略与克隆模板（天融信手册《配置访问控制策略》页）</t>
         </is>
       </c>
       <c r="E3" s="112" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="D4" s="113" t="inlineStr">
         <is>
-          <t>PA记录规则的审核注释历史/配置日志/规则更改历史，可CSV导出，用于策略变更审计；天融信仅规则描述字段，无审核注释存档</t>
+          <t>PA记录规则的审核注释历史/配置日志/规则更改历史，可CSV导出，用于策略变更审计（PA Web帮助p116-117）；天融信仅规则描述字段，无审核注释存档</t>
         </is>
       </c>
       <c r="E4" s="116" t="n"/>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="D5" s="113" t="inlineStr">
         <is>
-          <t>PA支持按时间段查询规则命中数，标识未使用规则以清理；含Reset Rule Hit Count重置功能；天融信策略统计开关可显示规则匹配情况[toc450050600]</t>
+          <t>PA支持按时间段查询规则命中数，标识未使用规则以清理；含Reset Rule Hit Count重置功能（PA Web帮助p118-119）；天融信策略统计开关可显示规则匹配情况（天融信手册《配置访问控制策略》页）</t>
         </is>
       </c>
       <c r="E5" s="116" t="n"/>
@@ -2948,7 +2948,7 @@
       </c>
       <c r="H5" s="116" t="n"/>
     </row>
-    <row r="6" ht="66" customHeight="1" s="101">
+    <row r="6" ht="111" customHeight="1" s="101">
       <c r="A6" s="116" t="n"/>
       <c r="B6" s="116" t="n"/>
       <c r="C6" s="113" t="inlineStr">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="D6" s="113" t="inlineStr">
         <is>
-          <t>PA在Panorama管理下策略分为前置规则（设备组共享）/本地规则/后置规则三层按序匹配；天融信为自上而下单层规则链[toc450050600]；迁移评估项：需拆解全局继承策略并映射到天融信策略表顺序</t>
+          <t>PA在Panorama集中管理下策略分为前置规则（设备组共享，最优先）/本地规则/后置规则三层按序匹配（层级机制属Panorama管理平台，PA两册手册未详载）；天融信为自上而下单层规则链一张表走到底（天融信手册《配置访问控制策略》页）；迁移评估项：需制定全局多级策略到单层扁平化策略的合并清洗规则（Pre→本地→Post按序展开映射）</t>
         </is>
       </c>
       <c r="E6" s="116" t="n"/>
@@ -2970,51 +2970,39 @@
       </c>
       <c r="H6" s="116" t="n"/>
     </row>
-    <row r="7" ht="51" customHeight="1" s="101">
+    <row r="7" ht="96" customHeight="1" s="101">
       <c r="A7" s="116" t="n"/>
-      <c r="B7" s="112" t="inlineStr">
+      <c r="B7" s="116" t="n"/>
+      <c r="C7" s="113" t="inlineStr">
+        <is>
+          <t>支持应用级会话超时覆盖（Application Timeout Override）</t>
+        </is>
+      </c>
+      <c r="D7" s="113" t="inlineStr">
+        <is>
+          <t>PA除全局TCP/UDP会话超时外，可在应用程序对象上定义专用超时，匹配该应用的流量覆盖全局值（PA Web帮助p215、p695）；天融信手册未见应用级超时覆盖（仅SSLVPN会话超时设置与黑名单老化）；迁移评估项：需排查现网PA为数据库/长连接业务单独配置的应用超时并逐条转换，否则长连接业务频繁中断</t>
+        </is>
+      </c>
+      <c r="E7" s="116" t="n"/>
+      <c r="F7" s="116" t="n"/>
+      <c r="G7" s="116" t="n"/>
+      <c r="H7" s="116" t="n"/>
+    </row>
+    <row r="8" ht="51" customHeight="1" s="101">
+      <c r="A8" s="116" t="n"/>
+      <c r="B8" s="112" t="inlineStr">
         <is>
           <t>安全策略(Security)</t>
         </is>
       </c>
-      <c r="C7" s="113" t="inlineStr">
+      <c r="C8" s="113" t="inlineStr">
         <is>
           <t>支持基于应用、源/目的区域和地址、用户或用户组、服务（端口/协议）的安全策略</t>
         </is>
       </c>
-      <c r="D7" s="113" t="inlineStr">
+      <c r="D8" s="113" t="inlineStr">
         <is>
           <t>PA安全策略规则基于App-ID应用、用户(User-ID)、区域地址、服务多维匹配并允许/拒绝/跟踪流量；对应矩阵#2/3/4</t>
-        </is>
-      </c>
-      <c r="E7" s="112" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="F7" s="113" t="inlineStr"/>
-      <c r="G7" s="112" t="inlineStr">
-        <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="H7" s="112" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1" s="101">
-      <c r="A8" s="116" t="n"/>
-      <c r="B8" s="116" t="n"/>
-      <c r="C8" s="113" t="inlineStr">
-        <is>
-          <t>支持安全策略规则构建块：源用户/HIP/设备/应用/服务/日志等</t>
-        </is>
-      </c>
-      <c r="D8" s="113" t="inlineStr">
-        <is>
-          <t>PA规则构建块含预登录用户、HIP配置文件、设备对象、应用默认端口规避、会话结束日志等；对应矩阵#3/4</t>
         </is>
       </c>
       <c r="E8" s="112" t="inlineStr">
@@ -3028,141 +3016,137 @@
           <t>已支持</t>
         </is>
       </c>
-      <c r="H8" s="112" t="inlineStr"/>
+      <c r="H8" s="112" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="36" customHeight="1" s="101">
       <c r="A9" s="116" t="n"/>
       <c r="B9" s="116" t="n"/>
       <c r="C9" s="113" t="inlineStr">
         <is>
-          <t>支持安全策略优化器（Policy Optimizer）</t>
+          <t>支持安全策略规则构建块：源用户/HIP/设备/应用/服务/日志等</t>
         </is>
       </c>
       <c r="D9" s="113" t="inlineStr">
         <is>
-          <t>PA新应用查看器+端口规则迁移至App-ID规则工作流+规则使用统计，减少攻击面；对应矩阵#132</t>
+          <t>PA规则构建块含预登录用户、HIP配置文件、设备对象、应用默认端口规避、会话结束日志等；对应矩阵#3/4</t>
         </is>
       </c>
       <c r="E9" s="112" t="inlineStr">
         <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="F9" s="116" t="n"/>
-      <c r="G9" s="116" t="n"/>
-      <c r="H9" s="116" t="n"/>
-    </row>
-    <row r="10" ht="36" customHeight="1" s="101">
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F9" s="113" t="inlineStr"/>
+      <c r="G9" s="112" t="inlineStr">
+        <is>
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="H9" s="112" t="inlineStr"/>
+    </row>
+    <row r="10" ht="51" customHeight="1" s="101">
       <c r="A10" s="116" t="n"/>
       <c r="B10" s="116" t="n"/>
       <c r="C10" s="113" t="inlineStr">
         <is>
-          <t>支持配置锁（Config Lock/Commit Lock）</t>
+          <t>支持安全策略优化器（Policy Optimizer）</t>
         </is>
       </c>
       <c r="D10" s="113" t="inlineStr">
         <is>
-          <t>PA可锁定待选配置或提交，防止他管理员并发更改；对应矩阵#135（天融信不支持，PA优势）</t>
-        </is>
-      </c>
-      <c r="E10" s="116" t="n"/>
+          <t>PA新应用查看器+端口规则迁移至App-ID规则工作流+规则使用统计，减少攻击面（PA Web帮助p142）；对应矩阵#132</t>
+        </is>
+      </c>
+      <c r="E10" s="112" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
       <c r="F10" s="116" t="n"/>
-      <c r="G10" s="112" t="inlineStr">
-        <is>
-          <t>待评估</t>
-        </is>
-      </c>
+      <c r="G10" s="116" t="n"/>
       <c r="H10" s="116" t="n"/>
     </row>
-    <row r="11" ht="81" customHeight="1" s="101">
+    <row r="11" ht="36" customHeight="1" s="101">
       <c r="A11" s="116" t="n"/>
       <c r="B11" s="116" t="n"/>
       <c r="C11" s="113" t="inlineStr">
         <is>
-          <t>支持应用默认端口绑定（Service: application-default）</t>
+          <t>支持配置锁（Config Lock/Commit Lock）</t>
         </is>
       </c>
       <c r="D11" s="113" t="inlineStr">
         <is>
-          <t>PA安全策略默认服务为application-default（应用走标准端口，非标准端口不匹配即拦截）；天融信策略为五元组+应用识别组合[toc450050600]；迁移评估项：策略转换若仅匹配应用不限端口将放宽安全边界，需制定非标准端口转换细则；对应矩阵#2</t>
-        </is>
-      </c>
-      <c r="E11" s="112" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
+          <t>PA可锁定待选配置或提交，防止他管理员并发更改；对应矩阵#135（天融信不支持，PA优势）</t>
+        </is>
+      </c>
+      <c r="E11" s="116" t="n"/>
       <c r="F11" s="116" t="n"/>
-      <c r="G11" s="116" t="n"/>
+      <c r="G11" s="112" t="inlineStr">
+        <is>
+          <t>待评估</t>
+        </is>
+      </c>
       <c r="H11" s="116" t="n"/>
     </row>
-    <row r="12" ht="81" customHeight="1" s="101">
+    <row r="12" ht="111" customHeight="1" s="101">
       <c r="A12" s="116" t="n"/>
       <c r="B12" s="116" t="n"/>
       <c r="C12" s="113" t="inlineStr">
         <is>
-          <t>支持安全策略绑定安全配置文件组（Profile Group）</t>
+          <t>支持应用默认端口绑定（Service: application-default）</t>
         </is>
       </c>
       <c r="D12" s="113" t="inlineStr">
         <is>
-          <t>PA安全策略Allow动作关联Profile组（反病毒/漏洞防护/URL过滤/文件阻止/WildFire等）；天融信一体化策略引擎自带检测项；迁移评估项：需评估Profile组到天融信各检测引擎的映射与缺省动作差异；对应矩阵#4</t>
+          <t>PA安全策略默认服务为application-default：放行应用同时强制其使用标准端口（如SSH仅22），非标准端口不匹配即拦截（PA管理指南p904）；天融信策略为五元组+应用识别组合（天融信手册《配置访问控制策略》页）；迁移评估项：直接转换若仅保留应用识别不限端口将扩大安全敞口，需制定应用标准端口映射限制（App-Default）转换方案；对应矩阵#2</t>
         </is>
       </c>
       <c r="E12" s="112" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="F12" s="116" t="n"/>
       <c r="G12" s="116" t="n"/>
       <c r="H12" s="116" t="n"/>
     </row>
-    <row r="13" ht="36" customHeight="1" s="101">
+    <row r="13" ht="81" customHeight="1" s="101">
       <c r="A13" s="116" t="n"/>
-      <c r="B13" s="112" t="inlineStr">
-        <is>
-          <t>NAT策略</t>
-        </is>
-      </c>
+      <c r="B13" s="116" t="n"/>
       <c r="C13" s="113" t="inlineStr">
         <is>
-          <t>支持源NAT（动态/PAT静态IP）与Hairpin回流</t>
+          <t>支持安全策略绑定安全配置文件组（Profile Group）</t>
         </is>
       </c>
       <c r="D13" s="113" t="inlineStr">
         <is>
-          <t>PA源NAT含DIPP动态IP+端口/静态IP/接口地址/持久NAT等；对应矩阵#6</t>
+          <t>PA安全策略Allow动作关联Profile组（反病毒/漏洞防护/URL过滤/文件阻止/WildFire等，PA Web帮助p304）；天融信一体化策略引擎自带检测项；迁移评估项：需评估Profile组到天融信各检测引擎的映射与缺省动作差异；对应矩阵#4</t>
         </is>
       </c>
       <c r="E13" s="112" t="inlineStr">
         <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="F13" s="113" t="inlineStr"/>
-      <c r="G13" s="112" t="inlineStr">
-        <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="H13" s="112" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="36" customHeight="1" s="101">
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F13" s="116" t="n"/>
+      <c r="G13" s="116" t="n"/>
+      <c r="H13" s="116" t="n"/>
+    </row>
+    <row r="14" ht="111" customHeight="1" s="101">
       <c r="A14" s="116" t="n"/>
       <c r="B14" s="116" t="n"/>
       <c r="C14" s="113" t="inlineStr">
         <is>
-          <t>支持目的NAT（端口映射/服务器发布）</t>
+          <t>支持隐式默认规则显式化迁移（intrazone/interzone-default）</t>
         </is>
       </c>
       <c r="D14" s="113" t="inlineStr">
         <is>
-          <t>PA目标NAT含静态/动态IP、端口转换、DNS Rewrite、FQDN目标；对应矩阵#7</t>
+          <t>PA安全策略库末尾自带两条隐式系统规则：区域内默认（同Zone默认放行）与区域间默认（跨Zone默认拒绝），可被替代配置（PA Web帮助p134）；天融信未见同区域默认放行的隐式规则机制；迁移评估项：必须提取intrazone-default同Zone互访需求并显式转换为放行规则，否则割接后同Zone不同网段/VLAN互访将被默认拦截</t>
         </is>
       </c>
       <c r="E14" s="112" t="inlineStr">
@@ -3170,113 +3154,117 @@
           <t>高</t>
         </is>
       </c>
-      <c r="F14" s="113" t="inlineStr"/>
-      <c r="G14" s="112" t="inlineStr">
+      <c r="F14" s="116" t="n"/>
+      <c r="G14" s="116" t="n"/>
+      <c r="H14" s="116" t="n"/>
+    </row>
+    <row r="15" ht="51" customHeight="1" s="101">
+      <c r="A15" s="116" t="n"/>
+      <c r="B15" s="112" t="inlineStr">
+        <is>
+          <t>NAT策略</t>
+        </is>
+      </c>
+      <c r="C15" s="113" t="inlineStr">
+        <is>
+          <t>支持源NAT（动态/PAT静态IP）与Hairpin回流</t>
+        </is>
+      </c>
+      <c r="D15" s="113" t="inlineStr">
+        <is>
+          <t>PA源NAT含DIPP动态IP+端口/静态IP/接口地址/持久NAT等（PA Web帮助p147）；对应矩阵#6</t>
+        </is>
+      </c>
+      <c r="E15" s="112" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F15" s="113" t="inlineStr"/>
+      <c r="G15" s="112" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H14" s="112" t="inlineStr"/>
-    </row>
-    <row r="15" ht="36" customHeight="1" s="101">
-      <c r="A15" s="116" t="n"/>
-      <c r="B15" s="116" t="n"/>
-      <c r="C15" s="113" t="inlineStr">
-        <is>
-          <t>支持静态/双向NAT一对一转换</t>
-        </is>
-      </c>
-      <c r="D15" s="113" t="inlineStr">
-        <is>
-          <t>PA支持静态IP转换与双向(Bi-directional)转换；对应矩阵#8</t>
-        </is>
-      </c>
-      <c r="E15" s="116" t="n"/>
-      <c r="F15" s="116" t="n"/>
-      <c r="G15" s="116" t="n"/>
-      <c r="H15" s="116" t="n"/>
-    </row>
-    <row r="16" ht="36" customHeight="1" s="101">
+      <c r="H15" s="112" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="51" customHeight="1" s="101">
       <c r="A16" s="116" t="n"/>
       <c r="B16" s="116" t="n"/>
       <c r="C16" s="113" t="inlineStr">
         <is>
-          <t>支持NAT与安全策略解耦独立配置</t>
+          <t>支持目的NAT（端口映射/服务器发布）</t>
         </is>
       </c>
       <c r="D16" s="113" t="inlineStr">
         <is>
-          <t>PA NAT策略库独立于安全策略库(Policies&gt;NAT)，先NAT后安全匹配；对应矩阵#9</t>
-        </is>
-      </c>
-      <c r="E16" s="116" t="n"/>
-      <c r="F16" s="116" t="n"/>
-      <c r="G16" s="116" t="n"/>
-      <c r="H16" s="116" t="n"/>
+          <t>PA目标NAT含静态/动态IP、端口转换、DNS Rewrite、FQDN目标（PA Web帮助p149）；对应矩阵#7</t>
+        </is>
+      </c>
+      <c r="E16" s="112" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F16" s="113" t="inlineStr"/>
+      <c r="G16" s="112" t="inlineStr">
+        <is>
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="H16" s="112" t="inlineStr"/>
     </row>
     <row r="17" ht="36" customHeight="1" s="101">
       <c r="A17" s="116" t="n"/>
       <c r="B17" s="116" t="n"/>
       <c r="C17" s="113" t="inlineStr">
         <is>
-          <t>支持IPv6/NAT64转换（nat64类型）</t>
+          <t>支持静态/双向NAT一对一转换</t>
         </is>
       </c>
       <c r="D17" s="113" t="inlineStr">
         <is>
-          <t>PA NAT规则支持IPv4/IPv6及NAT64转换类型（RFC6146）；对应矩阵#18</t>
-        </is>
-      </c>
-      <c r="E17" s="112" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
+          <t>PA支持静态IP转换与双向(Bi-directional)转换（PA Web帮助p148）；对应矩阵#8</t>
+        </is>
+      </c>
+      <c r="E17" s="116" t="n"/>
       <c r="F17" s="116" t="n"/>
       <c r="G17" s="116" t="n"/>
       <c r="H17" s="116" t="n"/>
     </row>
-    <row r="18" ht="81" customHeight="1" s="101">
+    <row r="18" ht="36" customHeight="1" s="101">
       <c r="A18" s="116" t="n"/>
       <c r="B18" s="116" t="n"/>
       <c r="C18" s="113" t="inlineStr">
         <is>
-          <t>支持NAT后目的区域路由回查匹配（Dest Zone by route lookup）</t>
+          <t>支持NAT与安全策略解耦独立配置</t>
         </is>
       </c>
       <c r="D18" s="113" t="inlineStr">
         <is>
-          <t>PA NAT策略目的区域按NAT后地址路由回查确定、源区域按NAT前区域；天融信地址转换为独立策略库常规匹配（安全策略&gt;地址转换）[toc398625673]；迁移评估项：Zone/IP匹配计算差异易引发业务不通，需专项评估NAT策略转换映射；对应矩阵#9</t>
-        </is>
-      </c>
-      <c r="E18" s="112" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
+          <t>PA NAT策略库独立于安全策略库(Policies&gt;NAT)，先NAT后安全匹配；对应矩阵#9</t>
+        </is>
+      </c>
+      <c r="E18" s="116" t="n"/>
       <c r="F18" s="116" t="n"/>
-      <c r="G18" s="112" t="inlineStr">
-        <is>
-          <t>待评估</t>
-        </is>
-      </c>
+      <c r="G18" s="116" t="n"/>
       <c r="H18" s="116" t="n"/>
     </row>
-    <row r="19" ht="51" customHeight="1" s="101">
+    <row r="19" ht="36" customHeight="1" s="101">
       <c r="A19" s="116" t="n"/>
-      <c r="B19" s="112" t="inlineStr">
-        <is>
-          <t>QoS策略</t>
-        </is>
-      </c>
+      <c r="B19" s="116" t="n"/>
       <c r="C19" s="113" t="inlineStr">
         <is>
-          <t>支持按应用/源地址/用户等定义QoS策略并划分优先级类</t>
+          <t>支持IPv6/NAT64转换（nat64类型）</t>
         </is>
       </c>
       <c r="D19" s="113" t="inlineStr">
         <is>
-          <t>PA QoS策略规则分配QoS类（8类+4级优先级），按Egress Guaranteed/Max控制带宽；对应矩阵#33/66</t>
+          <t>PA NAT规则支持IPv4/IPv6及NAT64转换类型（RFC6146）；对应矩阵#18</t>
         </is>
       </c>
       <c r="E19" s="112" t="inlineStr">
@@ -3284,64 +3272,56 @@
           <t>中</t>
         </is>
       </c>
-      <c r="F19" s="113" t="inlineStr"/>
-      <c r="G19" s="112" t="inlineStr">
-        <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="H19" s="112" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="96" customHeight="1" s="101">
+      <c r="F19" s="116" t="n"/>
+      <c r="G19" s="116" t="n"/>
+      <c r="H19" s="116" t="n"/>
+    </row>
+    <row r="20" ht="111" customHeight="1" s="101">
       <c r="A20" s="116" t="n"/>
       <c r="B20" s="116" t="n"/>
       <c r="C20" s="113" t="inlineStr">
         <is>
-          <t>支持基于DSCP/ToS值匹配的QoS</t>
+          <t>支持NAT后目的区域路由回查匹配（Dest Zone by route lookup）</t>
         </is>
       </c>
       <c r="D20" s="113" t="inlineStr">
         <is>
-          <t>PA QoS规则可选按DSCP值或IP优先级/ToS匹配；天融信有流量管理模块（虚拟通道+限制/保证带宽+每IP/每用户限速+通道优先级，匹配维度为应用/用户/区域/地址/服务/时间[toc450050609]），DSCP/CoS识别与重标记在现有NGFW手册未见（ACM产品/新版手册待补证）</t>
+          <t>PA底层为『先NAT判断后安全策略匹配』的因果倒置：安全策略要求源区域(NAT前)+源地址(NAT前)+目的地址(NAT前)+目的区域(NAT后按路由查找)，极其反直觉；天融信地址转换为独立策略库常规直观映射（安全策略&gt;地址转换，天融信手册《服务器映射》页）；迁移评估项：带目的NAT的策略平移后易因Zone填写错误不通，需制定NAT查表逻辑转换映射规范；对应矩阵#9</t>
         </is>
       </c>
       <c r="E20" s="112" t="inlineStr">
         <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="F20" s="113" t="inlineStr"/>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F20" s="116" t="n"/>
       <c r="G20" s="112" t="inlineStr">
         <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="H20" s="112" t="inlineStr"/>
-    </row>
-    <row r="21" ht="36" customHeight="1" s="101">
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="H20" s="116" t="n"/>
+    </row>
+    <row r="21" ht="66" customHeight="1" s="101">
       <c r="A21" s="116" t="n"/>
       <c r="B21" s="112" t="inlineStr">
         <is>
-          <t>基于策略转发(PBF)</t>
+          <t>QoS策略</t>
         </is>
       </c>
       <c r="C21" s="113" t="inlineStr">
         <is>
-          <t>支持按源区域/地址/用户/应用/服务+下一跳的基于策略转发</t>
+          <t>支持按应用/源地址/用户等定义QoS策略并划分优先级类</t>
         </is>
       </c>
       <c r="D21" s="113" t="inlineStr">
         <is>
-          <t>PA PBF策略绕过常规路由表选路，支持路径监控与失效切换、BFD、强制对称返回；对应矩阵#10</t>
+          <t>PA QoS策略规则分配QoS类（8类+4级优先级），按Egress Guaranteed/Max控制带宽（PA Web帮助p154-155）；对应矩阵#33/66</t>
         </is>
       </c>
       <c r="E21" s="112" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="F21" s="113" t="inlineStr"/>
@@ -3356,28 +3336,28 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="36" customHeight="1" s="101">
+    <row r="22" ht="96" customHeight="1" s="101">
       <c r="A22" s="116" t="n"/>
       <c r="B22" s="116" t="n"/>
       <c r="C22" s="113" t="inlineStr">
         <is>
-          <t>支持PBF强制对称返回（非对称路由环境）</t>
+          <t>支持基于DSCP/ToS值匹配的QoS</t>
         </is>
       </c>
       <c r="D22" s="113" t="inlineStr">
         <is>
-          <t>PA Enforce Symmetric Return确保返回流量对称</t>
+          <t>PA QoS规则可直接按DSCP值或IP优先级/ToS匹配调度（PA Web帮助p155）；天融信支持DSCP/802.1p(CoS)识别与重标记，但需在独立流量管理模块配置（虚拟通道+限制/保证带宽+通道优先级，天融信手册《流量管理》页），未直接耦合在基础访问控制策略表内（联网核实厂商流控资料，手册未详载）</t>
         </is>
       </c>
       <c r="E22" s="112" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="F22" s="113" t="inlineStr"/>
       <c r="G22" s="112" t="inlineStr">
         <is>
-          <t>已支持</t>
+          <t>部分支持</t>
         </is>
       </c>
       <c r="H22" s="112" t="inlineStr"/>
@@ -3386,17 +3366,17 @@
       <c r="A23" s="116" t="n"/>
       <c r="B23" s="112" t="inlineStr">
         <is>
-          <t>解密策略(Decryption)</t>
+          <t>基于策略转发(PBF)</t>
         </is>
       </c>
       <c r="C23" s="113" t="inlineStr">
         <is>
-          <t>支持SSL/TLS解密策略（出站正向/入站反向）</t>
+          <t>支持按源区域/地址/用户/应用/服务+下一跳的基于策略转发</t>
         </is>
       </c>
       <c r="D23" s="113" t="inlineStr">
         <is>
-          <t>PA解密策略区分SSL Forward Proxy/Inbound Inspection/SSH，可解密以获得流量可见性与深度检测；对应矩阵#29/30</t>
+          <t>PA PBF策略绕过常规路由表选路，支持路径监控与失效切换、BFD、强制对称返回（PA Web帮助p156）；对应矩阵#10</t>
         </is>
       </c>
       <c r="E23" s="112" t="inlineStr">
@@ -3421,12 +3401,12 @@
       <c r="B24" s="116" t="n"/>
       <c r="C24" s="113" t="inlineStr">
         <is>
-          <t>支持解密目标选择与证书配置</t>
+          <t>支持PBF强制对称返回（非对称路由环境）</t>
         </is>
       </c>
       <c r="D24" s="113" t="inlineStr">
         <is>
-          <t>PA解密目标允许指定数据包/会话；入站含Certificates证书配置；对应矩阵#31</t>
+          <t>PA Enforce Symmetric Return确保返回流量对称（PA管理指南p1294）</t>
         </is>
       </c>
       <c r="E24" s="112" t="inlineStr">
@@ -3442,103 +3422,99 @@
       </c>
       <c r="H24" s="112" t="inlineStr"/>
     </row>
-    <row r="25" ht="51" customHeight="1" s="101">
+    <row r="25" ht="66" customHeight="1" s="101">
       <c r="A25" s="116" t="n"/>
-      <c r="B25" s="116" t="n"/>
+      <c r="B25" s="112" t="inlineStr">
+        <is>
+          <t>解密策略(Decryption)</t>
+        </is>
+      </c>
       <c r="C25" s="113" t="inlineStr">
         <is>
-          <t>支持解密流量镜像到专用接口（Decryption Port Mirroring）</t>
+          <t>支持SSL/TLS解密策略（出站正向/入站反向）</t>
         </is>
       </c>
       <c r="D25" s="113" t="inlineStr">
         <is>
-          <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
-        </is>
-      </c>
-      <c r="E25" s="116" t="n"/>
-      <c r="F25" s="116" t="n"/>
+          <t>PA解密策略区分SSL Forward Proxy/Inbound Inspection/SSH，可解密以获得流量可见性与深度检测（PA Web帮助p164）；对应矩阵#29/30</t>
+        </is>
+      </c>
+      <c r="E25" s="112" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F25" s="113" t="inlineStr"/>
       <c r="G25" s="112" t="inlineStr">
         <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="H25" s="116" t="n"/>
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="H25" s="112" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="36" customHeight="1" s="101">
       <c r="A26" s="116" t="n"/>
-      <c r="B26" s="112" t="inlineStr">
-        <is>
-          <t>网络数据包代理(NPBroker)</t>
-        </is>
-      </c>
+      <c r="B26" s="116" t="n"/>
       <c r="C26" s="113" t="inlineStr">
         <is>
-          <t>支持按应用/用户/区域/设备/IP定义NPBroker规则转发到第三方安全链</t>
+          <t>支持解密目标选择与证书配置</t>
         </is>
       </c>
       <c r="D26" s="113" t="inlineStr">
         <is>
-          <t>PA网络数据包代理策略将已解密/未解密TLS/非TLS流量内联转发至第三方安全工具；对应矩阵#122</t>
+          <t>PA解密目标允许指定数据包/会话；入站含Certificates证书配置；对应矩阵#31</t>
         </is>
       </c>
       <c r="E26" s="112" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="F26" s="113" t="inlineStr"/>
       <c r="G26" s="112" t="inlineStr">
         <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="H26" s="112" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="H26" s="112" t="inlineStr"/>
     </row>
     <row r="27" ht="51" customHeight="1" s="101">
       <c r="A27" s="116" t="n"/>
       <c r="B27" s="116" t="n"/>
       <c r="C27" s="113" t="inlineStr">
         <is>
-          <t>支持NPBroker转发流量类型选择（TLS解密/未解密/非TLS）</t>
+          <t>支持解密流量镜像到专用接口（Decryption Port Mirroring）</t>
         </is>
       </c>
       <c r="D27" s="113" t="inlineStr">
         <is>
-          <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证；天融信无网络数据包代理模块（矩阵#122）</t>
-        </is>
-      </c>
-      <c r="E27" s="112" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="F27" s="113" t="inlineStr"/>
+          <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证（PA管理指南p1059）；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
+        </is>
+      </c>
+      <c r="E27" s="116" t="n"/>
+      <c r="F27" s="116" t="n"/>
       <c r="G27" s="112" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H27" s="112" t="inlineStr"/>
-    </row>
-    <row r="28" ht="36" customHeight="1" s="101">
+      <c r="H27" s="116" t="n"/>
+    </row>
+    <row r="28" ht="126" customHeight="1" s="101">
       <c r="A28" s="116" t="n"/>
-      <c r="B28" s="112" t="inlineStr">
-        <is>
-          <t>隧道检测(Tunnel Inspection)</t>
-        </is>
-      </c>
+      <c r="B28" s="116" t="n"/>
       <c r="C28" s="113" t="inlineStr">
         <is>
-          <t>支持GRE/GTP-U/HTTP2等明文隧道内层流量检测</t>
+          <t>支持解密不受信证书分离处理（Forward Untrust Certificate）</t>
         </is>
       </c>
       <c r="D28" s="113" t="inlineStr">
         <is>
-          <t>PA隧道检测策略解封装并深度检测GRE/GTP-U/HTTP2等明文隧道内容；对应矩阵#128/37</t>
+          <t>PA转发代理遇外部过期/不受信证书时，不用内部信任CA重签，而是专用Forward Untrust Certificate重签名，让浏览器保留不受信告警（PA管理指南p994、p1030）；天融信SSL解密（透明代理/服务器SSL解密，天融信手册《代理策略》页）未见受信/不受信双证书体系；迁移评估项：需验证天融信对外部无效证书的处理方式，避免直接阻断（白屏）或信任重签（掩盖风险）</t>
         </is>
       </c>
       <c r="E28" s="112" t="inlineStr">
@@ -3546,59 +3522,59 @@
           <t>高</t>
         </is>
       </c>
-      <c r="F28" s="113" t="inlineStr"/>
+      <c r="F28" s="116" t="n"/>
       <c r="G28" s="112" t="inlineStr">
         <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="H28" s="112" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="36" customHeight="1" s="101">
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="H28" s="116" t="n"/>
+    </row>
+    <row r="29" ht="51" customHeight="1" s="101">
       <c r="A29" s="116" t="n"/>
-      <c r="B29" s="116" t="n"/>
+      <c r="B29" s="112" t="inlineStr">
+        <is>
+          <t>网络数据包代理(NPBroker)</t>
+        </is>
+      </c>
       <c r="C29" s="113" t="inlineStr">
         <is>
-          <t>支持最大封装级数防护（max_encap）</t>
+          <t>支持按应用/用户/区域/设备/IP定义NPBroker规则转发到第三方安全链</t>
         </is>
       </c>
       <c r="D29" s="113" t="inlineStr">
         <is>
-          <t>PA对隧道最大封装级数超限丢包防护，防隧道嵌套绕过；天融信手册无封装级数防护（检索无命中）</t>
+          <t>PA网络数据包代理策略将已解密/未解密TLS/非TLS流量内联转发至第三方安全工具（PA Web帮助p167）；对应矩阵#122</t>
         </is>
       </c>
       <c r="E29" s="112" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="F29" s="113" t="inlineStr"/>
       <c r="G29" s="112" t="inlineStr">
         <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="H29" s="112" t="inlineStr"/>
-    </row>
-    <row r="30" ht="36" customHeight="1" s="101">
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="H29" s="112" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="66" customHeight="1" s="101">
       <c r="A30" s="116" t="n"/>
-      <c r="B30" s="112" t="inlineStr">
-        <is>
-          <t>应用覆盖(App Override)</t>
-        </is>
-      </c>
+      <c r="B30" s="116" t="n"/>
       <c r="C30" s="113" t="inlineStr">
         <is>
-          <t>支持通过Application Override重定义应用识别</t>
+          <t>支持NPBroker转发流量类型选择（TLS解密/未解密/非TLS）</t>
         </is>
       </c>
       <c r="D30" s="113" t="inlineStr">
         <is>
-          <t>PA应用替代策略改变防火墙对网络通信的应用分类方式（如指定明文协议/端口识别）；对应矩阵#26</t>
+          <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证（PA Web帮助p167）；天融信无网络数据包代理模块（矩阵#122）</t>
         </is>
       </c>
       <c r="E30" s="112" t="inlineStr">
@@ -3609,86 +3585,86 @@
       <c r="F30" s="113" t="inlineStr"/>
       <c r="G30" s="112" t="inlineStr">
         <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="H30" s="112" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="36" customHeight="1" s="101">
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="H30" s="112" t="inlineStr"/>
+    </row>
+    <row r="31" ht="51" customHeight="1" s="101">
       <c r="A31" s="116" t="n"/>
-      <c r="B31" s="116" t="n"/>
+      <c r="B31" s="112" t="inlineStr">
+        <is>
+          <t>隧道检测(Tunnel Inspection)</t>
+        </is>
+      </c>
       <c r="C31" s="113" t="inlineStr">
         <is>
-          <t>支持覆盖类型（端口映射类）识别</t>
+          <t>支持GRE/GTP-U/HTTP2等明文隧道内层流量检测</t>
         </is>
       </c>
       <c r="D31" s="113" t="inlineStr">
         <is>
-          <t>PA支持端口式应用覆盖识别（configurable自定义应用）</t>
+          <t>PA隧道检测策略解封装并深度检测GRE/GTP-U/HTTP2等明文隧道内容（PA Web帮助p172-173）；对应矩阵#128/37</t>
         </is>
       </c>
       <c r="E31" s="112" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>高</t>
         </is>
       </c>
       <c r="F31" s="113" t="inlineStr"/>
       <c r="G31" s="112" t="inlineStr">
         <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="H31" s="112" t="inlineStr"/>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="H31" s="112" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="51" customHeight="1" s="101">
       <c r="A32" s="116" t="n"/>
-      <c r="B32" s="112" t="inlineStr">
-        <is>
-          <t>身份验证(Authentication)</t>
-        </is>
-      </c>
+      <c r="B32" s="116" t="n"/>
       <c r="C32" s="113" t="inlineStr">
         <is>
-          <t>支持基于用户身份的身份验证策略（User-ID）</t>
+          <t>支持最大封装级数防护（max_encap）</t>
         </is>
       </c>
       <c r="D32" s="113" t="inlineStr">
         <is>
-          <t>PA身份验证策略在访问网络资源前对用户鉴权，配合User-ID多源映射（AD/XML/Syslog等）；对应矩阵#3/35</t>
+          <t>PA对隧道最大封装级数超限丢包防护，防隧道嵌套绕过（PA管理指南p655）；天融信手册无封装级数防护（检索无命中）</t>
         </is>
       </c>
       <c r="E32" s="112" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="F32" s="113" t="inlineStr"/>
       <c r="G32" s="112" t="inlineStr">
         <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="H32" s="112" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="36" customHeight="1" s="101">
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="H32" s="112" t="inlineStr"/>
+    </row>
+    <row r="33" ht="51" customHeight="1" s="101">
       <c r="A33" s="116" t="n"/>
-      <c r="B33" s="116" t="n"/>
+      <c r="B33" s="112" t="inlineStr">
+        <is>
+          <t>应用覆盖(App Override)</t>
+        </is>
+      </c>
       <c r="C33" s="113" t="inlineStr">
         <is>
-          <t>支持认证策略超时与单次认证（SSO）</t>
+          <t>支持通过Application Override重定义应用识别</t>
         </is>
       </c>
       <c r="D33" s="113" t="inlineStr">
         <is>
-          <t>PA支持认证超时减少重复质询、Kerberos/SAML/RADIUS等对接</t>
+          <t>PA应用替代策略改变防火墙对网络通信的应用分类方式（如指定明文协议/端口识别，PA Web帮助p178）；对应矩阵#26</t>
         </is>
       </c>
       <c r="E33" s="112" t="inlineStr">
@@ -3702,28 +3678,28 @@
           <t>已支持</t>
         </is>
       </c>
-      <c r="H33" s="112" t="inlineStr"/>
-    </row>
-    <row r="34" ht="51" customHeight="1" s="101">
+      <c r="H33" s="112" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="36" customHeight="1" s="101">
       <c r="A34" s="116" t="n"/>
-      <c r="B34" s="112" t="inlineStr">
-        <is>
-          <t>DoS防护(DoS Protection)</t>
-        </is>
-      </c>
+      <c r="B34" s="116" t="n"/>
       <c r="C34" s="113" t="inlineStr">
         <is>
-          <t>支持针对关键资源的分类/聚合DoS防护</t>
+          <t>支持覆盖类型（端口映射类）识别</t>
         </is>
       </c>
       <c r="D34" s="113" t="inlineStr">
         <is>
-          <t>PA DoS策略基于源/目的接口、区域、地址、服务定义允许/拒绝/告警，含分类与聚合双层阈值配置文件；对应矩阵#52/42</t>
+          <t>PA支持端口式应用覆盖识别（configurable自定义应用）</t>
         </is>
       </c>
       <c r="E34" s="112" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>低</t>
         </is>
       </c>
       <c r="F34" s="113" t="inlineStr"/>
@@ -3732,53 +3708,49 @@
           <t>已支持</t>
         </is>
       </c>
-      <c r="H34" s="112" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="36" customHeight="1" s="101">
+      <c r="H34" s="112" t="inlineStr"/>
+    </row>
+    <row r="35" ht="96" customHeight="1" s="101">
       <c r="A35" s="116" t="n"/>
       <c r="B35" s="116" t="n"/>
       <c r="C35" s="113" t="inlineStr">
         <is>
-          <t>支持DoS聚合配置文件（连接/秒阈值）</t>
+          <t>支持应用替代流量跳过七层检测等效配置</t>
         </is>
       </c>
       <c r="D35" s="113" t="inlineStr">
         <is>
-          <t>PA聚合DoS配置文件按传入连接数/秒触发告警与最大速率限制</t>
+          <t>PA应用替代策略明确绕过第7层处理与威胁检查，改用第4层状态检查以加速（PA管理指南p1307）；天融信自定义应用加入规则库后仍默认经安全引擎检测（天融信手册《自定义应用》页）；迁移评估项：PA应用替代多为私有大流量业务加速，转换时需同步关闭对应策略的IPS/七层检测，否则性能被拖垮或误阻断</t>
         </is>
       </c>
       <c r="E35" s="112" t="inlineStr">
         <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="F35" s="113" t="inlineStr"/>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F35" s="116" t="n"/>
       <c r="G35" s="112" t="inlineStr">
         <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="H35" s="112" t="inlineStr"/>
-    </row>
-    <row r="36" ht="36" customHeight="1" s="101">
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="H35" s="116" t="n"/>
+    </row>
+    <row r="36" ht="51" customHeight="1" s="101">
       <c r="A36" s="116" t="n"/>
       <c r="B36" s="112" t="inlineStr">
         <is>
-          <t>SD-WAN策略</t>
+          <t>身份验证(Authentication)</t>
         </is>
       </c>
       <c r="C36" s="113" t="inlineStr">
         <is>
-          <t>支持按应用配置链路路径管理与链路质量探测</t>
+          <t>支持基于用户身份的身份验证策略（User-ID）</t>
         </is>
       </c>
       <c r="D36" s="113" t="inlineStr">
         <is>
-          <t>PA SD-WAN策略按应用/抖动/延迟/丢包指标分配链路，流量分发；对应矩阵#129/120</t>
+          <t>PA身份验证策略在访问网络资源前对用户鉴权（PA Web帮助p182），配合User-ID多源映射（AD/XML/Syslog等）；对应矩阵#3/35</t>
         </is>
       </c>
       <c r="E36" s="112" t="inlineStr">
@@ -3789,7 +3761,7 @@
       <c r="F36" s="113" t="inlineStr"/>
       <c r="G36" s="112" t="inlineStr">
         <is>
-          <t>部分支持</t>
+          <t>已支持</t>
         </is>
       </c>
       <c r="H36" s="112" t="inlineStr">
@@ -3798,17 +3770,17 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="66" customHeight="1" s="101">
+    <row r="37" ht="36" customHeight="1" s="101">
       <c r="A37" s="116" t="n"/>
       <c r="B37" s="116" t="n"/>
       <c r="C37" s="113" t="inlineStr">
         <is>
-          <t>支持SD-WAN路径选择与链路质量监测（jitter/latency/loss）</t>
+          <t>支持认证策略超时与单次认证（SSO）</t>
         </is>
       </c>
       <c r="D37" s="113" t="inlineStr">
         <is>
-          <t>PA路径质量配置文件基于抖动/延迟/丢包等运行状况指标选路；天融信有链路探测(ping)+智能选路(最小延迟优先)[toc490041605]，无jitter/latency/loss多维指标</t>
+          <t>PA支持认证超时减少重复质询、Kerberos/SAML/RADIUS等对接</t>
         </is>
       </c>
       <c r="E37" s="112" t="inlineStr">
@@ -3819,41 +3791,189 @@
       <c r="F37" s="113" t="inlineStr"/>
       <c r="G37" s="112" t="inlineStr">
         <is>
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="H37" s="112" t="inlineStr"/>
+    </row>
+    <row r="38" ht="81" customHeight="1" s="101">
+      <c r="A38" s="116" t="n"/>
+      <c r="B38" s="116" t="n"/>
+      <c r="C38" s="113" t="inlineStr">
+        <is>
+          <t>支持User-ID动态映射时效性等效（AD日志毫秒级更新）</t>
+        </is>
+      </c>
+      <c r="D38" s="113" t="inlineStr">
+        <is>
+          <t>PA无代理架构通过读取域控事件日志实现IP-用户毫秒级动态映射，大规模部署有专项规划（PA管理指南p866-867）；天融信AD对接的轮询间隔与并发认证能力手册未量化；迁移评估项：数万AD用户且移动频繁场景需实测天融信映射更新时延，避免基于用户的策略出现间歇性未授权拦截</t>
+        </is>
+      </c>
+      <c r="E38" s="116" t="n"/>
+      <c r="F38" s="116" t="n"/>
+      <c r="G38" s="112" t="inlineStr">
+        <is>
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="H38" s="116" t="n"/>
+    </row>
+    <row r="39" ht="51" customHeight="1" s="101">
+      <c r="A39" s="116" t="n"/>
+      <c r="B39" s="112" t="inlineStr">
+        <is>
+          <t>DoS防护(DoS Protection)</t>
+        </is>
+      </c>
+      <c r="C39" s="113" t="inlineStr">
+        <is>
+          <t>支持针对关键资源的分类/聚合DoS防护</t>
+        </is>
+      </c>
+      <c r="D39" s="113" t="inlineStr">
+        <is>
+          <t>PA DoS策略基于源/目的接口、区域、地址、服务定义允许/拒绝/告警，含分类与聚合双层阈值配置文件（PA管理指南p1354）；对应矩阵#52/42</t>
+        </is>
+      </c>
+      <c r="E39" s="112" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F39" s="113" t="inlineStr"/>
+      <c r="G39" s="112" t="inlineStr">
+        <is>
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="H39" s="112" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="36" customHeight="1" s="101">
+      <c r="A40" s="116" t="n"/>
+      <c r="B40" s="116" t="n"/>
+      <c r="C40" s="113" t="inlineStr">
+        <is>
+          <t>支持DoS聚合配置文件（连接/秒阈值）</t>
+        </is>
+      </c>
+      <c r="D40" s="113" t="inlineStr">
+        <is>
+          <t>PA聚合DoS配置文件按传入连接数/秒触发告警与最大速率限制</t>
+        </is>
+      </c>
+      <c r="E40" s="112" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F40" s="113" t="inlineStr"/>
+      <c r="G40" s="112" t="inlineStr">
+        <is>
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="H40" s="112" t="inlineStr"/>
+    </row>
+    <row r="41" ht="51" customHeight="1" s="101">
+      <c r="A41" s="116" t="n"/>
+      <c r="B41" s="112" t="inlineStr">
+        <is>
+          <t>SD-WAN策略</t>
+        </is>
+      </c>
+      <c r="C41" s="113" t="inlineStr">
+        <is>
+          <t>支持按应用配置链路路径管理与链路质量探测</t>
+        </is>
+      </c>
+      <c r="D41" s="113" t="inlineStr">
+        <is>
+          <t>PA SD-WAN策略按应用/抖动/延迟/丢包指标分配链路，流量分发（PA Web帮助p197）；对应矩阵#129/120</t>
+        </is>
+      </c>
+      <c r="E41" s="112" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F41" s="113" t="inlineStr"/>
+      <c r="G41" s="112" t="inlineStr">
+        <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H37" s="112" t="inlineStr"/>
+      <c r="H41" s="112" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="81" customHeight="1" s="101">
+      <c r="A42" s="116" t="n"/>
+      <c r="B42" s="116" t="n"/>
+      <c r="C42" s="113" t="inlineStr">
+        <is>
+          <t>支持SD-WAN路径选择与链路质量监测（jitter/latency/loss）</t>
+        </is>
+      </c>
+      <c r="D42" s="113" t="inlineStr">
+        <is>
+          <t>PA路径质量配置文件基于抖动/延迟/丢包等运行状况指标选路（PA Web帮助p195）；天融信有链路探测(ping)+智能选路(最小延迟优先)（天融信手册《策略路由》页），无jitter/latency/loss多维指标</t>
+        </is>
+      </c>
+      <c r="E42" s="112" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F42" s="113" t="inlineStr"/>
+      <c r="G42" s="112" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="H42" s="112" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="A2:A37"/>
-    <mergeCell ref="B7:B12"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="F3:F6"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="H14:H18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="H8:H12"/>
-    <mergeCell ref="G14:G17"/>
-    <mergeCell ref="B13:B18"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="H24:H25"/>
-    <mergeCell ref="B2:B6"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="G10:G12"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="H3:H6"/>
-    <mergeCell ref="F8:F12"/>
-    <mergeCell ref="E3:E6"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="E24:E25"/>
+  <mergeCells count="34">
+    <mergeCell ref="H3:H7"/>
+    <mergeCell ref="H16:H20"/>
+    <mergeCell ref="B33:B35"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="H34:H35"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="H9:H14"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="B2:B7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="E3:E7"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="H37:H38"/>
+    <mergeCell ref="F3:F7"/>
+    <mergeCell ref="B15:B20"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="F16:F20"/>
+    <mergeCell ref="F26:F28"/>
+    <mergeCell ref="A2:A42"/>
+    <mergeCell ref="F9:F14"/>
+    <mergeCell ref="B8:B14"/>
+    <mergeCell ref="G16:G19"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="F34:F35"/>
     <mergeCell ref="B21:B22"/>
-    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="G11:G14"/>
+    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor(scripts): update excel sheet handling and strategy sheet data
1. update filter and add strategy scripts to support 9-column sheet with new comparison column
2. adjust column indices, headers, widths and cell formatting
3. update data model comments and row content for better clarity
4. fix status index reference in logging
5. simplify merge range printing output
</commit_message>
<xml_diff>
--- a/PA替代需求列表.xlsx
+++ b/PA替代需求列表.xlsx
@@ -3279,17 +3279,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.7" customWidth="1" style="1" min="1" max="1"/>
     <col width="19.7" customWidth="1" style="1" min="2" max="2"/>
-    <col width="48" customWidth="1" style="1" min="3" max="3"/>
-    <col width="55" customWidth="1" style="1" min="4" max="4"/>
-    <col width="7.7" customWidth="1" style="1" min="5" max="5"/>
-    <col width="20" customWidth="1" style="1" min="6" max="6"/>
-    <col width="12" customWidth="1" style="1" min="7" max="7"/>
-    <col width="9.699999999999999" customWidth="1" style="1" min="8" max="8"/>
+    <col width="40" customWidth="1" style="1" min="3" max="3"/>
+    <col width="30" customWidth="1" style="1" min="4" max="4"/>
+    <col width="62" customWidth="1" style="1" min="5" max="5"/>
+    <col width="7.7" customWidth="1" style="1" min="6" max="6"/>
+    <col width="18" customWidth="1" style="1" min="7" max="7"/>
+    <col width="10" customWidth="1" style="1" min="8" max="8"/>
+    <col width="9.699999999999999" customWidth="1" style="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" s="1">
@@ -3315,26 +3316,31 @@
       </c>
       <c r="E1" s="79" t="inlineStr">
         <is>
+          <t>对比依据（PA证据·天融信现状）</t>
+        </is>
+      </c>
+      <c r="F1" s="79" t="inlineStr">
+        <is>
           <t>优先级</t>
         </is>
       </c>
-      <c r="F1" s="79" t="inlineStr">
+      <c r="G1" s="79" t="inlineStr">
         <is>
           <t>交付/规划说明</t>
         </is>
       </c>
-      <c r="G1" s="79" t="inlineStr">
+      <c r="H1" s="79" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="H1" s="79" t="inlineStr">
+      <c r="I1" s="79" t="inlineStr">
         <is>
           <t>负责人</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="96" customHeight="1" s="1">
+    <row r="2" ht="111" customHeight="1" s="1">
       <c r="A2" s="80" t="inlineStr">
         <is>
           <t>策略</t>
@@ -3352,21 +3358,26 @@
       </c>
       <c r="D2" s="81" t="inlineStr">
         <is>
+          <t>安全/NAT/QoS/PBF/解密/隧道/应用覆盖/认证/DoS/SD-WAN各自独立策略库</t>
+        </is>
+      </c>
+      <c r="E2" s="81" t="inlineStr">
+        <is>
           <t>PA Web界面『策略』章节定义多种策略类型，按用途各自独立配置（PA Web帮助p113起）；天融信策略库按用途划分：访问控制策略/地址转换策略/流量管理/策略路由/代理策略各自独立（天融信手册《安全策略》《源NAT》《流量管理》《策略路由》《代理策略》页）；对应功能矩阵#2-9/33/52/122/128/129</t>
         </is>
       </c>
-      <c r="E2" s="80" t="inlineStr">
+      <c r="F2" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F2" s="81" t="inlineStr"/>
-      <c r="G2" s="80" t="inlineStr">
+      <c r="G2" s="81" t="inlineStr"/>
+      <c r="H2" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H2" s="80" t="inlineStr">
+      <c r="I2" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
@@ -3382,21 +3393,26 @@
       </c>
       <c r="D3" s="81" t="inlineStr">
         <is>
+          <t>策略可移动调整顺序、克隆复制，支持跨虚拟系统/设备组</t>
+        </is>
+      </c>
+      <c r="E3" s="81" t="inlineStr">
+        <is>
           <t>PA支持将策略规则移动/克隆到虚拟系统或Panorama设备组（含共享位置，PA Web帮助p115）；天融信访问控制策略支持移动策略与克隆模板（天融信手册《配置访问控制策略》页）</t>
         </is>
       </c>
-      <c r="E3" s="80" t="inlineStr">
+      <c r="F3" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F3" s="81" t="inlineStr"/>
-      <c r="G3" s="80" t="inlineStr">
+      <c r="G3" s="81" t="inlineStr"/>
+      <c r="H3" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H3" s="80" t="inlineStr"/>
+      <c r="I3" s="80" t="inlineStr"/>
     </row>
     <row r="4" ht="51" customHeight="1" s="1">
       <c r="A4" s="84" t="n"/>
@@ -3408,19 +3424,24 @@
       </c>
       <c r="D4" s="81" t="inlineStr">
         <is>
+          <t>提交/修改策略须填写审核注释并留存历史，可导出</t>
+        </is>
+      </c>
+      <c r="E4" s="81" t="inlineStr">
+        <is>
           <t>PA记录规则的审核注释历史/配置日志/规则更改历史，可CSV导出，用于策略变更审计（PA Web帮助p116-117）；天融信仅规则描述字段，无审核注释存档</t>
         </is>
       </c>
-      <c r="E4" s="84" t="n"/>
       <c r="F4" s="84" t="n"/>
-      <c r="G4" s="80" t="inlineStr">
+      <c r="G4" s="84" t="n"/>
+      <c r="H4" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H4" s="84" t="n"/>
-    </row>
-    <row r="5" ht="66" customHeight="1" s="1">
+      <c r="I4" s="84" t="n"/>
+    </row>
+    <row r="5" ht="81" customHeight="1" s="1">
       <c r="A5" s="84" t="n"/>
       <c r="B5" s="84" t="n"/>
       <c r="C5" s="81" t="inlineStr">
@@ -3430,17 +3451,22 @@
       </c>
       <c r="D5" s="81" t="inlineStr">
         <is>
+          <t>按时间段统计规则命中次数，识别未使用规则</t>
+        </is>
+      </c>
+      <c r="E5" s="81" t="inlineStr">
+        <is>
           <t>PA支持按时间段查询规则命中数，标识未使用规则以清理；含Reset Rule Hit Count重置功能（PA Web帮助p118-119）；天融信策略统计开关可显示规则匹配情况（天融信手册《配置访问控制策略》页）</t>
         </is>
       </c>
-      <c r="E5" s="84" t="n"/>
       <c r="F5" s="84" t="n"/>
-      <c r="G5" s="80" t="inlineStr">
+      <c r="G5" s="84" t="n"/>
+      <c r="H5" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H5" s="84" t="n"/>
+      <c r="I5" s="84" t="n"/>
     </row>
     <row r="6" ht="111" customHeight="1" s="1">
       <c r="A6" s="84" t="n"/>
@@ -3452,17 +3478,22 @@
       </c>
       <c r="D6" s="81" t="inlineStr">
         <is>
+          <t>前置规则→本地规则→后置规则三层按序合并为单层规则链</t>
+        </is>
+      </c>
+      <c r="E6" s="81" t="inlineStr">
+        <is>
           <t>PA在Panorama集中管理下策略分为前置规则（设备组共享，最优先）/本地规则/后置规则三层按序匹配（层级机制属Panorama管理平台，PA两册手册未详载）；天融信为自上而下单层规则链一张表走到底（天融信手册《配置访问控制策略》页）；迁移评估项：需制定全局多级策略到单层扁平化策略的合并清洗规则（Pre→本地→Post按序展开映射）</t>
         </is>
       </c>
-      <c r="E6" s="84" t="n"/>
       <c r="F6" s="84" t="n"/>
-      <c r="G6" s="80" t="inlineStr">
+      <c r="G6" s="84" t="n"/>
+      <c r="H6" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H6" s="84" t="n"/>
+      <c r="I6" s="84" t="n"/>
     </row>
     <row r="7" ht="96" customHeight="1" s="1">
       <c r="A7" s="84" t="n"/>
@@ -3474,13 +3505,18 @@
       </c>
       <c r="D7" s="81" t="inlineStr">
         <is>
+          <t>应用程序对象级会话超时，覆盖全局TCP/UDP超时</t>
+        </is>
+      </c>
+      <c r="E7" s="81" t="inlineStr">
+        <is>
           <t>PA除全局TCP/UDP会话超时外，可在应用程序对象上定义专用超时，匹配该应用的流量覆盖全局值（PA Web帮助p215、p695）；天融信手册未见应用级超时覆盖（仅SSLVPN会话超时设置与黑名单老化）；迁移评估项：需排查现网PA为数据库/长连接业务单独配置的应用超时并逐条转换，否则长连接业务频繁中断</t>
         </is>
       </c>
-      <c r="E7" s="85" t="n"/>
       <c r="F7" s="85" t="n"/>
       <c r="G7" s="85" t="n"/>
       <c r="H7" s="85" t="n"/>
+      <c r="I7" s="85" t="n"/>
     </row>
     <row r="8" ht="81" customHeight="1" s="1">
       <c r="A8" s="84" t="n"/>
@@ -3496,27 +3532,32 @@
       </c>
       <c r="D8" s="81" t="inlineStr">
         <is>
+          <t>源/目的区域+地址+用户/用户组+服务+应用+时间多维匹配</t>
+        </is>
+      </c>
+      <c r="E8" s="81" t="inlineStr">
+        <is>
           <t>PA安全策略规则基于App-ID应用、用户(User-ID)、区域地址、服务多维匹配并允许/拒绝/跟踪流量；天融信访问控制策略匹配条件含源/目的区域、地址、用户、服务、应用、时间、域名（天融信手册《配置访问控制策略》页）；对应矩阵#2/3/4</t>
         </is>
       </c>
-      <c r="E8" s="80" t="inlineStr">
+      <c r="F8" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F8" s="81" t="inlineStr"/>
-      <c r="G8" s="80" t="inlineStr">
+      <c r="G8" s="81" t="inlineStr"/>
+      <c r="H8" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H8" s="80" t="inlineStr">
+      <c r="I8" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="81" customHeight="1" s="1">
+    <row r="9" ht="96" customHeight="1" s="1">
       <c r="A9" s="84" t="n"/>
       <c r="B9" s="84" t="n"/>
       <c r="C9" s="81" t="inlineStr">
@@ -3526,21 +3567,26 @@
       </c>
       <c r="D9" s="81" t="inlineStr">
         <is>
+          <t>预登录用户/HIP主机信息/设备对象/应用默认端口规避/会话结束日志等构建块</t>
+        </is>
+      </c>
+      <c r="E9" s="81" t="inlineStr">
+        <is>
           <t>PA规则构建块含预登录用户、HIP配置文件、设备对象、应用默认端口规避、会话结束日志等；天融信支持用户/应用/服务/日志构建块，但无HIP主机信息配置文件与设备对象等价物，仅有EDR联动上报终端资产并下发管控策略（天融信手册《与EDR联动》页）；对应矩阵#3/4</t>
         </is>
       </c>
-      <c r="E9" s="80" t="inlineStr">
+      <c r="F9" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F9" s="81" t="inlineStr"/>
-      <c r="G9" s="80" t="inlineStr">
+      <c r="G9" s="81" t="inlineStr"/>
+      <c r="H9" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H9" s="80" t="inlineStr"/>
+      <c r="I9" s="80" t="inlineStr"/>
     </row>
     <row r="10" ht="81" customHeight="1" s="1">
       <c r="A10" s="84" t="n"/>
@@ -3552,13 +3598,18 @@
       </c>
       <c r="D10" s="81" t="inlineStr">
         <is>
+          <t>端口(L4)规则一键迁移为应用(L7)规则+新应用查看器</t>
+        </is>
+      </c>
+      <c r="E10" s="81" t="inlineStr">
+        <is>
           <t>PA新应用查看器+端口规则迁移至App-ID规则工作流+规则使用统计，减少攻击面（PA Web帮助p142）；天融信策略统计开关可显示规则匹配命中情况（天融信手册《配置访问控制策略》页），但无新应用查看器与端口→应用规则迁移工作流；对应矩阵#132</t>
         </is>
       </c>
-      <c r="E10" s="84" t="n"/>
       <c r="F10" s="84" t="n"/>
-      <c r="G10" s="85" t="n"/>
-      <c r="H10" s="84" t="n"/>
+      <c r="G10" s="84" t="n"/>
+      <c r="H10" s="85" t="n"/>
+      <c r="I10" s="84" t="n"/>
     </row>
     <row r="11" ht="36" customHeight="1" s="1">
       <c r="A11" s="84" t="n"/>
@@ -3570,17 +3621,22 @@
       </c>
       <c r="D11" s="81" t="inlineStr">
         <is>
+          <t>配置锁/提交锁，防止多管理员并发修改</t>
+        </is>
+      </c>
+      <c r="E11" s="81" t="inlineStr">
+        <is>
           <t>PA可锁定待选配置或提交，防止他管理员并发更改；对应矩阵#135（天融信不支持，PA优势）</t>
         </is>
       </c>
-      <c r="E11" s="85" t="n"/>
-      <c r="F11" s="84" t="n"/>
-      <c r="G11" s="80" t="inlineStr">
+      <c r="F11" s="85" t="n"/>
+      <c r="G11" s="84" t="n"/>
+      <c r="H11" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H11" s="84" t="n"/>
+      <c r="I11" s="84" t="n"/>
     </row>
     <row r="12" ht="111" customHeight="1" s="1">
       <c r="A12" s="84" t="n"/>
@@ -3592,17 +3648,22 @@
       </c>
       <c r="D12" s="81" t="inlineStr">
         <is>
+          <t>应用匹配同时强制使用标准端口，非标端口拒绝</t>
+        </is>
+      </c>
+      <c r="E12" s="81" t="inlineStr">
+        <is>
           <t>PA安全策略默认服务为application-default：放行应用同时强制其使用标准端口（如SSH仅22），非标准端口不匹配即拦截（PA管理指南p904）；天融信策略为五元组+应用识别组合（天融信手册《配置访问控制策略》页）；迁移评估项：直接转换若仅保留应用识别不限端口将扩大安全敞口，需制定应用标准端口映射限制（App-Default）转换方案；对应矩阵#2</t>
         </is>
       </c>
-      <c r="E12" s="80" t="inlineStr">
+      <c r="F12" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F12" s="84" t="n"/>
       <c r="G12" s="84" t="n"/>
       <c r="H12" s="84" t="n"/>
+      <c r="I12" s="84" t="n"/>
     </row>
     <row r="13" ht="81" customHeight="1" s="1">
       <c r="A13" s="84" t="n"/>
@@ -3614,17 +3675,22 @@
       </c>
       <c r="D13" s="81" t="inlineStr">
         <is>
+          <t>Allow动作关联反病毒/漏洞防护/URL过滤/文件阻断/WildFire配置文件组</t>
+        </is>
+      </c>
+      <c r="E13" s="81" t="inlineStr">
+        <is>
           <t>PA安全策略Allow动作关联Profile组（反病毒/漏洞防护/URL过滤/文件阻止/WildFire等，PA Web帮助p304）；天融信一体化策略引擎自带检测项；迁移评估项：需评估Profile组到天融信各检测引擎的映射与缺省动作差异；对应矩阵#4</t>
         </is>
       </c>
-      <c r="E13" s="80" t="inlineStr">
+      <c r="F13" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F13" s="84" t="n"/>
       <c r="G13" s="84" t="n"/>
       <c r="H13" s="84" t="n"/>
+      <c r="I13" s="84" t="n"/>
     </row>
     <row r="14" ht="156" customHeight="1" s="1">
       <c r="A14" s="84" t="n"/>
@@ -3636,17 +3702,22 @@
       </c>
       <c r="D14" s="81" t="inlineStr">
         <is>
+          <t>同区域默认放行/跨区域默认拒绝，支持替代与日志转发</t>
+        </is>
+      </c>
+      <c r="E14" s="81" t="inlineStr">
+        <is>
           <t>PA安全策略库末尾自带两条隐式系统规则：区域内默认（同Zone默认放行）与区域间默认（跨Zone默认拒绝），可被替代配置，替代字段含日志转发配置文件与Log at Session End在会话结束时记录（PA Web帮助p134-136）；天融信未见同区域默认放行的隐式规则机制；迁移评估项：①必须提取intrazone-default同Zone互访需求并显式转换为放行规则，否则割接后同Zone不同网段/VLAN互访将被默认拦截；②需在新设备补齐底部兜底Deny-All并开启日志，否则被拒流量查无日志、排障困难</t>
         </is>
       </c>
-      <c r="E14" s="80" t="inlineStr">
+      <c r="F14" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F14" s="85" t="n"/>
       <c r="G14" s="85" t="n"/>
       <c r="H14" s="85" t="n"/>
+      <c r="I14" s="85" t="n"/>
     </row>
     <row r="15" ht="81" customHeight="1" s="1">
       <c r="A15" s="84" t="n"/>
@@ -3662,21 +3733,26 @@
       </c>
       <c r="D15" s="81" t="inlineStr">
         <is>
+          <t>动态IP+端口(DIPP)/静态IP/接口地址，含回流(Hairpin)</t>
+        </is>
+      </c>
+      <c r="E15" s="81" t="inlineStr">
+        <is>
           <t>PA源NAT含DIPP动态IP+端口/静态IP/接口地址/持久NAT等（PA Web帮助p147）；天融信SNAT地址池（多对一/多对多/一对一/PAT）与仅源IP转换等（天融信手册《源NAT》《配置源转换》页）；对应矩阵#6</t>
         </is>
       </c>
-      <c r="E15" s="80" t="inlineStr">
+      <c r="F15" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F15" s="81" t="inlineStr"/>
-      <c r="G15" s="80" t="inlineStr">
+      <c r="G15" s="81" t="inlineStr"/>
+      <c r="H15" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H15" s="80" t="inlineStr">
+      <c r="I15" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
@@ -3692,23 +3768,28 @@
       </c>
       <c r="D16" s="81" t="inlineStr">
         <is>
+          <t>静态映射/端口转换/DNS重写/FQDN目标</t>
+        </is>
+      </c>
+      <c r="E16" s="81" t="inlineStr">
+        <is>
           <t>PA目标NAT含静态/动态IP、端口转换、DNS Rewrite、FQDN目标（PA Web帮助p149）；天融信服务器映射含静态映射+服务器负载均衡两种模式，NAT46/NAT66全系列（天融信手册《服务器映射》页）；对应矩阵#7</t>
         </is>
       </c>
-      <c r="E16" s="80" t="inlineStr">
+      <c r="F16" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F16" s="81" t="inlineStr"/>
-      <c r="G16" s="80" t="inlineStr">
+      <c r="G16" s="81" t="inlineStr"/>
+      <c r="H16" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H16" s="80" t="inlineStr"/>
-    </row>
-    <row r="17" ht="66" customHeight="1" s="1">
+      <c r="I16" s="80" t="inlineStr"/>
+    </row>
+    <row r="17" ht="81" customHeight="1" s="1">
       <c r="A17" s="84" t="n"/>
       <c r="B17" s="84" t="n"/>
       <c r="C17" s="81" t="inlineStr">
@@ -3718,15 +3799,20 @@
       </c>
       <c r="D17" s="81" t="inlineStr">
         <is>
+          <t>一对一转换，支持双向映射</t>
+        </is>
+      </c>
+      <c r="E17" s="81" t="inlineStr">
+        <is>
           <t>PA支持静态IP转换与双向(Bi-directional)转换（PA Web帮助p148）；天融信支持一对一转换（SNAT地址池一对一/NAT66一对一）（天融信手册《源NAT》《配置一对一转换》页）；对应矩阵#8</t>
         </is>
       </c>
-      <c r="E17" s="84" t="n"/>
       <c r="F17" s="84" t="n"/>
       <c r="G17" s="84" t="n"/>
       <c r="H17" s="84" t="n"/>
-    </row>
-    <row r="18" ht="66" customHeight="1" s="1">
+      <c r="I17" s="84" t="n"/>
+    </row>
+    <row r="18" ht="81" customHeight="1" s="1">
       <c r="A18" s="84" t="n"/>
       <c r="B18" s="84" t="n"/>
       <c r="C18" s="81" t="inlineStr">
@@ -3736,13 +3822,18 @@
       </c>
       <c r="D18" s="81" t="inlineStr">
         <is>
+          <t>NAT独立策略库，先NAT后安全策略匹配</t>
+        </is>
+      </c>
+      <c r="E18" s="81" t="inlineStr">
+        <is>
           <t>PA NAT策略库独立于安全策略库(Policies&gt;NAT)，先NAT后安全匹配；天融信地址转换为独立策略库（安全策略&gt;地址转换），与访问控制策略分离配置（天融信手册《安全策略》《工作原理》页）；对应矩阵#9</t>
         </is>
       </c>
-      <c r="E18" s="85" t="n"/>
-      <c r="F18" s="84" t="n"/>
+      <c r="F18" s="85" t="n"/>
       <c r="G18" s="84" t="n"/>
       <c r="H18" s="84" t="n"/>
+      <c r="I18" s="84" t="n"/>
     </row>
     <row r="19" ht="81" customHeight="1" s="1">
       <c r="A19" s="84" t="n"/>
@@ -3754,19 +3845,24 @@
       </c>
       <c r="D19" s="81" t="inlineStr">
         <is>
+          <t>IPv4↔IPv6转换类型（nat64）</t>
+        </is>
+      </c>
+      <c r="E19" s="81" t="inlineStr">
+        <is>
           <t>PA NAT规则支持IPv4/IPv6及NAT64转换类型（RFC6146）；天融信NAT64含静态转换+前缀转换+动态算法（IVI/普通前缀），另有NAT46（天融信手册《NAT64》《NAT46》页）；对应矩阵#18</t>
         </is>
       </c>
-      <c r="E19" s="80" t="inlineStr">
+      <c r="F19" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F19" s="84" t="n"/>
-      <c r="G19" s="85" t="n"/>
-      <c r="H19" s="84" t="n"/>
-    </row>
-    <row r="20" ht="111" customHeight="1" s="1">
+      <c r="G19" s="84" t="n"/>
+      <c r="H19" s="85" t="n"/>
+      <c r="I19" s="84" t="n"/>
+    </row>
+    <row r="20" ht="126" customHeight="1" s="1">
       <c r="A20" s="84" t="n"/>
       <c r="B20" s="84" t="n"/>
       <c r="C20" s="81" t="inlineStr">
@@ -3776,21 +3872,26 @@
       </c>
       <c r="D20" s="81" t="inlineStr">
         <is>
+          <t>目的区域按NAT后路由查找；源/目的地址用NAT前值</t>
+        </is>
+      </c>
+      <c r="E20" s="81" t="inlineStr">
+        <is>
           <t>PA底层为『先NAT判断后安全策略匹配』的因果倒置：安全策略要求源区域(NAT前)+源地址(NAT前)+目的地址(NAT前)+目的区域(NAT后按路由查找)，极其反直觉；天融信地址转换为独立策略库常规直观映射（安全策略&gt;地址转换，天融信手册《服务器映射》页）；迁移评估项：带目的NAT的策略平移后易因Zone填写错误不通，需制定NAT查表逻辑转换映射规范；对应矩阵#9</t>
         </is>
       </c>
-      <c r="E20" s="80" t="inlineStr">
+      <c r="F20" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F20" s="84" t="n"/>
-      <c r="G20" s="80" t="inlineStr">
+      <c r="G20" s="84" t="n"/>
+      <c r="H20" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H20" s="84" t="n"/>
+      <c r="I20" s="84" t="n"/>
     </row>
     <row r="21" ht="81" customHeight="1" s="1">
       <c r="A21" s="84" t="n"/>
@@ -3802,21 +3903,26 @@
       </c>
       <c r="D21" s="81" t="inlineStr">
         <is>
+          <t>主动/主动HA下NAT规则绑定会话所有者</t>
+        </is>
+      </c>
+      <c r="E21" s="81" t="inlineStr">
+        <is>
           <t>PA主动/主动HA配置下NAT规则可绑定会话所有者/会话设置，控制NAT会话的设备绑定，仅A/A模式可见（PA Web帮助p150）；天融信HA为主备双机热备模式（天融信手册《配置双机热备功能》页），无主动/主动模式及NAT规则绑定机制</t>
         </is>
       </c>
-      <c r="E21" s="80" t="inlineStr">
+      <c r="F21" s="80" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="F21" s="85" t="n"/>
-      <c r="G21" s="80" t="inlineStr">
+      <c r="G21" s="85" t="n"/>
+      <c r="H21" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H21" s="85" t="n"/>
+      <c r="I21" s="85" t="n"/>
     </row>
     <row r="22" ht="96" customHeight="1" s="1">
       <c r="A22" s="84" t="n"/>
@@ -3832,21 +3938,26 @@
       </c>
       <c r="D22" s="81" t="inlineStr">
         <is>
+          <t>8类流量分类+4级优先级，保证/最大带宽控制</t>
+        </is>
+      </c>
+      <c r="E22" s="81" t="inlineStr">
+        <is>
           <t>PA QoS策略规则分配QoS类（8类+4级优先级），按Egress Guaranteed/Max控制带宽（PA Web帮助p154-155）；天融信流量管理基于应用/用户/源目的区域/地址/服务/时间+通道优先级，虚拟通道限制与保证带宽（天融信手册《流量管理》页）；对应矩阵#33/66</t>
         </is>
       </c>
-      <c r="E22" s="80" t="inlineStr">
+      <c r="F22" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F22" s="81" t="inlineStr"/>
-      <c r="G22" s="80" t="inlineStr">
+      <c r="G22" s="81" t="inlineStr"/>
+      <c r="H22" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H22" s="80" t="inlineStr">
+      <c r="I22" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
@@ -3862,21 +3973,26 @@
       </c>
       <c r="D23" s="81" t="inlineStr">
         <is>
+          <t>QoS规则按DSCP/ToS值匹配调度</t>
+        </is>
+      </c>
+      <c r="E23" s="81" t="inlineStr">
+        <is>
           <t>PA QoS规则可直接按DSCP值或IP优先级/ToS匹配调度（PA Web帮助p155）；天融信支持DSCP/802.1p(CoS)识别与重标记，但需在独立流量管理模块配置（虚拟通道+限制/保证带宽+通道优先级，天融信手册《流量管理》页），未直接耦合在基础访问控制策略表内（联网核实厂商流控资料，手册未详载）</t>
         </is>
       </c>
-      <c r="E23" s="80" t="inlineStr">
+      <c r="F23" s="80" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="F23" s="81" t="inlineStr"/>
-      <c r="G23" s="80" t="inlineStr">
+      <c r="G23" s="81" t="inlineStr"/>
+      <c r="H23" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H23" s="80" t="inlineStr"/>
+      <c r="I23" s="80" t="inlineStr"/>
     </row>
     <row r="24" ht="81" customHeight="1" s="1">
       <c r="A24" s="84" t="n"/>
@@ -3892,27 +4008,32 @@
       </c>
       <c r="D24" s="81" t="inlineStr">
         <is>
+          <t>按源区域/地址/用户/应用/服务+下一跳转发，路径监控失效切换</t>
+        </is>
+      </c>
+      <c r="E24" s="81" t="inlineStr">
+        <is>
           <t>PA PBF策略绕过常规路由表选路，支持路径监控与失效切换、BFD、强制对称返回（PA Web帮助p156）；天融信策略路由按源/目的地址端口、ISP名称、协议、角色等参数选路（天融信手册《策略路由》页）；对应矩阵#10</t>
         </is>
       </c>
-      <c r="E24" s="80" t="inlineStr">
+      <c r="F24" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F24" s="81" t="inlineStr"/>
-      <c r="G24" s="80" t="inlineStr">
+      <c r="G24" s="81" t="inlineStr"/>
+      <c r="H24" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H24" s="80" t="inlineStr">
+      <c r="I24" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="96" customHeight="1" s="1">
+    <row r="25" ht="111" customHeight="1" s="1">
       <c r="A25" s="84" t="n"/>
       <c r="B25" s="85" t="n"/>
       <c r="C25" s="81" t="inlineStr">
@@ -3922,21 +4043,26 @@
       </c>
       <c r="D25" s="81" t="inlineStr">
         <is>
+          <t>记录入接口MAC，回包强制原路返回</t>
+        </is>
+      </c>
+      <c r="E25" s="81" t="inlineStr">
+        <is>
           <t>PA对称返回：虚拟路由器替代返回流量的路由查找，将流量引导回接收SYN数据包的MAC地址（ARP表确定下一跳），双ISP双活/非对称路由核心机制（PA管理指南p1294）；天融信手册检索无对称返回/回程机制命中，策略路由与LLB的回程保障能力待验证；迁移评估项：多ISP双活环境需实测天融信回包路由对称性，否则现网业务中断</t>
         </is>
       </c>
-      <c r="E25" s="80" t="inlineStr">
+      <c r="F25" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F25" s="81" t="inlineStr"/>
-      <c r="G25" s="80" t="inlineStr">
+      <c r="G25" s="81" t="inlineStr"/>
+      <c r="H25" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H25" s="80" t="inlineStr"/>
+      <c r="I25" s="80" t="inlineStr"/>
     </row>
     <row r="26" ht="96" customHeight="1" s="1">
       <c r="A26" s="84" t="n"/>
@@ -3952,27 +4078,32 @@
       </c>
       <c r="D26" s="81" t="inlineStr">
         <is>
+          <t>出站正向代理+入站检查双向解密</t>
+        </is>
+      </c>
+      <c r="E26" s="81" t="inlineStr">
+        <is>
           <t>PA解密策略区分SSL Forward Proxy/Inbound Inspection/SSH，可解密以获得流量可见性与深度检测（PA Web帮助p164）；天融信代理策略将NGFW作为代理服务器，对加密流量解密还原明文完成内容安全检查后重新加密（天融信手册《代理策略》页）；对应矩阵#29/30</t>
         </is>
       </c>
-      <c r="E26" s="80" t="inlineStr">
+      <c r="F26" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F26" s="81" t="inlineStr"/>
-      <c r="G26" s="80" t="inlineStr">
+      <c r="G26" s="81" t="inlineStr"/>
+      <c r="H26" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H26" s="80" t="inlineStr">
+      <c r="I26" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="51" customHeight="1" s="1">
+    <row r="27" ht="66" customHeight="1" s="1">
       <c r="A27" s="84" t="n"/>
       <c r="B27" s="84" t="n"/>
       <c r="C27" s="81" t="inlineStr">
@@ -3982,21 +4113,26 @@
       </c>
       <c r="D27" s="81" t="inlineStr">
         <is>
+          <t>入站证书配置/解密目标（数据包/会话）</t>
+        </is>
+      </c>
+      <c r="E27" s="81" t="inlineStr">
+        <is>
           <t>PA解密目标允许指定数据包/会话；入站含Certificates证书配置；对应矩阵#31；天融信代理模板支持证书选择与预置动态证书模板（天融信手册《代理模板》页）</t>
         </is>
       </c>
-      <c r="E27" s="80" t="inlineStr">
+      <c r="F27" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F27" s="81" t="inlineStr"/>
-      <c r="G27" s="80" t="inlineStr">
+      <c r="G27" s="81" t="inlineStr"/>
+      <c r="H27" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H27" s="80" t="inlineStr"/>
+      <c r="I27" s="80" t="inlineStr"/>
     </row>
     <row r="28" ht="51" customHeight="1" s="1">
       <c r="A28" s="84" t="n"/>
@@ -4008,17 +4144,22 @@
       </c>
       <c r="D28" s="81" t="inlineStr">
         <is>
+          <t>解密后明文流量镜像至专用接口供第三方分析</t>
+        </is>
+      </c>
+      <c r="E28" s="81" t="inlineStr">
+        <is>
           <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证（PA管理指南p1059）；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
         </is>
       </c>
-      <c r="E28" s="85" t="n"/>
-      <c r="F28" s="84" t="n"/>
-      <c r="G28" s="80" t="inlineStr">
+      <c r="F28" s="85" t="n"/>
+      <c r="G28" s="84" t="n"/>
+      <c r="H28" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H28" s="84" t="n"/>
+      <c r="I28" s="84" t="n"/>
     </row>
     <row r="29" ht="126" customHeight="1" s="1">
       <c r="A29" s="84" t="n"/>
@@ -4030,21 +4171,26 @@
       </c>
       <c r="D29" s="81" t="inlineStr">
         <is>
+          <t>外部无效证书以不受信转发证书重签，保留浏览器告警</t>
+        </is>
+      </c>
+      <c r="E29" s="81" t="inlineStr">
+        <is>
           <t>PA转发代理遇外部过期/不受信证书时，不用内部信任CA重签，而是专用Forward Untrust Certificate重签名，让浏览器保留不受信告警（PA管理指南p994、p1030）；天融信SSL解密（透明代理/服务器SSL解密，天融信手册《代理策略》页）未见受信/不受信双证书体系；迁移评估项：需验证天融信对外部无效证书的处理方式，避免直接阻断（白屏）或信任重签（掩盖风险）</t>
         </is>
       </c>
-      <c r="E29" s="80" t="inlineStr">
+      <c r="F29" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F29" s="84" t="n"/>
-      <c r="G29" s="80" t="inlineStr">
+      <c r="G29" s="84" t="n"/>
+      <c r="H29" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H29" s="84" t="n"/>
+      <c r="I29" s="84" t="n"/>
     </row>
     <row r="30" ht="66" customHeight="1" s="1">
       <c r="A30" s="84" t="n"/>
@@ -4056,21 +4202,26 @@
       </c>
       <c r="D30" s="81" t="inlineStr">
         <is>
+          <t>按URL类别圈定解密范围，排除银行/医疗等敏感类</t>
+        </is>
+      </c>
+      <c r="E30" s="81" t="inlineStr">
+        <is>
           <t>PA解密规则可按URL类别（含自定义类别）选择解密范围，可排除银行/医疗等敏感类别不解密（PA Web帮助p164）；天融信SSL解密（代理策略/代理模板）无按URL类别选择解密机制（检索无命中）</t>
         </is>
       </c>
-      <c r="E30" s="80" t="inlineStr">
+      <c r="F30" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F30" s="84" t="n"/>
-      <c r="G30" s="80" t="inlineStr">
+      <c r="G30" s="84" t="n"/>
+      <c r="H30" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H30" s="84" t="n"/>
+      <c r="I30" s="84" t="n"/>
     </row>
     <row r="31" ht="96" customHeight="1" s="1">
       <c r="A31" s="84" t="n"/>
@@ -4082,13 +4233,18 @@
       </c>
       <c r="D31" s="81" t="inlineStr">
         <is>
+          <t>SSH代理解密+SSH隧道(ssh-tunnel)识别控制</t>
+        </is>
+      </c>
+      <c r="E31" s="81" t="inlineStr">
+        <is>
           <t>PA解密策略SSH Proxy类型解密SSH通信，可通过ssh-tunnel App-ID在策略中控制SSH隧道（端口转发/内网穿透），正常SSH管理流量放行；含不受支持算法检查/资源不足阻断会话等防护（PA Web帮助p164、p318-319）；天融信手册检索无SSH代理/SSH隧道控制命中</t>
         </is>
       </c>
-      <c r="E31" s="85" t="n"/>
       <c r="F31" s="85" t="n"/>
       <c r="G31" s="85" t="n"/>
       <c r="H31" s="85" t="n"/>
+      <c r="I31" s="85" t="n"/>
     </row>
     <row r="32" ht="66" customHeight="1" s="1">
       <c r="A32" s="84" t="n"/>
@@ -4104,21 +4260,26 @@
       </c>
       <c r="D32" s="81" t="inlineStr">
         <is>
+          <t>已解密/未解密流量内联转发第三方安全链，L3路由转发</t>
+        </is>
+      </c>
+      <c r="E32" s="81" t="inlineStr">
+        <is>
           <t>PA网络数据包代理策略将已解密/未解密TLS/非TLS流量内联转发至第三方安全工具，路径选择选项卡应用数据包代理配置文件定义经路由L3安全链的转发方式（PA Web帮助p167-170）；对应矩阵#122</t>
         </is>
       </c>
-      <c r="E32" s="80" t="inlineStr">
+      <c r="F32" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F32" s="81" t="inlineStr"/>
-      <c r="G32" s="80" t="inlineStr">
+      <c r="G32" s="81" t="inlineStr"/>
+      <c r="H32" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H32" s="80" t="inlineStr">
+      <c r="I32" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
@@ -4134,21 +4295,26 @@
       </c>
       <c r="D33" s="81" t="inlineStr">
         <is>
+          <t>TLS解密/未解密/非TLS流量类型选择</t>
+        </is>
+      </c>
+      <c r="E33" s="81" t="inlineStr">
+        <is>
           <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证（PA Web帮助p167）；天融信无网络数据包代理模块（矩阵#122）</t>
         </is>
       </c>
-      <c r="E33" s="80" t="inlineStr">
+      <c r="F33" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F33" s="81" t="inlineStr"/>
-      <c r="G33" s="80" t="inlineStr">
+      <c r="G33" s="81" t="inlineStr"/>
+      <c r="H33" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H33" s="80" t="inlineStr"/>
+      <c r="I33" s="80" t="inlineStr"/>
     </row>
     <row r="34" ht="66" customHeight="1" s="1">
       <c r="A34" s="84" t="n"/>
@@ -4164,21 +4330,26 @@
       </c>
       <c r="D34" s="81" t="inlineStr">
         <is>
+          <t>GRE/GTP-U/VXLAN/非加密IPSec隧道内层流量解封装检测</t>
+        </is>
+      </c>
+      <c r="E34" s="81" t="inlineStr">
+        <is>
           <t>PA隧道检测策略解封装并深度检测GRE/GTP-U/VXLAN/非加密IPSec（NULL加密/AH传输模式）等明文隧道内容（PA Web帮助p172-173）；对应矩阵#128/37</t>
         </is>
       </c>
-      <c r="E34" s="80" t="inlineStr">
+      <c r="F34" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F34" s="81" t="inlineStr"/>
-      <c r="G34" s="80" t="inlineStr">
+      <c r="G34" s="81" t="inlineStr"/>
+      <c r="H34" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H34" s="80" t="inlineStr">
+      <c r="I34" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
@@ -4194,21 +4365,26 @@
       </c>
       <c r="D35" s="81" t="inlineStr">
         <is>
+          <t>隧道嵌套封装最大级数限制，超限丢弃</t>
+        </is>
+      </c>
+      <c r="E35" s="81" t="inlineStr">
+        <is>
           <t>PA对隧道最大封装级数超限丢包防护，防隧道嵌套绕过（PA管理指南p655）；天融信手册无封装级数防护（检索无命中）</t>
         </is>
       </c>
-      <c r="E35" s="80" t="inlineStr">
+      <c r="F35" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F35" s="81" t="inlineStr"/>
-      <c r="G35" s="80" t="inlineStr">
+      <c r="G35" s="81" t="inlineStr"/>
+      <c r="H35" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H35" s="80" t="inlineStr"/>
+      <c r="I35" s="80" t="inlineStr"/>
     </row>
     <row r="36" ht="81" customHeight="1" s="1">
       <c r="A36" s="84" t="n"/>
@@ -4224,21 +4400,26 @@
       </c>
       <c r="D36" s="81" t="inlineStr">
         <is>
+          <t>按协议/端口自定义应用识别结果</t>
+        </is>
+      </c>
+      <c r="E36" s="81" t="inlineStr">
+        <is>
           <t>PA应用替代策略改变防火墙对网络通信的应用分类方式（如指定明文协议/端口识别，PA Web帮助p178）；天融信自定义应用允许管理员按需自定义应用协议（含端口匹配）并加入应用规则库（天融信手册《自定义应用》页）；对应矩阵#26</t>
         </is>
       </c>
-      <c r="E36" s="80" t="inlineStr">
+      <c r="F36" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F36" s="81" t="inlineStr"/>
-      <c r="G36" s="80" t="inlineStr">
+      <c r="G36" s="81" t="inlineStr"/>
+      <c r="H36" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H36" s="80" t="inlineStr">
+      <c r="I36" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
@@ -4254,21 +4435,26 @@
       </c>
       <c r="D37" s="81" t="inlineStr">
         <is>
+          <t>端口映射类覆盖识别</t>
+        </is>
+      </c>
+      <c r="E37" s="81" t="inlineStr">
+        <is>
           <t>PA支持端口式应用覆盖识别（configurable自定义应用）；天融信自定义应用允许管理员按特定需要自行定义应用协议（含端口匹配），自动添加到应用规则库供安全策略引用（天融信手册《自定义应用》页）</t>
         </is>
       </c>
-      <c r="E37" s="80" t="inlineStr">
+      <c r="F37" s="80" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="F37" s="81" t="inlineStr"/>
-      <c r="G37" s="80" t="inlineStr">
+      <c r="G37" s="81" t="inlineStr"/>
+      <c r="H37" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H37" s="80" t="inlineStr"/>
+      <c r="I37" s="80" t="inlineStr"/>
     </row>
     <row r="38" ht="96" customHeight="1" s="1">
       <c r="A38" s="84" t="n"/>
@@ -4280,21 +4466,26 @@
       </c>
       <c r="D38" s="81" t="inlineStr">
         <is>
+          <t>匹配覆盖策略的流量跳过七层检测，四层快速转发</t>
+        </is>
+      </c>
+      <c r="E38" s="81" t="inlineStr">
+        <is>
           <t>PA应用替代策略明确绕过第7层处理与威胁检查，改用第4层状态检查以加速（PA管理指南p1307）；天融信自定义应用加入规则库后仍默认经安全引擎检测（天融信手册《自定义应用》页）；迁移评估项：PA应用替代多为私有大流量业务加速，转换时需同步关闭对应策略的IPS/七层检测，否则性能被拖垮或误阻断</t>
         </is>
       </c>
-      <c r="E38" s="80" t="inlineStr">
+      <c r="F38" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F38" s="85" t="n"/>
-      <c r="G38" s="80" t="inlineStr">
+      <c r="G38" s="85" t="n"/>
+      <c r="H38" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H38" s="85" t="n"/>
+      <c r="I38" s="85" t="n"/>
     </row>
     <row r="39" ht="111" customHeight="1" s="1">
       <c r="A39" s="84" t="n"/>
@@ -4310,21 +4501,26 @@
       </c>
       <c r="D39" s="81" t="inlineStr">
         <is>
+          <t>基于用户/用户组策略，多源IP-用户映射（AD/Syslog/XML API）</t>
+        </is>
+      </c>
+      <c r="E39" s="81" t="inlineStr">
+        <is>
           <t>PA身份验证策略在访问网络资源前对用户鉴权（PA Web帮助p182），配合User-ID多源映射（AD/XML/Syslog等）；天融信用户访问网络资源前经认证，认证通过后检查关联的用户访问策略，支持门户认证（本地/外部）与LDAP/RADIUS对接（天融信手册《管理用户》《添加Radius服务器》页）；对应矩阵#3/35</t>
         </is>
       </c>
-      <c r="E39" s="80" t="inlineStr">
+      <c r="F39" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F39" s="81" t="inlineStr"/>
-      <c r="G39" s="80" t="inlineStr">
+      <c r="G39" s="81" t="inlineStr"/>
+      <c r="H39" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H39" s="80" t="inlineStr">
+      <c r="I39" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
@@ -4340,21 +4536,26 @@
       </c>
       <c r="D40" s="81" t="inlineStr">
         <is>
+          <t>认证超时+单次认证(SSO)</t>
+        </is>
+      </c>
+      <c r="E40" s="81" t="inlineStr">
+        <is>
           <t>PA支持认证超时减少重复质询、Kerberos/SAML/RADIUS等对接（PA Web帮助p186）；天融信手册检索认证超时/单点登录/SSO无命中（仅在线用户在线时长查看与强制下线）；迁移评估项：需核实天融信认证会话有效期配置与SSO对接能力</t>
         </is>
       </c>
-      <c r="E40" s="80" t="inlineStr">
+      <c r="F40" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F40" s="81" t="inlineStr"/>
-      <c r="G40" s="80" t="inlineStr">
+      <c r="G40" s="81" t="inlineStr"/>
+      <c r="H40" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H40" s="80" t="inlineStr"/>
+      <c r="I40" s="80" t="inlineStr"/>
     </row>
     <row r="41" ht="126" customHeight="1" s="1">
       <c r="A41" s="84" t="n"/>
@@ -4366,19 +4567,24 @@
       </c>
       <c r="D41" s="81" t="inlineStr">
         <is>
+          <t>策略匹配触发多因素认证质询（MFA供应商API/RADIUS）</t>
+        </is>
+      </c>
+      <c r="E41" s="81" t="inlineStr">
+        <is>
           <t>PA身份验证策略通过Authentication Enforcement对象对匹配流量强制质询，支持多因素身份验证（每因素独立超时，防火墙记录时间戳），MFA供应商API/RADIUS对接（PA Web帮助p185-186、p310、p735-742）；天融信双因子认证（密码+短信/证书/Ukey）仅限管理员/用户登录场景（天融信手册《登录安全策略》页），未见流量策略触发MFA质询</t>
         </is>
       </c>
-      <c r="E41" s="84" t="n"/>
       <c r="F41" s="84" t="n"/>
-      <c r="G41" s="80" t="inlineStr">
+      <c r="G41" s="84" t="n"/>
+      <c r="H41" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H41" s="84" t="n"/>
-    </row>
-    <row r="42" ht="81" customHeight="1" s="1">
+      <c r="I41" s="84" t="n"/>
+    </row>
+    <row r="42" ht="96" customHeight="1" s="1">
       <c r="A42" s="84" t="n"/>
       <c r="B42" s="85" t="n"/>
       <c r="C42" s="81" t="inlineStr">
@@ -4388,17 +4594,22 @@
       </c>
       <c r="D42" s="81" t="inlineStr">
         <is>
+          <t>AD域事件日志毫秒级IP-用户映射更新</t>
+        </is>
+      </c>
+      <c r="E42" s="81" t="inlineStr">
+        <is>
           <t>PA无代理架构通过读取域控事件日志实现IP-用户毫秒级动态映射，大规模部署有专项规划（PA管理指南p866-867）；天融信AD对接的轮询间隔与并发认证能力手册未量化；迁移评估项：数万AD用户且移动频繁场景需实测天融信映射更新时延，避免基于用户的策略出现间歇性未授权拦截</t>
         </is>
       </c>
-      <c r="E42" s="85" t="n"/>
       <c r="F42" s="85" t="n"/>
-      <c r="G42" s="80" t="inlineStr">
+      <c r="G42" s="85" t="n"/>
+      <c r="H42" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H42" s="85" t="n"/>
+      <c r="I42" s="85" t="n"/>
     </row>
     <row r="43" ht="111" customHeight="1" s="1">
       <c r="A43" s="84" t="n"/>
@@ -4414,21 +4625,26 @@
       </c>
       <c r="D43" s="81" t="inlineStr">
         <is>
+          <t>分类(源/目的IP粒度)+聚合(全局)双层阈值限流</t>
+        </is>
+      </c>
+      <c r="E43" s="81" t="inlineStr">
+        <is>
           <t>PA DoS策略基于源/目的接口、区域、地址、服务定义允许/拒绝/告警，规则可选聚合与分类双层DoS保护配置文件设定阈值速率（PA Web帮助p189-191、PA管理指南p1354）；天融信DDoS防护模块按防护对象（目的服务器）设阈值（pps/bps），可达目的IP粒度（天融信手册《配置策略模板》《日志查看》页）；对应矩阵#52/42</t>
         </is>
       </c>
-      <c r="E43" s="80" t="inlineStr">
+      <c r="F43" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F43" s="81" t="inlineStr"/>
-      <c r="G43" s="80" t="inlineStr">
+      <c r="G43" s="81" t="inlineStr"/>
+      <c r="H43" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H43" s="80" t="inlineStr">
+      <c r="I43" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
@@ -4444,23 +4660,28 @@
       </c>
       <c r="D44" s="81" t="inlineStr">
         <is>
+          <t>连接数/秒阈值告警+最大速率限制</t>
+        </is>
+      </c>
+      <c r="E44" s="81" t="inlineStr">
+        <is>
           <t>PA聚合DoS配置文件按传入连接数/秒触发告警与最大速率限制；天融信DDoS防护模块按阈值（pps/bps）监视并触发防护（天融信手册《配置策略模板》页）</t>
         </is>
       </c>
-      <c r="E44" s="80" t="inlineStr">
+      <c r="F44" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F44" s="81" t="inlineStr"/>
-      <c r="G44" s="80" t="inlineStr">
+      <c r="G44" s="81" t="inlineStr"/>
+      <c r="H44" s="80" t="inlineStr">
         <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="H44" s="80" t="inlineStr"/>
-    </row>
-    <row r="45" ht="156" customHeight="1" s="1">
+      <c r="I44" s="80" t="inlineStr"/>
+    </row>
+    <row r="45" ht="171" customHeight="1" s="1">
       <c r="A45" s="84" t="n"/>
       <c r="B45" s="80" t="inlineStr">
         <is>
@@ -4474,21 +4695,26 @@
       </c>
       <c r="D45" s="81" t="inlineStr">
         <is>
+          <t>HTTP/HTTPS外部文本列表(IP/域名/URL)自动拉取，策略直接引用</t>
+        </is>
+      </c>
+      <c r="E45" s="81" t="inlineStr">
+        <is>
           <t>PA外部动态列表：基于HTTP/HTTPS托管的文本文件创建IP/URL/域名/IMEI/IMSI地址对象，防火墙定时自动拉取更新，策略中直接引用（Objects&gt;External Dynamic Lists，PA Web帮助p236-239；策略源/目标可直接选EDL，p196-197）；天融信手册检索外部动态列表/EDL无命中，仅内置威胁情报库与云端威胁情报库（规则集管理，天融信手册《威胁情报》《配置规则集》页），无策略直接引用任意外部文本列表机制；迁移评估项：PA策略中引用的EDL需转换为天融信静态地址组定期导入或威胁情报联动</t>
         </is>
       </c>
-      <c r="E45" s="80" t="inlineStr">
+      <c r="F45" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F45" s="81" t="inlineStr"/>
-      <c r="G45" s="80" t="inlineStr">
+      <c r="G45" s="81" t="inlineStr"/>
+      <c r="H45" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H45" s="80" t="inlineStr"/>
+      <c r="I45" s="80" t="inlineStr"/>
     </row>
     <row r="46" ht="126" customHeight="1" s="1">
       <c r="A46" s="84" t="n"/>
@@ -4500,21 +4726,26 @@
       </c>
       <c r="D46" s="81" t="inlineStr">
         <is>
+          <t>Tag标记过滤器动态地址组，成员随IP变化自动更新</t>
+        </is>
+      </c>
+      <c r="E46" s="81" t="inlineStr">
+        <is>
           <t>PA动态地址组：查找标记(Tag)+基于标记的过滤器（AND/OR匹配）动态填充成员，VM信息源注册或XML/REST API定义标记，IP变化时策略自动生效（PA Web帮助p207-208、p228）；天融信手册检索动态地址组/标签/SDN/云平台联动无命中，地址组为静态IP/子网绑定（天融信手册《地址》页）；迁移评估项：PA云环境Tag微隔离策略需转换为静态地址组，IP漂移场景需人工或API维护</t>
         </is>
       </c>
-      <c r="E46" s="80" t="inlineStr">
+      <c r="F46" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F46" s="81" t="inlineStr"/>
-      <c r="G46" s="80" t="inlineStr">
+      <c r="G46" s="81" t="inlineStr"/>
+      <c r="H46" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H46" s="80" t="inlineStr"/>
+      <c r="I46" s="80" t="inlineStr"/>
     </row>
     <row r="47" ht="51" customHeight="1" s="1">
       <c r="A47" s="84" t="n"/>
@@ -4530,21 +4761,26 @@
       </c>
       <c r="D47" s="81" t="inlineStr">
         <is>
+          <t>按应用/区域/地址分配链路与流量分发</t>
+        </is>
+      </c>
+      <c r="E47" s="81" t="inlineStr">
+        <is>
           <t>PA SD-WAN策略按应用/抖动/延迟/丢包指标分配链路，流量分发（PA Web帮助p197）；对应矩阵#129/120</t>
         </is>
       </c>
-      <c r="E47" s="80" t="inlineStr">
+      <c r="F47" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F47" s="81" t="inlineStr"/>
-      <c r="G47" s="80" t="inlineStr">
+      <c r="G47" s="81" t="inlineStr"/>
+      <c r="H47" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H47" s="80" t="inlineStr">
+      <c r="I47" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
@@ -4560,61 +4796,66 @@
       </c>
       <c r="D48" s="81" t="inlineStr">
         <is>
+          <t>抖动/延迟/丢包(jitter/latency/loss)指标选路</t>
+        </is>
+      </c>
+      <c r="E48" s="81" t="inlineStr">
+        <is>
           <t>PA路径质量配置文件基于抖动/延迟/丢包等运行状况指标选路（PA Web帮助p195）；天融信有链路探测(ping)+智能选路(最小延迟优先)（天融信手册《策略路由》页），无jitter/latency/loss多维指标</t>
         </is>
       </c>
-      <c r="E48" s="80" t="inlineStr">
+      <c r="F48" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F48" s="81" t="inlineStr"/>
-      <c r="G48" s="80" t="inlineStr">
+      <c r="G48" s="81" t="inlineStr"/>
+      <c r="H48" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H48" s="80" t="inlineStr"/>
+      <c r="I48" s="80" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="I9:I14"/>
     <mergeCell ref="B26:B31"/>
     <mergeCell ref="B47:B48"/>
+    <mergeCell ref="H9:H10"/>
     <mergeCell ref="B43:B44"/>
-    <mergeCell ref="H3:H7"/>
-    <mergeCell ref="F16:F21"/>
+    <mergeCell ref="H6:H7"/>
     <mergeCell ref="B15:B21"/>
-    <mergeCell ref="F27:F31"/>
     <mergeCell ref="B36:B38"/>
-    <mergeCell ref="H9:H14"/>
+    <mergeCell ref="F30:F31"/>
+    <mergeCell ref="F9:F11"/>
+    <mergeCell ref="G40:G42"/>
+    <mergeCell ref="I40:I42"/>
     <mergeCell ref="B39:B42"/>
-    <mergeCell ref="E16:E18"/>
     <mergeCell ref="B2:B7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="H27:H31"/>
+    <mergeCell ref="H11:H14"/>
+    <mergeCell ref="G37:G38"/>
+    <mergeCell ref="I16:I21"/>
     <mergeCell ref="B34:B35"/>
-    <mergeCell ref="E3:E7"/>
+    <mergeCell ref="I37:I38"/>
     <mergeCell ref="B24:B25"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="G30:G31"/>
+    <mergeCell ref="F27:F28"/>
     <mergeCell ref="F40:F42"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="H16:H21"/>
-    <mergeCell ref="H37:H38"/>
+    <mergeCell ref="F16:F18"/>
+    <mergeCell ref="H16:H19"/>
     <mergeCell ref="F3:F7"/>
+    <mergeCell ref="G27:G31"/>
+    <mergeCell ref="I27:I31"/>
     <mergeCell ref="B45:B46"/>
-    <mergeCell ref="H40:H42"/>
-    <mergeCell ref="G9:G10"/>
     <mergeCell ref="B32:B33"/>
+    <mergeCell ref="H30:H31"/>
     <mergeCell ref="B22:B23"/>
-    <mergeCell ref="F9:F14"/>
+    <mergeCell ref="G3:G7"/>
     <mergeCell ref="B8:B14"/>
-    <mergeCell ref="G16:G19"/>
+    <mergeCell ref="I3:I7"/>
+    <mergeCell ref="G16:G21"/>
     <mergeCell ref="A2:A48"/>
-    <mergeCell ref="G11:G14"/>
-    <mergeCell ref="E40:E42"/>
-    <mergeCell ref="E9:E11"/>
+    <mergeCell ref="G9:G14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4626,17 +4867,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15.2"/>
   <cols>
     <col width="11.7" customWidth="1" style="1" min="1" max="1"/>
     <col width="19.7" customWidth="1" style="1" min="2" max="2"/>
-    <col width="48" customWidth="1" style="1" min="3" max="3"/>
-    <col width="55" customWidth="1" style="1" min="4" max="4"/>
-    <col width="7.7" customWidth="1" style="1" min="5" max="5"/>
-    <col width="20" customWidth="1" style="1" min="6" max="6"/>
-    <col width="12" customWidth="1" style="1" min="7" max="7"/>
-    <col width="9.699999999999999" customWidth="1" style="1" min="8" max="8"/>
+    <col width="40" customWidth="1" style="1" min="3" max="3"/>
+    <col width="30" customWidth="1" style="1" min="4" max="4"/>
+    <col width="62" customWidth="1" style="1" min="5" max="5"/>
+    <col width="7.7" customWidth="1" style="1" min="6" max="6"/>
+    <col width="18" customWidth="1" style="1" min="7" max="7"/>
+    <col width="10" customWidth="1" style="1" min="8" max="8"/>
+    <col width="9.699999999999999" customWidth="1" style="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" s="1">
@@ -4662,20 +4904,25 @@
       </c>
       <c r="E1" s="79" t="inlineStr">
         <is>
+          <t>对比依据（PA证据·天融信现状）</t>
+        </is>
+      </c>
+      <c r="F1" s="79" t="inlineStr">
+        <is>
           <t>优先级</t>
         </is>
       </c>
-      <c r="F1" s="79" t="inlineStr">
+      <c r="G1" s="79" t="inlineStr">
         <is>
           <t>交付/规划说明</t>
         </is>
       </c>
-      <c r="G1" s="79" t="inlineStr">
+      <c r="H1" s="79" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="H1" s="79" t="inlineStr">
+      <c r="I1" s="79" t="inlineStr">
         <is>
           <t>负责人</t>
         </is>
@@ -4699,21 +4946,26 @@
       </c>
       <c r="D2" s="81" t="inlineStr">
         <is>
+          <t>提交/修改策略须填写审核注释并留存历史，可导出</t>
+        </is>
+      </c>
+      <c r="E2" s="81" t="inlineStr">
+        <is>
           <t>PA记录规则的审核注释历史/配置日志/规则更改历史，可CSV导出，用于策略变更审计（PA Web帮助p116-117）；天融信仅规则描述字段，无审核注释存档</t>
         </is>
       </c>
-      <c r="E2" s="80" t="inlineStr">
+      <c r="F2" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F2" s="81" t="inlineStr"/>
-      <c r="G2" s="80" t="inlineStr">
+      <c r="G2" s="81" t="inlineStr"/>
+      <c r="H2" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H2" s="80" t="inlineStr"/>
+      <c r="I2" s="80" t="inlineStr"/>
     </row>
     <row r="3" ht="111" customHeight="1" s="1">
       <c r="A3" s="82" t="n"/>
@@ -4725,21 +4977,26 @@
       </c>
       <c r="D3" s="81" t="inlineStr">
         <is>
+          <t>前置规则→本地规则→后置规则三层按序合并为单层规则链</t>
+        </is>
+      </c>
+      <c r="E3" s="81" t="inlineStr">
+        <is>
           <t>PA在Panorama集中管理下策略分为前置规则（设备组共享，最优先）/本地规则/后置规则三层按序匹配（层级机制属Panorama管理平台，PA两册手册未详载）；天融信为自上而下单层规则链一张表走到底（天融信手册《配置访问控制策略》页）；迁移评估项：需制定全局多级策略到单层扁平化策略的合并清洗规则（Pre→本地→Post按序展开映射）</t>
         </is>
       </c>
-      <c r="E3" s="80" t="inlineStr">
+      <c r="F3" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F3" s="81" t="inlineStr"/>
-      <c r="G3" s="80" t="inlineStr">
+      <c r="G3" s="81" t="inlineStr"/>
+      <c r="H3" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H3" s="80" t="inlineStr"/>
+      <c r="I3" s="80" t="inlineStr"/>
     </row>
     <row r="4" ht="96" customHeight="1" s="1">
       <c r="A4" s="82" t="n"/>
@@ -4751,15 +5008,20 @@
       </c>
       <c r="D4" s="81" t="inlineStr">
         <is>
+          <t>应用程序对象级会话超时，覆盖全局TCP/UDP超时</t>
+        </is>
+      </c>
+      <c r="E4" s="81" t="inlineStr">
+        <is>
           <t>PA除全局TCP/UDP会话超时外，可在应用程序对象上定义专用超时，匹配该应用的流量覆盖全局值（PA Web帮助p215、p695）；天融信手册未见应用级超时覆盖（仅SSLVPN会话超时设置与黑名单老化）；迁移评估项：需排查现网PA为数据库/长连接业务单独配置的应用超时并逐条转换，否则长连接业务频繁中断</t>
         </is>
       </c>
-      <c r="E4" s="82" t="n"/>
       <c r="F4" s="82" t="n"/>
       <c r="G4" s="82" t="n"/>
       <c r="H4" s="82" t="n"/>
-    </row>
-    <row r="5" ht="81" customHeight="1" s="1">
+      <c r="I4" s="82" t="n"/>
+    </row>
+    <row r="5" ht="96" customHeight="1" s="1">
       <c r="A5" s="82" t="n"/>
       <c r="B5" s="80" t="inlineStr">
         <is>
@@ -4773,21 +5035,26 @@
       </c>
       <c r="D5" s="81" t="inlineStr">
         <is>
+          <t>预登录用户/HIP主机信息/设备对象/应用默认端口规避/会话结束日志等构建块</t>
+        </is>
+      </c>
+      <c r="E5" s="81" t="inlineStr">
+        <is>
           <t>PA规则构建块含预登录用户、HIP配置文件、设备对象、应用默认端口规避、会话结束日志等；天融信支持用户/应用/服务/日志构建块，但无HIP主机信息配置文件与设备对象等价物，仅有EDR联动上报终端资产并下发管控策略（天融信手册《与EDR联动》页）；对应矩阵#3/4</t>
         </is>
       </c>
-      <c r="E5" s="80" t="inlineStr">
+      <c r="F5" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F5" s="81" t="inlineStr"/>
-      <c r="G5" s="80" t="inlineStr">
+      <c r="G5" s="81" t="inlineStr"/>
+      <c r="H5" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H5" s="80" t="inlineStr"/>
+      <c r="I5" s="80" t="inlineStr"/>
     </row>
     <row r="6" ht="81" customHeight="1" s="1">
       <c r="A6" s="82" t="n"/>
@@ -4799,21 +5066,26 @@
       </c>
       <c r="D6" s="81" t="inlineStr">
         <is>
+          <t>端口(L4)规则一键迁移为应用(L7)规则+新应用查看器</t>
+        </is>
+      </c>
+      <c r="E6" s="81" t="inlineStr">
+        <is>
           <t>PA新应用查看器+端口规则迁移至App-ID规则工作流+规则使用统计，减少攻击面（PA Web帮助p142）；天融信策略统计开关可显示规则匹配命中情况（天融信手册《配置访问控制策略》页），但无新应用查看器与端口→应用规则迁移工作流；对应矩阵#132</t>
         </is>
       </c>
-      <c r="E6" s="80" t="inlineStr">
+      <c r="F6" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F6" s="81" t="inlineStr"/>
-      <c r="G6" s="80" t="inlineStr">
+      <c r="G6" s="81" t="inlineStr"/>
+      <c r="H6" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H6" s="80" t="inlineStr"/>
+      <c r="I6" s="80" t="inlineStr"/>
     </row>
     <row r="7" ht="36" customHeight="1" s="1">
       <c r="A7" s="82" t="n"/>
@@ -4825,17 +5097,22 @@
       </c>
       <c r="D7" s="81" t="inlineStr">
         <is>
+          <t>配置锁/提交锁，防止多管理员并发修改</t>
+        </is>
+      </c>
+      <c r="E7" s="81" t="inlineStr">
+        <is>
           <t>PA可锁定待选配置或提交，防止他管理员并发更改；对应矩阵#135（天融信不支持，PA优势）</t>
         </is>
       </c>
-      <c r="E7" s="82" t="n"/>
       <c r="F7" s="82" t="n"/>
-      <c r="G7" s="80" t="inlineStr">
+      <c r="G7" s="82" t="n"/>
+      <c r="H7" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H7" s="82" t="n"/>
+      <c r="I7" s="82" t="n"/>
     </row>
     <row r="8" ht="111" customHeight="1" s="1">
       <c r="A8" s="82" t="n"/>
@@ -4847,17 +5124,22 @@
       </c>
       <c r="D8" s="81" t="inlineStr">
         <is>
+          <t>应用匹配同时强制使用标准端口，非标端口拒绝</t>
+        </is>
+      </c>
+      <c r="E8" s="81" t="inlineStr">
+        <is>
           <t>PA安全策略默认服务为application-default：放行应用同时强制其使用标准端口（如SSH仅22），非标准端口不匹配即拦截（PA管理指南p904）；天融信策略为五元组+应用识别组合（天融信手册《配置访问控制策略》页）；迁移评估项：直接转换若仅保留应用识别不限端口将扩大安全敞口，需制定应用标准端口映射限制（App-Default）转换方案；对应矩阵#2</t>
         </is>
       </c>
-      <c r="E8" s="80" t="inlineStr">
+      <c r="F8" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F8" s="82" t="n"/>
       <c r="G8" s="82" t="n"/>
       <c r="H8" s="82" t="n"/>
+      <c r="I8" s="82" t="n"/>
     </row>
     <row r="9" ht="81" customHeight="1" s="1">
       <c r="A9" s="82" t="n"/>
@@ -4869,17 +5151,22 @@
       </c>
       <c r="D9" s="81" t="inlineStr">
         <is>
+          <t>Allow动作关联反病毒/漏洞防护/URL过滤/文件阻断/WildFire配置文件组</t>
+        </is>
+      </c>
+      <c r="E9" s="81" t="inlineStr">
+        <is>
           <t>PA安全策略Allow动作关联Profile组（反病毒/漏洞防护/URL过滤/文件阻止/WildFire等，PA Web帮助p304）；天融信一体化策略引擎自带检测项；迁移评估项：需评估Profile组到天融信各检测引擎的映射与缺省动作差异；对应矩阵#4</t>
         </is>
       </c>
-      <c r="E9" s="80" t="inlineStr">
+      <c r="F9" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F9" s="82" t="n"/>
       <c r="G9" s="82" t="n"/>
       <c r="H9" s="82" t="n"/>
+      <c r="I9" s="82" t="n"/>
     </row>
     <row r="10" ht="156" customHeight="1" s="1">
       <c r="A10" s="82" t="n"/>
@@ -4891,19 +5178,24 @@
       </c>
       <c r="D10" s="81" t="inlineStr">
         <is>
+          <t>同区域默认放行/跨区域默认拒绝，支持替代与日志转发</t>
+        </is>
+      </c>
+      <c r="E10" s="81" t="inlineStr">
+        <is>
           <t>PA安全策略库末尾自带两条隐式系统规则：区域内默认（同Zone默认放行）与区域间默认（跨Zone默认拒绝），可被替代配置，替代字段含日志转发配置文件与Log at Session End在会话结束时记录（PA Web帮助p134-136）；天融信未见同区域默认放行的隐式规则机制；迁移评估项：①必须提取intrazone-default同Zone互访需求并显式转换为放行规则，否则割接后同Zone不同网段/VLAN互访将被默认拦截；②需在新设备补齐底部兜底Deny-All并开启日志，否则被拒流量查无日志、排障困难</t>
         </is>
       </c>
-      <c r="E10" s="80" t="inlineStr">
+      <c r="F10" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F10" s="82" t="n"/>
       <c r="G10" s="82" t="n"/>
       <c r="H10" s="82" t="n"/>
-    </row>
-    <row r="11" ht="111" customHeight="1" s="1">
+      <c r="I10" s="82" t="n"/>
+    </row>
+    <row r="11" ht="126" customHeight="1" s="1">
       <c r="A11" s="82" t="n"/>
       <c r="B11" s="80" t="inlineStr">
         <is>
@@ -4917,21 +5209,26 @@
       </c>
       <c r="D11" s="81" t="inlineStr">
         <is>
+          <t>目的区域按NAT后路由查找；源/目的地址用NAT前值</t>
+        </is>
+      </c>
+      <c r="E11" s="81" t="inlineStr">
+        <is>
           <t>PA底层为『先NAT判断后安全策略匹配』的因果倒置：安全策略要求源区域(NAT前)+源地址(NAT前)+目的地址(NAT前)+目的区域(NAT后按路由查找)，极其反直觉；天融信地址转换为独立策略库常规直观映射（安全策略&gt;地址转换，天融信手册《服务器映射》页）；迁移评估项：带目的NAT的策略平移后易因Zone填写错误不通，需制定NAT查表逻辑转换映射规范；对应矩阵#9</t>
         </is>
       </c>
-      <c r="E11" s="80" t="inlineStr">
+      <c r="F11" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F11" s="81" t="inlineStr"/>
-      <c r="G11" s="80" t="inlineStr">
+      <c r="G11" s="81" t="inlineStr"/>
+      <c r="H11" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H11" s="80" t="inlineStr"/>
+      <c r="I11" s="80" t="inlineStr"/>
     </row>
     <row r="12" ht="81" customHeight="1" s="1">
       <c r="A12" s="82" t="n"/>
@@ -4943,21 +5240,26 @@
       </c>
       <c r="D12" s="81" t="inlineStr">
         <is>
+          <t>主动/主动HA下NAT规则绑定会话所有者</t>
+        </is>
+      </c>
+      <c r="E12" s="81" t="inlineStr">
+        <is>
           <t>PA主动/主动HA配置下NAT规则可绑定会话所有者/会话设置，控制NAT会话的设备绑定，仅A/A模式可见（PA Web帮助p150）；天融信HA为主备双机热备模式（天融信手册《配置双机热备功能》页），无主动/主动模式及NAT规则绑定机制</t>
         </is>
       </c>
-      <c r="E12" s="80" t="inlineStr">
+      <c r="F12" s="80" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="F12" s="81" t="inlineStr"/>
-      <c r="G12" s="80" t="inlineStr">
+      <c r="G12" s="81" t="inlineStr"/>
+      <c r="H12" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H12" s="80" t="inlineStr"/>
+      <c r="I12" s="80" t="inlineStr"/>
     </row>
     <row r="13" ht="96" customHeight="1" s="1">
       <c r="A13" s="82" t="n"/>
@@ -4973,23 +5275,28 @@
       </c>
       <c r="D13" s="81" t="inlineStr">
         <is>
+          <t>QoS规则按DSCP/ToS值匹配调度</t>
+        </is>
+      </c>
+      <c r="E13" s="81" t="inlineStr">
+        <is>
           <t>PA QoS规则可直接按DSCP值或IP优先级/ToS匹配调度（PA Web帮助p155）；天融信支持DSCP/802.1p(CoS)识别与重标记，但需在独立流量管理模块配置（虚拟通道+限制/保证带宽+通道优先级，天融信手册《流量管理》页），未直接耦合在基础访问控制策略表内（联网核实厂商流控资料，手册未详载）</t>
         </is>
       </c>
-      <c r="E13" s="80" t="inlineStr">
+      <c r="F13" s="80" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="F13" s="81" t="inlineStr"/>
-      <c r="G13" s="80" t="inlineStr">
+      <c r="G13" s="81" t="inlineStr"/>
+      <c r="H13" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H13" s="80" t="inlineStr"/>
-    </row>
-    <row r="14" ht="96" customHeight="1" s="1">
+      <c r="I13" s="80" t="inlineStr"/>
+    </row>
+    <row r="14" ht="111" customHeight="1" s="1">
       <c r="A14" s="82" t="n"/>
       <c r="B14" s="80" t="inlineStr">
         <is>
@@ -5003,21 +5310,26 @@
       </c>
       <c r="D14" s="81" t="inlineStr">
         <is>
+          <t>记录入接口MAC，回包强制原路返回</t>
+        </is>
+      </c>
+      <c r="E14" s="81" t="inlineStr">
+        <is>
           <t>PA对称返回：虚拟路由器替代返回流量的路由查找，将流量引导回接收SYN数据包的MAC地址（ARP表确定下一跳），双ISP双活/非对称路由核心机制（PA管理指南p1294）；天融信手册检索无对称返回/回程机制命中，策略路由与LLB的回程保障能力待验证；迁移评估项：多ISP双活环境需实测天融信回包路由对称性，否则现网业务中断</t>
         </is>
       </c>
-      <c r="E14" s="80" t="inlineStr">
+      <c r="F14" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F14" s="81" t="inlineStr"/>
-      <c r="G14" s="80" t="inlineStr">
+      <c r="G14" s="81" t="inlineStr"/>
+      <c r="H14" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H14" s="80" t="inlineStr"/>
+      <c r="I14" s="80" t="inlineStr"/>
     </row>
     <row r="15" ht="51" customHeight="1" s="1">
       <c r="A15" s="82" t="n"/>
@@ -5033,21 +5345,26 @@
       </c>
       <c r="D15" s="81" t="inlineStr">
         <is>
+          <t>解密后明文流量镜像至专用接口供第三方分析</t>
+        </is>
+      </c>
+      <c r="E15" s="81" t="inlineStr">
+        <is>
           <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证（PA管理指南p1059）；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
         </is>
       </c>
-      <c r="E15" s="80" t="inlineStr">
+      <c r="F15" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F15" s="81" t="inlineStr"/>
-      <c r="G15" s="80" t="inlineStr">
+      <c r="G15" s="81" t="inlineStr"/>
+      <c r="H15" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H15" s="80" t="inlineStr"/>
+      <c r="I15" s="80" t="inlineStr"/>
     </row>
     <row r="16" ht="126" customHeight="1" s="1">
       <c r="A16" s="82" t="n"/>
@@ -5059,21 +5376,26 @@
       </c>
       <c r="D16" s="81" t="inlineStr">
         <is>
+          <t>外部无效证书以不受信转发证书重签，保留浏览器告警</t>
+        </is>
+      </c>
+      <c r="E16" s="81" t="inlineStr">
+        <is>
           <t>PA转发代理遇外部过期/不受信证书时，不用内部信任CA重签，而是专用Forward Untrust Certificate重签名，让浏览器保留不受信告警（PA管理指南p994、p1030）；天融信SSL解密（透明代理/服务器SSL解密，天融信手册《代理策略》页）未见受信/不受信双证书体系；迁移评估项：需验证天融信对外部无效证书的处理方式，避免直接阻断（白屏）或信任重签（掩盖风险）</t>
         </is>
       </c>
-      <c r="E16" s="80" t="inlineStr">
+      <c r="F16" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F16" s="81" t="inlineStr"/>
-      <c r="G16" s="80" t="inlineStr">
+      <c r="G16" s="81" t="inlineStr"/>
+      <c r="H16" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H16" s="80" t="inlineStr"/>
+      <c r="I16" s="80" t="inlineStr"/>
     </row>
     <row r="17" ht="66" customHeight="1" s="1">
       <c r="A17" s="82" t="n"/>
@@ -5085,21 +5407,26 @@
       </c>
       <c r="D17" s="81" t="inlineStr">
         <is>
+          <t>按URL类别圈定解密范围，排除银行/医疗等敏感类</t>
+        </is>
+      </c>
+      <c r="E17" s="81" t="inlineStr">
+        <is>
           <t>PA解密规则可按URL类别（含自定义类别）选择解密范围，可排除银行/医疗等敏感类别不解密（PA Web帮助p164）；天融信SSL解密（代理策略/代理模板）无按URL类别选择解密机制（检索无命中）</t>
         </is>
       </c>
-      <c r="E17" s="80" t="inlineStr">
+      <c r="F17" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F17" s="82" t="n"/>
-      <c r="G17" s="80" t="inlineStr">
+      <c r="G17" s="82" t="n"/>
+      <c r="H17" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H17" s="82" t="n"/>
+      <c r="I17" s="82" t="n"/>
     </row>
     <row r="18" ht="96" customHeight="1" s="1">
       <c r="A18" s="82" t="n"/>
@@ -5111,13 +5438,18 @@
       </c>
       <c r="D18" s="81" t="inlineStr">
         <is>
+          <t>SSH代理解密+SSH隧道(ssh-tunnel)识别控制</t>
+        </is>
+      </c>
+      <c r="E18" s="81" t="inlineStr">
+        <is>
           <t>PA解密策略SSH Proxy类型解密SSH通信，可通过ssh-tunnel App-ID在策略中控制SSH隧道（端口转发/内网穿透），正常SSH管理流量放行；含不受支持算法检查/资源不足阻断会话等防护（PA Web帮助p164、p318-319）；天融信手册检索无SSH代理/SSH隧道控制命中</t>
         </is>
       </c>
-      <c r="E18" s="82" t="n"/>
       <c r="F18" s="82" t="n"/>
       <c r="G18" s="82" t="n"/>
       <c r="H18" s="82" t="n"/>
+      <c r="I18" s="82" t="n"/>
     </row>
     <row r="19" ht="66" customHeight="1" s="1">
       <c r="A19" s="82" t="n"/>
@@ -5133,21 +5465,26 @@
       </c>
       <c r="D19" s="81" t="inlineStr">
         <is>
+          <t>已解密/未解密流量内联转发第三方安全链，L3路由转发</t>
+        </is>
+      </c>
+      <c r="E19" s="81" t="inlineStr">
+        <is>
           <t>PA网络数据包代理策略将已解密/未解密TLS/非TLS流量内联转发至第三方安全工具，路径选择选项卡应用数据包代理配置文件定义经路由L3安全链的转发方式（PA Web帮助p167-170）；对应矩阵#122</t>
         </is>
       </c>
-      <c r="E19" s="80" t="inlineStr">
+      <c r="F19" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F19" s="81" t="inlineStr"/>
-      <c r="G19" s="80" t="inlineStr">
+      <c r="G19" s="81" t="inlineStr"/>
+      <c r="H19" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H19" s="80" t="inlineStr">
+      <c r="I19" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
@@ -5163,21 +5500,26 @@
       </c>
       <c r="D20" s="81" t="inlineStr">
         <is>
+          <t>TLS解密/未解密/非TLS流量类型选择</t>
+        </is>
+      </c>
+      <c r="E20" s="81" t="inlineStr">
+        <is>
           <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证（PA Web帮助p167）；天融信无网络数据包代理模块（矩阵#122）</t>
         </is>
       </c>
-      <c r="E20" s="80" t="inlineStr">
+      <c r="F20" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F20" s="81" t="inlineStr"/>
-      <c r="G20" s="80" t="inlineStr">
+      <c r="G20" s="81" t="inlineStr"/>
+      <c r="H20" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H20" s="80" t="inlineStr"/>
+      <c r="I20" s="80" t="inlineStr"/>
     </row>
     <row r="21" ht="66" customHeight="1" s="1">
       <c r="A21" s="82" t="n"/>
@@ -5193,21 +5535,26 @@
       </c>
       <c r="D21" s="81" t="inlineStr">
         <is>
+          <t>GRE/GTP-U/VXLAN/非加密IPSec隧道内层流量解封装检测</t>
+        </is>
+      </c>
+      <c r="E21" s="81" t="inlineStr">
+        <is>
           <t>PA隧道检测策略解封装并深度检测GRE/GTP-U/VXLAN/非加密IPSec（NULL加密/AH传输模式）等明文隧道内容（PA Web帮助p172-173）；对应矩阵#128/37</t>
         </is>
       </c>
-      <c r="E21" s="80" t="inlineStr">
+      <c r="F21" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F21" s="81" t="inlineStr"/>
-      <c r="G21" s="80" t="inlineStr">
+      <c r="G21" s="81" t="inlineStr"/>
+      <c r="H21" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H21" s="80" t="inlineStr">
+      <c r="I21" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
@@ -5223,21 +5570,26 @@
       </c>
       <c r="D22" s="81" t="inlineStr">
         <is>
+          <t>隧道嵌套封装最大级数限制，超限丢弃</t>
+        </is>
+      </c>
+      <c r="E22" s="81" t="inlineStr">
+        <is>
           <t>PA对隧道最大封装级数超限丢包防护，防隧道嵌套绕过（PA管理指南p655）；天融信手册无封装级数防护（检索无命中）</t>
         </is>
       </c>
-      <c r="E22" s="80" t="inlineStr">
+      <c r="F22" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F22" s="81" t="inlineStr"/>
-      <c r="G22" s="80" t="inlineStr">
+      <c r="G22" s="81" t="inlineStr"/>
+      <c r="H22" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H22" s="80" t="inlineStr"/>
+      <c r="I22" s="80" t="inlineStr"/>
     </row>
     <row r="23" ht="96" customHeight="1" s="1">
       <c r="A23" s="82" t="n"/>
@@ -5253,21 +5605,26 @@
       </c>
       <c r="D23" s="81" t="inlineStr">
         <is>
+          <t>匹配覆盖策略的流量跳过七层检测，四层快速转发</t>
+        </is>
+      </c>
+      <c r="E23" s="81" t="inlineStr">
+        <is>
           <t>PA应用替代策略明确绕过第7层处理与威胁检查，改用第4层状态检查以加速（PA管理指南p1307）；天融信自定义应用加入规则库后仍默认经安全引擎检测（天融信手册《自定义应用》页）；迁移评估项：PA应用替代多为私有大流量业务加速，转换时需同步关闭对应策略的IPS/七层检测，否则性能被拖垮或误阻断</t>
         </is>
       </c>
-      <c r="E23" s="80" t="inlineStr">
+      <c r="F23" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F23" s="81" t="inlineStr"/>
-      <c r="G23" s="80" t="inlineStr">
+      <c r="G23" s="81" t="inlineStr"/>
+      <c r="H23" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H23" s="80" t="inlineStr"/>
+      <c r="I23" s="80" t="inlineStr"/>
     </row>
     <row r="24" ht="81" customHeight="1" s="1">
       <c r="A24" s="82" t="n"/>
@@ -5283,21 +5640,26 @@
       </c>
       <c r="D24" s="81" t="inlineStr">
         <is>
+          <t>认证超时+单次认证(SSO)</t>
+        </is>
+      </c>
+      <c r="E24" s="81" t="inlineStr">
+        <is>
           <t>PA支持认证超时减少重复质询、Kerberos/SAML/RADIUS等对接（PA Web帮助p186）；天融信手册检索认证超时/单点登录/SSO无命中（仅在线用户在线时长查看与强制下线）；迁移评估项：需核实天融信认证会话有效期配置与SSO对接能力</t>
         </is>
       </c>
-      <c r="E24" s="80" t="inlineStr">
+      <c r="F24" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F24" s="81" t="inlineStr"/>
-      <c r="G24" s="80" t="inlineStr">
+      <c r="G24" s="81" t="inlineStr"/>
+      <c r="H24" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H24" s="80" t="inlineStr"/>
+      <c r="I24" s="80" t="inlineStr"/>
     </row>
     <row r="25" ht="126" customHeight="1" s="1">
       <c r="A25" s="82" t="n"/>
@@ -5309,23 +5671,28 @@
       </c>
       <c r="D25" s="81" t="inlineStr">
         <is>
+          <t>策略匹配触发多因素认证质询（MFA供应商API/RADIUS）</t>
+        </is>
+      </c>
+      <c r="E25" s="81" t="inlineStr">
+        <is>
           <t>PA身份验证策略通过Authentication Enforcement对象对匹配流量强制质询，支持多因素身份验证（每因素独立超时，防火墙记录时间戳），MFA供应商API/RADIUS对接（PA Web帮助p185-186、p310、p735-742）；天融信双因子认证（密码+短信/证书/Ukey）仅限管理员/用户登录场景（天融信手册《登录安全策略》页），未见流量策略触发MFA质询</t>
         </is>
       </c>
-      <c r="E25" s="80" t="inlineStr">
+      <c r="F25" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F25" s="81" t="inlineStr"/>
-      <c r="G25" s="80" t="inlineStr">
+      <c r="G25" s="81" t="inlineStr"/>
+      <c r="H25" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H25" s="80" t="inlineStr"/>
-    </row>
-    <row r="26" ht="81" customHeight="1" s="1">
+      <c r="I25" s="80" t="inlineStr"/>
+    </row>
+    <row r="26" ht="96" customHeight="1" s="1">
       <c r="A26" s="82" t="n"/>
       <c r="B26" s="82" t="n"/>
       <c r="C26" s="81" t="inlineStr">
@@ -5335,19 +5702,24 @@
       </c>
       <c r="D26" s="81" t="inlineStr">
         <is>
+          <t>AD域事件日志毫秒级IP-用户映射更新</t>
+        </is>
+      </c>
+      <c r="E26" s="81" t="inlineStr">
+        <is>
           <t>PA无代理架构通过读取域控事件日志实现IP-用户毫秒级动态映射，大规模部署有专项规划（PA管理指南p866-867）；天融信AD对接的轮询间隔与并发认证能力手册未量化；迁移评估项：数万AD用户且移动频繁场景需实测天融信映射更新时延，避免基于用户的策略出现间歇性未授权拦截</t>
         </is>
       </c>
-      <c r="E26" s="82" t="n"/>
       <c r="F26" s="82" t="n"/>
-      <c r="G26" s="80" t="inlineStr">
+      <c r="G26" s="82" t="n"/>
+      <c r="H26" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="H26" s="82" t="n"/>
-    </row>
-    <row r="27" ht="156" customHeight="1" s="1">
+      <c r="I26" s="82" t="n"/>
+    </row>
+    <row r="27" ht="171" customHeight="1" s="1">
       <c r="A27" s="82" t="n"/>
       <c r="B27" s="80" t="inlineStr">
         <is>
@@ -5361,21 +5733,26 @@
       </c>
       <c r="D27" s="81" t="inlineStr">
         <is>
+          <t>HTTP/HTTPS外部文本列表(IP/域名/URL)自动拉取，策略直接引用</t>
+        </is>
+      </c>
+      <c r="E27" s="81" t="inlineStr">
+        <is>
           <t>PA外部动态列表：基于HTTP/HTTPS托管的文本文件创建IP/URL/域名/IMEI/IMSI地址对象，防火墙定时自动拉取更新，策略中直接引用（Objects&gt;External Dynamic Lists，PA Web帮助p236-239；策略源/目标可直接选EDL，p196-197）；天融信手册检索外部动态列表/EDL无命中，仅内置威胁情报库与云端威胁情报库（规则集管理，天融信手册《威胁情报》《配置规则集》页），无策略直接引用任意外部文本列表机制；迁移评估项：PA策略中引用的EDL需转换为天融信静态地址组定期导入或威胁情报联动</t>
         </is>
       </c>
-      <c r="E27" s="80" t="inlineStr">
+      <c r="F27" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F27" s="81" t="inlineStr"/>
-      <c r="G27" s="80" t="inlineStr">
+      <c r="G27" s="81" t="inlineStr"/>
+      <c r="H27" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H27" s="80" t="inlineStr"/>
+      <c r="I27" s="80" t="inlineStr"/>
     </row>
     <row r="28" ht="126" customHeight="1" s="1">
       <c r="A28" s="82" t="n"/>
@@ -5387,21 +5764,26 @@
       </c>
       <c r="D28" s="81" t="inlineStr">
         <is>
+          <t>Tag标记过滤器动态地址组，成员随IP变化自动更新</t>
+        </is>
+      </c>
+      <c r="E28" s="81" t="inlineStr">
+        <is>
           <t>PA动态地址组：查找标记(Tag)+基于标记的过滤器（AND/OR匹配）动态填充成员，VM信息源注册或XML/REST API定义标记，IP变化时策略自动生效（PA Web帮助p207-208、p228）；天融信手册检索动态地址组/标签/SDN/云平台联动无命中，地址组为静态IP/子网绑定（天融信手册《地址》页）；迁移评估项：PA云环境Tag微隔离策略需转换为静态地址组，IP漂移场景需人工或API维护</t>
         </is>
       </c>
-      <c r="E28" s="80" t="inlineStr">
+      <c r="F28" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F28" s="81" t="inlineStr"/>
-      <c r="G28" s="80" t="inlineStr">
+      <c r="G28" s="81" t="inlineStr"/>
+      <c r="H28" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="H28" s="80" t="inlineStr"/>
+      <c r="I28" s="80" t="inlineStr"/>
     </row>
     <row r="29" ht="51" customHeight="1" s="1">
       <c r="A29" s="82" t="n"/>
@@ -5417,21 +5799,26 @@
       </c>
       <c r="D29" s="81" t="inlineStr">
         <is>
+          <t>按应用/区域/地址分配链路与流量分发</t>
+        </is>
+      </c>
+      <c r="E29" s="81" t="inlineStr">
+        <is>
           <t>PA SD-WAN策略按应用/抖动/延迟/丢包指标分配链路，流量分发（PA Web帮助p197）；对应矩阵#129/120</t>
         </is>
       </c>
-      <c r="E29" s="80" t="inlineStr">
+      <c r="F29" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="F29" s="81" t="inlineStr"/>
-      <c r="G29" s="80" t="inlineStr">
+      <c r="G29" s="81" t="inlineStr"/>
+      <c r="H29" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H29" s="80" t="inlineStr">
+      <c r="I29" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
@@ -5447,49 +5834,54 @@
       </c>
       <c r="D30" s="81" t="inlineStr">
         <is>
+          <t>抖动/延迟/丢包(jitter/latency/loss)指标选路</t>
+        </is>
+      </c>
+      <c r="E30" s="81" t="inlineStr">
+        <is>
           <t>PA路径质量配置文件基于抖动/延迟/丢包等运行状况指标选路（PA Web帮助p195）；天融信有链路探测(ping)+智能选路(最小延迟优先)（天融信手册《策略路由》页），无jitter/latency/loss多维指标</t>
         </is>
       </c>
-      <c r="E30" s="80" t="inlineStr">
+      <c r="F30" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F30" s="81" t="inlineStr"/>
-      <c r="G30" s="80" t="inlineStr">
+      <c r="G30" s="81" t="inlineStr"/>
+      <c r="H30" s="80" t="inlineStr">
         <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="H30" s="80" t="inlineStr"/>
+      <c r="I30" s="80" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="25">
     <mergeCell ref="B27:B28"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="G17:G18"/>
     <mergeCell ref="F25:F26"/>
-    <mergeCell ref="H16:H18"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="B11:B12"/>
     <mergeCell ref="B24:B26"/>
-    <mergeCell ref="G7:G10"/>
     <mergeCell ref="B29:B30"/>
     <mergeCell ref="A2:A30"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="F17:F18"/>
     <mergeCell ref="G3:G4"/>
-    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="G16:G18"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="I6:I10"/>
     <mergeCell ref="B19:B20"/>
-    <mergeCell ref="F16:F18"/>
+    <mergeCell ref="H7:H10"/>
     <mergeCell ref="H3:H4"/>
-    <mergeCell ref="F6:F10"/>
     <mergeCell ref="B15:B18"/>
     <mergeCell ref="B2:B4"/>
-    <mergeCell ref="H6:H10"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="I16:I18"/>
     <mergeCell ref="B5:B10"/>
-    <mergeCell ref="H25:H26"/>
+    <mergeCell ref="G6:G10"/>
     <mergeCell ref="B21:B22"/>
+    <mergeCell ref="F6:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: update PA migration comparison spreadsheet rows
Rewrite and refine multiple comparison table entries for feature support status:
1. Fix HIP/device object support details for security policies
2. Correct NPBroker and tunnel inspection support levels
3. Update MFA enforcement and QoS DSCP matching descriptions
4. Adjust SD-WAN strategy comparison context
5. Update the main PA spreadsheet file binary
</commit_message>
<xml_diff>
--- a/PA替代需求列表.xlsx
+++ b/PA替代需求列表.xlsx
@@ -3279,7 +3279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.7" customWidth="1" style="1" min="1" max="1"/>
@@ -3557,22 +3557,22 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="96" customHeight="1" s="1">
+    <row r="9" ht="51" customHeight="1" s="1">
       <c r="A9" s="84" t="n"/>
       <c r="B9" s="84" t="n"/>
       <c r="C9" s="81" t="inlineStr">
         <is>
-          <t>支持安全策略规则构建块：源用户/HIP/设备/应用/服务/日志等</t>
+          <t>支持HIP主机信息配置文件策略匹配（Host Information Profile）</t>
         </is>
       </c>
       <c r="D9" s="81" t="inlineStr">
         <is>
-          <t>预登录用户/HIP主机信息/设备对象/应用默认端口规避/会话结束日志等构建块</t>
+          <t>终端安全态势（补丁/杀软/磁盘加密等）作为策略匹配条件</t>
         </is>
       </c>
       <c r="E9" s="81" t="inlineStr">
         <is>
-          <t>PA规则构建块含预登录用户、HIP配置文件、设备对象、应用默认端口规避、会话结束日志等；天融信支持用户/应用/服务/日志构建块，但无HIP主机信息配置文件与设备对象等价物，仅有EDR联动上报终端资产并下发管控策略（天融信手册《与EDR联动》页）；对应矩阵#3/4</t>
+          <t>PA规则构建块支持HIP配置文件匹配终端安全态势（对应矩阵#3/4）；天融信手册检索HIP/主机信息配置文件无命中，无终端安全态势匹配等价物</t>
         </is>
       </c>
       <c r="F9" s="80" t="inlineStr">
@@ -3583,197 +3583,201 @@
       <c r="G9" s="81" t="inlineStr"/>
       <c r="H9" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
+          <t>不支持</t>
         </is>
       </c>
       <c r="I9" s="80" t="inlineStr"/>
     </row>
-    <row r="10" ht="81" customHeight="1" s="1">
+    <row r="10" ht="51" customHeight="1" s="1">
       <c r="A10" s="84" t="n"/>
       <c r="B10" s="84" t="n"/>
       <c r="C10" s="81" t="inlineStr">
         <is>
-          <t>支持安全策略优化器（Policy Optimizer）</t>
+          <t>支持终端设备对象作为策略匹配条件</t>
         </is>
       </c>
       <c r="D10" s="81" t="inlineStr">
         <is>
-          <t>端口(L4)规则一键迁移为应用(L7)规则+新应用查看器</t>
+          <t>终端设备类型（手机/平板/IoT等设备对象）作为策略构建块</t>
         </is>
       </c>
       <c r="E10" s="81" t="inlineStr">
         <is>
-          <t>PA新应用查看器+端口规则迁移至App-ID规则工作流+规则使用统计，减少攻击面（PA Web帮助p142）；天融信策略统计开关可显示规则匹配命中情况（天融信手册《配置访问控制策略》页），但无新应用查看器与端口→应用规则迁移工作流；对应矩阵#132</t>
-        </is>
-      </c>
-      <c r="F10" s="84" t="n"/>
+          <t>PA支持设备对象构建块（对应矩阵#3/4）；天融信经EDR联动上报终端资产并下发管控策略（天融信手册《与EDR联动》页），无独立设备对象</t>
+        </is>
+      </c>
+      <c r="F10" s="80" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
       <c r="G10" s="84" t="n"/>
-      <c r="H10" s="85" t="n"/>
+      <c r="H10" s="80" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
       <c r="I10" s="84" t="n"/>
     </row>
-    <row r="11" ht="36" customHeight="1" s="1">
+    <row r="11" ht="81" customHeight="1" s="1">
       <c r="A11" s="84" t="n"/>
       <c r="B11" s="84" t="n"/>
       <c r="C11" s="81" t="inlineStr">
         <is>
-          <t>支持配置锁（Config Lock/Commit Lock）</t>
+          <t>支持端口(L4)规则向应用(L7)规则迁移工作流（Policy Optimizer）</t>
         </is>
       </c>
       <c r="D11" s="81" t="inlineStr">
         <is>
-          <t>配置锁/提交锁，防止多管理员并发修改</t>
+          <t>端口规则一键迁移为应用规则+新应用查看器</t>
         </is>
       </c>
       <c r="E11" s="81" t="inlineStr">
         <is>
-          <t>PA可锁定待选配置或提交，防止他管理员并发更改；对应矩阵#135（天融信不支持，PA优势）</t>
-        </is>
-      </c>
-      <c r="F11" s="85" t="n"/>
+          <t>PA策略优化器提供新应用查看器与端口→App-ID规则迁移工作流（PA Web帮助p142）；天融信策略统计仅显示规则命中数（天融信手册《配置访问控制策略》页），无迁移工具（命中统计能力已另列已支持行）；对应矩阵#132</t>
+        </is>
+      </c>
+      <c r="F11" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
       <c r="G11" s="84" t="n"/>
       <c r="H11" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>不支持</t>
         </is>
       </c>
       <c r="I11" s="84" t="n"/>
     </row>
-    <row r="12" ht="111" customHeight="1" s="1">
+    <row r="12" ht="36" customHeight="1" s="1">
       <c r="A12" s="84" t="n"/>
       <c r="B12" s="84" t="n"/>
       <c r="C12" s="81" t="inlineStr">
         <is>
-          <t>支持应用默认端口绑定（Service: application-default）</t>
+          <t>支持配置锁（Config Lock/Commit Lock）</t>
         </is>
       </c>
       <c r="D12" s="81" t="inlineStr">
         <is>
-          <t>应用匹配同时强制使用标准端口，非标端口拒绝</t>
+          <t>配置锁/提交锁，防止多管理员并发修改</t>
         </is>
       </c>
       <c r="E12" s="81" t="inlineStr">
         <is>
-          <t>PA安全策略默认服务为application-default：放行应用同时强制其使用标准端口（如SSH仅22），非标准端口不匹配即拦截（PA管理指南p904）；天融信策略为五元组+应用识别组合（天融信手册《配置访问控制策略》页）；迁移评估项：直接转换若仅保留应用识别不限端口将扩大安全敞口，需制定应用标准端口映射限制（App-Default）转换方案；对应矩阵#2</t>
-        </is>
-      </c>
-      <c r="F12" s="80" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
+          <t>PA可锁定待选配置或提交，防止他管理员并发更改；对应矩阵#135（天融信不支持，PA优势）</t>
+        </is>
+      </c>
+      <c r="F12" s="85" t="n"/>
       <c r="G12" s="84" t="n"/>
-      <c r="H12" s="84" t="n"/>
+      <c r="H12" s="80" t="inlineStr">
+        <is>
+          <t>待评估</t>
+        </is>
+      </c>
       <c r="I12" s="84" t="n"/>
     </row>
-    <row r="13" ht="81" customHeight="1" s="1">
+    <row r="13" ht="111" customHeight="1" s="1">
       <c r="A13" s="84" t="n"/>
       <c r="B13" s="84" t="n"/>
       <c r="C13" s="81" t="inlineStr">
         <is>
-          <t>支持安全策略绑定安全配置文件组（Profile Group）</t>
+          <t>支持应用默认端口绑定（Service: application-default）</t>
         </is>
       </c>
       <c r="D13" s="81" t="inlineStr">
         <is>
-          <t>Allow动作关联反病毒/漏洞防护/URL过滤/文件阻断/WildFire配置文件组</t>
+          <t>应用匹配同时强制使用标准端口，非标端口拒绝</t>
         </is>
       </c>
       <c r="E13" s="81" t="inlineStr">
         <is>
-          <t>PA安全策略Allow动作关联Profile组（反病毒/漏洞防护/URL过滤/文件阻止/WildFire等，PA Web帮助p304）；天融信一体化策略引擎自带检测项；迁移评估项：需评估Profile组到天融信各检测引擎的映射与缺省动作差异；对应矩阵#4</t>
+          <t>PA安全策略默认服务为application-default：放行应用同时强制其使用标准端口（如SSH仅22），非标准端口不匹配即拦截（PA管理指南p904）；天融信策略为五元组+应用识别组合（天融信手册《配置访问控制策略》页）；迁移评估项：直接转换若仅保留应用识别不限端口将扩大安全敞口，需制定应用标准端口映射限制（App-Default）转换方案；对应矩阵#2</t>
         </is>
       </c>
       <c r="F13" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G13" s="84" t="n"/>
       <c r="H13" s="84" t="n"/>
       <c r="I13" s="84" t="n"/>
     </row>
-    <row r="14" ht="156" customHeight="1" s="1">
+    <row r="14" ht="81" customHeight="1" s="1">
       <c r="A14" s="84" t="n"/>
-      <c r="B14" s="85" t="n"/>
+      <c r="B14" s="84" t="n"/>
       <c r="C14" s="81" t="inlineStr">
         <is>
+          <t>支持安全策略绑定安全配置文件组（Profile Group）</t>
+        </is>
+      </c>
+      <c r="D14" s="81" t="inlineStr">
+        <is>
+          <t>Allow动作关联反病毒/漏洞防护/URL过滤/文件阻断/WildFire配置文件组</t>
+        </is>
+      </c>
+      <c r="E14" s="81" t="inlineStr">
+        <is>
+          <t>PA安全策略Allow动作关联Profile组（反病毒/漏洞防护/URL过滤/文件阻止/WildFire等，PA Web帮助p304）；天融信一体化策略引擎自带检测项；迁移评估项：需评估Profile组到天融信各检测引擎的映射与缺省动作差异；对应矩阵#4</t>
+        </is>
+      </c>
+      <c r="F14" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G14" s="84" t="n"/>
+      <c r="H14" s="84" t="n"/>
+      <c r="I14" s="84" t="n"/>
+    </row>
+    <row r="15" ht="156" customHeight="1" s="1">
+      <c r="A15" s="84" t="n"/>
+      <c r="B15" s="85" t="n"/>
+      <c r="C15" s="81" t="inlineStr">
+        <is>
           <t>支持隐式默认规则显式化迁移（intrazone/interzone-default）</t>
         </is>
       </c>
-      <c r="D14" s="81" t="inlineStr">
+      <c r="D15" s="81" t="inlineStr">
         <is>
           <t>同区域默认放行/跨区域默认拒绝，支持替代与日志转发</t>
         </is>
       </c>
-      <c r="E14" s="81" t="inlineStr">
+      <c r="E15" s="81" t="inlineStr">
         <is>
           <t>PA安全策略库末尾自带两条隐式系统规则：区域内默认（同Zone默认放行）与区域间默认（跨Zone默认拒绝），可被替代配置，替代字段含日志转发配置文件与Log at Session End在会话结束时记录（PA Web帮助p134-136）；天融信未见同区域默认放行的隐式规则机制；迁移评估项：①必须提取intrazone-default同Zone互访需求并显式转换为放行规则，否则割接后同Zone不同网段/VLAN互访将被默认拦截；②需在新设备补齐底部兜底Deny-All并开启日志，否则被拒流量查无日志、排障困难</t>
         </is>
       </c>
-      <c r="F14" s="80" t="inlineStr">
+      <c r="F15" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="G14" s="85" t="n"/>
-      <c r="H14" s="85" t="n"/>
-      <c r="I14" s="85" t="n"/>
-    </row>
-    <row r="15" ht="81" customHeight="1" s="1">
-      <c r="A15" s="84" t="n"/>
-      <c r="B15" s="80" t="inlineStr">
-        <is>
-          <t>NAT策略</t>
-        </is>
-      </c>
-      <c r="C15" s="81" t="inlineStr">
-        <is>
-          <t>支持源NAT（动态/PAT静态IP）与Hairpin回流</t>
-        </is>
-      </c>
-      <c r="D15" s="81" t="inlineStr">
-        <is>
-          <t>动态IP+端口(DIPP)/静态IP/接口地址，含回流(Hairpin)</t>
-        </is>
-      </c>
-      <c r="E15" s="81" t="inlineStr">
-        <is>
-          <t>PA源NAT含DIPP动态IP+端口/静态IP/接口地址/持久NAT等（PA Web帮助p147）；天融信SNAT地址池（多对一/多对多/一对一/PAT）与仅源IP转换等（天融信手册《源NAT》《配置源转换》页）；对应矩阵#6</t>
-        </is>
-      </c>
-      <c r="F15" s="80" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="G15" s="81" t="inlineStr"/>
-      <c r="H15" s="80" t="inlineStr">
-        <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I15" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
+      <c r="G15" s="85" t="n"/>
+      <c r="H15" s="85" t="n"/>
+      <c r="I15" s="85" t="n"/>
     </row>
     <row r="16" ht="81" customHeight="1" s="1">
       <c r="A16" s="84" t="n"/>
-      <c r="B16" s="84" t="n"/>
+      <c r="B16" s="80" t="inlineStr">
+        <is>
+          <t>NAT策略</t>
+        </is>
+      </c>
       <c r="C16" s="81" t="inlineStr">
         <is>
-          <t>支持目的NAT（端口映射/服务器发布）</t>
+          <t>支持源NAT（动态/PAT静态IP）与Hairpin回流</t>
         </is>
       </c>
       <c r="D16" s="81" t="inlineStr">
         <is>
-          <t>静态映射/端口转换/DNS重写/FQDN目标</t>
+          <t>动态IP+端口(DIPP)/静态IP/接口地址，含回流(Hairpin)</t>
         </is>
       </c>
       <c r="E16" s="81" t="inlineStr">
         <is>
-          <t>PA目标NAT含静态/动态IP、端口转换、DNS Rewrite、FQDN目标（PA Web帮助p149）；天融信服务器映射含静态映射+服务器负载均衡两种模式，NAT46/NAT66全系列（天融信手册《服务器映射》页）；对应矩阵#7</t>
+          <t>PA源NAT含DIPP动态IP+端口/静态IP/接口地址/持久NAT等（PA Web帮助p147）；天融信SNAT地址池（多对一/多对多/一对一/PAT）与仅源IP转换等（天融信手册《源NAT》《配置源转换》页）；对应矩阵#6</t>
         </is>
       </c>
       <c r="F16" s="80" t="inlineStr">
@@ -3787,50 +3791,62 @@
           <t>已支持</t>
         </is>
       </c>
-      <c r="I16" s="80" t="inlineStr"/>
+      <c r="I16" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="81" customHeight="1" s="1">
       <c r="A17" s="84" t="n"/>
       <c r="B17" s="84" t="n"/>
       <c r="C17" s="81" t="inlineStr">
         <is>
-          <t>支持静态/双向NAT一对一转换</t>
+          <t>支持目的NAT（端口映射/服务器发布）</t>
         </is>
       </c>
       <c r="D17" s="81" t="inlineStr">
         <is>
-          <t>一对一转换，支持双向映射</t>
+          <t>静态映射/端口转换/DNS重写/FQDN目标</t>
         </is>
       </c>
       <c r="E17" s="81" t="inlineStr">
         <is>
-          <t>PA支持静态IP转换与双向(Bi-directional)转换（PA Web帮助p148）；天融信支持一对一转换（SNAT地址池一对一/NAT66一对一）（天融信手册《源NAT》《配置一对一转换》页）；对应矩阵#8</t>
-        </is>
-      </c>
-      <c r="F17" s="84" t="n"/>
-      <c r="G17" s="84" t="n"/>
-      <c r="H17" s="84" t="n"/>
-      <c r="I17" s="84" t="n"/>
+          <t>PA目标NAT含静态/动态IP、端口转换、DNS Rewrite、FQDN目标（PA Web帮助p149）；天融信服务器映射含静态映射+服务器负载均衡两种模式，NAT46/NAT66全系列（天融信手册《服务器映射》页）；对应矩阵#7</t>
+        </is>
+      </c>
+      <c r="F17" s="80" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="G17" s="81" t="inlineStr"/>
+      <c r="H17" s="80" t="inlineStr">
+        <is>
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I17" s="80" t="inlineStr"/>
     </row>
     <row r="18" ht="81" customHeight="1" s="1">
       <c r="A18" s="84" t="n"/>
       <c r="B18" s="84" t="n"/>
       <c r="C18" s="81" t="inlineStr">
         <is>
-          <t>支持NAT与安全策略解耦独立配置</t>
+          <t>支持静态/双向NAT一对一转换</t>
         </is>
       </c>
       <c r="D18" s="81" t="inlineStr">
         <is>
-          <t>NAT独立策略库，先NAT后安全策略匹配</t>
+          <t>一对一转换，支持双向映射</t>
         </is>
       </c>
       <c r="E18" s="81" t="inlineStr">
         <is>
-          <t>PA NAT策略库独立于安全策略库(Policies&gt;NAT)，先NAT后安全匹配；天融信地址转换为独立策略库（安全策略&gt;地址转换），与访问控制策略分离配置（天融信手册《安全策略》《工作原理》页）；对应矩阵#9</t>
-        </is>
-      </c>
-      <c r="F18" s="85" t="n"/>
+          <t>PA支持静态IP转换与双向(Bi-directional)转换（PA Web帮助p148）；天融信支持一对一转换（SNAT地址池一对一/NAT66一对一）（天融信手册《源NAT》《配置一对一转换》页）；对应矩阵#8</t>
+        </is>
+      </c>
+      <c r="F18" s="84" t="n"/>
       <c r="G18" s="84" t="n"/>
       <c r="H18" s="84" t="n"/>
       <c r="I18" s="84" t="n"/>
@@ -3840,215 +3856,203 @@
       <c r="B19" s="84" t="n"/>
       <c r="C19" s="81" t="inlineStr">
         <is>
-          <t>支持IPv6/NAT64转换（nat64类型）</t>
+          <t>支持NAT与安全策略解耦独立配置</t>
         </is>
       </c>
       <c r="D19" s="81" t="inlineStr">
         <is>
-          <t>IPv4↔IPv6转换类型（nat64）</t>
+          <t>NAT独立策略库，先NAT后安全策略匹配</t>
         </is>
       </c>
       <c r="E19" s="81" t="inlineStr">
         <is>
-          <t>PA NAT规则支持IPv4/IPv6及NAT64转换类型（RFC6146）；天融信NAT64含静态转换+前缀转换+动态算法（IVI/普通前缀），另有NAT46（天融信手册《NAT64》《NAT46》页）；对应矩阵#18</t>
-        </is>
-      </c>
-      <c r="F19" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
+          <t>PA NAT策略库独立于安全策略库(Policies&gt;NAT)，先NAT后安全匹配；天融信地址转换为独立策略库（安全策略&gt;地址转换），与访问控制策略分离配置（天融信手册《安全策略》《工作原理》页）；对应矩阵#9</t>
+        </is>
+      </c>
+      <c r="F19" s="85" t="n"/>
       <c r="G19" s="84" t="n"/>
-      <c r="H19" s="85" t="n"/>
+      <c r="H19" s="84" t="n"/>
       <c r="I19" s="84" t="n"/>
     </row>
-    <row r="20" ht="126" customHeight="1" s="1">
+    <row r="20" ht="81" customHeight="1" s="1">
       <c r="A20" s="84" t="n"/>
       <c r="B20" s="84" t="n"/>
       <c r="C20" s="81" t="inlineStr">
         <is>
+          <t>支持IPv6/NAT64转换（nat64类型）</t>
+        </is>
+      </c>
+      <c r="D20" s="81" t="inlineStr">
+        <is>
+          <t>IPv4↔IPv6转换类型（nat64）</t>
+        </is>
+      </c>
+      <c r="E20" s="81" t="inlineStr">
+        <is>
+          <t>PA NAT规则支持IPv4/IPv6及NAT64转换类型（RFC6146）；天融信NAT64含静态转换+前缀转换+动态算法（IVI/普通前缀），另有NAT46（天融信手册《NAT64》《NAT46》页）；对应矩阵#18</t>
+        </is>
+      </c>
+      <c r="F20" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G20" s="84" t="n"/>
+      <c r="H20" s="85" t="n"/>
+      <c r="I20" s="84" t="n"/>
+    </row>
+    <row r="21" ht="126" customHeight="1" s="1">
+      <c r="A21" s="84" t="n"/>
+      <c r="B21" s="84" t="n"/>
+      <c r="C21" s="81" t="inlineStr">
+        <is>
           <t>支持NAT后目的区域路由回查匹配（Dest Zone by route lookup）</t>
         </is>
       </c>
-      <c r="D20" s="81" t="inlineStr">
+      <c r="D21" s="81" t="inlineStr">
         <is>
           <t>目的区域按NAT后路由查找；源/目的地址用NAT前值</t>
         </is>
       </c>
-      <c r="E20" s="81" t="inlineStr">
+      <c r="E21" s="81" t="inlineStr">
         <is>
           <t>PA底层为『先NAT判断后安全策略匹配』的因果倒置：安全策略要求源区域(NAT前)+源地址(NAT前)+目的地址(NAT前)+目的区域(NAT后按路由查找)，极其反直觉；天融信地址转换为独立策略库常规直观映射（安全策略&gt;地址转换，天融信手册《服务器映射》页）；迁移评估项：带目的NAT的策略平移后易因Zone填写错误不通，需制定NAT查表逻辑转换映射规范；对应矩阵#9</t>
         </is>
       </c>
-      <c r="F20" s="80" t="inlineStr">
+      <c r="F21" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="G20" s="84" t="n"/>
-      <c r="H20" s="80" t="inlineStr">
+      <c r="G21" s="84" t="n"/>
+      <c r="H21" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="I20" s="84" t="n"/>
-    </row>
-    <row r="21" ht="81" customHeight="1" s="1">
-      <c r="A21" s="84" t="n"/>
-      <c r="B21" s="85" t="n"/>
-      <c r="C21" s="81" t="inlineStr">
+      <c r="I21" s="84" t="n"/>
+    </row>
+    <row r="22" ht="81" customHeight="1" s="1">
+      <c r="A22" s="84" t="n"/>
+      <c r="B22" s="85" t="n"/>
+      <c r="C22" s="81" t="inlineStr">
         <is>
           <t>支持NAT规则主动/主动HA绑定（Active/Active HA Binding）</t>
         </is>
       </c>
-      <c r="D21" s="81" t="inlineStr">
+      <c r="D22" s="81" t="inlineStr">
         <is>
           <t>主动/主动HA下NAT规则绑定会话所有者</t>
         </is>
       </c>
-      <c r="E21" s="81" t="inlineStr">
+      <c r="E22" s="81" t="inlineStr">
         <is>
           <t>PA主动/主动HA配置下NAT规则可绑定会话所有者/会话设置，控制NAT会话的设备绑定，仅A/A模式可见（PA Web帮助p150）；天融信HA为主备双机热备模式（天融信手册《配置双机热备功能》页），无主动/主动模式及NAT规则绑定机制</t>
         </is>
       </c>
-      <c r="F21" s="80" t="inlineStr">
+      <c r="F22" s="80" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="G21" s="85" t="n"/>
-      <c r="H21" s="80" t="inlineStr">
+      <c r="G22" s="85" t="n"/>
+      <c r="H22" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="I21" s="85" t="n"/>
-    </row>
-    <row r="22" ht="96" customHeight="1" s="1">
-      <c r="A22" s="84" t="n"/>
-      <c r="B22" s="80" t="inlineStr">
-        <is>
-          <t>QoS策略</t>
-        </is>
-      </c>
-      <c r="C22" s="81" t="inlineStr">
-        <is>
-          <t>支持按应用/源地址/用户等定义QoS策略并划分优先级类</t>
-        </is>
-      </c>
-      <c r="D22" s="81" t="inlineStr">
-        <is>
-          <t>8类流量分类+4级优先级，保证/最大带宽控制</t>
-        </is>
-      </c>
-      <c r="E22" s="81" t="inlineStr">
-        <is>
-          <t>PA QoS策略规则分配QoS类（8类+4级优先级），按Egress Guaranteed/Max控制带宽（PA Web帮助p154-155）；天融信流量管理基于应用/用户/源目的区域/地址/服务/时间+通道优先级，虚拟通道限制与保证带宽（天融信手册《流量管理》页）；对应矩阵#33/66</t>
-        </is>
-      </c>
-      <c r="F22" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="G22" s="81" t="inlineStr"/>
-      <c r="H22" s="80" t="inlineStr">
-        <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I22" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
+      <c r="I22" s="85" t="n"/>
     </row>
     <row r="23" ht="96" customHeight="1" s="1">
       <c r="A23" s="84" t="n"/>
-      <c r="B23" s="85" t="n"/>
+      <c r="B23" s="80" t="inlineStr">
+        <is>
+          <t>QoS策略</t>
+        </is>
+      </c>
       <c r="C23" s="81" t="inlineStr">
         <is>
-          <t>支持基于DSCP/ToS值匹配的QoS</t>
+          <t>支持按应用/源地址/用户等定义QoS策略并划分优先级类</t>
         </is>
       </c>
       <c r="D23" s="81" t="inlineStr">
         <is>
-          <t>QoS规则按DSCP/ToS值匹配调度</t>
+          <t>8类流量分类+4级优先级，保证/最大带宽控制</t>
         </is>
       </c>
       <c r="E23" s="81" t="inlineStr">
         <is>
-          <t>PA QoS规则可直接按DSCP值或IP优先级/ToS匹配调度（PA Web帮助p155）；天融信支持DSCP/802.1p(CoS)识别与重标记，但需在独立流量管理模块配置（虚拟通道+限制/保证带宽+通道优先级，天融信手册《流量管理》页），未直接耦合在基础访问控制策略表内（联网核实厂商流控资料，手册未详载）</t>
+          <t>PA QoS策略规则分配QoS类（8类+4级优先级），按Egress Guaranteed/Max控制带宽（PA Web帮助p154-155）；天融信流量管理基于应用/用户/源目的区域/地址/服务/时间+通道优先级，虚拟通道限制与保证带宽（天融信手册《流量管理》页）；对应矩阵#33/66</t>
         </is>
       </c>
       <c r="F23" s="80" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G23" s="81" t="inlineStr"/>
       <c r="H23" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="I23" s="80" t="inlineStr"/>
-    </row>
-    <row r="24" ht="81" customHeight="1" s="1">
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I23" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="96" customHeight="1" s="1">
       <c r="A24" s="84" t="n"/>
-      <c r="B24" s="80" t="inlineStr">
-        <is>
-          <t>基于策略转发(PBF)</t>
-        </is>
-      </c>
+      <c r="B24" s="85" t="n"/>
       <c r="C24" s="81" t="inlineStr">
         <is>
-          <t>支持按源区域/地址/用户/应用/服务+下一跳的基于策略转发</t>
+          <t>支持QoS策略规则内直接按DSCP/ToS匹配调度</t>
         </is>
       </c>
       <c r="D24" s="81" t="inlineStr">
         <is>
-          <t>按源区域/地址/用户/应用/服务+下一跳转发，路径监控失效切换</t>
+          <t>QoS策略规则DSCP/ToS直接匹配（非独立流控模块配置）</t>
         </is>
       </c>
       <c r="E24" s="81" t="inlineStr">
         <is>
-          <t>PA PBF策略绕过常规路由表选路，支持路径监控与失效切换、BFD、强制对称返回（PA Web帮助p156）；天融信策略路由按源/目的地址端口、ISP名称、协议、角色等参数选路（天融信手册《策略路由》页）；对应矩阵#10</t>
+          <t>PA QoS规则可直接按DSCP值或IP优先级/ToS匹配调度（PA Web帮助p155）；天融信支持DSCP/802.1p(CoS)识别与重标记，但需在独立流量管理模块配置（虚拟通道+限制/保证带宽+通道优先级，天融信手册《流量管理》页），未直接耦合在基础访问控制策略表内（联网核实厂商流控资料，手册未详载）</t>
         </is>
       </c>
       <c r="F24" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>低</t>
         </is>
       </c>
       <c r="G24" s="81" t="inlineStr"/>
       <c r="H24" s="80" t="inlineStr">
         <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I24" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="111" customHeight="1" s="1">
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="I24" s="80" t="inlineStr"/>
+    </row>
+    <row r="25" ht="81" customHeight="1" s="1">
       <c r="A25" s="84" t="n"/>
-      <c r="B25" s="85" t="n"/>
+      <c r="B25" s="80" t="inlineStr">
+        <is>
+          <t>基于策略转发(PBF)</t>
+        </is>
+      </c>
       <c r="C25" s="81" t="inlineStr">
         <is>
-          <t>支持PBF强制对称返回（非对称路由环境）</t>
+          <t>支持按源区域/地址/用户/应用/服务+下一跳的基于策略转发</t>
         </is>
       </c>
       <c r="D25" s="81" t="inlineStr">
         <is>
-          <t>记录入接口MAC，回包强制原路返回</t>
+          <t>按源区域/地址/用户/应用/服务+下一跳转发，路径监控失效切换</t>
         </is>
       </c>
       <c r="E25" s="81" t="inlineStr">
         <is>
-          <t>PA对称返回：虚拟路由器替代返回流量的路由查找，将流量引导回接收SYN数据包的MAC地址（ARP表确定下一跳），双ISP双活/非对称路由核心机制（PA管理指南p1294）；天融信手册检索无对称返回/回程机制命中，策略路由与LLB的回程保障能力待验证；迁移评估项：多ISP双活环境需实测天融信回包路由对称性，否则现网业务中断</t>
+          <t>PA PBF策略绕过常规路由表选路，支持路径监控与失效切换、BFD、强制对称返回（PA Web帮助p156）；天融信策略路由按源/目的地址端口、ISP名称、协议、角色等参数选路（天融信手册《策略路由》页）；对应矩阵#10</t>
         </is>
       </c>
       <c r="F25" s="80" t="inlineStr">
@@ -4059,31 +4063,31 @@
       <c r="G25" s="81" t="inlineStr"/>
       <c r="H25" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
-        </is>
-      </c>
-      <c r="I25" s="80" t="inlineStr"/>
-    </row>
-    <row r="26" ht="96" customHeight="1" s="1">
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I25" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="111" customHeight="1" s="1">
       <c r="A26" s="84" t="n"/>
-      <c r="B26" s="80" t="inlineStr">
-        <is>
-          <t>解密策略(Decryption)</t>
-        </is>
-      </c>
+      <c r="B26" s="85" t="n"/>
       <c r="C26" s="81" t="inlineStr">
         <is>
-          <t>支持SSL/TLS解密策略（出站正向/入站反向）</t>
+          <t>支持PBF强制对称返回（非对称路由环境）</t>
         </is>
       </c>
       <c r="D26" s="81" t="inlineStr">
         <is>
-          <t>出站正向代理+入站检查双向解密</t>
+          <t>记录入接口MAC，回包强制原路返回</t>
         </is>
       </c>
       <c r="E26" s="81" t="inlineStr">
         <is>
-          <t>PA解密策略区分SSL Forward Proxy/Inbound Inspection/SSH，可解密以获得流量可见性与深度检测（PA Web帮助p164）；天融信代理策略将NGFW作为代理服务器，对加密流量解密还原明文完成内容安全检查后重新加密（天融信手册《代理策略》页）；对应矩阵#29/30</t>
+          <t>PA对称返回：虚拟路由器替代返回流量的路由查找，将流量引导回接收SYN数据包的MAC地址（ARP表确定下一跳），双ISP双活/非对称路由核心机制（PA管理指南p1294）；天融信手册检索无对称返回/回程机制命中，策略路由与LLB的回程保障能力待验证；迁移评估项：多ISP双活环境需实测天融信回包路由对称性，否则现网业务中断</t>
         </is>
       </c>
       <c r="F26" s="80" t="inlineStr">
@@ -4094,36 +4098,36 @@
       <c r="G26" s="81" t="inlineStr"/>
       <c r="H26" s="80" t="inlineStr">
         <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I26" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="66" customHeight="1" s="1">
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="I26" s="80" t="inlineStr"/>
+    </row>
+    <row r="27" ht="96" customHeight="1" s="1">
       <c r="A27" s="84" t="n"/>
-      <c r="B27" s="84" t="n"/>
+      <c r="B27" s="80" t="inlineStr">
+        <is>
+          <t>解密策略(Decryption)</t>
+        </is>
+      </c>
       <c r="C27" s="81" t="inlineStr">
         <is>
-          <t>支持解密目标选择与证书配置</t>
+          <t>支持SSL/TLS解密策略（出站正向/入站反向）</t>
         </is>
       </c>
       <c r="D27" s="81" t="inlineStr">
         <is>
-          <t>入站证书配置/解密目标（数据包/会话）</t>
+          <t>出站正向代理+入站检查双向解密</t>
         </is>
       </c>
       <c r="E27" s="81" t="inlineStr">
         <is>
-          <t>PA解密目标允许指定数据包/会话；入站含Certificates证书配置；对应矩阵#31；天融信代理模板支持证书选择与预置动态证书模板（天融信手册《代理模板》页）</t>
+          <t>PA解密策略区分SSL Forward Proxy/Inbound Inspection/SSH，可解密以获得流量可见性与深度检测（PA Web帮助p164）；天融信代理策略将NGFW作为代理服务器，对加密流量解密还原明文完成内容安全检查后重新加密（天融信手册《代理策略》页）；对应矩阵#29/30</t>
         </is>
       </c>
       <c r="F27" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G27" s="81" t="inlineStr"/>
@@ -4132,180 +4136,180 @@
           <t>已支持</t>
         </is>
       </c>
-      <c r="I27" s="80" t="inlineStr"/>
-    </row>
-    <row r="28" ht="51" customHeight="1" s="1">
+      <c r="I27" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="66" customHeight="1" s="1">
       <c r="A28" s="84" t="n"/>
       <c r="B28" s="84" t="n"/>
       <c r="C28" s="81" t="inlineStr">
         <is>
-          <t>支持解密流量镜像到专用接口（Decryption Port Mirroring）</t>
+          <t>支持解密目标选择与证书配置</t>
         </is>
       </c>
       <c r="D28" s="81" t="inlineStr">
         <is>
-          <t>解密后明文流量镜像至专用接口供第三方分析</t>
+          <t>入站证书配置/解密目标（数据包/会话）</t>
         </is>
       </c>
       <c r="E28" s="81" t="inlineStr">
         <is>
-          <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证（PA管理指南p1059）；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
-        </is>
-      </c>
-      <c r="F28" s="85" t="n"/>
-      <c r="G28" s="84" t="n"/>
+          <t>PA解密目标允许指定数据包/会话；入站含Certificates证书配置；对应矩阵#31；天融信代理模板支持证书选择与预置动态证书模板（天融信手册《代理模板》页）</t>
+        </is>
+      </c>
+      <c r="F28" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G28" s="81" t="inlineStr"/>
       <c r="H28" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="I28" s="84" t="n"/>
-    </row>
-    <row r="29" ht="126" customHeight="1" s="1">
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I28" s="80" t="inlineStr"/>
+    </row>
+    <row r="29" ht="51" customHeight="1" s="1">
       <c r="A29" s="84" t="n"/>
       <c r="B29" s="84" t="n"/>
       <c r="C29" s="81" t="inlineStr">
         <is>
-          <t>支持解密不受信证书分离处理（Forward Untrust Certificate）</t>
+          <t>支持解密流量镜像到专用接口（Decryption Port Mirroring）</t>
         </is>
       </c>
       <c r="D29" s="81" t="inlineStr">
         <is>
-          <t>外部无效证书以不受信转发证书重签，保留浏览器告警</t>
+          <t>解密后明文流量镜像至专用接口供第三方分析</t>
         </is>
       </c>
       <c r="E29" s="81" t="inlineStr">
         <is>
-          <t>PA转发代理遇外部过期/不受信证书时，不用内部信任CA重签，而是专用Forward Untrust Certificate重签名，让浏览器保留不受信告警（PA管理指南p994、p1030）；天融信SSL解密（透明代理/服务器SSL解密，天融信手册《代理策略》页）未见受信/不受信双证书体系；迁移评估项：需验证天融信对外部无效证书的处理方式，避免直接阻断（白屏）或信任重签（掩盖风险）</t>
-        </is>
-      </c>
-      <c r="F29" s="80" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
+          <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证（PA管理指南p1059）；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
+        </is>
+      </c>
+      <c r="F29" s="85" t="n"/>
       <c r="G29" s="84" t="n"/>
       <c r="H29" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>不支持</t>
         </is>
       </c>
       <c r="I29" s="84" t="n"/>
     </row>
-    <row r="30" ht="66" customHeight="1" s="1">
+    <row r="30" ht="126" customHeight="1" s="1">
       <c r="A30" s="84" t="n"/>
       <c r="B30" s="84" t="n"/>
       <c r="C30" s="81" t="inlineStr">
         <is>
-          <t>支持解密规则按URL类别选择性解密（URL Category）</t>
+          <t>支持解密不受信证书分离处理（Forward Untrust Certificate）</t>
         </is>
       </c>
       <c r="D30" s="81" t="inlineStr">
         <is>
-          <t>按URL类别圈定解密范围，排除银行/医疗等敏感类</t>
+          <t>外部无效证书以不受信转发证书重签，保留浏览器告警</t>
         </is>
       </c>
       <c r="E30" s="81" t="inlineStr">
         <is>
-          <t>PA解密规则可按URL类别（含自定义类别）选择解密范围，可排除银行/医疗等敏感类别不解密（PA Web帮助p164）；天融信SSL解密（代理策略/代理模板）无按URL类别选择解密机制（检索无命中）</t>
+          <t>PA转发代理遇外部过期/不受信证书时，不用内部信任CA重签，而是专用Forward Untrust Certificate重签名，让浏览器保留不受信告警（PA管理指南p994、p1030）；天融信SSL解密（透明代理/服务器SSL解密，天融信手册《代理策略》页）未见受信/不受信双证书体系；迁移评估项：需验证天融信对外部无效证书的处理方式，避免直接阻断（白屏）或信任重签（掩盖风险）</t>
         </is>
       </c>
       <c r="F30" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G30" s="84" t="n"/>
       <c r="H30" s="80" t="inlineStr">
         <is>
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="I30" s="84" t="n"/>
+    </row>
+    <row r="31" ht="66" customHeight="1" s="1">
+      <c r="A31" s="84" t="n"/>
+      <c r="B31" s="84" t="n"/>
+      <c r="C31" s="81" t="inlineStr">
+        <is>
+          <t>支持解密规则按URL类别选择性解密（URL Category）</t>
+        </is>
+      </c>
+      <c r="D31" s="81" t="inlineStr">
+        <is>
+          <t>按URL类别圈定解密范围，排除银行/医疗等敏感类</t>
+        </is>
+      </c>
+      <c r="E31" s="81" t="inlineStr">
+        <is>
+          <t>PA解密规则可按URL类别（含自定义类别）选择解密范围，可排除银行/医疗等敏感类别不解密（PA Web帮助p164）；天融信SSL解密（代理策略/代理模板）无按URL类别选择解密机制（检索无命中）</t>
+        </is>
+      </c>
+      <c r="F31" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G31" s="84" t="n"/>
+      <c r="H31" s="80" t="inlineStr">
+        <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="I30" s="84" t="n"/>
-    </row>
-    <row r="31" ht="96" customHeight="1" s="1">
-      <c r="A31" s="84" t="n"/>
-      <c r="B31" s="85" t="n"/>
-      <c r="C31" s="81" t="inlineStr">
+      <c r="I31" s="84" t="n"/>
+    </row>
+    <row r="32" ht="96" customHeight="1" s="1">
+      <c r="A32" s="84" t="n"/>
+      <c r="B32" s="85" t="n"/>
+      <c r="C32" s="81" t="inlineStr">
         <is>
           <t>支持SSH代理解密与SSH隧道控制（SSH Proxy）</t>
         </is>
       </c>
-      <c r="D31" s="81" t="inlineStr">
+      <c r="D32" s="81" t="inlineStr">
         <is>
           <t>SSH代理解密+SSH隧道(ssh-tunnel)识别控制</t>
         </is>
       </c>
-      <c r="E31" s="81" t="inlineStr">
+      <c r="E32" s="81" t="inlineStr">
         <is>
           <t>PA解密策略SSH Proxy类型解密SSH通信，可通过ssh-tunnel App-ID在策略中控制SSH隧道（端口转发/内网穿透），正常SSH管理流量放行；含不受支持算法检查/资源不足阻断会话等防护（PA Web帮助p164、p318-319）；天融信手册检索无SSH代理/SSH隧道控制命中</t>
         </is>
       </c>
-      <c r="F31" s="85" t="n"/>
-      <c r="G31" s="85" t="n"/>
-      <c r="H31" s="85" t="n"/>
-      <c r="I31" s="85" t="n"/>
-    </row>
-    <row r="32" ht="66" customHeight="1" s="1">
-      <c r="A32" s="84" t="n"/>
-      <c r="B32" s="80" t="inlineStr">
+      <c r="F32" s="85" t="n"/>
+      <c r="G32" s="85" t="n"/>
+      <c r="H32" s="85" t="n"/>
+      <c r="I32" s="85" t="n"/>
+    </row>
+    <row r="33" ht="111" customHeight="1" s="1">
+      <c r="A33" s="84" t="n"/>
+      <c r="B33" s="80" t="inlineStr">
         <is>
           <t>网络数据包代理(NPBroker)</t>
         </is>
       </c>
-      <c r="C32" s="81" t="inlineStr">
-        <is>
-          <t>支持按应用/用户/区域/设备/IP定义NPBroker规则转发到第三方安全链</t>
-        </is>
-      </c>
-      <c r="D32" s="81" t="inlineStr">
+      <c r="C33" s="81" t="inlineStr">
+        <is>
+          <t>支持内联数据包代理策略将流量转发第三方安全链（NPBroker）</t>
+        </is>
+      </c>
+      <c r="D33" s="81" t="inlineStr">
         <is>
           <t>已解密/未解密流量内联转发第三方安全链，L3路由转发</t>
         </is>
       </c>
-      <c r="E32" s="81" t="inlineStr">
-        <is>
-          <t>PA网络数据包代理策略将已解密/未解密TLS/非TLS流量内联转发至第三方安全工具，路径选择选项卡应用数据包代理配置文件定义经路由L3安全链的转发方式（PA Web帮助p167-170）；对应矩阵#122</t>
-        </is>
-      </c>
-      <c r="F32" s="80" t="inlineStr">
+      <c r="E33" s="81" t="inlineStr">
+        <is>
+          <t>PA网络数据包代理策略将已解密/未解密TLS/非TLS流量内联转发至第三方安全工具，路径选择选项卡应用数据包代理配置文件定义经路由L3安全链的转发方式（PA Web帮助p167-170）；天融信无网络数据包代理模块，最接近手段为WAF旁路联动（经交换机镜像引流，天融信手册《与WAF联动》页），非内联且无回注路径；对应矩阵#122</t>
+        </is>
+      </c>
+      <c r="F33" s="80" t="inlineStr">
         <is>
           <t>高</t>
-        </is>
-      </c>
-      <c r="G32" s="81" t="inlineStr"/>
-      <c r="H32" s="80" t="inlineStr">
-        <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="I32" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="66" customHeight="1" s="1">
-      <c r="A33" s="84" t="n"/>
-      <c r="B33" s="85" t="n"/>
-      <c r="C33" s="81" t="inlineStr">
-        <is>
-          <t>支持NPBroker转发流量类型选择（TLS解密/未解密/非TLS）</t>
-        </is>
-      </c>
-      <c r="D33" s="81" t="inlineStr">
-        <is>
-          <t>TLS解密/未解密/非TLS流量类型选择</t>
-        </is>
-      </c>
-      <c r="E33" s="81" t="inlineStr">
-        <is>
-          <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证（PA Web帮助p167）；天融信无网络数据包代理模块（矩阵#122）</t>
-        </is>
-      </c>
-      <c r="F33" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
         </is>
       </c>
       <c r="G33" s="81" t="inlineStr"/>
@@ -4314,63 +4318,63 @@
           <t>不支持</t>
         </is>
       </c>
-      <c r="I33" s="80" t="inlineStr"/>
+      <c r="I33" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="66" customHeight="1" s="1">
       <c r="A34" s="84" t="n"/>
-      <c r="B34" s="80" t="inlineStr">
-        <is>
-          <t>隧道检测(Tunnel Inspection)</t>
-        </is>
-      </c>
+      <c r="B34" s="85" t="n"/>
       <c r="C34" s="81" t="inlineStr">
         <is>
-          <t>支持GRE/GTP-U/HTTP2等明文隧道内层流量检测</t>
+          <t>支持NPBroker转发流量类型选择（TLS解密/未解密/非TLS）</t>
         </is>
       </c>
       <c r="D34" s="81" t="inlineStr">
         <is>
-          <t>GRE/GTP-U/VXLAN/非加密IPSec隧道内层流量解封装检测</t>
+          <t>TLS解密/未解密/非TLS流量类型选择</t>
         </is>
       </c>
       <c r="E34" s="81" t="inlineStr">
         <is>
-          <t>PA隧道检测策略解封装并深度检测GRE/GTP-U/VXLAN/非加密IPSec（NULL加密/AH传输模式）等明文隧道内容（PA Web帮助p172-173）；对应矩阵#128/37</t>
+          <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证（PA Web帮助p167）；天融信无网络数据包代理模块（矩阵#122）</t>
         </is>
       </c>
       <c r="F34" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G34" s="81" t="inlineStr"/>
       <c r="H34" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="I34" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="51" customHeight="1" s="1">
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I34" s="80" t="inlineStr"/>
+    </row>
+    <row r="35" ht="66" customHeight="1" s="1">
       <c r="A35" s="84" t="n"/>
-      <c r="B35" s="85" t="n"/>
+      <c r="B35" s="80" t="inlineStr">
+        <is>
+          <t>隧道检测(Tunnel Inspection)</t>
+        </is>
+      </c>
       <c r="C35" s="81" t="inlineStr">
         <is>
-          <t>支持最大封装级数防护（max_encap）</t>
+          <t>支持GRE隧道终结与内层流量检测</t>
         </is>
       </c>
       <c r="D35" s="81" t="inlineStr">
         <is>
-          <t>隧道嵌套封装最大级数限制，超限丢弃</t>
+          <t>GRE隧道封装/解封装，内层流量按普通流量检测</t>
         </is>
       </c>
       <c r="E35" s="81" t="inlineStr">
         <is>
-          <t>PA对隧道最大封装级数超限丢包防护，防隧道嵌套绕过（PA管理指南p655）；天融信手册无封装级数防护（检索无命中）</t>
+          <t>PA隧道检测策略解封装并检测GRE隧道内容（PA Web帮助p172-173）；天融信GRE隧道支持封装与解封装，解封装后内层报文按普通流量处理检测（天融信手册《GRE隧道》页）；对应矩阵#128/37</t>
         </is>
       </c>
       <c r="F35" s="80" t="inlineStr">
@@ -4381,137 +4385,133 @@
       <c r="G35" s="81" t="inlineStr"/>
       <c r="H35" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="I35" s="80" t="inlineStr"/>
-    </row>
-    <row r="36" ht="81" customHeight="1" s="1">
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I35" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="96" customHeight="1" s="1">
       <c r="A36" s="84" t="n"/>
-      <c r="B36" s="80" t="inlineStr">
-        <is>
-          <t>应用覆盖(App Override)</t>
-        </is>
-      </c>
+      <c r="B36" s="84" t="n"/>
       <c r="C36" s="81" t="inlineStr">
         <is>
-          <t>支持通过Application Override重定义应用识别</t>
+          <t>支持GTP-U/VXLAN/非加密IPSec隧道内层检测</t>
         </is>
       </c>
       <c r="D36" s="81" t="inlineStr">
         <is>
-          <t>按协议/端口自定义应用识别结果</t>
+          <t>GTP-U/VXLAN/NULL加密IPSec(AH)隧道内层流量检测</t>
         </is>
       </c>
       <c r="E36" s="81" t="inlineStr">
         <is>
-          <t>PA应用替代策略改变防火墙对网络通信的应用分类方式（如指定明文协议/端口识别，PA Web帮助p178）；天融信自定义应用允许管理员按需自定义应用协议（含端口匹配）并加入应用规则库（天融信手册《自定义应用》页）；对应矩阵#26</t>
+          <t>PA隧道检测支持GTP-U/VXLAN/非加密IPSec（NULL加密/AH传输模式）内层检测（PA Web帮助p172-173）；天融信VXLAN仅隧道封装转发与三层网关（天融信手册《业务接入端》《三层VXLAN网关》页），无内层安全检测，GTP检测检索无命中；对应矩阵#128/37</t>
         </is>
       </c>
       <c r="F36" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G36" s="81" t="inlineStr"/>
       <c r="H36" s="80" t="inlineStr">
         <is>
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I36" s="80" t="inlineStr"/>
+    </row>
+    <row r="37" ht="51" customHeight="1" s="1">
+      <c r="A37" s="84" t="n"/>
+      <c r="B37" s="85" t="n"/>
+      <c r="C37" s="81" t="inlineStr">
+        <is>
+          <t>支持最大封装级数防护（max_encap）</t>
+        </is>
+      </c>
+      <c r="D37" s="81" t="inlineStr">
+        <is>
+          <t>隧道嵌套封装最大级数限制，超限丢弃</t>
+        </is>
+      </c>
+      <c r="E37" s="81" t="inlineStr">
+        <is>
+          <t>PA对隧道最大封装级数超限丢包防护，防隧道嵌套绕过（PA管理指南p655）；天融信手册无封装级数防护（检索无命中）</t>
+        </is>
+      </c>
+      <c r="F37" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G37" s="85" t="n"/>
+      <c r="H37" s="85" t="n"/>
+      <c r="I37" s="85" t="n"/>
+    </row>
+    <row r="38" ht="81" customHeight="1" s="1">
+      <c r="A38" s="84" t="n"/>
+      <c r="B38" s="80" t="inlineStr">
+        <is>
+          <t>应用覆盖(App Override)</t>
+        </is>
+      </c>
+      <c r="C38" s="81" t="inlineStr">
+        <is>
+          <t>支持通过Application Override重定义应用识别</t>
+        </is>
+      </c>
+      <c r="D38" s="81" t="inlineStr">
+        <is>
+          <t>按协议/端口自定义应用识别结果</t>
+        </is>
+      </c>
+      <c r="E38" s="81" t="inlineStr">
+        <is>
+          <t>PA应用替代策略改变防火墙对网络通信的应用分类方式（如指定明文协议/端口识别，PA Web帮助p178）；天融信自定义应用允许管理员按需自定义应用协议（含端口匹配）并加入应用规则库（天融信手册《自定义应用》页）；对应矩阵#26</t>
+        </is>
+      </c>
+      <c r="F38" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G38" s="81" t="inlineStr"/>
+      <c r="H38" s="80" t="inlineStr">
+        <is>
           <t>已支持</t>
         </is>
       </c>
-      <c r="I36" s="80" t="inlineStr">
+      <c r="I38" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="66" customHeight="1" s="1">
-      <c r="A37" s="84" t="n"/>
-      <c r="B37" s="84" t="n"/>
-      <c r="C37" s="81" t="inlineStr">
+    <row r="39" ht="66" customHeight="1" s="1">
+      <c r="A39" s="84" t="n"/>
+      <c r="B39" s="84" t="n"/>
+      <c r="C39" s="81" t="inlineStr">
         <is>
           <t>支持覆盖类型（端口映射类）识别</t>
         </is>
       </c>
-      <c r="D37" s="81" t="inlineStr">
+      <c r="D39" s="81" t="inlineStr">
         <is>
           <t>端口映射类覆盖识别</t>
         </is>
       </c>
-      <c r="E37" s="81" t="inlineStr">
+      <c r="E39" s="81" t="inlineStr">
         <is>
           <t>PA支持端口式应用覆盖识别（configurable自定义应用）；天融信自定义应用允许管理员按特定需要自行定义应用协议（含端口匹配），自动添加到应用规则库供安全策略引用（天融信手册《自定义应用》页）</t>
         </is>
       </c>
-      <c r="F37" s="80" t="inlineStr">
+      <c r="F39" s="80" t="inlineStr">
         <is>
           <t>低</t>
-        </is>
-      </c>
-      <c r="G37" s="81" t="inlineStr"/>
-      <c r="H37" s="80" t="inlineStr">
-        <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I37" s="80" t="inlineStr"/>
-    </row>
-    <row r="38" ht="96" customHeight="1" s="1">
-      <c r="A38" s="84" t="n"/>
-      <c r="B38" s="85" t="n"/>
-      <c r="C38" s="81" t="inlineStr">
-        <is>
-          <t>支持应用替代流量跳过七层检测等效配置</t>
-        </is>
-      </c>
-      <c r="D38" s="81" t="inlineStr">
-        <is>
-          <t>匹配覆盖策略的流量跳过七层检测，四层快速转发</t>
-        </is>
-      </c>
-      <c r="E38" s="81" t="inlineStr">
-        <is>
-          <t>PA应用替代策略明确绕过第7层处理与威胁检查，改用第4层状态检查以加速（PA管理指南p1307）；天融信自定义应用加入规则库后仍默认经安全引擎检测（天融信手册《自定义应用》页）；迁移评估项：PA应用替代多为私有大流量业务加速，转换时需同步关闭对应策略的IPS/七层检测，否则性能被拖垮或误阻断</t>
-        </is>
-      </c>
-      <c r="F38" s="80" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="G38" s="85" t="n"/>
-      <c r="H38" s="80" t="inlineStr">
-        <is>
-          <t>待评估</t>
-        </is>
-      </c>
-      <c r="I38" s="85" t="n"/>
-    </row>
-    <row r="39" ht="111" customHeight="1" s="1">
-      <c r="A39" s="84" t="n"/>
-      <c r="B39" s="80" t="inlineStr">
-        <is>
-          <t>身份验证(Authentication)</t>
-        </is>
-      </c>
-      <c r="C39" s="81" t="inlineStr">
-        <is>
-          <t>支持基于用户身份的身份验证策略（User-ID）</t>
-        </is>
-      </c>
-      <c r="D39" s="81" t="inlineStr">
-        <is>
-          <t>基于用户/用户组策略，多源IP-用户映射（AD/Syslog/XML API）</t>
-        </is>
-      </c>
-      <c r="E39" s="81" t="inlineStr">
-        <is>
-          <t>PA身份验证策略在访问网络资源前对用户鉴权（PA Web帮助p182），配合User-ID多源映射（AD/XML/Syslog等）；天融信用户访问网络资源前经认证，认证通过后检查关联的用户访问策略，支持门户认证（本地/外部）与LDAP/RADIUS对接（天融信手册《管理用户》《添加Radius服务器》页）；对应矩阵#3/35</t>
-        </is>
-      </c>
-      <c r="F39" s="80" t="inlineStr">
-        <is>
-          <t>高</t>
         </is>
       </c>
       <c r="G39" s="81" t="inlineStr"/>
@@ -4520,218 +4520,218 @@
           <t>已支持</t>
         </is>
       </c>
-      <c r="I39" s="80" t="inlineStr">
+      <c r="I39" s="80" t="inlineStr"/>
+    </row>
+    <row r="40" ht="96" customHeight="1" s="1">
+      <c r="A40" s="84" t="n"/>
+      <c r="B40" s="85" t="n"/>
+      <c r="C40" s="81" t="inlineStr">
+        <is>
+          <t>支持应用替代流量跳过七层检测等效配置</t>
+        </is>
+      </c>
+      <c r="D40" s="81" t="inlineStr">
+        <is>
+          <t>匹配覆盖策略的流量跳过七层检测，四层快速转发</t>
+        </is>
+      </c>
+      <c r="E40" s="81" t="inlineStr">
+        <is>
+          <t>PA应用替代策略明确绕过第7层处理与威胁检查，改用第4层状态检查以加速（PA管理指南p1307）；天融信自定义应用加入规则库后仍默认经安全引擎检测（天融信手册《自定义应用》页）；迁移评估项：PA应用替代多为私有大流量业务加速，转换时需同步关闭对应策略的IPS/七层检测，否则性能被拖垮或误阻断</t>
+        </is>
+      </c>
+      <c r="F40" s="80" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="G40" s="85" t="n"/>
+      <c r="H40" s="80" t="inlineStr">
+        <is>
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="I40" s="85" t="n"/>
+    </row>
+    <row r="41" ht="111" customHeight="1" s="1">
+      <c r="A41" s="84" t="n"/>
+      <c r="B41" s="80" t="inlineStr">
+        <is>
+          <t>身份验证(Authentication)</t>
+        </is>
+      </c>
+      <c r="C41" s="81" t="inlineStr">
+        <is>
+          <t>支持基于用户身份的身份验证策略（User-ID）</t>
+        </is>
+      </c>
+      <c r="D41" s="81" t="inlineStr">
+        <is>
+          <t>基于用户/用户组策略，多源IP-用户映射（AD/Syslog/XML API）</t>
+        </is>
+      </c>
+      <c r="E41" s="81" t="inlineStr">
+        <is>
+          <t>PA身份验证策略在访问网络资源前对用户鉴权（PA Web帮助p182），配合User-ID多源映射（AD/XML/Syslog等）；天融信用户访问网络资源前经认证，认证通过后检查关联的用户访问策略，支持门户认证（本地/外部）与LDAP/RADIUS对接（天融信手册《管理用户》《添加Radius服务器》页）；对应矩阵#3/35</t>
+        </is>
+      </c>
+      <c r="F41" s="80" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="G41" s="81" t="inlineStr"/>
+      <c r="H41" s="80" t="inlineStr">
+        <is>
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I41" s="80" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="81" customHeight="1" s="1">
-      <c r="A40" s="84" t="n"/>
-      <c r="B40" s="84" t="n"/>
-      <c r="C40" s="81" t="inlineStr">
+    <row r="42" ht="81" customHeight="1" s="1">
+      <c r="A42" s="84" t="n"/>
+      <c r="B42" s="84" t="n"/>
+      <c r="C42" s="81" t="inlineStr">
         <is>
           <t>支持认证策略超时与单次认证（SSO）</t>
         </is>
       </c>
-      <c r="D40" s="81" t="inlineStr">
+      <c r="D42" s="81" t="inlineStr">
         <is>
           <t>认证超时+单次认证(SSO)</t>
         </is>
       </c>
-      <c r="E40" s="81" t="inlineStr">
+      <c r="E42" s="81" t="inlineStr">
         <is>
           <t>PA支持认证超时减少重复质询、Kerberos/SAML/RADIUS等对接（PA Web帮助p186）；天融信手册检索认证超时/单点登录/SSO无命中（仅在线用户在线时长查看与强制下线）；迁移评估项：需核实天融信认证会话有效期配置与SSO对接能力</t>
         </is>
       </c>
-      <c r="F40" s="80" t="inlineStr">
+      <c r="F42" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="G40" s="81" t="inlineStr"/>
-      <c r="H40" s="80" t="inlineStr">
+      <c r="G42" s="81" t="inlineStr"/>
+      <c r="H42" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="I40" s="80" t="inlineStr"/>
-    </row>
-    <row r="41" ht="126" customHeight="1" s="1">
-      <c r="A41" s="84" t="n"/>
-      <c r="B41" s="84" t="n"/>
-      <c r="C41" s="81" t="inlineStr">
-        <is>
-          <t>支持基于策略触发多因素认证质询（MFA Enforcement）</t>
-        </is>
-      </c>
-      <c r="D41" s="81" t="inlineStr">
-        <is>
-          <t>策略匹配触发多因素认证质询（MFA供应商API/RADIUS）</t>
-        </is>
-      </c>
-      <c r="E41" s="81" t="inlineStr">
-        <is>
-          <t>PA身份验证策略通过Authentication Enforcement对象对匹配流量强制质询，支持多因素身份验证（每因素独立超时，防火墙记录时间戳），MFA供应商API/RADIUS对接（PA Web帮助p185-186、p310、p735-742）；天融信双因子认证（密码+短信/证书/Ukey）仅限管理员/用户登录场景（天融信手册《登录安全策略》页），未见流量策略触发MFA质询</t>
-        </is>
-      </c>
-      <c r="F41" s="84" t="n"/>
-      <c r="G41" s="84" t="n"/>
-      <c r="H41" s="80" t="inlineStr">
-        <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="I41" s="84" t="n"/>
-    </row>
-    <row r="42" ht="96" customHeight="1" s="1">
-      <c r="A42" s="84" t="n"/>
-      <c r="B42" s="85" t="n"/>
-      <c r="C42" s="81" t="inlineStr">
-        <is>
-          <t>支持User-ID动态映射时效性等效（AD日志毫秒级更新）</t>
-        </is>
-      </c>
-      <c r="D42" s="81" t="inlineStr">
-        <is>
-          <t>AD域事件日志毫秒级IP-用户映射更新</t>
-        </is>
-      </c>
-      <c r="E42" s="81" t="inlineStr">
-        <is>
-          <t>PA无代理架构通过读取域控事件日志实现IP-用户毫秒级动态映射，大规模部署有专项规划（PA管理指南p866-867）；天融信AD对接的轮询间隔与并发认证能力手册未量化；迁移评估项：数万AD用户且移动频繁场景需实测天融信映射更新时延，避免基于用户的策略出现间歇性未授权拦截</t>
-        </is>
-      </c>
-      <c r="F42" s="85" t="n"/>
-      <c r="G42" s="85" t="n"/>
-      <c r="H42" s="80" t="inlineStr">
-        <is>
-          <t>待评估</t>
-        </is>
-      </c>
-      <c r="I42" s="85" t="n"/>
-    </row>
-    <row r="43" ht="111" customHeight="1" s="1">
+      <c r="I42" s="80" t="inlineStr"/>
+    </row>
+    <row r="43" ht="126" customHeight="1" s="1">
       <c r="A43" s="84" t="n"/>
-      <c r="B43" s="80" t="inlineStr">
-        <is>
-          <t>DoS防护(DoS Protection)</t>
-        </is>
-      </c>
+      <c r="B43" s="84" t="n"/>
       <c r="C43" s="81" t="inlineStr">
         <is>
-          <t>支持针对关键资源的分类/聚合DoS防护</t>
+          <t>支持流量策略触发多因素认证质询（MFA Enforcement）</t>
         </is>
       </c>
       <c r="D43" s="81" t="inlineStr">
         <is>
-          <t>分类(源/目的IP粒度)+聚合(全局)双层阈值限流</t>
+          <t>流量策略匹配触发MFA质询（非登录场景，MFA供应商API/RADIUS）</t>
         </is>
       </c>
       <c r="E43" s="81" t="inlineStr">
         <is>
-          <t>PA DoS策略基于源/目的接口、区域、地址、服务定义允许/拒绝/告警，规则可选聚合与分类双层DoS保护配置文件设定阈值速率（PA Web帮助p189-191、PA管理指南p1354）；天融信DDoS防护模块按防护对象（目的服务器）设阈值（pps/bps），可达目的IP粒度（天融信手册《配置策略模板》《日志查看》页）；对应矩阵#52/42</t>
-        </is>
-      </c>
-      <c r="F43" s="80" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="G43" s="81" t="inlineStr"/>
+          <t>PA身份验证策略通过Authentication Enforcement对象对匹配流量强制质询，支持多因素身份验证（每因素独立超时，防火墙记录时间戳），MFA供应商API/RADIUS对接（PA Web帮助p185-186、p310、p735-742）；天融信双因子认证（密码+短信/证书/Ukey）仅限管理员/用户登录场景（天融信手册《登录安全策略》页），无流量策略触发MFA质询</t>
+        </is>
+      </c>
+      <c r="F43" s="84" t="n"/>
+      <c r="G43" s="84" t="n"/>
       <c r="H43" s="80" t="inlineStr">
         <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I43" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="51" customHeight="1" s="1">
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I43" s="84" t="n"/>
+    </row>
+    <row r="44" ht="96" customHeight="1" s="1">
       <c r="A44" s="84" t="n"/>
       <c r="B44" s="85" t="n"/>
       <c r="C44" s="81" t="inlineStr">
         <is>
-          <t>支持DoS聚合配置文件（连接/秒阈值）</t>
+          <t>支持User-ID动态映射时效性等效（AD日志毫秒级更新）</t>
         </is>
       </c>
       <c r="D44" s="81" t="inlineStr">
         <is>
-          <t>连接数/秒阈值告警+最大速率限制</t>
+          <t>AD域事件日志毫秒级IP-用户映射更新</t>
         </is>
       </c>
       <c r="E44" s="81" t="inlineStr">
         <is>
-          <t>PA聚合DoS配置文件按传入连接数/秒触发告警与最大速率限制；天融信DDoS防护模块按阈值（pps/bps）监视并触发防护（天融信手册《配置策略模板》页）</t>
-        </is>
-      </c>
-      <c r="F44" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="G44" s="81" t="inlineStr"/>
+          <t>PA无代理架构通过读取域控事件日志实现IP-用户毫秒级动态映射，大规模部署有专项规划（PA管理指南p866-867）；天融信AD对接的轮询间隔与并发认证能力手册未量化；迁移评估项：数万AD用户且移动频繁场景需实测天融信映射更新时延，避免基于用户的策略出现间歇性未授权拦截</t>
+        </is>
+      </c>
+      <c r="F44" s="85" t="n"/>
+      <c r="G44" s="85" t="n"/>
       <c r="H44" s="80" t="inlineStr">
         <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I44" s="80" t="inlineStr"/>
-    </row>
-    <row r="45" ht="171" customHeight="1" s="1">
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="I44" s="85" t="n"/>
+    </row>
+    <row r="45" ht="111" customHeight="1" s="1">
       <c r="A45" s="84" t="n"/>
       <c r="B45" s="80" t="inlineStr">
         <is>
-          <t>动态对象(Dynamic Objects)</t>
+          <t>DoS防护(DoS Protection)</t>
         </is>
       </c>
       <c r="C45" s="81" t="inlineStr">
         <is>
-          <t>支持外部动态列表作为策略地址对象（EDL）</t>
+          <t>支持针对关键资源的分类/聚合DoS防护</t>
         </is>
       </c>
       <c r="D45" s="81" t="inlineStr">
         <is>
-          <t>HTTP/HTTPS外部文本列表(IP/域名/URL)自动拉取，策略直接引用</t>
+          <t>分类(源/目的IP粒度)+聚合(全局)双层阈值限流</t>
         </is>
       </c>
       <c r="E45" s="81" t="inlineStr">
         <is>
-          <t>PA外部动态列表：基于HTTP/HTTPS托管的文本文件创建IP/URL/域名/IMEI/IMSI地址对象，防火墙定时自动拉取更新，策略中直接引用（Objects&gt;External Dynamic Lists，PA Web帮助p236-239；策略源/目标可直接选EDL，p196-197）；天融信手册检索外部动态列表/EDL无命中，仅内置威胁情报库与云端威胁情报库（规则集管理，天融信手册《威胁情报》《配置规则集》页），无策略直接引用任意外部文本列表机制；迁移评估项：PA策略中引用的EDL需转换为天融信静态地址组定期导入或威胁情报联动</t>
+          <t>PA DoS策略基于源/目的接口、区域、地址、服务定义允许/拒绝/告警，规则可选聚合与分类双层DoS保护配置文件设定阈值速率（PA Web帮助p189-191、PA管理指南p1354）；天融信DDoS防护模块按防护对象（目的服务器）设阈值（pps/bps），可达目的IP粒度（天融信手册《配置策略模板》《日志查看》页）；对应矩阵#52/42</t>
         </is>
       </c>
       <c r="F45" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G45" s="81" t="inlineStr"/>
       <c r="H45" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="I45" s="80" t="inlineStr"/>
-    </row>
-    <row r="46" ht="126" customHeight="1" s="1">
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I45" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="51" customHeight="1" s="1">
       <c r="A46" s="84" t="n"/>
       <c r="B46" s="85" t="n"/>
       <c r="C46" s="81" t="inlineStr">
         <is>
-          <t>支持基于标记的动态地址组（DAG）</t>
+          <t>支持DoS聚合配置文件（连接/秒阈值）</t>
         </is>
       </c>
       <c r="D46" s="81" t="inlineStr">
         <is>
-          <t>Tag标记过滤器动态地址组，成员随IP变化自动更新</t>
+          <t>连接数/秒阈值告警+最大速率限制</t>
         </is>
       </c>
       <c r="E46" s="81" t="inlineStr">
         <is>
-          <t>PA动态地址组：查找标记(Tag)+基于标记的过滤器（AND/OR匹配）动态填充成员，VM信息源注册或XML/REST API定义标记，IP变化时策略自动生效（PA Web帮助p207-208、p228）；天融信手册检索动态地址组/标签/SDN/云平台联动无命中，地址组为静态IP/子网绑定（天融信手册《地址》页）；迁移评估项：PA云环境Tag微隔离策略需转换为静态地址组，IP漂移场景需人工或API维护</t>
+          <t>PA聚合DoS配置文件按传入连接数/秒触发告警与最大速率限制；天融信DDoS防护模块按阈值（pps/bps）监视并触发防护（天融信手册《配置策略模板》页）</t>
         </is>
       </c>
       <c r="F46" s="80" t="inlineStr">
@@ -4742,66 +4742,62 @@
       <c r="G46" s="81" t="inlineStr"/>
       <c r="H46" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
+          <t>已支持</t>
         </is>
       </c>
       <c r="I46" s="80" t="inlineStr"/>
     </row>
-    <row r="47" ht="51" customHeight="1" s="1">
+    <row r="47" ht="171" customHeight="1" s="1">
       <c r="A47" s="84" t="n"/>
       <c r="B47" s="80" t="inlineStr">
         <is>
-          <t>SD-WAN策略</t>
+          <t>动态对象(Dynamic Objects)</t>
         </is>
       </c>
       <c r="C47" s="81" t="inlineStr">
         <is>
-          <t>支持按应用配置链路路径管理与链路质量探测</t>
+          <t>支持外部动态列表作为策略地址对象（EDL）</t>
         </is>
       </c>
       <c r="D47" s="81" t="inlineStr">
         <is>
-          <t>按应用/区域/地址分配链路与流量分发</t>
+          <t>HTTP/HTTPS外部文本列表(IP/域名/URL)自动拉取，策略直接引用</t>
         </is>
       </c>
       <c r="E47" s="81" t="inlineStr">
         <is>
-          <t>PA SD-WAN策略按应用/抖动/延迟/丢包指标分配链路，流量分发（PA Web帮助p197）；对应矩阵#129/120</t>
+          <t>PA外部动态列表：基于HTTP/HTTPS托管的文本文件创建IP/URL/域名/IMEI/IMSI地址对象，防火墙定时自动拉取更新，策略中直接引用（Objects&gt;External Dynamic Lists，PA Web帮助p236-239；策略源/目标可直接选EDL，p196-197）；天融信手册检索外部动态列表/EDL无命中，仅内置威胁情报库与云端威胁情报库（规则集管理，天融信手册《威胁情报》《配置规则集》页），无策略直接引用任意外部文本列表机制；迁移评估项：PA策略中引用的EDL需转换为天融信静态地址组定期导入或威胁情报联动</t>
         </is>
       </c>
       <c r="F47" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G47" s="81" t="inlineStr"/>
       <c r="H47" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="I47" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="81" customHeight="1" s="1">
-      <c r="A48" s="85" t="n"/>
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I47" s="80" t="inlineStr"/>
+    </row>
+    <row r="48" ht="126" customHeight="1" s="1">
+      <c r="A48" s="84" t="n"/>
       <c r="B48" s="85" t="n"/>
       <c r="C48" s="81" t="inlineStr">
         <is>
-          <t>支持SD-WAN路径选择与链路质量监测（jitter/latency/loss）</t>
+          <t>支持基于标记的动态地址组（DAG）</t>
         </is>
       </c>
       <c r="D48" s="81" t="inlineStr">
         <is>
-          <t>抖动/延迟/丢包(jitter/latency/loss)指标选路</t>
+          <t>Tag标记过滤器动态地址组，成员随IP变化自动更新</t>
         </is>
       </c>
       <c r="E48" s="81" t="inlineStr">
         <is>
-          <t>PA路径质量配置文件基于抖动/延迟/丢包等运行状况指标选路（PA Web帮助p195）；天融信有链路探测(ping)+智能选路(最小延迟优先)（天融信手册《策略路由》页），无jitter/latency/loss多维指标</t>
+          <t>PA动态地址组：查找标记(Tag)+基于标记的过滤器（AND/OR匹配）动态填充成员，VM信息源注册或XML/REST API定义标记，IP变化时策略自动生效（PA Web帮助p207-208、p228）；天融信手册检索动态地址组/标签/SDN/云平台联动无命中，地址组为静态IP/子网绑定（天融信手册《地址》页）；迁移评估项：PA云环境Tag微隔离策略需转换为静态地址组，IP漂移场景需人工或API维护</t>
         </is>
       </c>
       <c r="F48" s="80" t="inlineStr">
@@ -4812,50 +4808,122 @@
       <c r="G48" s="81" t="inlineStr"/>
       <c r="H48" s="80" t="inlineStr">
         <is>
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I48" s="80" t="inlineStr"/>
+    </row>
+    <row r="49" ht="81" customHeight="1" s="1">
+      <c r="A49" s="84" t="n"/>
+      <c r="B49" s="80" t="inlineStr">
+        <is>
+          <t>SD-WAN策略</t>
+        </is>
+      </c>
+      <c r="C49" s="81" t="inlineStr">
+        <is>
+          <t>支持按应用配置链路路径管理与链路质量探测</t>
+        </is>
+      </c>
+      <c r="D49" s="81" t="inlineStr">
+        <is>
+          <t>按应用分配链路与流量分发（天融信以策略路由+LLB近似实现）</t>
+        </is>
+      </c>
+      <c r="E49" s="81" t="inlineStr">
+        <is>
+          <t>PA SD-WAN策略按应用/抖动/延迟/丢包指标分配链路，流量分发（PA Web帮助p197）；天融信为策略路由+链路负载均衡近似实现（天融信手册《策略路由》《链路负载均衡》页），无SD-WAN策略模型；对应矩阵#129/120</t>
+        </is>
+      </c>
+      <c r="F49" s="80" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="G49" s="81" t="inlineStr"/>
+      <c r="H49" s="80" t="inlineStr">
+        <is>
           <t>部分支持</t>
         </is>
       </c>
-      <c r="I48" s="80" t="inlineStr"/>
+      <c r="I49" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="81" customHeight="1" s="1">
+      <c r="A50" s="85" t="n"/>
+      <c r="B50" s="85" t="n"/>
+      <c r="C50" s="81" t="inlineStr">
+        <is>
+          <t>支持SD-WAN路径选择与链路质量监测（jitter/latency/loss）</t>
+        </is>
+      </c>
+      <c r="D50" s="81" t="inlineStr">
+        <is>
+          <t>抖动/延迟/丢包多维指标选路（天融信现仅延迟探测）</t>
+        </is>
+      </c>
+      <c r="E50" s="81" t="inlineStr">
+        <is>
+          <t>PA路径质量配置文件基于抖动/延迟/丢包等运行状况指标选路（PA Web帮助p195）；天融信有链路探测(ping)+智能选路(最小延迟优先)（天融信手册《策略路由》页），无jitter/latency/loss多维指标</t>
+        </is>
+      </c>
+      <c r="F50" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G50" s="81" t="inlineStr"/>
+      <c r="H50" s="80" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="I50" s="80" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="37">
-    <mergeCell ref="I9:I14"/>
-    <mergeCell ref="B26:B31"/>
+  <mergeCells count="39">
+    <mergeCell ref="F17:F19"/>
     <mergeCell ref="B47:B48"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="A2:A50"/>
     <mergeCell ref="H6:H7"/>
-    <mergeCell ref="B15:B21"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="F30:F31"/>
-    <mergeCell ref="F9:F11"/>
-    <mergeCell ref="G40:G42"/>
-    <mergeCell ref="I40:I42"/>
-    <mergeCell ref="B39:B42"/>
+    <mergeCell ref="I36:I37"/>
+    <mergeCell ref="G39:G40"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="B27:B32"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="G17:G22"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="H17:H20"/>
     <mergeCell ref="B2:B7"/>
-    <mergeCell ref="H11:H14"/>
-    <mergeCell ref="G37:G38"/>
-    <mergeCell ref="I16:I21"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="I37:I38"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="F40:F42"/>
-    <mergeCell ref="F16:F18"/>
-    <mergeCell ref="H16:H19"/>
+    <mergeCell ref="H36:H37"/>
+    <mergeCell ref="B8:B15"/>
+    <mergeCell ref="B16:B22"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="G9:G15"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="I9:I15"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="G42:G44"/>
+    <mergeCell ref="H12:H15"/>
     <mergeCell ref="F3:F7"/>
-    <mergeCell ref="G27:G31"/>
-    <mergeCell ref="I27:I31"/>
+    <mergeCell ref="F11:F12"/>
     <mergeCell ref="B45:B46"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="H30:H31"/>
-    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="I17:I22"/>
     <mergeCell ref="G3:G7"/>
-    <mergeCell ref="B8:B14"/>
     <mergeCell ref="I3:I7"/>
-    <mergeCell ref="G16:G21"/>
-    <mergeCell ref="A2:A48"/>
-    <mergeCell ref="G9:G14"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="F42:F44"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="G28:G32"/>
+    <mergeCell ref="B41:B44"/>
+    <mergeCell ref="I28:I32"/>
+    <mergeCell ref="G36:G37"/>
+    <mergeCell ref="I42:I44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4867,7 +4935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15.2"/>
   <cols>
     <col width="11.7" customWidth="1" style="1" min="1" max="1"/>
@@ -5021,7 +5089,7 @@
       <c r="H4" s="82" t="n"/>
       <c r="I4" s="82" t="n"/>
     </row>
-    <row r="5" ht="96" customHeight="1" s="1">
+    <row r="5" ht="51" customHeight="1" s="1">
       <c r="A5" s="82" t="n"/>
       <c r="B5" s="80" t="inlineStr">
         <is>
@@ -5030,17 +5098,17 @@
       </c>
       <c r="C5" s="81" t="inlineStr">
         <is>
-          <t>支持安全策略规则构建块：源用户/HIP/设备/应用/服务/日志等</t>
+          <t>支持HIP主机信息配置文件策略匹配（Host Information Profile）</t>
         </is>
       </c>
       <c r="D5" s="81" t="inlineStr">
         <is>
-          <t>预登录用户/HIP主机信息/设备对象/应用默认端口规避/会话结束日志等构建块</t>
+          <t>终端安全态势（补丁/杀软/磁盘加密等）作为策略匹配条件</t>
         </is>
       </c>
       <c r="E5" s="81" t="inlineStr">
         <is>
-          <t>PA规则构建块含预登录用户、HIP配置文件、设备对象、应用默认端口规避、会话结束日志等；天融信支持用户/应用/服务/日志构建块，但无HIP主机信息配置文件与设备对象等价物，仅有EDR联动上报终端资产并下发管控策略（天融信手册《与EDR联动》页）；对应矩阵#3/4</t>
+          <t>PA规则构建块支持HIP配置文件匹配终端安全态势（对应矩阵#3/4）；天融信手册检索HIP/主机信息配置文件无命中，无终端安全态势匹配等价物</t>
         </is>
       </c>
       <c r="F5" s="80" t="inlineStr">
@@ -5051,32 +5119,32 @@
       <c r="G5" s="81" t="inlineStr"/>
       <c r="H5" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
+          <t>不支持</t>
         </is>
       </c>
       <c r="I5" s="80" t="inlineStr"/>
     </row>
-    <row r="6" ht="81" customHeight="1" s="1">
+    <row r="6" ht="51" customHeight="1" s="1">
       <c r="A6" s="82" t="n"/>
       <c r="B6" s="82" t="n"/>
       <c r="C6" s="81" t="inlineStr">
         <is>
-          <t>支持安全策略优化器（Policy Optimizer）</t>
+          <t>支持终端设备对象作为策略匹配条件</t>
         </is>
       </c>
       <c r="D6" s="81" t="inlineStr">
         <is>
-          <t>端口(L4)规则一键迁移为应用(L7)规则+新应用查看器</t>
+          <t>终端设备类型（手机/平板/IoT等设备对象）作为策略构建块</t>
         </is>
       </c>
       <c r="E6" s="81" t="inlineStr">
         <is>
-          <t>PA新应用查看器+端口规则迁移至App-ID规则工作流+规则使用统计，减少攻击面（PA Web帮助p142）；天融信策略统计开关可显示规则匹配命中情况（天融信手册《配置访问控制策略》页），但无新应用查看器与端口→应用规则迁移工作流；对应矩阵#132</t>
+          <t>PA支持设备对象构建块（对应矩阵#3/4）；天融信经EDR联动上报终端资产并下发管控策略（天融信手册《与EDR联动》页），无独立设备对象</t>
         </is>
       </c>
       <c r="F6" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>低</t>
         </is>
       </c>
       <c r="G6" s="81" t="inlineStr"/>
@@ -5087,200 +5155,196 @@
       </c>
       <c r="I6" s="80" t="inlineStr"/>
     </row>
-    <row r="7" ht="36" customHeight="1" s="1">
+    <row r="7" ht="81" customHeight="1" s="1">
       <c r="A7" s="82" t="n"/>
       <c r="B7" s="82" t="n"/>
       <c r="C7" s="81" t="inlineStr">
         <is>
-          <t>支持配置锁（Config Lock/Commit Lock）</t>
+          <t>支持端口(L4)规则向应用(L7)规则迁移工作流（Policy Optimizer）</t>
         </is>
       </c>
       <c r="D7" s="81" t="inlineStr">
         <is>
-          <t>配置锁/提交锁，防止多管理员并发修改</t>
+          <t>端口规则一键迁移为应用规则+新应用查看器</t>
         </is>
       </c>
       <c r="E7" s="81" t="inlineStr">
         <is>
-          <t>PA可锁定待选配置或提交，防止他管理员并发更改；对应矩阵#135（天融信不支持，PA优势）</t>
-        </is>
-      </c>
-      <c r="F7" s="82" t="n"/>
+          <t>PA策略优化器提供新应用查看器与端口→App-ID规则迁移工作流（PA Web帮助p142）；天融信策略统计仅显示规则命中数（天融信手册《配置访问控制策略》页），无迁移工具（命中统计能力已另列已支持行）；对应矩阵#132</t>
+        </is>
+      </c>
+      <c r="F7" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
       <c r="G7" s="82" t="n"/>
       <c r="H7" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>不支持</t>
         </is>
       </c>
       <c r="I7" s="82" t="n"/>
     </row>
-    <row r="8" ht="111" customHeight="1" s="1">
+    <row r="8" ht="36" customHeight="1" s="1">
       <c r="A8" s="82" t="n"/>
       <c r="B8" s="82" t="n"/>
       <c r="C8" s="81" t="inlineStr">
         <is>
-          <t>支持应用默认端口绑定（Service: application-default）</t>
+          <t>支持配置锁（Config Lock/Commit Lock）</t>
         </is>
       </c>
       <c r="D8" s="81" t="inlineStr">
         <is>
-          <t>应用匹配同时强制使用标准端口，非标端口拒绝</t>
+          <t>配置锁/提交锁，防止多管理员并发修改</t>
         </is>
       </c>
       <c r="E8" s="81" t="inlineStr">
         <is>
-          <t>PA安全策略默认服务为application-default：放行应用同时强制其使用标准端口（如SSH仅22），非标准端口不匹配即拦截（PA管理指南p904）；天融信策略为五元组+应用识别组合（天融信手册《配置访问控制策略》页）；迁移评估项：直接转换若仅保留应用识别不限端口将扩大安全敞口，需制定应用标准端口映射限制（App-Default）转换方案；对应矩阵#2</t>
-        </is>
-      </c>
-      <c r="F8" s="80" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
+          <t>PA可锁定待选配置或提交，防止他管理员并发更改；对应矩阵#135（天融信不支持，PA优势）</t>
+        </is>
+      </c>
+      <c r="F8" s="82" t="n"/>
       <c r="G8" s="82" t="n"/>
-      <c r="H8" s="82" t="n"/>
+      <c r="H8" s="80" t="inlineStr">
+        <is>
+          <t>待评估</t>
+        </is>
+      </c>
       <c r="I8" s="82" t="n"/>
     </row>
-    <row r="9" ht="81" customHeight="1" s="1">
+    <row r="9" ht="111" customHeight="1" s="1">
       <c r="A9" s="82" t="n"/>
       <c r="B9" s="82" t="n"/>
       <c r="C9" s="81" t="inlineStr">
         <is>
-          <t>支持安全策略绑定安全配置文件组（Profile Group）</t>
+          <t>支持应用默认端口绑定（Service: application-default）</t>
         </is>
       </c>
       <c r="D9" s="81" t="inlineStr">
         <is>
-          <t>Allow动作关联反病毒/漏洞防护/URL过滤/文件阻断/WildFire配置文件组</t>
+          <t>应用匹配同时强制使用标准端口，非标端口拒绝</t>
         </is>
       </c>
       <c r="E9" s="81" t="inlineStr">
         <is>
-          <t>PA安全策略Allow动作关联Profile组（反病毒/漏洞防护/URL过滤/文件阻止/WildFire等，PA Web帮助p304）；天融信一体化策略引擎自带检测项；迁移评估项：需评估Profile组到天融信各检测引擎的映射与缺省动作差异；对应矩阵#4</t>
+          <t>PA安全策略默认服务为application-default：放行应用同时强制其使用标准端口（如SSH仅22），非标准端口不匹配即拦截（PA管理指南p904）；天融信策略为五元组+应用识别组合（天融信手册《配置访问控制策略》页）；迁移评估项：直接转换若仅保留应用识别不限端口将扩大安全敞口，需制定应用标准端口映射限制（App-Default）转换方案；对应矩阵#2</t>
         </is>
       </c>
       <c r="F9" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G9" s="82" t="n"/>
       <c r="H9" s="82" t="n"/>
       <c r="I9" s="82" t="n"/>
     </row>
-    <row r="10" ht="156" customHeight="1" s="1">
+    <row r="10" ht="81" customHeight="1" s="1">
       <c r="A10" s="82" t="n"/>
       <c r="B10" s="82" t="n"/>
       <c r="C10" s="81" t="inlineStr">
         <is>
-          <t>支持隐式默认规则显式化迁移（intrazone/interzone-default）</t>
+          <t>支持安全策略绑定安全配置文件组（Profile Group）</t>
         </is>
       </c>
       <c r="D10" s="81" t="inlineStr">
         <is>
-          <t>同区域默认放行/跨区域默认拒绝，支持替代与日志转发</t>
+          <t>Allow动作关联反病毒/漏洞防护/URL过滤/文件阻断/WildFire配置文件组</t>
         </is>
       </c>
       <c r="E10" s="81" t="inlineStr">
         <is>
-          <t>PA安全策略库末尾自带两条隐式系统规则：区域内默认（同Zone默认放行）与区域间默认（跨Zone默认拒绝），可被替代配置，替代字段含日志转发配置文件与Log at Session End在会话结束时记录（PA Web帮助p134-136）；天融信未见同区域默认放行的隐式规则机制；迁移评估项：①必须提取intrazone-default同Zone互访需求并显式转换为放行规则，否则割接后同Zone不同网段/VLAN互访将被默认拦截；②需在新设备补齐底部兜底Deny-All并开启日志，否则被拒流量查无日志、排障困难</t>
+          <t>PA安全策略Allow动作关联Profile组（反病毒/漏洞防护/URL过滤/文件阻止/WildFire等，PA Web帮助p304）；天融信一体化策略引擎自带检测项；迁移评估项：需评估Profile组到天融信各检测引擎的映射与缺省动作差异；对应矩阵#4</t>
         </is>
       </c>
       <c r="F10" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G10" s="82" t="n"/>
       <c r="H10" s="82" t="n"/>
       <c r="I10" s="82" t="n"/>
     </row>
-    <row r="11" ht="126" customHeight="1" s="1">
+    <row r="11" ht="156" customHeight="1" s="1">
       <c r="A11" s="82" t="n"/>
-      <c r="B11" s="80" t="inlineStr">
+      <c r="B11" s="82" t="n"/>
+      <c r="C11" s="81" t="inlineStr">
+        <is>
+          <t>支持隐式默认规则显式化迁移（intrazone/interzone-default）</t>
+        </is>
+      </c>
+      <c r="D11" s="81" t="inlineStr">
+        <is>
+          <t>同区域默认放行/跨区域默认拒绝，支持替代与日志转发</t>
+        </is>
+      </c>
+      <c r="E11" s="81" t="inlineStr">
+        <is>
+          <t>PA安全策略库末尾自带两条隐式系统规则：区域内默认（同Zone默认放行）与区域间默认（跨Zone默认拒绝），可被替代配置，替代字段含日志转发配置文件与Log at Session End在会话结束时记录（PA Web帮助p134-136）；天融信未见同区域默认放行的隐式规则机制；迁移评估项：①必须提取intrazone-default同Zone互访需求并显式转换为放行规则，否则割接后同Zone不同网段/VLAN互访将被默认拦截；②需在新设备补齐底部兜底Deny-All并开启日志，否则被拒流量查无日志、排障困难</t>
+        </is>
+      </c>
+      <c r="F11" s="80" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="G11" s="82" t="n"/>
+      <c r="H11" s="82" t="n"/>
+      <c r="I11" s="82" t="n"/>
+    </row>
+    <row r="12" ht="126" customHeight="1" s="1">
+      <c r="A12" s="82" t="n"/>
+      <c r="B12" s="80" t="inlineStr">
         <is>
           <t>NAT策略</t>
         </is>
       </c>
-      <c r="C11" s="81" t="inlineStr">
+      <c r="C12" s="81" t="inlineStr">
         <is>
           <t>支持NAT后目的区域路由回查匹配（Dest Zone by route lookup）</t>
         </is>
       </c>
-      <c r="D11" s="81" t="inlineStr">
+      <c r="D12" s="81" t="inlineStr">
         <is>
           <t>目的区域按NAT后路由查找；源/目的地址用NAT前值</t>
         </is>
       </c>
-      <c r="E11" s="81" t="inlineStr">
+      <c r="E12" s="81" t="inlineStr">
         <is>
           <t>PA底层为『先NAT判断后安全策略匹配』的因果倒置：安全策略要求源区域(NAT前)+源地址(NAT前)+目的地址(NAT前)+目的区域(NAT后按路由查找)，极其反直觉；天融信地址转换为独立策略库常规直观映射（安全策略&gt;地址转换，天融信手册《服务器映射》页）；迁移评估项：带目的NAT的策略平移后易因Zone填写错误不通，需制定NAT查表逻辑转换映射规范；对应矩阵#9</t>
         </is>
       </c>
-      <c r="F11" s="80" t="inlineStr">
+      <c r="F12" s="80" t="inlineStr">
         <is>
           <t>高</t>
-        </is>
-      </c>
-      <c r="G11" s="81" t="inlineStr"/>
-      <c r="H11" s="80" t="inlineStr">
-        <is>
-          <t>待评估</t>
-        </is>
-      </c>
-      <c r="I11" s="80" t="inlineStr"/>
-    </row>
-    <row r="12" ht="81" customHeight="1" s="1">
-      <c r="A12" s="82" t="n"/>
-      <c r="B12" s="82" t="n"/>
-      <c r="C12" s="81" t="inlineStr">
-        <is>
-          <t>支持NAT规则主动/主动HA绑定（Active/Active HA Binding）</t>
-        </is>
-      </c>
-      <c r="D12" s="81" t="inlineStr">
-        <is>
-          <t>主动/主动HA下NAT规则绑定会话所有者</t>
-        </is>
-      </c>
-      <c r="E12" s="81" t="inlineStr">
-        <is>
-          <t>PA主动/主动HA配置下NAT规则可绑定会话所有者/会话设置，控制NAT会话的设备绑定，仅A/A模式可见（PA Web帮助p150）；天融信HA为主备双机热备模式（天融信手册《配置双机热备功能》页），无主动/主动模式及NAT规则绑定机制</t>
-        </is>
-      </c>
-      <c r="F12" s="80" t="inlineStr">
-        <is>
-          <t>低</t>
         </is>
       </c>
       <c r="G12" s="81" t="inlineStr"/>
       <c r="H12" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
+          <t>待评估</t>
         </is>
       </c>
       <c r="I12" s="80" t="inlineStr"/>
     </row>
-    <row r="13" ht="96" customHeight="1" s="1">
+    <row r="13" ht="81" customHeight="1" s="1">
       <c r="A13" s="82" t="n"/>
-      <c r="B13" s="80" t="inlineStr">
-        <is>
-          <t>QoS策略</t>
-        </is>
-      </c>
+      <c r="B13" s="82" t="n"/>
       <c r="C13" s="81" t="inlineStr">
         <is>
-          <t>支持基于DSCP/ToS值匹配的QoS</t>
+          <t>支持NAT规则主动/主动HA绑定（Active/Active HA Binding）</t>
         </is>
       </c>
       <c r="D13" s="81" t="inlineStr">
         <is>
-          <t>QoS规则按DSCP/ToS值匹配调度</t>
+          <t>主动/主动HA下NAT规则绑定会话所有者</t>
         </is>
       </c>
       <c r="E13" s="81" t="inlineStr">
         <is>
-          <t>PA QoS规则可直接按DSCP值或IP优先级/ToS匹配调度（PA Web帮助p155）；天融信支持DSCP/802.1p(CoS)识别与重标记，但需在独立流量管理模块配置（虚拟通道+限制/保证带宽+通道优先级，天融信手册《流量管理》页），未直接耦合在基础访问控制策略表内（联网核实厂商流控资料，手册未详载）</t>
+          <t>PA主动/主动HA配置下NAT规则可绑定会话所有者/会话设置，控制NAT会话的设备绑定，仅A/A模式可见（PA Web帮助p150）；天融信HA为主备双机热备模式（天融信手册《配置双机热备功能》页），无主动/主动模式及NAT规则绑定机制</t>
         </is>
       </c>
       <c r="F13" s="80" t="inlineStr">
@@ -5291,226 +5355,226 @@
       <c r="G13" s="81" t="inlineStr"/>
       <c r="H13" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
+          <t>不支持</t>
         </is>
       </c>
       <c r="I13" s="80" t="inlineStr"/>
     </row>
-    <row r="14" ht="111" customHeight="1" s="1">
+    <row r="14" ht="96" customHeight="1" s="1">
       <c r="A14" s="82" t="n"/>
       <c r="B14" s="80" t="inlineStr">
         <is>
-          <t>基于策略转发(PBF)</t>
+          <t>QoS策略</t>
         </is>
       </c>
       <c r="C14" s="81" t="inlineStr">
         <is>
-          <t>支持PBF强制对称返回（非对称路由环境）</t>
+          <t>支持QoS策略规则内直接按DSCP/ToS匹配调度</t>
         </is>
       </c>
       <c r="D14" s="81" t="inlineStr">
         <is>
-          <t>记录入接口MAC，回包强制原路返回</t>
+          <t>QoS策略规则DSCP/ToS直接匹配（非独立流控模块配置）</t>
         </is>
       </c>
       <c r="E14" s="81" t="inlineStr">
         <is>
-          <t>PA对称返回：虚拟路由器替代返回流量的路由查找，将流量引导回接收SYN数据包的MAC地址（ARP表确定下一跳），双ISP双活/非对称路由核心机制（PA管理指南p1294）；天融信手册检索无对称返回/回程机制命中，策略路由与LLB的回程保障能力待验证；迁移评估项：多ISP双活环境需实测天融信回包路由对称性，否则现网业务中断</t>
+          <t>PA QoS规则可直接按DSCP值或IP优先级/ToS匹配调度（PA Web帮助p155）；天融信支持DSCP/802.1p(CoS)识别与重标记，但需在独立流量管理模块配置（虚拟通道+限制/保证带宽+通道优先级，天融信手册《流量管理》页），未直接耦合在基础访问控制策略表内（联网核实厂商流控资料，手册未详载）</t>
         </is>
       </c>
       <c r="F14" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>低</t>
         </is>
       </c>
       <c r="G14" s="81" t="inlineStr"/>
       <c r="H14" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>部分支持</t>
         </is>
       </c>
       <c r="I14" s="80" t="inlineStr"/>
     </row>
-    <row r="15" ht="51" customHeight="1" s="1">
+    <row r="15" ht="111" customHeight="1" s="1">
       <c r="A15" s="82" t="n"/>
       <c r="B15" s="80" t="inlineStr">
         <is>
-          <t>解密策略(Decryption)</t>
+          <t>基于策略转发(PBF)</t>
         </is>
       </c>
       <c r="C15" s="81" t="inlineStr">
         <is>
-          <t>支持解密流量镜像到专用接口（Decryption Port Mirroring）</t>
+          <t>支持PBF强制对称返回（非对称路由环境）</t>
         </is>
       </c>
       <c r="D15" s="81" t="inlineStr">
         <is>
-          <t>解密后明文流量镜像至专用接口供第三方分析</t>
+          <t>记录入接口MAC，回包强制原路返回</t>
         </is>
       </c>
       <c r="E15" s="81" t="inlineStr">
         <is>
-          <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证（PA管理指南p1059）；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
+          <t>PA对称返回：虚拟路由器替代返回流量的路由查找，将流量引导回接收SYN数据包的MAC地址（ARP表确定下一跳），双ISP双活/非对称路由核心机制（PA管理指南p1294）；天融信手册检索无对称返回/回程机制命中，策略路由与LLB的回程保障能力待验证；迁移评估项：多ISP双活环境需实测天融信回包路由对称性，否则现网业务中断</t>
         </is>
       </c>
       <c r="F15" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G15" s="81" t="inlineStr"/>
       <c r="H15" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
+          <t>待评估</t>
         </is>
       </c>
       <c r="I15" s="80" t="inlineStr"/>
     </row>
-    <row r="16" ht="126" customHeight="1" s="1">
+    <row r="16" ht="51" customHeight="1" s="1">
       <c r="A16" s="82" t="n"/>
-      <c r="B16" s="82" t="n"/>
+      <c r="B16" s="80" t="inlineStr">
+        <is>
+          <t>解密策略(Decryption)</t>
+        </is>
+      </c>
       <c r="C16" s="81" t="inlineStr">
         <is>
-          <t>支持解密不受信证书分离处理（Forward Untrust Certificate）</t>
+          <t>支持解密流量镜像到专用接口（Decryption Port Mirroring）</t>
         </is>
       </c>
       <c r="D16" s="81" t="inlineStr">
         <is>
-          <t>外部无效证书以不受信转发证书重签，保留浏览器告警</t>
+          <t>解密后明文流量镜像至专用接口供第三方分析</t>
         </is>
       </c>
       <c r="E16" s="81" t="inlineStr">
         <is>
-          <t>PA转发代理遇外部过期/不受信证书时，不用内部信任CA重签，而是专用Forward Untrust Certificate重签名，让浏览器保留不受信告警（PA管理指南p994、p1030）；天融信SSL解密（透明代理/服务器SSL解密，天融信手册《代理策略》页）未见受信/不受信双证书体系；迁移评估项：需验证天融信对外部无效证书的处理方式，避免直接阻断（白屏）或信任重签（掩盖风险）</t>
+          <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证（PA管理指南p1059）；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
         </is>
       </c>
       <c r="F16" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G16" s="81" t="inlineStr"/>
       <c r="H16" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>不支持</t>
         </is>
       </c>
       <c r="I16" s="80" t="inlineStr"/>
     </row>
-    <row r="17" ht="66" customHeight="1" s="1">
+    <row r="17" ht="126" customHeight="1" s="1">
       <c r="A17" s="82" t="n"/>
       <c r="B17" s="82" t="n"/>
       <c r="C17" s="81" t="inlineStr">
         <is>
-          <t>支持解密规则按URL类别选择性解密（URL Category）</t>
+          <t>支持解密不受信证书分离处理（Forward Untrust Certificate）</t>
         </is>
       </c>
       <c r="D17" s="81" t="inlineStr">
         <is>
-          <t>按URL类别圈定解密范围，排除银行/医疗等敏感类</t>
+          <t>外部无效证书以不受信转发证书重签，保留浏览器告警</t>
         </is>
       </c>
       <c r="E17" s="81" t="inlineStr">
         <is>
-          <t>PA解密规则可按URL类别（含自定义类别）选择解密范围，可排除银行/医疗等敏感类别不解密（PA Web帮助p164）；天融信SSL解密（代理策略/代理模板）无按URL类别选择解密机制（检索无命中）</t>
+          <t>PA转发代理遇外部过期/不受信证书时，不用内部信任CA重签，而是专用Forward Untrust Certificate重签名，让浏览器保留不受信告警（PA管理指南p994、p1030）；天融信SSL解密（透明代理/服务器SSL解密，天融信手册《代理策略》页）未见受信/不受信双证书体系；迁移评估项：需验证天融信对外部无效证书的处理方式，避免直接阻断（白屏）或信任重签（掩盖风险）</t>
         </is>
       </c>
       <c r="F17" s="80" t="inlineStr">
         <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="G17" s="82" t="n"/>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="G17" s="81" t="inlineStr"/>
       <c r="H17" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="I17" s="82" t="n"/>
-    </row>
-    <row r="18" ht="96" customHeight="1" s="1">
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="I17" s="80" t="inlineStr"/>
+    </row>
+    <row r="18" ht="66" customHeight="1" s="1">
       <c r="A18" s="82" t="n"/>
       <c r="B18" s="82" t="n"/>
       <c r="C18" s="81" t="inlineStr">
         <is>
+          <t>支持解密规则按URL类别选择性解密（URL Category）</t>
+        </is>
+      </c>
+      <c r="D18" s="81" t="inlineStr">
+        <is>
+          <t>按URL类别圈定解密范围，排除银行/医疗等敏感类</t>
+        </is>
+      </c>
+      <c r="E18" s="81" t="inlineStr">
+        <is>
+          <t>PA解密规则可按URL类别（含自定义类别）选择解密范围，可排除银行/医疗等敏感类别不解密（PA Web帮助p164）；天融信SSL解密（代理策略/代理模板）无按URL类别选择解密机制（检索无命中）</t>
+        </is>
+      </c>
+      <c r="F18" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G18" s="82" t="n"/>
+      <c r="H18" s="80" t="inlineStr">
+        <is>
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I18" s="82" t="n"/>
+    </row>
+    <row r="19" ht="96" customHeight="1" s="1">
+      <c r="A19" s="82" t="n"/>
+      <c r="B19" s="82" t="n"/>
+      <c r="C19" s="81" t="inlineStr">
+        <is>
           <t>支持SSH代理解密与SSH隧道控制（SSH Proxy）</t>
         </is>
       </c>
-      <c r="D18" s="81" t="inlineStr">
+      <c r="D19" s="81" t="inlineStr">
         <is>
           <t>SSH代理解密+SSH隧道(ssh-tunnel)识别控制</t>
         </is>
       </c>
-      <c r="E18" s="81" t="inlineStr">
+      <c r="E19" s="81" t="inlineStr">
         <is>
           <t>PA解密策略SSH Proxy类型解密SSH通信，可通过ssh-tunnel App-ID在策略中控制SSH隧道（端口转发/内网穿透），正常SSH管理流量放行；含不受支持算法检查/资源不足阻断会话等防护（PA Web帮助p164、p318-319）；天融信手册检索无SSH代理/SSH隧道控制命中</t>
         </is>
       </c>
-      <c r="F18" s="82" t="n"/>
-      <c r="G18" s="82" t="n"/>
-      <c r="H18" s="82" t="n"/>
-      <c r="I18" s="82" t="n"/>
-    </row>
-    <row r="19" ht="66" customHeight="1" s="1">
-      <c r="A19" s="82" t="n"/>
-      <c r="B19" s="80" t="inlineStr">
+      <c r="F19" s="82" t="n"/>
+      <c r="G19" s="82" t="n"/>
+      <c r="H19" s="82" t="n"/>
+      <c r="I19" s="82" t="n"/>
+    </row>
+    <row r="20" ht="111" customHeight="1" s="1">
+      <c r="A20" s="82" t="n"/>
+      <c r="B20" s="80" t="inlineStr">
         <is>
           <t>网络数据包代理(NPBroker)</t>
         </is>
       </c>
-      <c r="C19" s="81" t="inlineStr">
-        <is>
-          <t>支持按应用/用户/区域/设备/IP定义NPBroker规则转发到第三方安全链</t>
-        </is>
-      </c>
-      <c r="D19" s="81" t="inlineStr">
+      <c r="C20" s="81" t="inlineStr">
+        <is>
+          <t>支持内联数据包代理策略将流量转发第三方安全链（NPBroker）</t>
+        </is>
+      </c>
+      <c r="D20" s="81" t="inlineStr">
         <is>
           <t>已解密/未解密流量内联转发第三方安全链，L3路由转发</t>
         </is>
       </c>
-      <c r="E19" s="81" t="inlineStr">
-        <is>
-          <t>PA网络数据包代理策略将已解密/未解密TLS/非TLS流量内联转发至第三方安全工具，路径选择选项卡应用数据包代理配置文件定义经路由L3安全链的转发方式（PA Web帮助p167-170）；对应矩阵#122</t>
-        </is>
-      </c>
-      <c r="F19" s="80" t="inlineStr">
+      <c r="E20" s="81" t="inlineStr">
+        <is>
+          <t>PA网络数据包代理策略将已解密/未解密TLS/非TLS流量内联转发至第三方安全工具，路径选择选项卡应用数据包代理配置文件定义经路由L3安全链的转发方式（PA Web帮助p167-170）；天融信无网络数据包代理模块，最接近手段为WAF旁路联动（经交换机镜像引流，天融信手册《与WAF联动》页），非内联且无回注路径；对应矩阵#122</t>
+        </is>
+      </c>
+      <c r="F20" s="80" t="inlineStr">
         <is>
           <t>高</t>
-        </is>
-      </c>
-      <c r="G19" s="81" t="inlineStr"/>
-      <c r="H19" s="80" t="inlineStr">
-        <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="I19" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="66" customHeight="1" s="1">
-      <c r="A20" s="82" t="n"/>
-      <c r="B20" s="82" t="n"/>
-      <c r="C20" s="81" t="inlineStr">
-        <is>
-          <t>支持NPBroker转发流量类型选择（TLS解密/未解密/非TLS）</t>
-        </is>
-      </c>
-      <c r="D20" s="81" t="inlineStr">
-        <is>
-          <t>TLS解密/未解密/非TLS流量类型选择</t>
-        </is>
-      </c>
-      <c r="E20" s="81" t="inlineStr">
-        <is>
-          <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证（PA Web帮助p167）；天融信无网络数据包代理模块（矩阵#122）</t>
-        </is>
-      </c>
-      <c r="F20" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
         </is>
       </c>
       <c r="G20" s="81" t="inlineStr"/>
@@ -5519,68 +5583,68 @@
           <t>不支持</t>
         </is>
       </c>
-      <c r="I20" s="80" t="inlineStr"/>
+      <c r="I20" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="66" customHeight="1" s="1">
       <c r="A21" s="82" t="n"/>
-      <c r="B21" s="80" t="inlineStr">
-        <is>
-          <t>隧道检测(Tunnel Inspection)</t>
-        </is>
-      </c>
+      <c r="B21" s="82" t="n"/>
       <c r="C21" s="81" t="inlineStr">
         <is>
-          <t>支持GRE/GTP-U/HTTP2等明文隧道内层流量检测</t>
+          <t>支持NPBroker转发流量类型选择（TLS解密/未解密/非TLS）</t>
         </is>
       </c>
       <c r="D21" s="81" t="inlineStr">
         <is>
-          <t>GRE/GTP-U/VXLAN/非加密IPSec隧道内层流量解封装检测</t>
+          <t>TLS解密/未解密/非TLS流量类型选择</t>
         </is>
       </c>
       <c r="E21" s="81" t="inlineStr">
         <is>
-          <t>PA隧道检测策略解封装并深度检测GRE/GTP-U/VXLAN/非加密IPSec（NULL加密/AH传输模式）等明文隧道内容（PA Web帮助p172-173）；对应矩阵#128/37</t>
+          <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证（PA Web帮助p167）；天融信无网络数据包代理模块（矩阵#122）</t>
         </is>
       </c>
       <c r="F21" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G21" s="81" t="inlineStr"/>
       <c r="H21" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="I21" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="51" customHeight="1" s="1">
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I21" s="80" t="inlineStr"/>
+    </row>
+    <row r="22" ht="96" customHeight="1" s="1">
       <c r="A22" s="82" t="n"/>
-      <c r="B22" s="82" t="n"/>
+      <c r="B22" s="80" t="inlineStr">
+        <is>
+          <t>隧道检测(Tunnel Inspection)</t>
+        </is>
+      </c>
       <c r="C22" s="81" t="inlineStr">
         <is>
-          <t>支持最大封装级数防护（max_encap）</t>
+          <t>支持GTP-U/VXLAN/非加密IPSec隧道内层检测</t>
         </is>
       </c>
       <c r="D22" s="81" t="inlineStr">
         <is>
-          <t>隧道嵌套封装最大级数限制，超限丢弃</t>
+          <t>GTP-U/VXLAN/NULL加密IPSec(AH)隧道内层流量检测</t>
         </is>
       </c>
       <c r="E22" s="81" t="inlineStr">
         <is>
-          <t>PA对隧道最大封装级数超限丢包防护，防隧道嵌套绕过（PA管理指南p655）；天融信手册无封装级数防护（检索无命中）</t>
+          <t>PA隧道检测支持GTP-U/VXLAN/非加密IPSec（NULL加密/AH传输模式）内层检测（PA Web帮助p172-173）；天融信VXLAN仅隧道封装转发与三层网关（天融信手册《业务接入端》《三层VXLAN网关》页），无内层安全检测，GTP检测检索无命中；对应矩阵#128/37</t>
         </is>
       </c>
       <c r="F22" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G22" s="81" t="inlineStr"/>
@@ -5591,66 +5655,62 @@
       </c>
       <c r="I22" s="80" t="inlineStr"/>
     </row>
-    <row r="23" ht="96" customHeight="1" s="1">
+    <row r="23" ht="51" customHeight="1" s="1">
       <c r="A23" s="82" t="n"/>
-      <c r="B23" s="80" t="inlineStr">
-        <is>
-          <t>应用覆盖(App Override)</t>
-        </is>
-      </c>
+      <c r="B23" s="82" t="n"/>
       <c r="C23" s="81" t="inlineStr">
         <is>
-          <t>支持应用替代流量跳过七层检测等效配置</t>
+          <t>支持最大封装级数防护（max_encap）</t>
         </is>
       </c>
       <c r="D23" s="81" t="inlineStr">
         <is>
-          <t>匹配覆盖策略的流量跳过七层检测，四层快速转发</t>
+          <t>隧道嵌套封装最大级数限制，超限丢弃</t>
         </is>
       </c>
       <c r="E23" s="81" t="inlineStr">
         <is>
-          <t>PA应用替代策略明确绕过第7层处理与威胁检查，改用第4层状态检查以加速（PA管理指南p1307）；天融信自定义应用加入规则库后仍默认经安全引擎检测（天融信手册《自定义应用》页）；迁移评估项：PA应用替代多为私有大流量业务加速，转换时需同步关闭对应策略的IPS/七层检测，否则性能被拖垮或误阻断</t>
+          <t>PA对隧道最大封装级数超限丢包防护，防隧道嵌套绕过（PA管理指南p655）；天融信手册无封装级数防护（检索无命中）</t>
         </is>
       </c>
       <c r="F23" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G23" s="81" t="inlineStr"/>
       <c r="H23" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>不支持</t>
         </is>
       </c>
       <c r="I23" s="80" t="inlineStr"/>
     </row>
-    <row r="24" ht="81" customHeight="1" s="1">
+    <row r="24" ht="96" customHeight="1" s="1">
       <c r="A24" s="82" t="n"/>
       <c r="B24" s="80" t="inlineStr">
         <is>
-          <t>身份验证(Authentication)</t>
+          <t>应用覆盖(App Override)</t>
         </is>
       </c>
       <c r="C24" s="81" t="inlineStr">
         <is>
-          <t>支持认证策略超时与单次认证（SSO）</t>
+          <t>支持应用替代流量跳过七层检测等效配置</t>
         </is>
       </c>
       <c r="D24" s="81" t="inlineStr">
         <is>
-          <t>认证超时+单次认证(SSO)</t>
+          <t>匹配覆盖策略的流量跳过七层检测，四层快速转发</t>
         </is>
       </c>
       <c r="E24" s="81" t="inlineStr">
         <is>
-          <t>PA支持认证超时减少重复质询、Kerberos/SAML/RADIUS等对接（PA Web帮助p186）；天融信手册检索认证超时/单点登录/SSO无命中（仅在线用户在线时长查看与强制下线）；迁移评估项：需核实天融信认证会话有效期配置与SSO对接能力</t>
+          <t>PA应用替代策略明确绕过第7层处理与威胁检查，改用第4层状态检查以加速（PA管理指南p1307）；天融信自定义应用加入规则库后仍默认经安全引擎检测（天融信手册《自定义应用》页）；迁移评估项：PA应用替代多为私有大流量业务加速，转换时需同步关闭对应策略的IPS/七层检测，否则性能被拖垮或误阻断</t>
         </is>
       </c>
       <c r="F24" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G24" s="81" t="inlineStr"/>
@@ -5661,22 +5721,26 @@
       </c>
       <c r="I24" s="80" t="inlineStr"/>
     </row>
-    <row r="25" ht="126" customHeight="1" s="1">
+    <row r="25" ht="81" customHeight="1" s="1">
       <c r="A25" s="82" t="n"/>
-      <c r="B25" s="82" t="n"/>
+      <c r="B25" s="80" t="inlineStr">
+        <is>
+          <t>身份验证(Authentication)</t>
+        </is>
+      </c>
       <c r="C25" s="81" t="inlineStr">
         <is>
-          <t>支持基于策略触发多因素认证质询（MFA Enforcement）</t>
+          <t>支持认证策略超时与单次认证（SSO）</t>
         </is>
       </c>
       <c r="D25" s="81" t="inlineStr">
         <is>
-          <t>策略匹配触发多因素认证质询（MFA供应商API/RADIUS）</t>
+          <t>认证超时+单次认证(SSO)</t>
         </is>
       </c>
       <c r="E25" s="81" t="inlineStr">
         <is>
-          <t>PA身份验证策略通过Authentication Enforcement对象对匹配流量强制质询，支持多因素身份验证（每因素独立超时，防火墙记录时间戳），MFA供应商API/RADIUS对接（PA Web帮助p185-186、p310、p735-742）；天融信双因子认证（密码+短信/证书/Ukey）仅限管理员/用户登录场景（天融信手册《登录安全策略》页），未见流量策略触发MFA质询</t>
+          <t>PA支持认证超时减少重复质询、Kerberos/SAML/RADIUS等对接（PA Web帮助p186）；天融信手册检索认证超时/单点登录/SSO无命中（仅在线用户在线时长查看与强制下线）；迁移评估项：需核实天融信认证会话有效期配置与SSO对接能力</t>
         </is>
       </c>
       <c r="F25" s="80" t="inlineStr">
@@ -5687,89 +5751,89 @@
       <c r="G25" s="81" t="inlineStr"/>
       <c r="H25" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
+          <t>待评估</t>
         </is>
       </c>
       <c r="I25" s="80" t="inlineStr"/>
     </row>
-    <row r="26" ht="96" customHeight="1" s="1">
+    <row r="26" ht="126" customHeight="1" s="1">
       <c r="A26" s="82" t="n"/>
       <c r="B26" s="82" t="n"/>
       <c r="C26" s="81" t="inlineStr">
         <is>
+          <t>支持流量策略触发多因素认证质询（MFA Enforcement）</t>
+        </is>
+      </c>
+      <c r="D26" s="81" t="inlineStr">
+        <is>
+          <t>流量策略匹配触发MFA质询（非登录场景，MFA供应商API/RADIUS）</t>
+        </is>
+      </c>
+      <c r="E26" s="81" t="inlineStr">
+        <is>
+          <t>PA身份验证策略通过Authentication Enforcement对象对匹配流量强制质询，支持多因素身份验证（每因素独立超时，防火墙记录时间戳），MFA供应商API/RADIUS对接（PA Web帮助p185-186、p310、p735-742）；天融信双因子认证（密码+短信/证书/Ukey）仅限管理员/用户登录场景（天融信手册《登录安全策略》页），无流量策略触发MFA质询</t>
+        </is>
+      </c>
+      <c r="F26" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G26" s="81" t="inlineStr"/>
+      <c r="H26" s="80" t="inlineStr">
+        <is>
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I26" s="80" t="inlineStr"/>
+    </row>
+    <row r="27" ht="96" customHeight="1" s="1">
+      <c r="A27" s="82" t="n"/>
+      <c r="B27" s="82" t="n"/>
+      <c r="C27" s="81" t="inlineStr">
+        <is>
           <t>支持User-ID动态映射时效性等效（AD日志毫秒级更新）</t>
         </is>
       </c>
-      <c r="D26" s="81" t="inlineStr">
+      <c r="D27" s="81" t="inlineStr">
         <is>
           <t>AD域事件日志毫秒级IP-用户映射更新</t>
         </is>
       </c>
-      <c r="E26" s="81" t="inlineStr">
+      <c r="E27" s="81" t="inlineStr">
         <is>
           <t>PA无代理架构通过读取域控事件日志实现IP-用户毫秒级动态映射，大规模部署有专项规划（PA管理指南p866-867）；天融信AD对接的轮询间隔与并发认证能力手册未量化；迁移评估项：数万AD用户且移动频繁场景需实测天融信映射更新时延，避免基于用户的策略出现间歇性未授权拦截</t>
         </is>
       </c>
-      <c r="F26" s="82" t="n"/>
-      <c r="G26" s="82" t="n"/>
-      <c r="H26" s="80" t="inlineStr">
+      <c r="F27" s="82" t="n"/>
+      <c r="G27" s="82" t="n"/>
+      <c r="H27" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="I26" s="82" t="n"/>
-    </row>
-    <row r="27" ht="171" customHeight="1" s="1">
-      <c r="A27" s="82" t="n"/>
-      <c r="B27" s="80" t="inlineStr">
+      <c r="I27" s="82" t="n"/>
+    </row>
+    <row r="28" ht="171" customHeight="1" s="1">
+      <c r="A28" s="82" t="n"/>
+      <c r="B28" s="80" t="inlineStr">
         <is>
           <t>动态对象(Dynamic Objects)</t>
         </is>
       </c>
-      <c r="C27" s="81" t="inlineStr">
+      <c r="C28" s="81" t="inlineStr">
         <is>
           <t>支持外部动态列表作为策略地址对象（EDL）</t>
         </is>
       </c>
-      <c r="D27" s="81" t="inlineStr">
+      <c r="D28" s="81" t="inlineStr">
         <is>
           <t>HTTP/HTTPS外部文本列表(IP/域名/URL)自动拉取，策略直接引用</t>
         </is>
       </c>
-      <c r="E27" s="81" t="inlineStr">
+      <c r="E28" s="81" t="inlineStr">
         <is>
           <t>PA外部动态列表：基于HTTP/HTTPS托管的文本文件创建IP/URL/域名/IMEI/IMSI地址对象，防火墙定时自动拉取更新，策略中直接引用（Objects&gt;External Dynamic Lists，PA Web帮助p236-239；策略源/目标可直接选EDL，p196-197）；天融信手册检索外部动态列表/EDL无命中，仅内置威胁情报库与云端威胁情报库（规则集管理，天融信手册《威胁情报》《配置规则集》页），无策略直接引用任意外部文本列表机制；迁移评估项：PA策略中引用的EDL需转换为天融信静态地址组定期导入或威胁情报联动</t>
-        </is>
-      </c>
-      <c r="F27" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="G27" s="81" t="inlineStr"/>
-      <c r="H27" s="80" t="inlineStr">
-        <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="I27" s="80" t="inlineStr"/>
-    </row>
-    <row r="28" ht="126" customHeight="1" s="1">
-      <c r="A28" s="82" t="n"/>
-      <c r="B28" s="82" t="n"/>
-      <c r="C28" s="81" t="inlineStr">
-        <is>
-          <t>支持基于标记的动态地址组（DAG）</t>
-        </is>
-      </c>
-      <c r="D28" s="81" t="inlineStr">
-        <is>
-          <t>Tag标记过滤器动态地址组，成员随IP变化自动更新</t>
-        </is>
-      </c>
-      <c r="E28" s="81" t="inlineStr">
-        <is>
-          <t>PA动态地址组：查找标记(Tag)+基于标记的过滤器（AND/OR匹配）动态填充成员，VM信息源注册或XML/REST API定义标记，IP变化时策略自动生效（PA Web帮助p207-208、p228）；天融信手册检索动态地址组/标签/SDN/云平台联动无命中，地址组为静态IP/子网绑定（天融信手册《地址》页）；迁移评估项：PA云环境Tag微隔离策略需转换为静态地址组，IP漂移场景需人工或API维护</t>
         </is>
       </c>
       <c r="F28" s="80" t="inlineStr">
@@ -5785,66 +5849,62 @@
       </c>
       <c r="I28" s="80" t="inlineStr"/>
     </row>
-    <row r="29" ht="51" customHeight="1" s="1">
+    <row r="29" ht="126" customHeight="1" s="1">
       <c r="A29" s="82" t="n"/>
-      <c r="B29" s="80" t="inlineStr">
-        <is>
-          <t>SD-WAN策略</t>
-        </is>
-      </c>
+      <c r="B29" s="82" t="n"/>
       <c r="C29" s="81" t="inlineStr">
         <is>
-          <t>支持按应用配置链路路径管理与链路质量探测</t>
+          <t>支持基于标记的动态地址组（DAG）</t>
         </is>
       </c>
       <c r="D29" s="81" t="inlineStr">
         <is>
-          <t>按应用/区域/地址分配链路与流量分发</t>
+          <t>Tag标记过滤器动态地址组，成员随IP变化自动更新</t>
         </is>
       </c>
       <c r="E29" s="81" t="inlineStr">
         <is>
-          <t>PA SD-WAN策略按应用/抖动/延迟/丢包指标分配链路，流量分发（PA Web帮助p197）；对应矩阵#129/120</t>
+          <t>PA动态地址组：查找标记(Tag)+基于标记的过滤器（AND/OR匹配）动态填充成员，VM信息源注册或XML/REST API定义标记，IP变化时策略自动生效（PA Web帮助p207-208、p228）；天融信手册检索动态地址组/标签/SDN/云平台联动无命中，地址组为静态IP/子网绑定（天融信手册《地址》页）；迁移评估项：PA云环境Tag微隔离策略需转换为静态地址组，IP漂移场景需人工或API维护</t>
         </is>
       </c>
       <c r="F29" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G29" s="81" t="inlineStr"/>
       <c r="H29" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="I29" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I29" s="80" t="inlineStr"/>
     </row>
     <row r="30" ht="81" customHeight="1" s="1">
       <c r="A30" s="82" t="n"/>
-      <c r="B30" s="82" t="n"/>
+      <c r="B30" s="80" t="inlineStr">
+        <is>
+          <t>SD-WAN策略</t>
+        </is>
+      </c>
       <c r="C30" s="81" t="inlineStr">
         <is>
-          <t>支持SD-WAN路径选择与链路质量监测（jitter/latency/loss）</t>
+          <t>支持按应用配置链路路径管理与链路质量探测</t>
         </is>
       </c>
       <c r="D30" s="81" t="inlineStr">
         <is>
-          <t>抖动/延迟/丢包(jitter/latency/loss)指标选路</t>
+          <t>按应用分配链路与流量分发（天融信以策略路由+LLB近似实现）</t>
         </is>
       </c>
       <c r="E30" s="81" t="inlineStr">
         <is>
-          <t>PA路径质量配置文件基于抖动/延迟/丢包等运行状况指标选路（PA Web帮助p195）；天融信有链路探测(ping)+智能选路(最小延迟优先)（天融信手册《策略路由》页），无jitter/latency/loss多维指标</t>
+          <t>PA SD-WAN策略按应用/抖动/延迟/丢包指标分配链路，流量分发（PA Web帮助p197）；天融信为策略路由+链路负载均衡近似实现（天融信手册《策略路由》《链路负载均衡》页），无SD-WAN策略模型；对应矩阵#129/120</t>
         </is>
       </c>
       <c r="F30" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G30" s="81" t="inlineStr"/>
@@ -5853,35 +5913,70 @@
           <t>部分支持</t>
         </is>
       </c>
-      <c r="I30" s="80" t="inlineStr"/>
+      <c r="I30" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="81" customHeight="1" s="1">
+      <c r="A31" s="82" t="n"/>
+      <c r="B31" s="82" t="n"/>
+      <c r="C31" s="81" t="inlineStr">
+        <is>
+          <t>支持SD-WAN路径选择与链路质量监测（jitter/latency/loss）</t>
+        </is>
+      </c>
+      <c r="D31" s="81" t="inlineStr">
+        <is>
+          <t>抖动/延迟/丢包多维指标选路（天融信现仅延迟探测）</t>
+        </is>
+      </c>
+      <c r="E31" s="81" t="inlineStr">
+        <is>
+          <t>PA路径质量配置文件基于抖动/延迟/丢包等运行状况指标选路（PA Web帮助p195）；天融信有链路探测(ping)+智能选路(最小延迟优先)（天融信手册《策略路由》页），无jitter/latency/loss多维指标</t>
+        </is>
+      </c>
+      <c r="F31" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G31" s="81" t="inlineStr"/>
+      <c r="H31" s="80" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="I31" s="80" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="I17:I19"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="I6:I11"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="A2:A30"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="I26:I27"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="B5:B11"/>
+    <mergeCell ref="F26:F27"/>
     <mergeCell ref="G3:G4"/>
-    <mergeCell ref="G16:G18"/>
     <mergeCell ref="I3:I4"/>
-    <mergeCell ref="I6:I10"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="H7:H10"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="G17:G19"/>
     <mergeCell ref="H3:H4"/>
-    <mergeCell ref="B15:B18"/>
+    <mergeCell ref="G6:G11"/>
+    <mergeCell ref="B20:B21"/>
     <mergeCell ref="B2:B4"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="I16:I18"/>
-    <mergeCell ref="B5:B10"/>
-    <mergeCell ref="G6:G10"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="A2:A31"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="H8:H11"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="B16:B19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: update PA strategy migration spreadsheet
add WildFire cloud sandbox detection migration entry to the strategy sheet, update related evaluation status and notes
</commit_message>
<xml_diff>
--- a/PA替代需求列表.xlsx
+++ b/PA替代需求列表.xlsx
@@ -3279,7 +3279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.7" customWidth="1" style="1" min="1" max="1"/>
@@ -3733,7 +3733,7 @@
     </row>
     <row r="15" ht="156" customHeight="1" s="1">
       <c r="A15" s="84" t="n"/>
-      <c r="B15" s="85" t="n"/>
+      <c r="B15" s="84" t="n"/>
       <c r="C15" s="81" t="inlineStr">
         <is>
           <t>支持隐式默认规则显式化迁移（intrazone/interzone-default）</t>
@@ -3754,41 +3754,33 @@
           <t>高</t>
         </is>
       </c>
-      <c r="G15" s="85" t="n"/>
+      <c r="G15" s="84" t="n"/>
       <c r="H15" s="85" t="n"/>
       <c r="I15" s="85" t="n"/>
     </row>
-    <row r="16" ht="81" customHeight="1" s="1">
+    <row r="16" ht="171" customHeight="1" s="1">
       <c r="A16" s="84" t="n"/>
-      <c r="B16" s="80" t="inlineStr">
-        <is>
-          <t>NAT策略</t>
-        </is>
-      </c>
+      <c r="B16" s="85" t="n"/>
       <c r="C16" s="81" t="inlineStr">
         <is>
-          <t>支持源NAT（动态/PAT静态IP）与Hairpin回流</t>
+          <t>支持WildFire云沙箱文件检测联动（Advanced WildFire）</t>
         </is>
       </c>
       <c r="D16" s="81" t="inlineStr">
         <is>
-          <t>动态IP+端口(DIPP)/静态IP/接口地址，含回流(Hairpin)</t>
+          <t>未知文件云沙箱实时分析+签名秒级下发，策略Actions绑定WildFire配置文件</t>
         </is>
       </c>
       <c r="E16" s="81" t="inlineStr">
         <is>
-          <t>PA源NAT含DIPP动态IP+端口/静态IP/接口地址/持久NAT等（PA Web帮助p147）；天融信SNAT地址池（多对一/多对多/一对一/PAT）与仅源IP转换等（天融信手册《源NAT》《配置源转换》页）；对应矩阵#6</t>
-        </is>
-      </c>
-      <c r="F16" s="80" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="G16" s="81" t="inlineStr"/>
+          <t>PA策略Actions可绑定WildFire Analysis配置文件（安全配置文件组含反病毒/漏洞/URL/文件阻断/WildFire，PA Web帮助p304；WildFire提交日志转发p305-306），云沙箱动态分析未知/零日威胁并秒级下发签名；天融信有内置APT沙箱（虚拟运行环境检测未知漏洞威胁）与沙箱联动（天融信手册《高级威胁防护》《APT联动配置》页），无云端动态分析与秒级签名下发证据；工作表1已登记云沙箱联动需求（不支持：公司无此产品），勿重复跟踪；迁移评估项：评估天融信本地APT沙箱与PA云沙箱检测能力等效性</t>
+        </is>
+      </c>
+      <c r="F16" s="85" t="n"/>
+      <c r="G16" s="85" t="n"/>
       <c r="H16" s="80" t="inlineStr">
         <is>
-          <t>已支持</t>
+          <t>部分支持</t>
         </is>
       </c>
       <c r="I16" s="80" t="inlineStr">
@@ -3799,20 +3791,24 @@
     </row>
     <row r="17" ht="81" customHeight="1" s="1">
       <c r="A17" s="84" t="n"/>
-      <c r="B17" s="84" t="n"/>
+      <c r="B17" s="80" t="inlineStr">
+        <is>
+          <t>NAT策略</t>
+        </is>
+      </c>
       <c r="C17" s="81" t="inlineStr">
         <is>
-          <t>支持目的NAT（端口映射/服务器发布）</t>
+          <t>支持源NAT（动态/PAT静态IP）与Hairpin回流</t>
         </is>
       </c>
       <c r="D17" s="81" t="inlineStr">
         <is>
-          <t>静态映射/端口转换/DNS重写/FQDN目标</t>
+          <t>动态IP+端口(DIPP)/静态IP/接口地址，含回流(Hairpin)</t>
         </is>
       </c>
       <c r="E17" s="81" t="inlineStr">
         <is>
-          <t>PA目标NAT含静态/动态IP、端口转换、DNS Rewrite、FQDN目标（PA Web帮助p149）；天融信服务器映射含静态映射+服务器负载均衡两种模式，NAT46/NAT66全系列（天融信手册《服务器映射》页）；对应矩阵#7</t>
+          <t>PA源NAT含DIPP动态IP+端口/静态IP/接口地址/持久NAT等（PA Web帮助p147）；天融信SNAT地址池（多对一/多对多/一对一/PAT）与仅源IP转换等（天融信手册《源NAT》《配置源转换》页）；对应矩阵#6</t>
         </is>
       </c>
       <c r="F17" s="80" t="inlineStr">
@@ -3826,50 +3822,62 @@
           <t>已支持</t>
         </is>
       </c>
-      <c r="I17" s="80" t="inlineStr"/>
+      <c r="I17" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="81" customHeight="1" s="1">
       <c r="A18" s="84" t="n"/>
       <c r="B18" s="84" t="n"/>
       <c r="C18" s="81" t="inlineStr">
         <is>
-          <t>支持静态/双向NAT一对一转换</t>
+          <t>支持目的NAT（端口映射/服务器发布）</t>
         </is>
       </c>
       <c r="D18" s="81" t="inlineStr">
         <is>
-          <t>一对一转换，支持双向映射</t>
+          <t>静态映射/端口转换/DNS重写/FQDN目标</t>
         </is>
       </c>
       <c r="E18" s="81" t="inlineStr">
         <is>
-          <t>PA支持静态IP转换与双向(Bi-directional)转换（PA Web帮助p148）；天融信支持一对一转换（SNAT地址池一对一/NAT66一对一）（天融信手册《源NAT》《配置一对一转换》页）；对应矩阵#8</t>
-        </is>
-      </c>
-      <c r="F18" s="84" t="n"/>
-      <c r="G18" s="84" t="n"/>
-      <c r="H18" s="84" t="n"/>
-      <c r="I18" s="84" t="n"/>
+          <t>PA目标NAT含静态/动态IP、端口转换、DNS Rewrite、FQDN目标（PA Web帮助p149）；天融信服务器映射含静态映射+服务器负载均衡两种模式，NAT46/NAT66全系列（天融信手册《服务器映射》页）；对应矩阵#7</t>
+        </is>
+      </c>
+      <c r="F18" s="80" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="G18" s="81" t="inlineStr"/>
+      <c r="H18" s="80" t="inlineStr">
+        <is>
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I18" s="80" t="inlineStr"/>
     </row>
     <row r="19" ht="81" customHeight="1" s="1">
       <c r="A19" s="84" t="n"/>
       <c r="B19" s="84" t="n"/>
       <c r="C19" s="81" t="inlineStr">
         <is>
-          <t>支持NAT与安全策略解耦独立配置</t>
+          <t>支持静态/双向NAT一对一转换</t>
         </is>
       </c>
       <c r="D19" s="81" t="inlineStr">
         <is>
-          <t>NAT独立策略库，先NAT后安全策略匹配</t>
+          <t>一对一转换，支持双向映射</t>
         </is>
       </c>
       <c r="E19" s="81" t="inlineStr">
         <is>
-          <t>PA NAT策略库独立于安全策略库(Policies&gt;NAT)，先NAT后安全匹配；天融信地址转换为独立策略库（安全策略&gt;地址转换），与访问控制策略分离配置（天融信手册《安全策略》《工作原理》页）；对应矩阵#9</t>
-        </is>
-      </c>
-      <c r="F19" s="85" t="n"/>
+          <t>PA支持静态IP转换与双向(Bi-directional)转换（PA Web帮助p148）；天融信支持一对一转换（SNAT地址池一对一/NAT66一对一）（天融信手册《源NAT》《配置一对一转换》页）；对应矩阵#8</t>
+        </is>
+      </c>
+      <c r="F19" s="84" t="n"/>
       <c r="G19" s="84" t="n"/>
       <c r="H19" s="84" t="n"/>
       <c r="I19" s="84" t="n"/>
@@ -3879,215 +3887,203 @@
       <c r="B20" s="84" t="n"/>
       <c r="C20" s="81" t="inlineStr">
         <is>
-          <t>支持IPv6/NAT64转换（nat64类型）</t>
+          <t>支持NAT与安全策略解耦独立配置</t>
         </is>
       </c>
       <c r="D20" s="81" t="inlineStr">
         <is>
-          <t>IPv4↔IPv6转换类型（nat64）</t>
+          <t>NAT独立策略库，先NAT后安全策略匹配</t>
         </is>
       </c>
       <c r="E20" s="81" t="inlineStr">
         <is>
-          <t>PA NAT规则支持IPv4/IPv6及NAT64转换类型（RFC6146）；天融信NAT64含静态转换+前缀转换+动态算法（IVI/普通前缀），另有NAT46（天融信手册《NAT64》《NAT46》页）；对应矩阵#18</t>
-        </is>
-      </c>
-      <c r="F20" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
+          <t>PA NAT策略库独立于安全策略库(Policies&gt;NAT)，先NAT后安全匹配；天融信地址转换为独立策略库（安全策略&gt;地址转换），与访问控制策略分离配置（天融信手册《安全策略》《工作原理》页）；对应矩阵#9</t>
+        </is>
+      </c>
+      <c r="F20" s="85" t="n"/>
       <c r="G20" s="84" t="n"/>
-      <c r="H20" s="85" t="n"/>
+      <c r="H20" s="84" t="n"/>
       <c r="I20" s="84" t="n"/>
     </row>
-    <row r="21" ht="126" customHeight="1" s="1">
+    <row r="21" ht="81" customHeight="1" s="1">
       <c r="A21" s="84" t="n"/>
       <c r="B21" s="84" t="n"/>
       <c r="C21" s="81" t="inlineStr">
         <is>
+          <t>支持IPv6/NAT64转换（nat64类型）</t>
+        </is>
+      </c>
+      <c r="D21" s="81" t="inlineStr">
+        <is>
+          <t>IPv4↔IPv6转换类型（nat64）</t>
+        </is>
+      </c>
+      <c r="E21" s="81" t="inlineStr">
+        <is>
+          <t>PA NAT规则支持IPv4/IPv6及NAT64转换类型（RFC6146）；天融信NAT64含静态转换+前缀转换+动态算法（IVI/普通前缀），另有NAT46（天融信手册《NAT64》《NAT46》页）；对应矩阵#18</t>
+        </is>
+      </c>
+      <c r="F21" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G21" s="84" t="n"/>
+      <c r="H21" s="85" t="n"/>
+      <c r="I21" s="84" t="n"/>
+    </row>
+    <row r="22" ht="126" customHeight="1" s="1">
+      <c r="A22" s="84" t="n"/>
+      <c r="B22" s="84" t="n"/>
+      <c r="C22" s="81" t="inlineStr">
+        <is>
           <t>支持NAT后目的区域路由回查匹配（Dest Zone by route lookup）</t>
         </is>
       </c>
-      <c r="D21" s="81" t="inlineStr">
+      <c r="D22" s="81" t="inlineStr">
         <is>
           <t>目的区域按NAT后路由查找；源/目的地址用NAT前值</t>
         </is>
       </c>
-      <c r="E21" s="81" t="inlineStr">
+      <c r="E22" s="81" t="inlineStr">
         <is>
           <t>PA底层为『先NAT判断后安全策略匹配』的因果倒置：安全策略要求源区域(NAT前)+源地址(NAT前)+目的地址(NAT前)+目的区域(NAT后按路由查找)，极其反直觉；天融信地址转换为独立策略库常规直观映射（安全策略&gt;地址转换，天融信手册《服务器映射》页）；迁移评估项：带目的NAT的策略平移后易因Zone填写错误不通，需制定NAT查表逻辑转换映射规范；对应矩阵#9</t>
         </is>
       </c>
-      <c r="F21" s="80" t="inlineStr">
+      <c r="F22" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="G21" s="84" t="n"/>
-      <c r="H21" s="80" t="inlineStr">
+      <c r="G22" s="84" t="n"/>
+      <c r="H22" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="I21" s="84" t="n"/>
-    </row>
-    <row r="22" ht="81" customHeight="1" s="1">
-      <c r="A22" s="84" t="n"/>
-      <c r="B22" s="85" t="n"/>
-      <c r="C22" s="81" t="inlineStr">
+      <c r="I22" s="84" t="n"/>
+    </row>
+    <row r="23" ht="81" customHeight="1" s="1">
+      <c r="A23" s="84" t="n"/>
+      <c r="B23" s="85" t="n"/>
+      <c r="C23" s="81" t="inlineStr">
         <is>
           <t>支持NAT规则主动/主动HA绑定（Active/Active HA Binding）</t>
         </is>
       </c>
-      <c r="D22" s="81" t="inlineStr">
+      <c r="D23" s="81" t="inlineStr">
         <is>
           <t>主动/主动HA下NAT规则绑定会话所有者</t>
         </is>
       </c>
-      <c r="E22" s="81" t="inlineStr">
+      <c r="E23" s="81" t="inlineStr">
         <is>
           <t>PA主动/主动HA配置下NAT规则可绑定会话所有者/会话设置，控制NAT会话的设备绑定，仅A/A模式可见（PA Web帮助p150）；天融信HA为主备双机热备模式（天融信手册《配置双机热备功能》页），无主动/主动模式及NAT规则绑定机制</t>
         </is>
       </c>
-      <c r="F22" s="80" t="inlineStr">
+      <c r="F23" s="80" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="G22" s="85" t="n"/>
-      <c r="H22" s="80" t="inlineStr">
+      <c r="G23" s="85" t="n"/>
+      <c r="H23" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="I22" s="85" t="n"/>
-    </row>
-    <row r="23" ht="96" customHeight="1" s="1">
-      <c r="A23" s="84" t="n"/>
-      <c r="B23" s="80" t="inlineStr">
-        <is>
-          <t>QoS策略</t>
-        </is>
-      </c>
-      <c r="C23" s="81" t="inlineStr">
-        <is>
-          <t>支持按应用/源地址/用户等定义QoS策略并划分优先级类</t>
-        </is>
-      </c>
-      <c r="D23" s="81" t="inlineStr">
-        <is>
-          <t>8类流量分类+4级优先级，保证/最大带宽控制</t>
-        </is>
-      </c>
-      <c r="E23" s="81" t="inlineStr">
-        <is>
-          <t>PA QoS策略规则分配QoS类（8类+4级优先级），按Egress Guaranteed/Max控制带宽（PA Web帮助p154-155）；天融信流量管理基于应用/用户/源目的区域/地址/服务/时间+通道优先级，虚拟通道限制与保证带宽（天融信手册《流量管理》页）；对应矩阵#33/66</t>
-        </is>
-      </c>
-      <c r="F23" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="G23" s="81" t="inlineStr"/>
-      <c r="H23" s="80" t="inlineStr">
-        <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I23" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
+      <c r="I23" s="85" t="n"/>
     </row>
     <row r="24" ht="96" customHeight="1" s="1">
       <c r="A24" s="84" t="n"/>
-      <c r="B24" s="85" t="n"/>
+      <c r="B24" s="80" t="inlineStr">
+        <is>
+          <t>QoS策略</t>
+        </is>
+      </c>
       <c r="C24" s="81" t="inlineStr">
         <is>
-          <t>支持QoS策略规则内直接按DSCP/ToS匹配调度</t>
+          <t>支持按应用/源地址/用户等定义QoS策略并划分优先级类</t>
         </is>
       </c>
       <c r="D24" s="81" t="inlineStr">
         <is>
-          <t>QoS策略规则DSCP/ToS直接匹配（非独立流控模块配置）</t>
+          <t>8类流量分类+4级优先级，保证/最大带宽控制</t>
         </is>
       </c>
       <c r="E24" s="81" t="inlineStr">
         <is>
-          <t>PA QoS规则可直接按DSCP值或IP优先级/ToS匹配调度（PA Web帮助p155）；天融信支持DSCP/802.1p(CoS)识别与重标记，但需在独立流量管理模块配置（虚拟通道+限制/保证带宽+通道优先级，天融信手册《流量管理》页），未直接耦合在基础访问控制策略表内（联网核实厂商流控资料，手册未详载）</t>
+          <t>PA QoS策略规则分配QoS类（8类+4级优先级），按Egress Guaranteed/Max控制带宽（PA Web帮助p154-155）；天融信流量管理基于应用/用户/源目的区域/地址/服务/时间+通道优先级，虚拟通道限制与保证带宽（天融信手册《流量管理》页）；对应矩阵#33/66</t>
         </is>
       </c>
       <c r="F24" s="80" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G24" s="81" t="inlineStr"/>
       <c r="H24" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="I24" s="80" t="inlineStr"/>
-    </row>
-    <row r="25" ht="81" customHeight="1" s="1">
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I24" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="96" customHeight="1" s="1">
       <c r="A25" s="84" t="n"/>
-      <c r="B25" s="80" t="inlineStr">
-        <is>
-          <t>基于策略转发(PBF)</t>
-        </is>
-      </c>
+      <c r="B25" s="85" t="n"/>
       <c r="C25" s="81" t="inlineStr">
         <is>
-          <t>支持按源区域/地址/用户/应用/服务+下一跳的基于策略转发</t>
+          <t>支持QoS策略规则内直接按DSCP/ToS匹配调度</t>
         </is>
       </c>
       <c r="D25" s="81" t="inlineStr">
         <is>
-          <t>按源区域/地址/用户/应用/服务+下一跳转发，路径监控失效切换</t>
+          <t>QoS策略规则DSCP/ToS直接匹配（非独立流控模块配置）</t>
         </is>
       </c>
       <c r="E25" s="81" t="inlineStr">
         <is>
-          <t>PA PBF策略绕过常规路由表选路，支持路径监控与失效切换、BFD、强制对称返回（PA Web帮助p156）；天融信策略路由按源/目的地址端口、ISP名称、协议、角色等参数选路（天融信手册《策略路由》页）；对应矩阵#10</t>
+          <t>PA QoS规则可直接按DSCP值或IP优先级/ToS匹配调度（PA Web帮助p155）；天融信支持DSCP/802.1p(CoS)识别与重标记，但需在独立流量管理模块配置（虚拟通道+限制/保证带宽+通道优先级，天融信手册《流量管理》页），未直接耦合在基础访问控制策略表内（联网核实厂商流控资料，手册未详载）</t>
         </is>
       </c>
       <c r="F25" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>低</t>
         </is>
       </c>
       <c r="G25" s="81" t="inlineStr"/>
       <c r="H25" s="80" t="inlineStr">
         <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I25" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="111" customHeight="1" s="1">
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="I25" s="80" t="inlineStr"/>
+    </row>
+    <row r="26" ht="81" customHeight="1" s="1">
       <c r="A26" s="84" t="n"/>
-      <c r="B26" s="85" t="n"/>
+      <c r="B26" s="80" t="inlineStr">
+        <is>
+          <t>基于策略转发(PBF)</t>
+        </is>
+      </c>
       <c r="C26" s="81" t="inlineStr">
         <is>
-          <t>支持PBF强制对称返回（非对称路由环境）</t>
+          <t>支持按源区域/地址/用户/应用/服务+下一跳的基于策略转发</t>
         </is>
       </c>
       <c r="D26" s="81" t="inlineStr">
         <is>
-          <t>记录入接口MAC，回包强制原路返回</t>
+          <t>按源区域/地址/用户/应用/服务+下一跳转发，路径监控失效切换</t>
         </is>
       </c>
       <c r="E26" s="81" t="inlineStr">
         <is>
-          <t>PA对称返回：虚拟路由器替代返回流量的路由查找，将流量引导回接收SYN数据包的MAC地址（ARP表确定下一跳），双ISP双活/非对称路由核心机制（PA管理指南p1294）；天融信手册检索无对称返回/回程机制命中，策略路由与LLB的回程保障能力待验证；迁移评估项：多ISP双活环境需实测天融信回包路由对称性，否则现网业务中断</t>
+          <t>PA PBF策略绕过常规路由表选路，支持路径监控与失效切换、BFD、强制对称返回（PA Web帮助p156）；天融信策略路由按源/目的地址端口、ISP名称、协议、角色等参数选路（天融信手册《策略路由》页）；对应矩阵#10</t>
         </is>
       </c>
       <c r="F26" s="80" t="inlineStr">
@@ -4098,31 +4094,31 @@
       <c r="G26" s="81" t="inlineStr"/>
       <c r="H26" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
-        </is>
-      </c>
-      <c r="I26" s="80" t="inlineStr"/>
-    </row>
-    <row r="27" ht="96" customHeight="1" s="1">
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I26" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="111" customHeight="1" s="1">
       <c r="A27" s="84" t="n"/>
-      <c r="B27" s="80" t="inlineStr">
-        <is>
-          <t>解密策略(Decryption)</t>
-        </is>
-      </c>
+      <c r="B27" s="85" t="n"/>
       <c r="C27" s="81" t="inlineStr">
         <is>
-          <t>支持SSL/TLS解密策略（出站正向/入站反向）</t>
+          <t>支持PBF强制对称返回（非对称路由环境）</t>
         </is>
       </c>
       <c r="D27" s="81" t="inlineStr">
         <is>
-          <t>出站正向代理+入站检查双向解密</t>
+          <t>记录入接口MAC，回包强制原路返回</t>
         </is>
       </c>
       <c r="E27" s="81" t="inlineStr">
         <is>
-          <t>PA解密策略区分SSL Forward Proxy/Inbound Inspection/SSH，可解密以获得流量可见性与深度检测（PA Web帮助p164）；天融信代理策略将NGFW作为代理服务器，对加密流量解密还原明文完成内容安全检查后重新加密（天融信手册《代理策略》页）；对应矩阵#29/30</t>
+          <t>PA对称返回：虚拟路由器替代返回流量的路由查找，将流量引导回接收SYN数据包的MAC地址（ARP表确定下一跳），双ISP双活/非对称路由核心机制（PA管理指南p1294）；天融信手册检索无对称返回/回程机制命中，策略路由与LLB的回程保障能力待验证；迁移评估项：多ISP双活环境需实测天融信回包路由对称性，否则现网业务中断</t>
         </is>
       </c>
       <c r="F27" s="80" t="inlineStr">
@@ -4133,36 +4129,36 @@
       <c r="G27" s="81" t="inlineStr"/>
       <c r="H27" s="80" t="inlineStr">
         <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I27" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="66" customHeight="1" s="1">
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="I27" s="80" t="inlineStr"/>
+    </row>
+    <row r="28" ht="96" customHeight="1" s="1">
       <c r="A28" s="84" t="n"/>
-      <c r="B28" s="84" t="n"/>
+      <c r="B28" s="80" t="inlineStr">
+        <is>
+          <t>解密策略(Decryption)</t>
+        </is>
+      </c>
       <c r="C28" s="81" t="inlineStr">
         <is>
-          <t>支持解密目标选择与证书配置</t>
+          <t>支持SSL/TLS解密策略（出站正向/入站反向）</t>
         </is>
       </c>
       <c r="D28" s="81" t="inlineStr">
         <is>
-          <t>入站证书配置/解密目标（数据包/会话）</t>
+          <t>出站正向代理+入站检查双向解密</t>
         </is>
       </c>
       <c r="E28" s="81" t="inlineStr">
         <is>
-          <t>PA解密目标允许指定数据包/会话；入站含Certificates证书配置；对应矩阵#31；天融信代理模板支持证书选择与预置动态证书模板（天融信手册《代理模板》页）</t>
+          <t>PA解密策略区分SSL Forward Proxy/Inbound Inspection/SSH，可解密以获得流量可见性与深度检测（PA Web帮助p164）；天融信代理策略将NGFW作为代理服务器，对加密流量解密还原明文完成内容安全检查后重新加密（天融信手册《代理策略》页）；对应矩阵#29/30</t>
         </is>
       </c>
       <c r="F28" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G28" s="81" t="inlineStr"/>
@@ -4171,180 +4167,180 @@
           <t>已支持</t>
         </is>
       </c>
-      <c r="I28" s="80" t="inlineStr"/>
-    </row>
-    <row r="29" ht="51" customHeight="1" s="1">
+      <c r="I28" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="66" customHeight="1" s="1">
       <c r="A29" s="84" t="n"/>
       <c r="B29" s="84" t="n"/>
       <c r="C29" s="81" t="inlineStr">
         <is>
-          <t>支持解密流量镜像到专用接口（Decryption Port Mirroring）</t>
+          <t>支持解密目标选择与证书配置</t>
         </is>
       </c>
       <c r="D29" s="81" t="inlineStr">
         <is>
-          <t>解密后明文流量镜像至专用接口供第三方分析</t>
+          <t>入站证书配置/解密目标（数据包/会话）</t>
         </is>
       </c>
       <c r="E29" s="81" t="inlineStr">
         <is>
-          <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证（PA管理指南p1059）；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
-        </is>
-      </c>
-      <c r="F29" s="85" t="n"/>
-      <c r="G29" s="84" t="n"/>
+          <t>PA解密目标允许指定数据包/会话；入站含Certificates证书配置；对应矩阵#31；天融信代理模板支持证书选择与预置动态证书模板（天融信手册《代理模板》页）</t>
+        </is>
+      </c>
+      <c r="F29" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G29" s="81" t="inlineStr"/>
       <c r="H29" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="I29" s="84" t="n"/>
-    </row>
-    <row r="30" ht="126" customHeight="1" s="1">
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I29" s="80" t="inlineStr"/>
+    </row>
+    <row r="30" ht="51" customHeight="1" s="1">
       <c r="A30" s="84" t="n"/>
       <c r="B30" s="84" t="n"/>
       <c r="C30" s="81" t="inlineStr">
         <is>
-          <t>支持解密不受信证书分离处理（Forward Untrust Certificate）</t>
+          <t>支持解密流量镜像到专用接口（Decryption Port Mirroring）</t>
         </is>
       </c>
       <c r="D30" s="81" t="inlineStr">
         <is>
-          <t>外部无效证书以不受信转发证书重签，保留浏览器告警</t>
+          <t>解密后明文流量镜像至专用接口供第三方分析</t>
         </is>
       </c>
       <c r="E30" s="81" t="inlineStr">
         <is>
-          <t>PA转发代理遇外部过期/不受信证书时，不用内部信任CA重签，而是专用Forward Untrust Certificate重签名，让浏览器保留不受信告警（PA管理指南p994、p1030）；天融信SSL解密（透明代理/服务器SSL解密，天融信手册《代理策略》页）未见受信/不受信双证书体系；迁移评估项：需验证天融信对外部无效证书的处理方式，避免直接阻断（白屏）或信任重签（掩盖风险）</t>
-        </is>
-      </c>
-      <c r="F30" s="80" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
+          <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证（PA管理指南p1059）；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
+        </is>
+      </c>
+      <c r="F30" s="85" t="n"/>
       <c r="G30" s="84" t="n"/>
       <c r="H30" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>不支持</t>
         </is>
       </c>
       <c r="I30" s="84" t="n"/>
     </row>
-    <row r="31" ht="66" customHeight="1" s="1">
+    <row r="31" ht="126" customHeight="1" s="1">
       <c r="A31" s="84" t="n"/>
       <c r="B31" s="84" t="n"/>
       <c r="C31" s="81" t="inlineStr">
         <is>
-          <t>支持解密规则按URL类别选择性解密（URL Category）</t>
+          <t>支持解密不受信证书分离处理（Forward Untrust Certificate）</t>
         </is>
       </c>
       <c r="D31" s="81" t="inlineStr">
         <is>
-          <t>按URL类别圈定解密范围，排除银行/医疗等敏感类</t>
+          <t>外部无效证书以不受信转发证书重签，保留浏览器告警</t>
         </is>
       </c>
       <c r="E31" s="81" t="inlineStr">
         <is>
-          <t>PA解密规则可按URL类别（含自定义类别）选择解密范围，可排除银行/医疗等敏感类别不解密（PA Web帮助p164）；天融信SSL解密（代理策略/代理模板）无按URL类别选择解密机制（检索无命中）</t>
+          <t>PA转发代理遇外部过期/不受信证书时，不用内部信任CA重签，而是专用Forward Untrust Certificate重签名，让浏览器保留不受信告警（PA管理指南p994、p1030）；天融信SSL解密（透明代理/服务器SSL解密，天融信手册《代理策略》页）未见受信/不受信双证书体系；迁移评估项：需验证天融信对外部无效证书的处理方式，避免直接阻断（白屏）或信任重签（掩盖风险）</t>
         </is>
       </c>
       <c r="F31" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G31" s="84" t="n"/>
       <c r="H31" s="80" t="inlineStr">
         <is>
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="I31" s="84" t="n"/>
+    </row>
+    <row r="32" ht="66" customHeight="1" s="1">
+      <c r="A32" s="84" t="n"/>
+      <c r="B32" s="84" t="n"/>
+      <c r="C32" s="81" t="inlineStr">
+        <is>
+          <t>支持解密规则按URL类别选择性解密（URL Category）</t>
+        </is>
+      </c>
+      <c r="D32" s="81" t="inlineStr">
+        <is>
+          <t>按URL类别圈定解密范围，排除银行/医疗等敏感类</t>
+        </is>
+      </c>
+      <c r="E32" s="81" t="inlineStr">
+        <is>
+          <t>PA解密规则可按URL类别（含自定义类别）选择解密范围，可排除银行/医疗等敏感类别不解密（PA Web帮助p164）；天融信SSL解密（代理策略/代理模板）无按URL类别选择解密机制（检索无命中）</t>
+        </is>
+      </c>
+      <c r="F32" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G32" s="84" t="n"/>
+      <c r="H32" s="80" t="inlineStr">
+        <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="I31" s="84" t="n"/>
-    </row>
-    <row r="32" ht="96" customHeight="1" s="1">
-      <c r="A32" s="84" t="n"/>
-      <c r="B32" s="85" t="n"/>
-      <c r="C32" s="81" t="inlineStr">
+      <c r="I32" s="84" t="n"/>
+    </row>
+    <row r="33" ht="96" customHeight="1" s="1">
+      <c r="A33" s="84" t="n"/>
+      <c r="B33" s="85" t="n"/>
+      <c r="C33" s="81" t="inlineStr">
         <is>
           <t>支持SSH代理解密与SSH隧道控制（SSH Proxy）</t>
         </is>
       </c>
-      <c r="D32" s="81" t="inlineStr">
+      <c r="D33" s="81" t="inlineStr">
         <is>
           <t>SSH代理解密+SSH隧道(ssh-tunnel)识别控制</t>
         </is>
       </c>
-      <c r="E32" s="81" t="inlineStr">
+      <c r="E33" s="81" t="inlineStr">
         <is>
           <t>PA解密策略SSH Proxy类型解密SSH通信，可通过ssh-tunnel App-ID在策略中控制SSH隧道（端口转发/内网穿透），正常SSH管理流量放行；含不受支持算法检查/资源不足阻断会话等防护（PA Web帮助p164、p318-319）；天融信手册检索无SSH代理/SSH隧道控制命中</t>
         </is>
       </c>
-      <c r="F32" s="85" t="n"/>
-      <c r="G32" s="85" t="n"/>
-      <c r="H32" s="85" t="n"/>
-      <c r="I32" s="85" t="n"/>
-    </row>
-    <row r="33" ht="111" customHeight="1" s="1">
-      <c r="A33" s="84" t="n"/>
-      <c r="B33" s="80" t="inlineStr">
+      <c r="F33" s="85" t="n"/>
+      <c r="G33" s="85" t="n"/>
+      <c r="H33" s="85" t="n"/>
+      <c r="I33" s="85" t="n"/>
+    </row>
+    <row r="34" ht="111" customHeight="1" s="1">
+      <c r="A34" s="84" t="n"/>
+      <c r="B34" s="80" t="inlineStr">
         <is>
           <t>网络数据包代理(NPBroker)</t>
         </is>
       </c>
-      <c r="C33" s="81" t="inlineStr">
+      <c r="C34" s="81" t="inlineStr">
         <is>
           <t>支持内联数据包代理策略将流量转发第三方安全链（NPBroker）</t>
         </is>
       </c>
-      <c r="D33" s="81" t="inlineStr">
+      <c r="D34" s="81" t="inlineStr">
         <is>
           <t>已解密/未解密流量内联转发第三方安全链，L3路由转发</t>
         </is>
       </c>
-      <c r="E33" s="81" t="inlineStr">
+      <c r="E34" s="81" t="inlineStr">
         <is>
           <t>PA网络数据包代理策略将已解密/未解密TLS/非TLS流量内联转发至第三方安全工具，路径选择选项卡应用数据包代理配置文件定义经路由L3安全链的转发方式（PA Web帮助p167-170）；天融信无网络数据包代理模块，最接近手段为WAF旁路联动（经交换机镜像引流，天融信手册《与WAF联动》页），非内联且无回注路径；对应矩阵#122</t>
         </is>
       </c>
-      <c r="F33" s="80" t="inlineStr">
+      <c r="F34" s="80" t="inlineStr">
         <is>
           <t>高</t>
-        </is>
-      </c>
-      <c r="G33" s="81" t="inlineStr"/>
-      <c r="H33" s="80" t="inlineStr">
-        <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="I33" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="66" customHeight="1" s="1">
-      <c r="A34" s="84" t="n"/>
-      <c r="B34" s="85" t="n"/>
-      <c r="C34" s="81" t="inlineStr">
-        <is>
-          <t>支持NPBroker转发流量类型选择（TLS解密/未解密/非TLS）</t>
-        </is>
-      </c>
-      <c r="D34" s="81" t="inlineStr">
-        <is>
-          <t>TLS解密/未解密/非TLS流量类型选择</t>
-        </is>
-      </c>
-      <c r="E34" s="81" t="inlineStr">
-        <is>
-          <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证（PA Web帮助p167）；天融信无网络数据包代理模块（矩阵#122）</t>
-        </is>
-      </c>
-      <c r="F34" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
         </is>
       </c>
       <c r="G34" s="81" t="inlineStr"/>
@@ -4353,28 +4349,28 @@
           <t>不支持</t>
         </is>
       </c>
-      <c r="I34" s="80" t="inlineStr"/>
+      <c r="I34" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="66" customHeight="1" s="1">
       <c r="A35" s="84" t="n"/>
-      <c r="B35" s="80" t="inlineStr">
-        <is>
-          <t>隧道检测(Tunnel Inspection)</t>
-        </is>
-      </c>
+      <c r="B35" s="85" t="n"/>
       <c r="C35" s="81" t="inlineStr">
         <is>
-          <t>支持GRE隧道终结与内层流量检测</t>
+          <t>支持NPBroker转发流量类型选择（TLS解密/未解密/非TLS）</t>
         </is>
       </c>
       <c r="D35" s="81" t="inlineStr">
         <is>
-          <t>GRE隧道封装/解封装，内层流量按普通流量检测</t>
+          <t>TLS解密/未解密/非TLS流量类型选择</t>
         </is>
       </c>
       <c r="E35" s="81" t="inlineStr">
         <is>
-          <t>PA隧道检测策略解封装并检测GRE隧道内容（PA Web帮助p172-173）；天融信GRE隧道支持封装与解封装，解封装后内层报文按普通流量处理检测（天融信手册《GRE隧道》页）；对应矩阵#128/37</t>
+          <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证（PA Web帮助p167）；天融信无网络数据包代理模块（矩阵#122）</t>
         </is>
       </c>
       <c r="F35" s="80" t="inlineStr">
@@ -4385,133 +4381,133 @@
       <c r="G35" s="81" t="inlineStr"/>
       <c r="H35" s="80" t="inlineStr">
         <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I35" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="96" customHeight="1" s="1">
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I35" s="80" t="inlineStr"/>
+    </row>
+    <row r="36" ht="66" customHeight="1" s="1">
       <c r="A36" s="84" t="n"/>
-      <c r="B36" s="84" t="n"/>
+      <c r="B36" s="80" t="inlineStr">
+        <is>
+          <t>隧道检测(Tunnel Inspection)</t>
+        </is>
+      </c>
       <c r="C36" s="81" t="inlineStr">
         <is>
-          <t>支持GTP-U/VXLAN/非加密IPSec隧道内层检测</t>
+          <t>支持GRE隧道终结与内层流量检测</t>
         </is>
       </c>
       <c r="D36" s="81" t="inlineStr">
         <is>
-          <t>GTP-U/VXLAN/NULL加密IPSec(AH)隧道内层流量检测</t>
+          <t>GRE隧道封装/解封装，内层流量按普通流量检测</t>
         </is>
       </c>
       <c r="E36" s="81" t="inlineStr">
         <is>
-          <t>PA隧道检测支持GTP-U/VXLAN/非加密IPSec（NULL加密/AH传输模式）内层检测（PA Web帮助p172-173）；天融信VXLAN仅隧道封装转发与三层网关（天融信手册《业务接入端》《三层VXLAN网关》页），无内层安全检测，GTP检测检索无命中；对应矩阵#128/37</t>
+          <t>PA隧道检测策略解封装并检测GRE隧道内容（PA Web帮助p172-173）；天融信GRE隧道支持封装与解封装，解封装后内层报文按普通流量处理检测（天融信手册《GRE隧道》页）；对应矩阵#128/37</t>
         </is>
       </c>
       <c r="F36" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G36" s="81" t="inlineStr"/>
       <c r="H36" s="80" t="inlineStr">
         <is>
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I36" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="96" customHeight="1" s="1">
+      <c r="A37" s="84" t="n"/>
+      <c r="B37" s="84" t="n"/>
+      <c r="C37" s="81" t="inlineStr">
+        <is>
+          <t>支持GTP-U/VXLAN/非加密IPSec隧道内层检测</t>
+        </is>
+      </c>
+      <c r="D37" s="81" t="inlineStr">
+        <is>
+          <t>GTP-U/VXLAN/NULL加密IPSec(AH)隧道内层流量检测</t>
+        </is>
+      </c>
+      <c r="E37" s="81" t="inlineStr">
+        <is>
+          <t>PA隧道检测支持GTP-U/VXLAN/非加密IPSec（NULL加密/AH传输模式）内层检测（PA Web帮助p172-173）；天融信VXLAN仅隧道封装转发与三层网关（天融信手册《业务接入端》《三层VXLAN网关》页），无内层安全检测，GTP检测检索无命中；对应矩阵#128/37</t>
+        </is>
+      </c>
+      <c r="F37" s="80" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="G37" s="81" t="inlineStr"/>
+      <c r="H37" s="80" t="inlineStr">
+        <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="I36" s="80" t="inlineStr"/>
-    </row>
-    <row r="37" ht="51" customHeight="1" s="1">
-      <c r="A37" s="84" t="n"/>
-      <c r="B37" s="85" t="n"/>
-      <c r="C37" s="81" t="inlineStr">
+      <c r="I37" s="80" t="inlineStr"/>
+    </row>
+    <row r="38" ht="51" customHeight="1" s="1">
+      <c r="A38" s="84" t="n"/>
+      <c r="B38" s="85" t="n"/>
+      <c r="C38" s="81" t="inlineStr">
         <is>
           <t>支持最大封装级数防护（max_encap）</t>
         </is>
       </c>
-      <c r="D37" s="81" t="inlineStr">
+      <c r="D38" s="81" t="inlineStr">
         <is>
           <t>隧道嵌套封装最大级数限制，超限丢弃</t>
         </is>
       </c>
-      <c r="E37" s="81" t="inlineStr">
+      <c r="E38" s="81" t="inlineStr">
         <is>
           <t>PA对隧道最大封装级数超限丢包防护，防隧道嵌套绕过（PA管理指南p655）；天融信手册无封装级数防护（检索无命中）</t>
         </is>
       </c>
-      <c r="F37" s="80" t="inlineStr">
+      <c r="F38" s="80" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="G37" s="85" t="n"/>
-      <c r="H37" s="85" t="n"/>
-      <c r="I37" s="85" t="n"/>
-    </row>
-    <row r="38" ht="81" customHeight="1" s="1">
-      <c r="A38" s="84" t="n"/>
-      <c r="B38" s="80" t="inlineStr">
+      <c r="G38" s="85" t="n"/>
+      <c r="H38" s="85" t="n"/>
+      <c r="I38" s="85" t="n"/>
+    </row>
+    <row r="39" ht="81" customHeight="1" s="1">
+      <c r="A39" s="84" t="n"/>
+      <c r="B39" s="80" t="inlineStr">
         <is>
           <t>应用覆盖(App Override)</t>
         </is>
       </c>
-      <c r="C38" s="81" t="inlineStr">
+      <c r="C39" s="81" t="inlineStr">
         <is>
           <t>支持通过Application Override重定义应用识别</t>
         </is>
       </c>
-      <c r="D38" s="81" t="inlineStr">
+      <c r="D39" s="81" t="inlineStr">
         <is>
           <t>按协议/端口自定义应用识别结果</t>
         </is>
       </c>
-      <c r="E38" s="81" t="inlineStr">
+      <c r="E39" s="81" t="inlineStr">
         <is>
           <t>PA应用替代策略改变防火墙对网络通信的应用分类方式（如指定明文协议/端口识别，PA Web帮助p178）；天融信自定义应用允许管理员按需自定义应用协议（含端口匹配）并加入应用规则库（天融信手册《自定义应用》页）；对应矩阵#26</t>
         </is>
       </c>
-      <c r="F38" s="80" t="inlineStr">
+      <c r="F39" s="80" t="inlineStr">
         <is>
           <t>中</t>
-        </is>
-      </c>
-      <c r="G38" s="81" t="inlineStr"/>
-      <c r="H38" s="80" t="inlineStr">
-        <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I38" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="66" customHeight="1" s="1">
-      <c r="A39" s="84" t="n"/>
-      <c r="B39" s="84" t="n"/>
-      <c r="C39" s="81" t="inlineStr">
-        <is>
-          <t>支持覆盖类型（端口映射类）识别</t>
-        </is>
-      </c>
-      <c r="D39" s="81" t="inlineStr">
-        <is>
-          <t>端口映射类覆盖识别</t>
-        </is>
-      </c>
-      <c r="E39" s="81" t="inlineStr">
-        <is>
-          <t>PA支持端口式应用覆盖识别（configurable自定义应用）；天融信自定义应用允许管理员按特定需要自行定义应用协议（含端口匹配），自动添加到应用规则库供安全策略引用（天融信手册《自定义应用》页）</t>
-        </is>
-      </c>
-      <c r="F39" s="80" t="inlineStr">
-        <is>
-          <t>低</t>
         </is>
       </c>
       <c r="G39" s="81" t="inlineStr"/>
@@ -4520,223 +4516,223 @@
           <t>已支持</t>
         </is>
       </c>
-      <c r="I39" s="80" t="inlineStr"/>
-    </row>
-    <row r="40" ht="96" customHeight="1" s="1">
+      <c r="I39" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="66" customHeight="1" s="1">
       <c r="A40" s="84" t="n"/>
-      <c r="B40" s="85" t="n"/>
+      <c r="B40" s="84" t="n"/>
       <c r="C40" s="81" t="inlineStr">
         <is>
+          <t>支持覆盖类型（端口映射类）识别</t>
+        </is>
+      </c>
+      <c r="D40" s="81" t="inlineStr">
+        <is>
+          <t>端口映射类覆盖识别</t>
+        </is>
+      </c>
+      <c r="E40" s="81" t="inlineStr">
+        <is>
+          <t>PA支持端口式应用覆盖识别（configurable自定义应用）；天融信自定义应用允许管理员按特定需要自行定义应用协议（含端口匹配），自动添加到应用规则库供安全策略引用（天融信手册《自定义应用》页）</t>
+        </is>
+      </c>
+      <c r="F40" s="80" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="G40" s="81" t="inlineStr"/>
+      <c r="H40" s="80" t="inlineStr">
+        <is>
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I40" s="80" t="inlineStr"/>
+    </row>
+    <row r="41" ht="96" customHeight="1" s="1">
+      <c r="A41" s="84" t="n"/>
+      <c r="B41" s="85" t="n"/>
+      <c r="C41" s="81" t="inlineStr">
+        <is>
           <t>支持应用替代流量跳过七层检测等效配置</t>
         </is>
       </c>
-      <c r="D40" s="81" t="inlineStr">
+      <c r="D41" s="81" t="inlineStr">
         <is>
           <t>匹配覆盖策略的流量跳过七层检测，四层快速转发</t>
         </is>
       </c>
-      <c r="E40" s="81" t="inlineStr">
+      <c r="E41" s="81" t="inlineStr">
         <is>
           <t>PA应用替代策略明确绕过第7层处理与威胁检查，改用第4层状态检查以加速（PA管理指南p1307）；天融信自定义应用加入规则库后仍默认经安全引擎检测（天融信手册《自定义应用》页）；迁移评估项：PA应用替代多为私有大流量业务加速，转换时需同步关闭对应策略的IPS/七层检测，否则性能被拖垮或误阻断</t>
         </is>
       </c>
-      <c r="F40" s="80" t="inlineStr">
+      <c r="F41" s="80" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="G40" s="85" t="n"/>
-      <c r="H40" s="80" t="inlineStr">
+      <c r="G41" s="85" t="n"/>
+      <c r="H41" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="I40" s="85" t="n"/>
-    </row>
-    <row r="41" ht="111" customHeight="1" s="1">
-      <c r="A41" s="84" t="n"/>
-      <c r="B41" s="80" t="inlineStr">
+      <c r="I41" s="85" t="n"/>
+    </row>
+    <row r="42" ht="111" customHeight="1" s="1">
+      <c r="A42" s="84" t="n"/>
+      <c r="B42" s="80" t="inlineStr">
         <is>
           <t>身份验证(Authentication)</t>
         </is>
       </c>
-      <c r="C41" s="81" t="inlineStr">
+      <c r="C42" s="81" t="inlineStr">
         <is>
           <t>支持基于用户身份的身份验证策略（User-ID）</t>
         </is>
       </c>
-      <c r="D41" s="81" t="inlineStr">
+      <c r="D42" s="81" t="inlineStr">
         <is>
           <t>基于用户/用户组策略，多源IP-用户映射（AD/Syslog/XML API）</t>
         </is>
       </c>
-      <c r="E41" s="81" t="inlineStr">
+      <c r="E42" s="81" t="inlineStr">
         <is>
           <t>PA身份验证策略在访问网络资源前对用户鉴权（PA Web帮助p182），配合User-ID多源映射（AD/XML/Syslog等）；天融信用户访问网络资源前经认证，认证通过后检查关联的用户访问策略，支持门户认证（本地/外部）与LDAP/RADIUS对接（天融信手册《管理用户》《添加Radius服务器》页）；对应矩阵#3/35</t>
         </is>
       </c>
-      <c r="F41" s="80" t="inlineStr">
+      <c r="F42" s="80" t="inlineStr">
         <is>
           <t>高</t>
-        </is>
-      </c>
-      <c r="G41" s="81" t="inlineStr"/>
-      <c r="H41" s="80" t="inlineStr">
-        <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I41" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="81" customHeight="1" s="1">
-      <c r="A42" s="84" t="n"/>
-      <c r="B42" s="84" t="n"/>
-      <c r="C42" s="81" t="inlineStr">
-        <is>
-          <t>支持认证策略超时与单次认证（SSO）</t>
-        </is>
-      </c>
-      <c r="D42" s="81" t="inlineStr">
-        <is>
-          <t>认证超时+单次认证(SSO)</t>
-        </is>
-      </c>
-      <c r="E42" s="81" t="inlineStr">
-        <is>
-          <t>PA支持认证超时减少重复质询、Kerberos/SAML/RADIUS等对接（PA Web帮助p186）；天融信手册检索认证超时/单点登录/SSO无命中（仅在线用户在线时长查看与强制下线）；迁移评估项：需核实天融信认证会话有效期配置与SSO对接能力</t>
-        </is>
-      </c>
-      <c r="F42" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
         </is>
       </c>
       <c r="G42" s="81" t="inlineStr"/>
       <c r="H42" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
-        </is>
-      </c>
-      <c r="I42" s="80" t="inlineStr"/>
-    </row>
-    <row r="43" ht="126" customHeight="1" s="1">
+          <t>已支持</t>
+        </is>
+      </c>
+      <c r="I42" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="81" customHeight="1" s="1">
       <c r="A43" s="84" t="n"/>
       <c r="B43" s="84" t="n"/>
       <c r="C43" s="81" t="inlineStr">
         <is>
+          <t>支持认证策略超时与单次认证（SSO）</t>
+        </is>
+      </c>
+      <c r="D43" s="81" t="inlineStr">
+        <is>
+          <t>认证超时+单次认证(SSO)</t>
+        </is>
+      </c>
+      <c r="E43" s="81" t="inlineStr">
+        <is>
+          <t>PA支持认证超时减少重复质询、Kerberos/SAML/RADIUS等对接（PA Web帮助p186）；天融信手册检索认证超时/单点登录/SSO无命中（仅在线用户在线时长查看与强制下线）；迁移评估项：需核实天融信认证会话有效期配置与SSO对接能力</t>
+        </is>
+      </c>
+      <c r="F43" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G43" s="81" t="inlineStr"/>
+      <c r="H43" s="80" t="inlineStr">
+        <is>
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="I43" s="80" t="inlineStr"/>
+    </row>
+    <row r="44" ht="126" customHeight="1" s="1">
+      <c r="A44" s="84" t="n"/>
+      <c r="B44" s="84" t="n"/>
+      <c r="C44" s="81" t="inlineStr">
+        <is>
           <t>支持流量策略触发多因素认证质询（MFA Enforcement）</t>
         </is>
       </c>
-      <c r="D43" s="81" t="inlineStr">
+      <c r="D44" s="81" t="inlineStr">
         <is>
           <t>流量策略匹配触发MFA质询（非登录场景，MFA供应商API/RADIUS）</t>
         </is>
       </c>
-      <c r="E43" s="81" t="inlineStr">
+      <c r="E44" s="81" t="inlineStr">
         <is>
           <t>PA身份验证策略通过Authentication Enforcement对象对匹配流量强制质询，支持多因素身份验证（每因素独立超时，防火墙记录时间戳），MFA供应商API/RADIUS对接（PA Web帮助p185-186、p310、p735-742）；天融信双因子认证（密码+短信/证书/Ukey）仅限管理员/用户登录场景（天融信手册《登录安全策略》页），无流量策略触发MFA质询</t>
         </is>
       </c>
-      <c r="F43" s="84" t="n"/>
-      <c r="G43" s="84" t="n"/>
-      <c r="H43" s="80" t="inlineStr">
+      <c r="F44" s="84" t="n"/>
+      <c r="G44" s="84" t="n"/>
+      <c r="H44" s="80" t="inlineStr">
         <is>
           <t>不支持</t>
         </is>
       </c>
-      <c r="I43" s="84" t="n"/>
-    </row>
-    <row r="44" ht="96" customHeight="1" s="1">
-      <c r="A44" s="84" t="n"/>
-      <c r="B44" s="85" t="n"/>
-      <c r="C44" s="81" t="inlineStr">
+      <c r="I44" s="84" t="n"/>
+    </row>
+    <row r="45" ht="96" customHeight="1" s="1">
+      <c r="A45" s="84" t="n"/>
+      <c r="B45" s="85" t="n"/>
+      <c r="C45" s="81" t="inlineStr">
         <is>
           <t>支持User-ID动态映射时效性等效（AD日志毫秒级更新）</t>
         </is>
       </c>
-      <c r="D44" s="81" t="inlineStr">
+      <c r="D45" s="81" t="inlineStr">
         <is>
           <t>AD域事件日志毫秒级IP-用户映射更新</t>
         </is>
       </c>
-      <c r="E44" s="81" t="inlineStr">
+      <c r="E45" s="81" t="inlineStr">
         <is>
           <t>PA无代理架构通过读取域控事件日志实现IP-用户毫秒级动态映射，大规模部署有专项规划（PA管理指南p866-867）；天融信AD对接的轮询间隔与并发认证能力手册未量化；迁移评估项：数万AD用户且移动频繁场景需实测天融信映射更新时延，避免基于用户的策略出现间歇性未授权拦截</t>
         </is>
       </c>
-      <c r="F44" s="85" t="n"/>
-      <c r="G44" s="85" t="n"/>
-      <c r="H44" s="80" t="inlineStr">
+      <c r="F45" s="85" t="n"/>
+      <c r="G45" s="85" t="n"/>
+      <c r="H45" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="I44" s="85" t="n"/>
-    </row>
-    <row r="45" ht="111" customHeight="1" s="1">
-      <c r="A45" s="84" t="n"/>
-      <c r="B45" s="80" t="inlineStr">
+      <c r="I45" s="85" t="n"/>
+    </row>
+    <row r="46" ht="111" customHeight="1" s="1">
+      <c r="A46" s="84" t="n"/>
+      <c r="B46" s="80" t="inlineStr">
         <is>
           <t>DoS防护(DoS Protection)</t>
         </is>
       </c>
-      <c r="C45" s="81" t="inlineStr">
+      <c r="C46" s="81" t="inlineStr">
         <is>
           <t>支持针对关键资源的分类/聚合DoS防护</t>
         </is>
       </c>
-      <c r="D45" s="81" t="inlineStr">
+      <c r="D46" s="81" t="inlineStr">
         <is>
           <t>分类(源/目的IP粒度)+聚合(全局)双层阈值限流</t>
         </is>
       </c>
-      <c r="E45" s="81" t="inlineStr">
+      <c r="E46" s="81" t="inlineStr">
         <is>
           <t>PA DoS策略基于源/目的接口、区域、地址、服务定义允许/拒绝/告警，规则可选聚合与分类双层DoS保护配置文件设定阈值速率（PA Web帮助p189-191、PA管理指南p1354）；天融信DDoS防护模块按防护对象（目的服务器）设阈值（pps/bps），可达目的IP粒度（天融信手册《配置策略模板》《日志查看》页）；对应矩阵#52/42</t>
         </is>
       </c>
-      <c r="F45" s="80" t="inlineStr">
+      <c r="F46" s="80" t="inlineStr">
         <is>
           <t>高</t>
-        </is>
-      </c>
-      <c r="G45" s="81" t="inlineStr"/>
-      <c r="H45" s="80" t="inlineStr">
-        <is>
-          <t>已支持</t>
-        </is>
-      </c>
-      <c r="I45" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="51" customHeight="1" s="1">
-      <c r="A46" s="84" t="n"/>
-      <c r="B46" s="85" t="n"/>
-      <c r="C46" s="81" t="inlineStr">
-        <is>
-          <t>支持DoS聚合配置文件（连接/秒阈值）</t>
-        </is>
-      </c>
-      <c r="D46" s="81" t="inlineStr">
-        <is>
-          <t>连接数/秒阈值告警+最大速率限制</t>
-        </is>
-      </c>
-      <c r="E46" s="81" t="inlineStr">
-        <is>
-          <t>PA聚合DoS配置文件按传入连接数/秒触发告警与最大速率限制；天融信DDoS防护模块按阈值（pps/bps）监视并触发防护（天融信手册《配置策略模板》页）</t>
-        </is>
-      </c>
-      <c r="F46" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
         </is>
       </c>
       <c r="G46" s="81" t="inlineStr"/>
@@ -4745,28 +4741,28 @@
           <t>已支持</t>
         </is>
       </c>
-      <c r="I46" s="80" t="inlineStr"/>
-    </row>
-    <row r="47" ht="171" customHeight="1" s="1">
+      <c r="I46" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="51" customHeight="1" s="1">
       <c r="A47" s="84" t="n"/>
-      <c r="B47" s="80" t="inlineStr">
-        <is>
-          <t>动态对象(Dynamic Objects)</t>
-        </is>
-      </c>
+      <c r="B47" s="85" t="n"/>
       <c r="C47" s="81" t="inlineStr">
         <is>
-          <t>支持外部动态列表作为策略地址对象（EDL）</t>
+          <t>支持DoS聚合配置文件（连接/秒阈值）</t>
         </is>
       </c>
       <c r="D47" s="81" t="inlineStr">
         <is>
-          <t>HTTP/HTTPS外部文本列表(IP/域名/URL)自动拉取，策略直接引用</t>
+          <t>连接数/秒阈值告警+最大速率限制</t>
         </is>
       </c>
       <c r="E47" s="81" t="inlineStr">
         <is>
-          <t>PA外部动态列表：基于HTTP/HTTPS托管的文本文件创建IP/URL/域名/IMEI/IMSI地址对象，防火墙定时自动拉取更新，策略中直接引用（Objects&gt;External Dynamic Lists，PA Web帮助p236-239；策略源/目标可直接选EDL，p196-197）；天融信手册检索外部动态列表/EDL无命中，仅内置威胁情报库与云端威胁情报库（规则集管理，天融信手册《威胁情报》《配置规则集》页），无策略直接引用任意外部文本列表机制；迁移评估项：PA策略中引用的EDL需转换为天融信静态地址组定期导入或威胁情报联动</t>
+          <t>PA聚合DoS配置文件按传入连接数/秒触发告警与最大速率限制；天融信DDoS防护模块按阈值（pps/bps）监视并触发防护（天融信手册《配置策略模板》页）</t>
         </is>
       </c>
       <c r="F47" s="80" t="inlineStr">
@@ -4777,27 +4773,31 @@
       <c r="G47" s="81" t="inlineStr"/>
       <c r="H47" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
+          <t>已支持</t>
         </is>
       </c>
       <c r="I47" s="80" t="inlineStr"/>
     </row>
-    <row r="48" ht="126" customHeight="1" s="1">
+    <row r="48" ht="171" customHeight="1" s="1">
       <c r="A48" s="84" t="n"/>
-      <c r="B48" s="85" t="n"/>
+      <c r="B48" s="80" t="inlineStr">
+        <is>
+          <t>动态对象(Dynamic Objects)</t>
+        </is>
+      </c>
       <c r="C48" s="81" t="inlineStr">
         <is>
-          <t>支持基于标记的动态地址组（DAG）</t>
+          <t>支持外部动态列表作为策略地址对象（EDL）</t>
         </is>
       </c>
       <c r="D48" s="81" t="inlineStr">
         <is>
-          <t>Tag标记过滤器动态地址组，成员随IP变化自动更新</t>
+          <t>HTTP/HTTPS外部文本列表(IP/域名/URL)自动拉取，策略直接引用</t>
         </is>
       </c>
       <c r="E48" s="81" t="inlineStr">
         <is>
-          <t>PA动态地址组：查找标记(Tag)+基于标记的过滤器（AND/OR匹配）动态填充成员，VM信息源注册或XML/REST API定义标记，IP变化时策略自动生效（PA Web帮助p207-208、p228）；天融信手册检索动态地址组/标签/SDN/云平台联动无命中，地址组为静态IP/子网绑定（天融信手册《地址》页）；迁移评估项：PA云环境Tag微隔离策略需转换为静态地址组，IP漂移场景需人工或API维护</t>
+          <t>PA外部动态列表：基于HTTP/HTTPS托管的文本文件创建IP/URL/域名/IMEI/IMSI地址对象，防火墙定时自动拉取更新，策略中直接引用（Objects&gt;External Dynamic Lists，PA Web帮助p236-239；策略源/目标可直接选EDL，p196-197）；天融信手册检索外部动态列表/EDL无命中，仅内置威胁情报库与云端威胁情报库（规则集管理，天融信手册《威胁情报》《配置规则集》页），无策略直接引用任意外部文本列表机制；迁移评估项：PA策略中引用的EDL需转换为天融信静态地址组定期导入或威胁情报联动</t>
         </is>
       </c>
       <c r="F48" s="80" t="inlineStr">
@@ -4813,66 +4813,62 @@
       </c>
       <c r="I48" s="80" t="inlineStr"/>
     </row>
-    <row r="49" ht="81" customHeight="1" s="1">
+    <row r="49" ht="126" customHeight="1" s="1">
       <c r="A49" s="84" t="n"/>
-      <c r="B49" s="80" t="inlineStr">
-        <is>
-          <t>SD-WAN策略</t>
-        </is>
-      </c>
+      <c r="B49" s="85" t="n"/>
       <c r="C49" s="81" t="inlineStr">
         <is>
-          <t>支持按应用配置链路路径管理与链路质量探测</t>
+          <t>支持基于标记的动态地址组（DAG）</t>
         </is>
       </c>
       <c r="D49" s="81" t="inlineStr">
         <is>
-          <t>按应用分配链路与流量分发（天融信以策略路由+LLB近似实现）</t>
+          <t>Tag标记过滤器动态地址组，成员随IP变化自动更新</t>
         </is>
       </c>
       <c r="E49" s="81" t="inlineStr">
         <is>
-          <t>PA SD-WAN策略按应用/抖动/延迟/丢包指标分配链路，流量分发（PA Web帮助p197）；天融信为策略路由+链路负载均衡近似实现（天融信手册《策略路由》《链路负载均衡》页），无SD-WAN策略模型；对应矩阵#129/120</t>
+          <t>PA动态地址组：查找标记(Tag)+基于标记的过滤器（AND/OR匹配）动态填充成员，VM信息源注册或XML/REST API定义标记，IP变化时策略自动生效（PA Web帮助p207-208、p228）；天融信手册检索动态地址组/标签/SDN/云平台联动无命中，地址组为静态IP/子网绑定（天融信手册《地址》页）；迁移评估项：PA云环境Tag微隔离策略需转换为静态地址组，IP漂移场景需人工或API维护</t>
         </is>
       </c>
       <c r="F49" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G49" s="81" t="inlineStr"/>
       <c r="H49" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="I49" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I49" s="80" t="inlineStr"/>
     </row>
     <row r="50" ht="81" customHeight="1" s="1">
-      <c r="A50" s="85" t="n"/>
-      <c r="B50" s="85" t="n"/>
+      <c r="A50" s="84" t="n"/>
+      <c r="B50" s="80" t="inlineStr">
+        <is>
+          <t>SD-WAN策略</t>
+        </is>
+      </c>
       <c r="C50" s="81" t="inlineStr">
         <is>
-          <t>支持SD-WAN路径选择与链路质量监测（jitter/latency/loss）</t>
+          <t>支持按应用配置链路路径管理与链路质量探测</t>
         </is>
       </c>
       <c r="D50" s="81" t="inlineStr">
         <is>
-          <t>抖动/延迟/丢包多维指标选路（天融信现仅延迟探测）</t>
+          <t>按应用分配链路与流量分发（天融信以策略路由+LLB近似实现）</t>
         </is>
       </c>
       <c r="E50" s="81" t="inlineStr">
         <is>
-          <t>PA路径质量配置文件基于抖动/延迟/丢包等运行状况指标选路（PA Web帮助p195）；天融信有链路探测(ping)+智能选路(最小延迟优先)（天融信手册《策略路由》页），无jitter/latency/loss多维指标</t>
+          <t>PA SD-WAN策略按应用/抖动/延迟/丢包指标分配链路，流量分发（PA Web帮助p197）；天融信为策略路由+链路负载均衡近似实现（天融信手册《策略路由》《链路负载均衡》页），无SD-WAN策略模型；对应矩阵#129/120</t>
         </is>
       </c>
       <c r="F50" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G50" s="81" t="inlineStr"/>
@@ -4881,49 +4877,85 @@
           <t>部分支持</t>
         </is>
       </c>
-      <c r="I50" s="80" t="inlineStr"/>
+      <c r="I50" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="81" customHeight="1" s="1">
+      <c r="A51" s="85" t="n"/>
+      <c r="B51" s="85" t="n"/>
+      <c r="C51" s="81" t="inlineStr">
+        <is>
+          <t>支持SD-WAN路径选择与链路质量监测（jitter/latency/loss）</t>
+        </is>
+      </c>
+      <c r="D51" s="81" t="inlineStr">
+        <is>
+          <t>抖动/延迟/丢包多维指标选路（天融信现仅延迟探测）</t>
+        </is>
+      </c>
+      <c r="E51" s="81" t="inlineStr">
+        <is>
+          <t>PA路径质量配置文件基于抖动/延迟/丢包等运行状况指标选路（PA Web帮助p195）；天融信有链路探测(ping)+智能选路(最小延迟优先)（天融信手册《策略路由》页），无jitter/latency/loss多维指标</t>
+        </is>
+      </c>
+      <c r="F51" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G51" s="81" t="inlineStr"/>
+      <c r="H51" s="80" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="I51" s="80" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="39">
-    <mergeCell ref="F17:F19"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="A2:A50"/>
+  <mergeCells count="40">
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="G9:G16"/>
+    <mergeCell ref="B8:B16"/>
+    <mergeCell ref="F43:F45"/>
     <mergeCell ref="H6:H7"/>
-    <mergeCell ref="I36:I37"/>
-    <mergeCell ref="G39:G40"/>
-    <mergeCell ref="H31:H32"/>
-    <mergeCell ref="B27:B32"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="G17:G22"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="H17:H20"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="F32:F33"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="G29:G33"/>
+    <mergeCell ref="I29:I33"/>
+    <mergeCell ref="G43:G45"/>
     <mergeCell ref="B2:B7"/>
-    <mergeCell ref="H36:H37"/>
-    <mergeCell ref="B8:B15"/>
-    <mergeCell ref="B16:B22"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="G9:G15"/>
-    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="G37:G38"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="I37:I38"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="G18:G23"/>
+    <mergeCell ref="I18:I23"/>
     <mergeCell ref="I9:I15"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="F28:F29"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="G42:G44"/>
+    <mergeCell ref="H32:H33"/>
     <mergeCell ref="H12:H15"/>
+    <mergeCell ref="B28:B33"/>
+    <mergeCell ref="H37:H38"/>
     <mergeCell ref="F3:F7"/>
     <mergeCell ref="F11:F12"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="I17:I22"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="A2:A51"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="B17:B23"/>
     <mergeCell ref="G3:G7"/>
+    <mergeCell ref="I43:I45"/>
     <mergeCell ref="I3:I7"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="F42:F44"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="G28:G32"/>
-    <mergeCell ref="B41:B44"/>
-    <mergeCell ref="I28:I32"/>
-    <mergeCell ref="G36:G37"/>
-    <mergeCell ref="I42:I44"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="G40:G41"/>
+    <mergeCell ref="I40:I41"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4935,7 +4967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15.2"/>
   <cols>
     <col width="11.7" customWidth="1" style="1" min="1" max="1"/>
@@ -5294,92 +5326,88 @@
       <c r="H11" s="82" t="n"/>
       <c r="I11" s="82" t="n"/>
     </row>
-    <row r="12" ht="126" customHeight="1" s="1">
+    <row r="12" ht="171" customHeight="1" s="1">
       <c r="A12" s="82" t="n"/>
-      <c r="B12" s="80" t="inlineStr">
+      <c r="B12" s="82" t="n"/>
+      <c r="C12" s="81" t="inlineStr">
+        <is>
+          <t>支持WildFire云沙箱文件检测联动（Advanced WildFire）</t>
+        </is>
+      </c>
+      <c r="D12" s="81" t="inlineStr">
+        <is>
+          <t>未知文件云沙箱实时分析+签名秒级下发，策略Actions绑定WildFire配置文件</t>
+        </is>
+      </c>
+      <c r="E12" s="81" t="inlineStr">
+        <is>
+          <t>PA策略Actions可绑定WildFire Analysis配置文件（安全配置文件组含反病毒/漏洞/URL/文件阻断/WildFire，PA Web帮助p304；WildFire提交日志转发p305-306），云沙箱动态分析未知/零日威胁并秒级下发签名；天融信有内置APT沙箱（虚拟运行环境检测未知漏洞威胁）与沙箱联动（天融信手册《高级威胁防护》《APT联动配置》页），无云端动态分析与秒级签名下发证据；工作表1已登记云沙箱联动需求（不支持：公司无此产品），勿重复跟踪；迁移评估项：评估天融信本地APT沙箱与PA云沙箱检测能力等效性</t>
+        </is>
+      </c>
+      <c r="F12" s="82" t="n"/>
+      <c r="G12" s="82" t="n"/>
+      <c r="H12" s="80" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="I12" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="126" customHeight="1" s="1">
+      <c r="A13" s="82" t="n"/>
+      <c r="B13" s="80" t="inlineStr">
         <is>
           <t>NAT策略</t>
         </is>
       </c>
-      <c r="C12" s="81" t="inlineStr">
+      <c r="C13" s="81" t="inlineStr">
         <is>
           <t>支持NAT后目的区域路由回查匹配（Dest Zone by route lookup）</t>
         </is>
       </c>
-      <c r="D12" s="81" t="inlineStr">
+      <c r="D13" s="81" t="inlineStr">
         <is>
           <t>目的区域按NAT后路由查找；源/目的地址用NAT前值</t>
         </is>
       </c>
-      <c r="E12" s="81" t="inlineStr">
+      <c r="E13" s="81" t="inlineStr">
         <is>
           <t>PA底层为『先NAT判断后安全策略匹配』的因果倒置：安全策略要求源区域(NAT前)+源地址(NAT前)+目的地址(NAT前)+目的区域(NAT后按路由查找)，极其反直觉；天融信地址转换为独立策略库常规直观映射（安全策略&gt;地址转换，天融信手册《服务器映射》页）；迁移评估项：带目的NAT的策略平移后易因Zone填写错误不通，需制定NAT查表逻辑转换映射规范；对应矩阵#9</t>
         </is>
       </c>
-      <c r="F12" s="80" t="inlineStr">
+      <c r="F13" s="80" t="inlineStr">
         <is>
           <t>高</t>
-        </is>
-      </c>
-      <c r="G12" s="81" t="inlineStr"/>
-      <c r="H12" s="80" t="inlineStr">
-        <is>
-          <t>待评估</t>
-        </is>
-      </c>
-      <c r="I12" s="80" t="inlineStr"/>
-    </row>
-    <row r="13" ht="81" customHeight="1" s="1">
-      <c r="A13" s="82" t="n"/>
-      <c r="B13" s="82" t="n"/>
-      <c r="C13" s="81" t="inlineStr">
-        <is>
-          <t>支持NAT规则主动/主动HA绑定（Active/Active HA Binding）</t>
-        </is>
-      </c>
-      <c r="D13" s="81" t="inlineStr">
-        <is>
-          <t>主动/主动HA下NAT规则绑定会话所有者</t>
-        </is>
-      </c>
-      <c r="E13" s="81" t="inlineStr">
-        <is>
-          <t>PA主动/主动HA配置下NAT规则可绑定会话所有者/会话设置，控制NAT会话的设备绑定，仅A/A模式可见（PA Web帮助p150）；天融信HA为主备双机热备模式（天融信手册《配置双机热备功能》页），无主动/主动模式及NAT规则绑定机制</t>
-        </is>
-      </c>
-      <c r="F13" s="80" t="inlineStr">
-        <is>
-          <t>低</t>
         </is>
       </c>
       <c r="G13" s="81" t="inlineStr"/>
       <c r="H13" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
+          <t>待评估</t>
         </is>
       </c>
       <c r="I13" s="80" t="inlineStr"/>
     </row>
-    <row r="14" ht="96" customHeight="1" s="1">
+    <row r="14" ht="81" customHeight="1" s="1">
       <c r="A14" s="82" t="n"/>
-      <c r="B14" s="80" t="inlineStr">
-        <is>
-          <t>QoS策略</t>
-        </is>
-      </c>
+      <c r="B14" s="82" t="n"/>
       <c r="C14" s="81" t="inlineStr">
         <is>
-          <t>支持QoS策略规则内直接按DSCP/ToS匹配调度</t>
+          <t>支持NAT规则主动/主动HA绑定（Active/Active HA Binding）</t>
         </is>
       </c>
       <c r="D14" s="81" t="inlineStr">
         <is>
-          <t>QoS策略规则DSCP/ToS直接匹配（非独立流控模块配置）</t>
+          <t>主动/主动HA下NAT规则绑定会话所有者</t>
         </is>
       </c>
       <c r="E14" s="81" t="inlineStr">
         <is>
-          <t>PA QoS规则可直接按DSCP值或IP优先级/ToS匹配调度（PA Web帮助p155）；天融信支持DSCP/802.1p(CoS)识别与重标记，但需在独立流量管理模块配置（虚拟通道+限制/保证带宽+通道优先级，天融信手册《流量管理》页），未直接耦合在基础访问控制策略表内（联网核实厂商流控资料，手册未详载）</t>
+          <t>PA主动/主动HA配置下NAT规则可绑定会话所有者/会话设置，控制NAT会话的设备绑定，仅A/A模式可见（PA Web帮助p150）；天融信HA为主备双机热备模式（天融信手册《配置双机热备功能》页），无主动/主动模式及NAT规则绑定机制</t>
         </is>
       </c>
       <c r="F14" s="80" t="inlineStr">
@@ -5390,226 +5418,226 @@
       <c r="G14" s="81" t="inlineStr"/>
       <c r="H14" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
+          <t>不支持</t>
         </is>
       </c>
       <c r="I14" s="80" t="inlineStr"/>
     </row>
-    <row r="15" ht="111" customHeight="1" s="1">
+    <row r="15" ht="96" customHeight="1" s="1">
       <c r="A15" s="82" t="n"/>
       <c r="B15" s="80" t="inlineStr">
         <is>
-          <t>基于策略转发(PBF)</t>
+          <t>QoS策略</t>
         </is>
       </c>
       <c r="C15" s="81" t="inlineStr">
         <is>
-          <t>支持PBF强制对称返回（非对称路由环境）</t>
+          <t>支持QoS策略规则内直接按DSCP/ToS匹配调度</t>
         </is>
       </c>
       <c r="D15" s="81" t="inlineStr">
         <is>
-          <t>记录入接口MAC，回包强制原路返回</t>
+          <t>QoS策略规则DSCP/ToS直接匹配（非独立流控模块配置）</t>
         </is>
       </c>
       <c r="E15" s="81" t="inlineStr">
         <is>
-          <t>PA对称返回：虚拟路由器替代返回流量的路由查找，将流量引导回接收SYN数据包的MAC地址（ARP表确定下一跳），双ISP双活/非对称路由核心机制（PA管理指南p1294）；天融信手册检索无对称返回/回程机制命中，策略路由与LLB的回程保障能力待验证；迁移评估项：多ISP双活环境需实测天融信回包路由对称性，否则现网业务中断</t>
+          <t>PA QoS规则可直接按DSCP值或IP优先级/ToS匹配调度（PA Web帮助p155）；天融信支持DSCP/802.1p(CoS)识别与重标记，但需在独立流量管理模块配置（虚拟通道+限制/保证带宽+通道优先级，天融信手册《流量管理》页），未直接耦合在基础访问控制策略表内（联网核实厂商流控资料，手册未详载）</t>
         </is>
       </c>
       <c r="F15" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>低</t>
         </is>
       </c>
       <c r="G15" s="81" t="inlineStr"/>
       <c r="H15" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>部分支持</t>
         </is>
       </c>
       <c r="I15" s="80" t="inlineStr"/>
     </row>
-    <row r="16" ht="51" customHeight="1" s="1">
+    <row r="16" ht="111" customHeight="1" s="1">
       <c r="A16" s="82" t="n"/>
       <c r="B16" s="80" t="inlineStr">
         <is>
-          <t>解密策略(Decryption)</t>
+          <t>基于策略转发(PBF)</t>
         </is>
       </c>
       <c r="C16" s="81" t="inlineStr">
         <is>
-          <t>支持解密流量镜像到专用接口（Decryption Port Mirroring）</t>
+          <t>支持PBF强制对称返回（非对称路由环境）</t>
         </is>
       </c>
       <c r="D16" s="81" t="inlineStr">
         <is>
-          <t>解密后明文流量镜像至专用接口供第三方分析</t>
+          <t>记录入接口MAC，回包强制原路返回</t>
         </is>
       </c>
       <c r="E16" s="81" t="inlineStr">
         <is>
-          <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证（PA管理指南p1059）；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
+          <t>PA对称返回：虚拟路由器替代返回流量的路由查找，将流量引导回接收SYN数据包的MAC地址（ARP表确定下一跳），双ISP双活/非对称路由核心机制（PA管理指南p1294）；天融信手册检索无对称返回/回程机制命中，策略路由与LLB的回程保障能力待验证；迁移评估项：多ISP双活环境需实测天融信回包路由对称性，否则现网业务中断</t>
         </is>
       </c>
       <c r="F16" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G16" s="81" t="inlineStr"/>
       <c r="H16" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
+          <t>待评估</t>
         </is>
       </c>
       <c r="I16" s="80" t="inlineStr"/>
     </row>
-    <row r="17" ht="126" customHeight="1" s="1">
+    <row r="17" ht="51" customHeight="1" s="1">
       <c r="A17" s="82" t="n"/>
-      <c r="B17" s="82" t="n"/>
+      <c r="B17" s="80" t="inlineStr">
+        <is>
+          <t>解密策略(Decryption)</t>
+        </is>
+      </c>
       <c r="C17" s="81" t="inlineStr">
         <is>
-          <t>支持解密不受信证书分离处理（Forward Untrust Certificate）</t>
+          <t>支持解密流量镜像到专用接口（Decryption Port Mirroring）</t>
         </is>
       </c>
       <c r="D17" s="81" t="inlineStr">
         <is>
-          <t>外部无效证书以不受信转发证书重签，保留浏览器告警</t>
+          <t>解密后明文流量镜像至专用接口供第三方分析</t>
         </is>
       </c>
       <c r="E17" s="81" t="inlineStr">
         <is>
-          <t>PA转发代理遇外部过期/不受信证书时，不用内部信任CA重签，而是专用Forward Untrust Certificate重签名，让浏览器保留不受信告警（PA管理指南p994、p1030）；天融信SSL解密（透明代理/服务器SSL解密，天融信手册《代理策略》页）未见受信/不受信双证书体系；迁移评估项：需验证天融信对外部无效证书的处理方式，避免直接阻断（白屏）或信任重签（掩盖风险）</t>
+          <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证（PA管理指南p1059）；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
         </is>
       </c>
       <c r="F17" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G17" s="81" t="inlineStr"/>
       <c r="H17" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>不支持</t>
         </is>
       </c>
       <c r="I17" s="80" t="inlineStr"/>
     </row>
-    <row r="18" ht="66" customHeight="1" s="1">
+    <row r="18" ht="126" customHeight="1" s="1">
       <c r="A18" s="82" t="n"/>
       <c r="B18" s="82" t="n"/>
       <c r="C18" s="81" t="inlineStr">
         <is>
-          <t>支持解密规则按URL类别选择性解密（URL Category）</t>
+          <t>支持解密不受信证书分离处理（Forward Untrust Certificate）</t>
         </is>
       </c>
       <c r="D18" s="81" t="inlineStr">
         <is>
-          <t>按URL类别圈定解密范围，排除银行/医疗等敏感类</t>
+          <t>外部无效证书以不受信转发证书重签，保留浏览器告警</t>
         </is>
       </c>
       <c r="E18" s="81" t="inlineStr">
         <is>
-          <t>PA解密规则可按URL类别（含自定义类别）选择解密范围，可排除银行/医疗等敏感类别不解密（PA Web帮助p164）；天融信SSL解密（代理策略/代理模板）无按URL类别选择解密机制（检索无命中）</t>
+          <t>PA转发代理遇外部过期/不受信证书时，不用内部信任CA重签，而是专用Forward Untrust Certificate重签名，让浏览器保留不受信告警（PA管理指南p994、p1030）；天融信SSL解密（透明代理/服务器SSL解密，天融信手册《代理策略》页）未见受信/不受信双证书体系；迁移评估项：需验证天融信对外部无效证书的处理方式，避免直接阻断（白屏）或信任重签（掩盖风险）</t>
         </is>
       </c>
       <c r="F18" s="80" t="inlineStr">
         <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="G18" s="82" t="n"/>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="G18" s="81" t="inlineStr"/>
       <c r="H18" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="I18" s="82" t="n"/>
-    </row>
-    <row r="19" ht="96" customHeight="1" s="1">
+          <t>待评估</t>
+        </is>
+      </c>
+      <c r="I18" s="80" t="inlineStr"/>
+    </row>
+    <row r="19" ht="66" customHeight="1" s="1">
       <c r="A19" s="82" t="n"/>
       <c r="B19" s="82" t="n"/>
       <c r="C19" s="81" t="inlineStr">
         <is>
+          <t>支持解密规则按URL类别选择性解密（URL Category）</t>
+        </is>
+      </c>
+      <c r="D19" s="81" t="inlineStr">
+        <is>
+          <t>按URL类别圈定解密范围，排除银行/医疗等敏感类</t>
+        </is>
+      </c>
+      <c r="E19" s="81" t="inlineStr">
+        <is>
+          <t>PA解密规则可按URL类别（含自定义类别）选择解密范围，可排除银行/医疗等敏感类别不解密（PA Web帮助p164）；天融信SSL解密（代理策略/代理模板）无按URL类别选择解密机制（检索无命中）</t>
+        </is>
+      </c>
+      <c r="F19" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G19" s="82" t="n"/>
+      <c r="H19" s="80" t="inlineStr">
+        <is>
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I19" s="82" t="n"/>
+    </row>
+    <row r="20" ht="96" customHeight="1" s="1">
+      <c r="A20" s="82" t="n"/>
+      <c r="B20" s="82" t="n"/>
+      <c r="C20" s="81" t="inlineStr">
+        <is>
           <t>支持SSH代理解密与SSH隧道控制（SSH Proxy）</t>
         </is>
       </c>
-      <c r="D19" s="81" t="inlineStr">
+      <c r="D20" s="81" t="inlineStr">
         <is>
           <t>SSH代理解密+SSH隧道(ssh-tunnel)识别控制</t>
         </is>
       </c>
-      <c r="E19" s="81" t="inlineStr">
+      <c r="E20" s="81" t="inlineStr">
         <is>
           <t>PA解密策略SSH Proxy类型解密SSH通信，可通过ssh-tunnel App-ID在策略中控制SSH隧道（端口转发/内网穿透），正常SSH管理流量放行；含不受支持算法检查/资源不足阻断会话等防护（PA Web帮助p164、p318-319）；天融信手册检索无SSH代理/SSH隧道控制命中</t>
         </is>
       </c>
-      <c r="F19" s="82" t="n"/>
-      <c r="G19" s="82" t="n"/>
-      <c r="H19" s="82" t="n"/>
-      <c r="I19" s="82" t="n"/>
-    </row>
-    <row r="20" ht="111" customHeight="1" s="1">
-      <c r="A20" s="82" t="n"/>
-      <c r="B20" s="80" t="inlineStr">
+      <c r="F20" s="82" t="n"/>
+      <c r="G20" s="82" t="n"/>
+      <c r="H20" s="82" t="n"/>
+      <c r="I20" s="82" t="n"/>
+    </row>
+    <row r="21" ht="111" customHeight="1" s="1">
+      <c r="A21" s="82" t="n"/>
+      <c r="B21" s="80" t="inlineStr">
         <is>
           <t>网络数据包代理(NPBroker)</t>
         </is>
       </c>
-      <c r="C20" s="81" t="inlineStr">
+      <c r="C21" s="81" t="inlineStr">
         <is>
           <t>支持内联数据包代理策略将流量转发第三方安全链（NPBroker）</t>
         </is>
       </c>
-      <c r="D20" s="81" t="inlineStr">
+      <c r="D21" s="81" t="inlineStr">
         <is>
           <t>已解密/未解密流量内联转发第三方安全链，L3路由转发</t>
         </is>
       </c>
-      <c r="E20" s="81" t="inlineStr">
+      <c r="E21" s="81" t="inlineStr">
         <is>
           <t>PA网络数据包代理策略将已解密/未解密TLS/非TLS流量内联转发至第三方安全工具，路径选择选项卡应用数据包代理配置文件定义经路由L3安全链的转发方式（PA Web帮助p167-170）；天融信无网络数据包代理模块，最接近手段为WAF旁路联动（经交换机镜像引流，天融信手册《与WAF联动》页），非内联且无回注路径；对应矩阵#122</t>
         </is>
       </c>
-      <c r="F20" s="80" t="inlineStr">
+      <c r="F21" s="80" t="inlineStr">
         <is>
           <t>高</t>
-        </is>
-      </c>
-      <c r="G20" s="81" t="inlineStr"/>
-      <c r="H20" s="80" t="inlineStr">
-        <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="I20" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="66" customHeight="1" s="1">
-      <c r="A21" s="82" t="n"/>
-      <c r="B21" s="82" t="n"/>
-      <c r="C21" s="81" t="inlineStr">
-        <is>
-          <t>支持NPBroker转发流量类型选择（TLS解密/未解密/非TLS）</t>
-        </is>
-      </c>
-      <c r="D21" s="81" t="inlineStr">
-        <is>
-          <t>TLS解密/未解密/非TLS流量类型选择</t>
-        </is>
-      </c>
-      <c r="E21" s="81" t="inlineStr">
-        <is>
-          <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证（PA Web帮助p167）；天融信无网络数据包代理模块（矩阵#122）</t>
-        </is>
-      </c>
-      <c r="F21" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
         </is>
       </c>
       <c r="G21" s="81" t="inlineStr"/>
@@ -5618,33 +5646,33 @@
           <t>不支持</t>
         </is>
       </c>
-      <c r="I21" s="80" t="inlineStr"/>
-    </row>
-    <row r="22" ht="96" customHeight="1" s="1">
+      <c r="I21" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="66" customHeight="1" s="1">
       <c r="A22" s="82" t="n"/>
-      <c r="B22" s="80" t="inlineStr">
-        <is>
-          <t>隧道检测(Tunnel Inspection)</t>
-        </is>
-      </c>
+      <c r="B22" s="82" t="n"/>
       <c r="C22" s="81" t="inlineStr">
         <is>
-          <t>支持GTP-U/VXLAN/非加密IPSec隧道内层检测</t>
+          <t>支持NPBroker转发流量类型选择（TLS解密/未解密/非TLS）</t>
         </is>
       </c>
       <c r="D22" s="81" t="inlineStr">
         <is>
-          <t>GTP-U/VXLAN/NULL加密IPSec(AH)隧道内层流量检测</t>
+          <t>TLS解密/未解密/非TLS流量类型选择</t>
         </is>
       </c>
       <c r="E22" s="81" t="inlineStr">
         <is>
-          <t>PA隧道检测支持GTP-U/VXLAN/非加密IPSec（NULL加密/AH传输模式）内层检测（PA Web帮助p172-173）；天融信VXLAN仅隧道封装转发与三层网关（天融信手册《业务接入端》《三层VXLAN网关》页），无内层安全检测，GTP检测检索无命中；对应矩阵#128/37</t>
+          <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证（PA Web帮助p167）；天融信无网络数据包代理模块（矩阵#122）</t>
         </is>
       </c>
       <c r="F22" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G22" s="81" t="inlineStr"/>
@@ -5655,27 +5683,31 @@
       </c>
       <c r="I22" s="80" t="inlineStr"/>
     </row>
-    <row r="23" ht="51" customHeight="1" s="1">
+    <row r="23" ht="96" customHeight="1" s="1">
       <c r="A23" s="82" t="n"/>
-      <c r="B23" s="82" t="n"/>
+      <c r="B23" s="80" t="inlineStr">
+        <is>
+          <t>隧道检测(Tunnel Inspection)</t>
+        </is>
+      </c>
       <c r="C23" s="81" t="inlineStr">
         <is>
-          <t>支持最大封装级数防护（max_encap）</t>
+          <t>支持GTP-U/VXLAN/非加密IPSec隧道内层检测</t>
         </is>
       </c>
       <c r="D23" s="81" t="inlineStr">
         <is>
-          <t>隧道嵌套封装最大级数限制，超限丢弃</t>
+          <t>GTP-U/VXLAN/NULL加密IPSec(AH)隧道内层流量检测</t>
         </is>
       </c>
       <c r="E23" s="81" t="inlineStr">
         <is>
-          <t>PA对隧道最大封装级数超限丢包防护，防隧道嵌套绕过（PA管理指南p655）；天融信手册无封装级数防护（检索无命中）</t>
+          <t>PA隧道检测支持GTP-U/VXLAN/非加密IPSec（NULL加密/AH传输模式）内层检测（PA Web帮助p172-173）；天融信VXLAN仅隧道封装转发与三层网关（天融信手册《业务接入端》《三层VXLAN网关》页），无内层安全检测，GTP检测检索无命中；对应矩阵#128/37</t>
         </is>
       </c>
       <c r="F23" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G23" s="81" t="inlineStr"/>
@@ -5686,66 +5718,62 @@
       </c>
       <c r="I23" s="80" t="inlineStr"/>
     </row>
-    <row r="24" ht="96" customHeight="1" s="1">
+    <row r="24" ht="51" customHeight="1" s="1">
       <c r="A24" s="82" t="n"/>
-      <c r="B24" s="80" t="inlineStr">
-        <is>
-          <t>应用覆盖(App Override)</t>
-        </is>
-      </c>
+      <c r="B24" s="82" t="n"/>
       <c r="C24" s="81" t="inlineStr">
         <is>
-          <t>支持应用替代流量跳过七层检测等效配置</t>
+          <t>支持最大封装级数防护（max_encap）</t>
         </is>
       </c>
       <c r="D24" s="81" t="inlineStr">
         <is>
-          <t>匹配覆盖策略的流量跳过七层检测，四层快速转发</t>
+          <t>隧道嵌套封装最大级数限制，超限丢弃</t>
         </is>
       </c>
       <c r="E24" s="81" t="inlineStr">
         <is>
-          <t>PA应用替代策略明确绕过第7层处理与威胁检查，改用第4层状态检查以加速（PA管理指南p1307）；天融信自定义应用加入规则库后仍默认经安全引擎检测（天融信手册《自定义应用》页）；迁移评估项：PA应用替代多为私有大流量业务加速，转换时需同步关闭对应策略的IPS/七层检测，否则性能被拖垮或误阻断</t>
+          <t>PA对隧道最大封装级数超限丢包防护，防隧道嵌套绕过（PA管理指南p655）；天融信手册无封装级数防护（检索无命中）</t>
         </is>
       </c>
       <c r="F24" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G24" s="81" t="inlineStr"/>
       <c r="H24" s="80" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>不支持</t>
         </is>
       </c>
       <c r="I24" s="80" t="inlineStr"/>
     </row>
-    <row r="25" ht="81" customHeight="1" s="1">
+    <row r="25" ht="96" customHeight="1" s="1">
       <c r="A25" s="82" t="n"/>
       <c r="B25" s="80" t="inlineStr">
         <is>
-          <t>身份验证(Authentication)</t>
+          <t>应用覆盖(App Override)</t>
         </is>
       </c>
       <c r="C25" s="81" t="inlineStr">
         <is>
-          <t>支持认证策略超时与单次认证（SSO）</t>
+          <t>支持应用替代流量跳过七层检测等效配置</t>
         </is>
       </c>
       <c r="D25" s="81" t="inlineStr">
         <is>
-          <t>认证超时+单次认证(SSO)</t>
+          <t>匹配覆盖策略的流量跳过七层检测，四层快速转发</t>
         </is>
       </c>
       <c r="E25" s="81" t="inlineStr">
         <is>
-          <t>PA支持认证超时减少重复质询、Kerberos/SAML/RADIUS等对接（PA Web帮助p186）；天融信手册检索认证超时/单点登录/SSO无命中（仅在线用户在线时长查看与强制下线）；迁移评估项：需核实天融信认证会话有效期配置与SSO对接能力</t>
+          <t>PA应用替代策略明确绕过第7层处理与威胁检查，改用第4层状态检查以加速（PA管理指南p1307）；天融信自定义应用加入规则库后仍默认经安全引擎检测（天融信手册《自定义应用》页）；迁移评估项：PA应用替代多为私有大流量业务加速，转换时需同步关闭对应策略的IPS/七层检测，否则性能被拖垮或误阻断</t>
         </is>
       </c>
       <c r="F25" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G25" s="81" t="inlineStr"/>
@@ -5756,22 +5784,26 @@
       </c>
       <c r="I25" s="80" t="inlineStr"/>
     </row>
-    <row r="26" ht="126" customHeight="1" s="1">
+    <row r="26" ht="81" customHeight="1" s="1">
       <c r="A26" s="82" t="n"/>
-      <c r="B26" s="82" t="n"/>
+      <c r="B26" s="80" t="inlineStr">
+        <is>
+          <t>身份验证(Authentication)</t>
+        </is>
+      </c>
       <c r="C26" s="81" t="inlineStr">
         <is>
-          <t>支持流量策略触发多因素认证质询（MFA Enforcement）</t>
+          <t>支持认证策略超时与单次认证（SSO）</t>
         </is>
       </c>
       <c r="D26" s="81" t="inlineStr">
         <is>
-          <t>流量策略匹配触发MFA质询（非登录场景，MFA供应商API/RADIUS）</t>
+          <t>认证超时+单次认证(SSO)</t>
         </is>
       </c>
       <c r="E26" s="81" t="inlineStr">
         <is>
-          <t>PA身份验证策略通过Authentication Enforcement对象对匹配流量强制质询，支持多因素身份验证（每因素独立超时，防火墙记录时间戳），MFA供应商API/RADIUS对接（PA Web帮助p185-186、p310、p735-742）；天融信双因子认证（密码+短信/证书/Ukey）仅限管理员/用户登录场景（天融信手册《登录安全策略》页），无流量策略触发MFA质询</t>
+          <t>PA支持认证超时减少重复质询、Kerberos/SAML/RADIUS等对接（PA Web帮助p186）；天融信手册检索认证超时/单点登录/SSO无命中（仅在线用户在线时长查看与强制下线）；迁移评估项：需核实天融信认证会话有效期配置与SSO对接能力</t>
         </is>
       </c>
       <c r="F26" s="80" t="inlineStr">
@@ -5782,89 +5814,89 @@
       <c r="G26" s="81" t="inlineStr"/>
       <c r="H26" s="80" t="inlineStr">
         <is>
-          <t>不支持</t>
+          <t>待评估</t>
         </is>
       </c>
       <c r="I26" s="80" t="inlineStr"/>
     </row>
-    <row r="27" ht="96" customHeight="1" s="1">
+    <row r="27" ht="126" customHeight="1" s="1">
       <c r="A27" s="82" t="n"/>
       <c r="B27" s="82" t="n"/>
       <c r="C27" s="81" t="inlineStr">
         <is>
+          <t>支持流量策略触发多因素认证质询（MFA Enforcement）</t>
+        </is>
+      </c>
+      <c r="D27" s="81" t="inlineStr">
+        <is>
+          <t>流量策略匹配触发MFA质询（非登录场景，MFA供应商API/RADIUS）</t>
+        </is>
+      </c>
+      <c r="E27" s="81" t="inlineStr">
+        <is>
+          <t>PA身份验证策略通过Authentication Enforcement对象对匹配流量强制质询，支持多因素身份验证（每因素独立超时，防火墙记录时间戳），MFA供应商API/RADIUS对接（PA Web帮助p185-186、p310、p735-742）；天融信双因子认证（密码+短信/证书/Ukey）仅限管理员/用户登录场景（天融信手册《登录安全策略》页），无流量策略触发MFA质询</t>
+        </is>
+      </c>
+      <c r="F27" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G27" s="81" t="inlineStr"/>
+      <c r="H27" s="80" t="inlineStr">
+        <is>
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I27" s="80" t="inlineStr"/>
+    </row>
+    <row r="28" ht="96" customHeight="1" s="1">
+      <c r="A28" s="82" t="n"/>
+      <c r="B28" s="82" t="n"/>
+      <c r="C28" s="81" t="inlineStr">
+        <is>
           <t>支持User-ID动态映射时效性等效（AD日志毫秒级更新）</t>
         </is>
       </c>
-      <c r="D27" s="81" t="inlineStr">
+      <c r="D28" s="81" t="inlineStr">
         <is>
           <t>AD域事件日志毫秒级IP-用户映射更新</t>
         </is>
       </c>
-      <c r="E27" s="81" t="inlineStr">
+      <c r="E28" s="81" t="inlineStr">
         <is>
           <t>PA无代理架构通过读取域控事件日志实现IP-用户毫秒级动态映射，大规模部署有专项规划（PA管理指南p866-867）；天融信AD对接的轮询间隔与并发认证能力手册未量化；迁移评估项：数万AD用户且移动频繁场景需实测天融信映射更新时延，避免基于用户的策略出现间歇性未授权拦截</t>
         </is>
       </c>
-      <c r="F27" s="82" t="n"/>
-      <c r="G27" s="82" t="n"/>
-      <c r="H27" s="80" t="inlineStr">
+      <c r="F28" s="82" t="n"/>
+      <c r="G28" s="82" t="n"/>
+      <c r="H28" s="80" t="inlineStr">
         <is>
           <t>待评估</t>
         </is>
       </c>
-      <c r="I27" s="82" t="n"/>
-    </row>
-    <row r="28" ht="171" customHeight="1" s="1">
-      <c r="A28" s="82" t="n"/>
-      <c r="B28" s="80" t="inlineStr">
+      <c r="I28" s="82" t="n"/>
+    </row>
+    <row r="29" ht="171" customHeight="1" s="1">
+      <c r="A29" s="82" t="n"/>
+      <c r="B29" s="80" t="inlineStr">
         <is>
           <t>动态对象(Dynamic Objects)</t>
         </is>
       </c>
-      <c r="C28" s="81" t="inlineStr">
+      <c r="C29" s="81" t="inlineStr">
         <is>
           <t>支持外部动态列表作为策略地址对象（EDL）</t>
         </is>
       </c>
-      <c r="D28" s="81" t="inlineStr">
+      <c r="D29" s="81" t="inlineStr">
         <is>
           <t>HTTP/HTTPS外部文本列表(IP/域名/URL)自动拉取，策略直接引用</t>
         </is>
       </c>
-      <c r="E28" s="81" t="inlineStr">
+      <c r="E29" s="81" t="inlineStr">
         <is>
           <t>PA外部动态列表：基于HTTP/HTTPS托管的文本文件创建IP/URL/域名/IMEI/IMSI地址对象，防火墙定时自动拉取更新，策略中直接引用（Objects&gt;External Dynamic Lists，PA Web帮助p236-239；策略源/目标可直接选EDL，p196-197）；天融信手册检索外部动态列表/EDL无命中，仅内置威胁情报库与云端威胁情报库（规则集管理，天融信手册《威胁情报》《配置规则集》页），无策略直接引用任意外部文本列表机制；迁移评估项：PA策略中引用的EDL需转换为天融信静态地址组定期导入或威胁情报联动</t>
-        </is>
-      </c>
-      <c r="F28" s="80" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="G28" s="81" t="inlineStr"/>
-      <c r="H28" s="80" t="inlineStr">
-        <is>
-          <t>不支持</t>
-        </is>
-      </c>
-      <c r="I28" s="80" t="inlineStr"/>
-    </row>
-    <row r="29" ht="126" customHeight="1" s="1">
-      <c r="A29" s="82" t="n"/>
-      <c r="B29" s="82" t="n"/>
-      <c r="C29" s="81" t="inlineStr">
-        <is>
-          <t>支持基于标记的动态地址组（DAG）</t>
-        </is>
-      </c>
-      <c r="D29" s="81" t="inlineStr">
-        <is>
-          <t>Tag标记过滤器动态地址组，成员随IP变化自动更新</t>
-        </is>
-      </c>
-      <c r="E29" s="81" t="inlineStr">
-        <is>
-          <t>PA动态地址组：查找标记(Tag)+基于标记的过滤器（AND/OR匹配）动态填充成员，VM信息源注册或XML/REST API定义标记，IP变化时策略自动生效（PA Web帮助p207-208、p228）；天融信手册检索动态地址组/标签/SDN/云平台联动无命中，地址组为静态IP/子网绑定（天融信手册《地址》页）；迁移评估项：PA云环境Tag微隔离策略需转换为静态地址组，IP漂移场景需人工或API维护</t>
         </is>
       </c>
       <c r="F29" s="80" t="inlineStr">
@@ -5880,66 +5912,62 @@
       </c>
       <c r="I29" s="80" t="inlineStr"/>
     </row>
-    <row r="30" ht="81" customHeight="1" s="1">
+    <row r="30" ht="126" customHeight="1" s="1">
       <c r="A30" s="82" t="n"/>
-      <c r="B30" s="80" t="inlineStr">
-        <is>
-          <t>SD-WAN策略</t>
-        </is>
-      </c>
+      <c r="B30" s="82" t="n"/>
       <c r="C30" s="81" t="inlineStr">
         <is>
-          <t>支持按应用配置链路路径管理与链路质量探测</t>
+          <t>支持基于标记的动态地址组（DAG）</t>
         </is>
       </c>
       <c r="D30" s="81" t="inlineStr">
         <is>
-          <t>按应用分配链路与流量分发（天融信以策略路由+LLB近似实现）</t>
+          <t>Tag标记过滤器动态地址组，成员随IP变化自动更新</t>
         </is>
       </c>
       <c r="E30" s="81" t="inlineStr">
         <is>
-          <t>PA SD-WAN策略按应用/抖动/延迟/丢包指标分配链路，流量分发（PA Web帮助p197）；天融信为策略路由+链路负载均衡近似实现（天融信手册《策略路由》《链路负载均衡》页），无SD-WAN策略模型；对应矩阵#129/120</t>
+          <t>PA动态地址组：查找标记(Tag)+基于标记的过滤器（AND/OR匹配）动态填充成员，VM信息源注册或XML/REST API定义标记，IP变化时策略自动生效（PA Web帮助p207-208、p228）；天融信手册检索动态地址组/标签/SDN/云平台联动无命中，地址组为静态IP/子网绑定（天融信手册《地址》页）；迁移评估项：PA云环境Tag微隔离策略需转换为静态地址组，IP漂移场景需人工或API维护</t>
         </is>
       </c>
       <c r="F30" s="80" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="G30" s="81" t="inlineStr"/>
       <c r="H30" s="80" t="inlineStr">
         <is>
-          <t>部分支持</t>
-        </is>
-      </c>
-      <c r="I30" s="80" t="inlineStr">
-        <is>
-          <t>产品线</t>
-        </is>
-      </c>
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I30" s="80" t="inlineStr"/>
     </row>
     <row r="31" ht="81" customHeight="1" s="1">
       <c r="A31" s="82" t="n"/>
-      <c r="B31" s="82" t="n"/>
+      <c r="B31" s="80" t="inlineStr">
+        <is>
+          <t>SD-WAN策略</t>
+        </is>
+      </c>
       <c r="C31" s="81" t="inlineStr">
         <is>
-          <t>支持SD-WAN路径选择与链路质量监测（jitter/latency/loss）</t>
+          <t>支持按应用配置链路路径管理与链路质量探测</t>
         </is>
       </c>
       <c r="D31" s="81" t="inlineStr">
         <is>
-          <t>抖动/延迟/丢包多维指标选路（天融信现仅延迟探测）</t>
+          <t>按应用分配链路与流量分发（天融信以策略路由+LLB近似实现）</t>
         </is>
       </c>
       <c r="E31" s="81" t="inlineStr">
         <is>
-          <t>PA路径质量配置文件基于抖动/延迟/丢包等运行状况指标选路（PA Web帮助p195）；天融信有链路探测(ping)+智能选路(最小延迟优先)（天融信手册《策略路由》页），无jitter/latency/loss多维指标</t>
+          <t>PA SD-WAN策略按应用/抖动/延迟/丢包指标分配链路，流量分发（PA Web帮助p197）；天融信为策略路由+链路负载均衡近似实现（天融信手册《策略路由》《链路负载均衡》页），无SD-WAN策略模型；对应矩阵#129/120</t>
         </is>
       </c>
       <c r="F31" s="80" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="G31" s="81" t="inlineStr"/>
@@ -5948,35 +5976,71 @@
           <t>部分支持</t>
         </is>
       </c>
-      <c r="I31" s="80" t="inlineStr"/>
+      <c r="I31" s="80" t="inlineStr">
+        <is>
+          <t>产品线</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="81" customHeight="1" s="1">
+      <c r="A32" s="82" t="n"/>
+      <c r="B32" s="82" t="n"/>
+      <c r="C32" s="81" t="inlineStr">
+        <is>
+          <t>支持SD-WAN路径选择与链路质量监测（jitter/latency/loss）</t>
+        </is>
+      </c>
+      <c r="D32" s="81" t="inlineStr">
+        <is>
+          <t>抖动/延迟/丢包多维指标选路（天融信现仅延迟探测）</t>
+        </is>
+      </c>
+      <c r="E32" s="81" t="inlineStr">
+        <is>
+          <t>PA路径质量配置文件基于抖动/延迟/丢包等运行状况指标选路（PA Web帮助p195）；天融信有链路探测(ping)+智能选路(最小延迟优先)（天融信手册《策略路由》页），无jitter/latency/loss多维指标</t>
+        </is>
+      </c>
+      <c r="F32" s="80" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="G32" s="81" t="inlineStr"/>
+      <c r="H32" s="80" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="I32" s="80" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="I17:I19"/>
-    <mergeCell ref="B12:B13"/>
+  <mergeCells count="26">
+    <mergeCell ref="I18:I20"/>
     <mergeCell ref="I6:I11"/>
+    <mergeCell ref="G6:G12"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="I26:I27"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="B5:B11"/>
-    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A2:A32"/>
+    <mergeCell ref="B26:B28"/>
     <mergeCell ref="G3:G4"/>
     <mergeCell ref="I3:I4"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="G17:G19"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="F27:F28"/>
     <mergeCell ref="H3:H4"/>
-    <mergeCell ref="G6:G11"/>
-    <mergeCell ref="B20:B21"/>
     <mergeCell ref="B2:B4"/>
-    <mergeCell ref="A2:A31"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="G27:G28"/>
     <mergeCell ref="H8:H11"/>
     <mergeCell ref="F7:F8"/>
-    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="B5:B12"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: update PA project schedule excel file
update the binary excel file that contains the PA project schedule data
</commit_message>
<xml_diff>
--- a/PA替代需求列表.xlsx
+++ b/PA替代需求列表.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="261">
   <si>
     <t>一级需求</t>
   </si>
@@ -576,43 +576,43 @@
     <t>PA支持设备对象构建块（对应矩阵#3/4）；天融信经EDR联动上报终端资产并下发管控策略（天融信手册《与EDR联动》页），无独立设备对象</t>
   </si>
   <si>
+    <t>支持端口(L4)规则向应用(L7)规则迁移工作流</t>
+  </si>
+  <si>
+    <t>端口规则一键迁移为应用规则</t>
+  </si>
+  <si>
+    <t>PA策略优化器提供新应用查看器与端口→App-ID规则迁移工作流（PA Web帮助p142）；天融信策略统计仅显示规则命中数（天融信手册《配置访问控制策略》页），无迁移工具（命中统计能力已另列已支持行）；对应矩阵#132</t>
+  </si>
+  <si>
+    <t>支持应用匹配时强制校验标准端口</t>
+  </si>
+  <si>
+    <t>应用规则匹配时同时校验应用的标准端口，非标准端口流量不匹配</t>
+  </si>
+  <si>
+    <t>PA安全策略默认服务为application-default：放行应用同时强制其使用标准端口（如SSH仅22），非标准端口不匹配即拦截（PA管理指南p904）；天融信策略为五元组+应用识别组合（天融信手册《配置访问控制策略》页）；迁移评估项：直接转换若仅保留应用识别不限端口将扩大安全敞口，需制定应用标准端口映射限制（App-Default）转换方案；对应矩阵#2</t>
+  </si>
+  <si>
+    <t>支持将隐式默认规则显式化</t>
+  </si>
+  <si>
+    <t>同区域默认放行/跨区域默认拒绝的两条隐式系统规则可被提取为显式规则</t>
+  </si>
+  <si>
+    <t>PA安全策略库末尾自带两条隐式系统规则：区域内默认（同Zone默认放行）与区域间默认（跨Zone默认拒绝），可被替代配置，替代字段含日志转发配置文件与Log at Session End在会话结束时记录（PA Web帮助p134-136）；天融信未见同区域默认放行的隐式规则机制；迁移评估项：①必须提取intrazone-default同Zone互访需求并显式转换为放行规则，否则割接后同Zone不同网段/VLAN互访将被默认拦截；②需在新设备补齐底部兜底Deny-All并开启日志，否则被拒流量查无日志、排障困难</t>
+  </si>
+  <si>
+    <t>支持WildFire云沙箱文件检测联动</t>
+  </si>
+  <si>
+    <t>策略动作绑定WildFire配置文件</t>
+  </si>
+  <si>
+    <t>PA策略Actions可绑定WildFire Analysis配置文件（安全配置文件组含反病毒/漏洞/URL/文件阻断/WildFire，PA Web帮助p304；WildFire提交日志转发p305-306），云沙箱动态分析未知/零日威胁并秒级下发签名；天融信有内置APT沙箱（虚拟运行环境检测未知漏洞威胁）与沙箱联动（天融信手册《高级威胁防护》《APT联动配置》页），无云端动态分析与秒级签名下发证据；工作表1已登记云沙箱联动需求（不支持：公司无此产品），勿重复跟踪；迁移评估项：评估天融信本地APT沙箱与PA云沙箱检测能力等效性</t>
+  </si>
+  <si>
     <t>部分支持</t>
-  </si>
-  <si>
-    <t>支持端口(L4)规则向应用(L7)规则迁移工作流</t>
-  </si>
-  <si>
-    <t>端口规则一键迁移为应用规则</t>
-  </si>
-  <si>
-    <t>PA策略优化器提供新应用查看器与端口→App-ID规则迁移工作流（PA Web帮助p142）；天融信策略统计仅显示规则命中数（天融信手册《配置访问控制策略》页），无迁移工具（命中统计能力已另列已支持行）；对应矩阵#132</t>
-  </si>
-  <si>
-    <t>支持应用匹配时强制校验标准端口</t>
-  </si>
-  <si>
-    <t>应用规则匹配时同时校验应用的标准端口，非标准端口流量不匹配</t>
-  </si>
-  <si>
-    <t>PA安全策略默认服务为application-default：放行应用同时强制其使用标准端口（如SSH仅22），非标准端口不匹配即拦截（PA管理指南p904）；天融信策略为五元组+应用识别组合（天融信手册《配置访问控制策略》页）；迁移评估项：直接转换若仅保留应用识别不限端口将扩大安全敞口，需制定应用标准端口映射限制（App-Default）转换方案；对应矩阵#2</t>
-  </si>
-  <si>
-    <t>支持将隐式默认规则显式化</t>
-  </si>
-  <si>
-    <t>同区域默认放行/跨区域默认拒绝的两条隐式系统规则可被提取为显式规则</t>
-  </si>
-  <si>
-    <t>PA安全策略库末尾自带两条隐式系统规则：区域内默认（同Zone默认放行）与区域间默认（跨Zone默认拒绝），可被替代配置，替代字段含日志转发配置文件与Log at Session End在会话结束时记录（PA Web帮助p134-136）；天融信未见同区域默认放行的隐式规则机制；迁移评估项：①必须提取intrazone-default同Zone互访需求并显式转换为放行规则，否则割接后同Zone不同网段/VLAN互访将被默认拦截；②需在新设备补齐底部兜底Deny-All并开启日志，否则被拒流量查无日志、排障困难</t>
-  </si>
-  <si>
-    <t>支持WildFire云沙箱文件检测联动</t>
-  </si>
-  <si>
-    <t>策略动作绑定WildFire配置文件</t>
-  </si>
-  <si>
-    <t>PA策略Actions可绑定WildFire Analysis配置文件（安全配置文件组含反病毒/漏洞/URL/文件阻断/WildFire，PA Web帮助p304；WildFire提交日志转发p305-306），云沙箱动态分析未知/零日威胁并秒级下发签名；天融信有内置APT沙箱（虚拟运行环境检测未知漏洞威胁）与沙箱联动（天融信手册《高级威胁防护》《APT联动配置》页），无云端动态分析与秒级签名下发证据；工作表1已登记云沙箱联动需求（不支持：公司无此产品），勿重复跟踪；迁移评估项：评估天融信本地APT沙箱与PA云沙箱检测能力等效性</t>
   </si>
   <si>
     <t>支持配置源、目的域名</t>
@@ -1648,6 +1648,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1679,9 +1685,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1745,9 +1748,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2205,88 +2205,88 @@
     <col min="5" max="5" width="7.70909090909091" style="1" customWidth="1"/>
     <col min="6" max="6" width="37.8545454545455" style="1" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="9.70909090909091" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.70909090909091" style="10" customWidth="1"/>
+    <col min="8" max="8" width="9.70909090909091" style="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="12" t="s">
+      <c r="F1" s="15"/>
+      <c r="G1" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="16"/>
-      <c r="E2" s="17" t="s">
+      <c r="D2" s="18"/>
+      <c r="E2" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1" spans="1:8">
       <c r="A3" s="6"/>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1" spans="1:8">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="18" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="6"/>
@@ -2297,10 +2297,10 @@
     <row r="5" ht="36" customHeight="1" spans="1:8">
       <c r="A5" s="6"/>
       <c r="B5" s="7"/>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="18" t="s">
         <v>21</v>
       </c>
       <c r="E5" s="7"/>
@@ -2310,35 +2310,35 @@
     </row>
     <row r="6" ht="14.25" customHeight="1" spans="1:8">
       <c r="A6" s="6"/>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="G6" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1" spans="1:8">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="6"/>
@@ -2349,10 +2349,10 @@
     <row r="8" ht="14.25" customHeight="1" spans="1:8">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="6"/>
@@ -2363,10 +2363,10 @@
     <row r="9" ht="14.25" customHeight="1" spans="1:8">
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E9" s="6"/>
@@ -2377,10 +2377,10 @@
     <row r="10" ht="14.25" customHeight="1" spans="1:8">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="16"/>
+      <c r="D10" s="18"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
@@ -2389,10 +2389,10 @@
     <row r="11" ht="14.25" customHeight="1" spans="1:8">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="16"/>
+      <c r="D11" s="18"/>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
@@ -2401,10 +2401,10 @@
     <row r="12" ht="14.25" customHeight="1" spans="1:8">
       <c r="A12" s="6"/>
       <c r="B12" s="7"/>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="16"/>
+      <c r="D12" s="18"/>
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
@@ -2412,58 +2412,58 @@
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:8">
       <c r="A13" s="7"/>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="16" t="s">
+      <c r="G13" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="H13" s="19" t="s">
+      <c r="H13" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="F14" s="18" t="s">
+      <c r="F14" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="16" t="s">
+      <c r="G14" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="H14" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A15" s="24"/>
+      <c r="A15" s="25"/>
       <c r="B15" s="6"/>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D15" s="6"/>
@@ -2473,9 +2473,9 @@
       <c r="H15" s="6"/>
     </row>
     <row r="16" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A16" s="24"/>
+      <c r="A16" s="25"/>
       <c r="B16" s="6"/>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="18" t="s">
         <v>44</v>
       </c>
       <c r="D16" s="6"/>
@@ -2485,9 +2485,9 @@
       <c r="H16" s="6"/>
     </row>
     <row r="17" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A17" s="24"/>
+      <c r="A17" s="25"/>
       <c r="B17" s="6"/>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="18" t="s">
         <v>45</v>
       </c>
       <c r="D17" s="6"/>
@@ -2497,9 +2497,9 @@
       <c r="H17" s="6"/>
     </row>
     <row r="18" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A18" s="24"/>
+      <c r="A18" s="25"/>
       <c r="B18" s="6"/>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="18" t="s">
         <v>46</v>
       </c>
       <c r="D18" s="6"/>
@@ -2509,9 +2509,9 @@
       <c r="H18" s="6"/>
     </row>
     <row r="19" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A19" s="24"/>
+      <c r="A19" s="25"/>
       <c r="B19" s="6"/>
-      <c r="C19" s="16" t="s">
+      <c r="C19" s="18" t="s">
         <v>47</v>
       </c>
       <c r="D19" s="6"/>
@@ -2521,9 +2521,9 @@
       <c r="H19" s="6"/>
     </row>
     <row r="20" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A20" s="24"/>
+      <c r="A20" s="25"/>
       <c r="B20" s="6"/>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="18" t="s">
         <v>48</v>
       </c>
       <c r="D20" s="6"/>
@@ -2533,9 +2533,9 @@
       <c r="H20" s="6"/>
     </row>
     <row r="21" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A21" s="24"/>
+      <c r="A21" s="25"/>
       <c r="B21" s="6"/>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="18" t="s">
         <v>49</v>
       </c>
       <c r="D21" s="6"/>
@@ -2545,9 +2545,9 @@
       <c r="H21" s="6"/>
     </row>
     <row r="22" ht="32.25" customHeight="1" spans="1:8">
-      <c r="A22" s="25"/>
+      <c r="A22" s="26"/>
       <c r="B22" s="7"/>
-      <c r="C22" s="16" t="s">
+      <c r="C22" s="18" t="s">
         <v>50</v>
       </c>
       <c r="D22" s="7"/>
@@ -2557,125 +2557,125 @@
       <c r="H22" s="7"/>
     </row>
     <row r="23" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="21" t="s">
+      <c r="B23" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="16" t="s">
+      <c r="C23" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="16" t="s">
+      <c r="D23" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="E23" s="17" t="s">
+      <c r="E23" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="26" t="s">
+      <c r="F23" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="G23" s="16" t="s">
+      <c r="G23" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H23" s="19" t="s">
+      <c r="H23" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="16" t="s">
+      <c r="D24" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="E24" s="17" t="s">
+      <c r="E24" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="F24" s="27" t="s">
+      <c r="F24" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="G24" s="16" t="s">
+      <c r="G24" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H24" s="19" t="s">
+      <c r="H24" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="16" t="s">
+      <c r="C25" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="28" t="s">
+      <c r="D25" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="E25" s="17" t="s">
+      <c r="E25" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="F25" s="18" t="s">
+      <c r="F25" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="G25" s="16" t="s">
+      <c r="G25" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H25" s="19" t="s">
+      <c r="H25" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="26" s="9" customFormat="1" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A26" s="24"/>
-      <c r="B26" s="21" t="s">
+    <row r="26" s="11" customFormat="1" ht="28.5" customHeight="1" spans="1:8">
+      <c r="A26" s="25"/>
+      <c r="B26" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="C26" s="19" t="s">
+      <c r="C26" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="28"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="16"/>
-      <c r="H26" s="19"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="30"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="8"/>
     </row>
     <row r="27" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A27" s="24"/>
-      <c r="B27" s="21" t="s">
+      <c r="A27" s="25"/>
+      <c r="B27" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C27" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="D27" s="16" t="s">
+      <c r="D27" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="E27" s="17" t="s">
+      <c r="E27" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="F27" s="18" t="s">
+      <c r="F27" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="G27" s="16" t="s">
+      <c r="G27" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H27" s="19" t="s">
+      <c r="H27" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A28" s="24"/>
+      <c r="A28" s="25"/>
       <c r="B28" s="7"/>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="18" t="s">
         <v>71</v>
       </c>
       <c r="D28" s="7"/>
@@ -2685,99 +2685,99 @@
       <c r="H28" s="7"/>
     </row>
     <row r="29" ht="60" customHeight="1" spans="1:8">
-      <c r="A29" s="24"/>
-      <c r="B29" s="21" t="s">
+      <c r="A29" s="25"/>
+      <c r="B29" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="C29" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="D29" s="19" t="s">
+      <c r="D29" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E29" s="17" t="s">
+      <c r="E29" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="F29" s="30" t="s">
+      <c r="F29" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="G29" s="16" t="s">
+      <c r="G29" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="H29" s="19" t="s">
+      <c r="H29" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A30" s="24"/>
+      <c r="A30" s="25"/>
       <c r="B30" s="6"/>
-      <c r="C30" s="16" t="s">
+      <c r="C30" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D30" s="16" t="s">
+      <c r="D30" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="E30" s="17" t="s">
+      <c r="E30" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F30" s="6"/>
-      <c r="G30" s="16" t="s">
+      <c r="G30" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H30" s="19" t="s">
+      <c r="H30" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A31" s="25"/>
+      <c r="A31" s="26"/>
       <c r="B31" s="7"/>
-      <c r="C31" s="16" t="s">
+      <c r="C31" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="D31" s="16" t="s">
+      <c r="D31" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="E31" s="31" t="s">
+      <c r="E31" s="32" t="s">
         <v>10</v>
       </c>
       <c r="F31" s="7"/>
-      <c r="G31" s="16" t="s">
+      <c r="G31" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H31" s="19" t="s">
+      <c r="H31" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A32" s="22" t="s">
+      <c r="A32" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="21" t="s">
+      <c r="B32" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="C32" s="16" t="s">
+      <c r="C32" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="D32" s="16" t="s">
+      <c r="D32" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="E32" s="17" t="s">
+      <c r="E32" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="F32" s="18" t="s">
+      <c r="F32" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="G32" s="16" t="s">
+      <c r="G32" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H32" s="19" t="s">
+      <c r="H32" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A33" s="25"/>
+      <c r="A33" s="26"/>
       <c r="B33" s="7"/>
-      <c r="C33" s="16" t="s">
+      <c r="C33" s="18" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="7"/>
@@ -2787,99 +2787,99 @@
       <c r="H33" s="7"/>
     </row>
     <row r="34" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A34" s="22" t="s">
+      <c r="A34" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="B34" s="21" t="s">
+      <c r="B34" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="C34" s="16" t="s">
+      <c r="C34" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="D34" s="16"/>
-      <c r="E34" s="17" t="s">
+      <c r="D34" s="18"/>
+      <c r="E34" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="F34" s="18" t="s">
+      <c r="F34" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="G34" s="16" t="s">
+      <c r="G34" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H34" s="19" t="s">
+      <c r="H34" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A35" s="24"/>
+      <c r="A35" s="25"/>
       <c r="B35" s="6"/>
-      <c r="C35" s="16" t="s">
+      <c r="C35" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="D35" s="16"/>
+      <c r="D35" s="18"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
     </row>
     <row r="36" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A36" s="24"/>
+      <c r="A36" s="25"/>
       <c r="B36" s="6"/>
-      <c r="C36" s="16" t="s">
+      <c r="C36" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="D36" s="16"/>
+      <c r="D36" s="18"/>
       <c r="E36" s="6"/>
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
     </row>
     <row r="37" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A37" s="25"/>
+      <c r="A37" s="26"/>
       <c r="B37" s="7"/>
-      <c r="C37" s="32" t="s">
+      <c r="C37" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="D37" s="32"/>
+      <c r="D37" s="33"/>
       <c r="E37" s="7"/>
       <c r="F37" s="7"/>
       <c r="G37" s="7"/>
       <c r="H37" s="7"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A38" s="21" t="s">
+      <c r="A38" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="B38" s="21" t="s">
+      <c r="B38" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="C38" s="33" t="s">
+      <c r="C38" s="34" t="s">
         <v>93</v>
       </c>
-      <c r="D38" s="33"/>
-      <c r="E38" s="31" t="s">
+      <c r="D38" s="34"/>
+      <c r="E38" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="F38" s="34" t="s">
+      <c r="F38" s="35" t="s">
         <v>61</v>
       </c>
-      <c r="G38" s="16" t="s">
+      <c r="G38" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H38" s="19" t="s">
+      <c r="H38" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" spans="1:8">
       <c r="A39" s="6"/>
-      <c r="B39" s="21" t="s">
+      <c r="B39" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="C39" s="33" t="s">
+      <c r="C39" s="34" t="s">
         <v>95</v>
       </c>
-      <c r="D39" s="33"/>
-      <c r="E39" s="31" t="s">
+      <c r="D39" s="34"/>
+      <c r="E39" s="32" t="s">
         <v>60</v>
       </c>
       <c r="F39" s="7"/>
@@ -2888,176 +2888,176 @@
     </row>
     <row r="40" ht="28.5" customHeight="1" spans="1:8">
       <c r="A40" s="6"/>
-      <c r="B40" s="21" t="s">
+      <c r="B40" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="C40" s="33" t="s">
+      <c r="C40" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="D40" s="35" t="s">
+      <c r="D40" s="36" t="s">
         <v>98</v>
       </c>
-      <c r="E40" s="31" t="s">
+      <c r="E40" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="F40" s="30" t="s">
+      <c r="F40" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="G40" s="16" t="s">
+      <c r="G40" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="H40" s="19" t="s">
+      <c r="H40" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" spans="1:8">
       <c r="A41" s="6"/>
-      <c r="B41" s="21" t="s">
+      <c r="B41" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="C41" s="16" t="s">
+      <c r="C41" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="D41" s="33" t="s">
+      <c r="D41" s="34" t="s">
         <v>101</v>
       </c>
-      <c r="E41" s="31" t="s">
+      <c r="E41" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="F41" s="30" t="s">
+      <c r="F41" s="31" t="s">
         <v>102</v>
       </c>
-      <c r="G41" s="16" t="s">
+      <c r="G41" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="H41" s="19" t="s">
+      <c r="H41" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" spans="1:8">
       <c r="A42" s="6"/>
-      <c r="B42" s="21" t="s">
+      <c r="B42" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="C42" s="16" t="s">
+      <c r="C42" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="D42" s="33"/>
-      <c r="E42" s="31"/>
-      <c r="F42" s="30"/>
-      <c r="G42" s="16"/>
-      <c r="H42" s="19"/>
+      <c r="D42" s="34"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="31"/>
+      <c r="G42" s="18"/>
+      <c r="H42" s="8"/>
     </row>
     <row r="43" ht="15.75" customHeight="1" spans="1:8">
       <c r="A43" s="7"/>
-      <c r="B43" s="21" t="s">
+      <c r="B43" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="C43" s="33" t="s">
+      <c r="C43" s="34" t="s">
         <v>107</v>
       </c>
-      <c r="D43" s="33"/>
-      <c r="E43" s="31" t="s">
+      <c r="D43" s="34"/>
+      <c r="E43" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="F43" s="30" t="s">
+      <c r="F43" s="31" t="s">
         <v>108</v>
       </c>
-      <c r="G43" s="16" t="s">
+      <c r="G43" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="H43" s="19" t="s">
+      <c r="H43" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A44" s="36" t="s">
+      <c r="A44" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="B44" s="37" t="s">
+      <c r="B44" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="C44" s="38" t="s">
+      <c r="C44" s="39" t="s">
         <v>112</v>
       </c>
-      <c r="D44" s="38" t="s">
+      <c r="D44" s="39" t="s">
         <v>113</v>
       </c>
-      <c r="E44" s="39" t="s">
+      <c r="E44" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="F44" s="40" t="s">
+      <c r="F44" s="41" t="s">
         <v>114</v>
       </c>
-      <c r="G44" s="41" t="s">
+      <c r="G44" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="H44" s="42" t="s">
+      <c r="H44" s="9" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A45" s="24"/>
+      <c r="A45" s="25"/>
       <c r="B45" s="6"/>
-      <c r="C45" s="33" t="s">
+      <c r="C45" s="34" t="s">
         <v>115</v>
       </c>
-      <c r="D45" s="33" t="s">
+      <c r="D45" s="34" t="s">
         <v>116</v>
       </c>
       <c r="E45" s="6"/>
       <c r="F45" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="G45" s="16" t="s">
+      <c r="G45" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H45" s="19" t="s">
+      <c r="H45" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A46" s="24"/>
+      <c r="A46" s="25"/>
       <c r="B46" s="6"/>
-      <c r="C46" s="33" t="s">
+      <c r="C46" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="D46" s="33"/>
+      <c r="D46" s="34"/>
       <c r="E46" s="6"/>
       <c r="F46" s="7"/>
       <c r="G46" s="7"/>
       <c r="H46" s="7"/>
     </row>
     <row r="47" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A47" s="24"/>
+      <c r="A47" s="25"/>
       <c r="B47" s="6"/>
-      <c r="C47" s="33" t="s">
+      <c r="C47" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="D47" s="33"/>
+      <c r="D47" s="34"/>
       <c r="E47" s="6"/>
       <c r="F47" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="G47" s="16" t="s">
+      <c r="G47" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H47" s="19" t="s">
+      <c r="H47" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A48" s="25"/>
+      <c r="A48" s="26"/>
       <c r="B48" s="7"/>
       <c r="C48" s="44" t="s">
         <v>119</v>
       </c>
       <c r="D48" s="44"/>
       <c r="E48" s="7"/>
-      <c r="F48" s="26" t="s">
+      <c r="F48" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="G48" s="32" t="s">
+      <c r="G48" s="33" t="s">
         <v>12</v>
       </c>
       <c r="H48" s="45" t="s">
@@ -3145,122 +3145,122 @@
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A53" s="37" t="s">
+      <c r="A53" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B53" s="37" t="s">
+      <c r="B53" s="38" t="s">
         <v>131</v>
       </c>
-      <c r="C53" s="38" t="s">
+      <c r="C53" s="39" t="s">
         <v>132</v>
       </c>
-      <c r="D53" s="38"/>
-      <c r="E53" s="39" t="s">
+      <c r="D53" s="39"/>
+      <c r="E53" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="F53" s="40" t="s">
+      <c r="F53" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="G53" s="41" t="s">
+      <c r="G53" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="H53" s="42" t="s">
+      <c r="H53" s="9" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="54" ht="28.5" customHeight="1" spans="1:8">
       <c r="A54" s="7"/>
-      <c r="B54" s="21" t="s">
+      <c r="B54" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="C54" s="19" t="s">
+      <c r="C54" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="D54" s="35" t="s">
+      <c r="D54" s="36" t="s">
         <v>135</v>
       </c>
-      <c r="E54" s="31" t="s">
+      <c r="E54" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="F54" s="30" t="s">
+      <c r="F54" s="31" t="s">
         <v>136</v>
       </c>
-      <c r="G54" s="16" t="s">
+      <c r="G54" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="H54" s="19" t="s">
+      <c r="H54" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A55" s="22" t="s">
+      <c r="A55" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="B55" s="21" t="s">
+      <c r="B55" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="C55" s="33" t="s">
+      <c r="C55" s="34" t="s">
         <v>139</v>
       </c>
-      <c r="D55" s="33"/>
-      <c r="E55" s="31" t="s">
+      <c r="D55" s="34"/>
+      <c r="E55" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="F55" s="30"/>
-      <c r="G55" s="16" t="s">
+      <c r="F55" s="31"/>
+      <c r="G55" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="H55" s="19" t="s">
+      <c r="H55" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="56" ht="42.75" customHeight="1" spans="1:8">
-      <c r="A56" s="22" t="s">
+      <c r="A56" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="B56" s="21" t="s">
+      <c r="B56" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="C56" s="33" t="s">
+      <c r="C56" s="34" t="s">
         <v>143</v>
       </c>
-      <c r="D56" s="35" t="s">
+      <c r="D56" s="36" t="s">
         <v>144</v>
       </c>
-      <c r="E56" s="31" t="s">
+      <c r="E56" s="32" t="s">
         <v>40</v>
       </c>
       <c r="F56" s="43" t="s">
         <v>145</v>
       </c>
-      <c r="G56" s="16"/>
-      <c r="H56" s="19" t="s">
+      <c r="G56" s="18"/>
+      <c r="H56" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="57" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A57" s="21" t="s">
+      <c r="A57" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="B57" s="21" t="s">
+      <c r="B57" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="C57" s="33" t="s">
+      <c r="C57" s="34" t="s">
         <v>147</v>
       </c>
-      <c r="D57" s="33" t="s">
+      <c r="D57" s="34" t="s">
         <v>148</v>
       </c>
-      <c r="E57" s="31" t="s">
+      <c r="E57" s="32" t="s">
         <v>60</v>
       </c>
       <c r="F57" s="43" t="s">
         <v>149</v>
       </c>
-      <c r="G57" s="16" t="s">
+      <c r="G57" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="H57" s="19" t="s">
+      <c r="H57" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
       <c r="B58" s="61" t="s">
         <v>150</v>
       </c>
-      <c r="C58" s="32" t="s">
+      <c r="C58" s="33" t="s">
         <v>151</v>
       </c>
       <c r="D58" s="44" t="s">
@@ -3283,7 +3283,7 @@
       <c r="F58" s="63" t="s">
         <v>153</v>
       </c>
-      <c r="G58" s="32" t="s">
+      <c r="G58" s="33" t="s">
         <v>103</v>
       </c>
       <c r="H58" s="45" t="s">
@@ -3305,7 +3305,7 @@
         <v>10</v>
       </c>
       <c r="F59" s="56"/>
-      <c r="G59" s="32" t="s">
+      <c r="G59" s="33" t="s">
         <v>103</v>
       </c>
       <c r="H59" s="57" t="s">
@@ -3496,7 +3496,7 @@
         <v>172</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>109</v>
@@ -3521,7 +3521,7 @@
         <v>60</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>176</v>
+        <v>109</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>162</v>
@@ -3531,13 +3531,13 @@
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="C7" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>178</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>179</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>10</v>
@@ -3551,13 +3551,13 @@
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>181</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>182</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>40</v>
@@ -3569,16 +3569,16 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>40</v>
+      <c r="F9" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
@@ -3587,17 +3587,19 @@
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="F10" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>188</v>
-      </c>
-      <c r="F10" s="7"/>
-      <c r="G10" s="4" t="s">
-        <v>176</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>13</v>
@@ -3606,15 +3608,15 @@
     <row r="11" ht="56" customHeight="1" spans="1:8">
       <c r="A11" s="6"/>
       <c r="B11" s="7"/>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8" t="s">
+      <c r="D11" s="10"/>
+      <c r="E11" s="10" t="s">
         <v>190</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>109</v>
@@ -3687,7 +3689,7 @@
         <v>60</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>162</v>
@@ -4043,7 +4045,7 @@
         <v>40</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>13</v>
@@ -4065,14 +4067,14 @@
         <v>10</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>162</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="20">
     <mergeCell ref="A2:A31"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="B5:B11"/>
@@ -4084,7 +4086,6 @@
     <mergeCell ref="B28:B29"/>
     <mergeCell ref="B30:B31"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F9:F10"/>
     <mergeCell ref="F18:F19"/>
     <mergeCell ref="F26:F27"/>
     <mergeCell ref="G3:G4"/>

</xml_diff>

<commit_message>
chore: update PA product price list excel file
binary file change for updated price list spreadsheet
</commit_message>
<xml_diff>
--- a/PA替代需求列表.xlsx
+++ b/PA替代需求列表.xlsx
@@ -1,15 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\zt\ggz\研发部\3.7项目\需求分析\PA-替代需求\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowHeight="18390" activeTab="1"/>
+    <workbookView windowHeight="15880" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -33,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="258">
   <si>
     <t>一级需求</t>
   </si>
@@ -622,15 +617,6 @@
   </si>
   <si>
     <t>NAT策略</t>
-  </si>
-  <si>
-    <t>支持NAT后目的区域路由回查匹配（Dest Zone by route lookup）</t>
-  </si>
-  <si>
-    <t>目的区域按NAT后路由查找；源/目的地址用NAT前值</t>
-  </si>
-  <si>
-    <t>PA底层为『先NAT判断后安全策略匹配』的因果倒置：安全策略要求源区域(NAT前)+源地址(NAT前)+目的地址(NAT前)+目的区域(NAT后按路由查找)，极其反直觉；天融信地址转换为独立策略库常规直观映射（安全策略&gt;地址转换，天融信手册《服务器映射》页）；迁移评估项：带目的NAT的策略平移后易因Zone填写错误不通，需制定NAT查表逻辑转换映射规范；对应矩阵#9</t>
   </si>
   <si>
     <t>支持NAT规则主动/主动HA绑定（Active/Active HA Binding）</t>
@@ -1629,7 +1615,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1656,6 +1642,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1892,7 +1884,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6799580" y="6399530"/>
+          <a:off x="6471920" y="6399530"/>
           <a:ext cx="2200275" cy="349885"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1915,7 +1907,7 @@
                   <a:alpha val="19999"/>
                 </a:srgbClr>
               </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204"/>
+              <a:latin typeface="Arial" panose="020B0604020202090204"/>
               <a:ea typeface="宋体" panose="02010600030101010101" pitchFamily="7" charset="-122"/>
             </a:rPr>
             <a:t>AI 生成</a:t>
@@ -1926,7 +1918,7 @@
                 <a:alpha val="19999"/>
               </a:srgbClr>
             </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204"/>
+            <a:latin typeface="Arial" panose="020B0604020202090204"/>
             <a:ea typeface="宋体" panose="02010600030101010101" pitchFamily="7" charset="-122"/>
           </a:endParaRPr>
         </a:p>
@@ -2196,60 +2188,60 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H59"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.2" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="11.7090909090909" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7090909090909" style="1" customWidth="1"/>
-    <col min="3" max="3" width="54.7090909090909" style="1" customWidth="1"/>
-    <col min="4" max="4" width="45.2909090909091" style="1" customWidth="1"/>
-    <col min="5" max="5" width="7.70909090909091" style="1" customWidth="1"/>
-    <col min="6" max="6" width="37.8545454545455" style="1" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="9.70909090909091" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.70909090909091" style="12" customWidth="1"/>
+    <col min="1" max="1" width="11.7115384615385" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7115384615385" style="1" customWidth="1"/>
+    <col min="3" max="3" width="54.7115384615385" style="1" customWidth="1"/>
+    <col min="4" max="4" width="45.2884615384615" style="1" customWidth="1"/>
+    <col min="5" max="5" width="7.71153846153846" style="1" customWidth="1"/>
+    <col min="6" max="6" width="37.8557692307692" style="1" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="9.71153846153846" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.71153846153846" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="15"/>
-      <c r="G1" s="14" t="s">
+      <c r="F1" s="17"/>
+      <c r="G1" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="16" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="19" t="s">
+      <c r="D2" s="20"/>
+      <c r="E2" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H2" s="8" t="s">
@@ -2258,22 +2250,22 @@
     </row>
     <row r="3" ht="36" customHeight="1" spans="1:8">
       <c r="A3" s="6"/>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="F3" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="20" t="s">
         <v>18</v>
       </c>
       <c r="H3" s="8" t="s">
@@ -2283,10 +2275,10 @@
     <row r="4" ht="36" customHeight="1" spans="1:8">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="20" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="6"/>
@@ -2297,10 +2289,10 @@
     <row r="5" ht="36" customHeight="1" spans="1:8">
       <c r="A5" s="6"/>
       <c r="B5" s="7"/>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="20" t="s">
         <v>21</v>
       </c>
       <c r="E5" s="7"/>
@@ -2310,22 +2302,22 @@
     </row>
     <row r="6" ht="14.25" customHeight="1" spans="1:8">
       <c r="A6" s="6"/>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H6" s="8" t="s">
@@ -2335,10 +2327,10 @@
     <row r="7" ht="14.25" customHeight="1" spans="1:8">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="20" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="6"/>
@@ -2349,10 +2341,10 @@
     <row r="8" ht="14.25" customHeight="1" spans="1:8">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="20" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="6"/>
@@ -2363,10 +2355,10 @@
     <row r="9" ht="14.25" customHeight="1" spans="1:8">
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="20" t="s">
         <v>24</v>
       </c>
       <c r="E9" s="6"/>
@@ -2377,10 +2369,10 @@
     <row r="10" ht="14.25" customHeight="1" spans="1:8">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="18"/>
+      <c r="D10" s="20"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
@@ -2389,10 +2381,10 @@
     <row r="11" ht="14.25" customHeight="1" spans="1:8">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="18"/>
+      <c r="D11" s="20"/>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
@@ -2401,10 +2393,10 @@
     <row r="12" ht="14.25" customHeight="1" spans="1:8">
       <c r="A12" s="6"/>
       <c r="B12" s="7"/>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="18"/>
+      <c r="D12" s="20"/>
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
@@ -2412,22 +2404,22 @@
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:8">
       <c r="A13" s="7"/>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="20" t="s">
+      <c r="F13" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="18" t="s">
+      <c r="G13" s="20" t="s">
         <v>35</v>
       </c>
       <c r="H13" s="8" t="s">
@@ -2435,25 +2427,25 @@
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="20" t="s">
         <v>38</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="F14" s="20" t="s">
+      <c r="F14" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="18" t="s">
+      <c r="G14" s="20" t="s">
         <v>42</v>
       </c>
       <c r="H14" s="8" t="s">
@@ -2461,9 +2453,9 @@
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A15" s="25"/>
+      <c r="A15" s="27"/>
       <c r="B15" s="6"/>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="20" t="s">
         <v>43</v>
       </c>
       <c r="D15" s="6"/>
@@ -2473,9 +2465,9 @@
       <c r="H15" s="6"/>
     </row>
     <row r="16" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A16" s="25"/>
+      <c r="A16" s="27"/>
       <c r="B16" s="6"/>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="20" t="s">
         <v>44</v>
       </c>
       <c r="D16" s="6"/>
@@ -2485,9 +2477,9 @@
       <c r="H16" s="6"/>
     </row>
     <row r="17" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A17" s="25"/>
+      <c r="A17" s="27"/>
       <c r="B17" s="6"/>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="20" t="s">
         <v>45</v>
       </c>
       <c r="D17" s="6"/>
@@ -2497,9 +2489,9 @@
       <c r="H17" s="6"/>
     </row>
     <row r="18" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A18" s="25"/>
+      <c r="A18" s="27"/>
       <c r="B18" s="6"/>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="20" t="s">
         <v>46</v>
       </c>
       <c r="D18" s="6"/>
@@ -2509,9 +2501,9 @@
       <c r="H18" s="6"/>
     </row>
     <row r="19" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A19" s="25"/>
+      <c r="A19" s="27"/>
       <c r="B19" s="6"/>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="20" t="s">
         <v>47</v>
       </c>
       <c r="D19" s="6"/>
@@ -2521,9 +2513,9 @@
       <c r="H19" s="6"/>
     </row>
     <row r="20" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A20" s="25"/>
+      <c r="A20" s="27"/>
       <c r="B20" s="6"/>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="20" t="s">
         <v>48</v>
       </c>
       <c r="D20" s="6"/>
@@ -2533,9 +2525,9 @@
       <c r="H20" s="6"/>
     </row>
     <row r="21" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A21" s="25"/>
+      <c r="A21" s="27"/>
       <c r="B21" s="6"/>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="20" t="s">
         <v>49</v>
       </c>
       <c r="D21" s="6"/>
@@ -2545,9 +2537,9 @@
       <c r="H21" s="6"/>
     </row>
     <row r="22" ht="32.25" customHeight="1" spans="1:8">
-      <c r="A22" s="26"/>
+      <c r="A22" s="28"/>
       <c r="B22" s="7"/>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="20" t="s">
         <v>50</v>
       </c>
       <c r="D22" s="7"/>
@@ -2557,25 +2549,25 @@
       <c r="H22" s="7"/>
     </row>
     <row r="23" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A23" s="23" t="s">
+      <c r="A23" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="18" t="s">
+      <c r="D23" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="E23" s="19" t="s">
+      <c r="E23" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="27" t="s">
+      <c r="F23" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="G23" s="18" t="s">
+      <c r="G23" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H23" s="8" t="s">
@@ -2583,25 +2575,25 @@
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A24" s="23" t="s">
+      <c r="A24" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="E24" s="19" t="s">
+      <c r="E24" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="F24" s="28" t="s">
+      <c r="F24" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="G24" s="18" t="s">
+      <c r="G24" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H24" s="8" t="s">
@@ -2609,63 +2601,63 @@
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A25" s="23" t="s">
+      <c r="A25" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="22" t="s">
+      <c r="B25" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="29" t="s">
+      <c r="D25" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="E25" s="19" t="s">
+      <c r="E25" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="F25" s="20" t="s">
+      <c r="F25" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="G25" s="18" t="s">
+      <c r="G25" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H25" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="26" s="11" customFormat="1" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A26" s="25"/>
-      <c r="B26" s="22" t="s">
+    <row r="26" s="13" customFormat="1" ht="28.5" customHeight="1" spans="1:8">
+      <c r="A26" s="27"/>
+      <c r="B26" s="24" t="s">
         <v>66</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="29"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="18"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="20"/>
       <c r="H26" s="8"/>
     </row>
     <row r="27" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A27" s="25"/>
-      <c r="B27" s="22" t="s">
+      <c r="A27" s="27"/>
+      <c r="B27" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="D27" s="18" t="s">
+      <c r="D27" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="E27" s="19" t="s">
+      <c r="E27" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="F27" s="20" t="s">
+      <c r="F27" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="G27" s="18" t="s">
+      <c r="G27" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H27" s="8" t="s">
@@ -2673,9 +2665,9 @@
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A28" s="25"/>
+      <c r="A28" s="27"/>
       <c r="B28" s="7"/>
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="20" t="s">
         <v>71</v>
       </c>
       <c r="D28" s="7"/>
@@ -2685,23 +2677,23 @@
       <c r="H28" s="7"/>
     </row>
     <row r="29" ht="60" customHeight="1" spans="1:8">
-      <c r="A29" s="25"/>
-      <c r="B29" s="22" t="s">
+      <c r="A29" s="27"/>
+      <c r="B29" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="C29" s="18" t="s">
+      <c r="C29" s="20" t="s">
         <v>73</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E29" s="19" t="s">
+      <c r="E29" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="F29" s="31" t="s">
+      <c r="F29" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="G29" s="18" t="s">
+      <c r="G29" s="20" t="s">
         <v>35</v>
       </c>
       <c r="H29" s="8" t="s">
@@ -2709,19 +2701,19 @@
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A30" s="25"/>
+      <c r="A30" s="27"/>
       <c r="B30" s="6"/>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="D30" s="18" t="s">
+      <c r="D30" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="E30" s="19" t="s">
+      <c r="E30" s="21" t="s">
         <v>10</v>
       </c>
       <c r="F30" s="6"/>
-      <c r="G30" s="18" t="s">
+      <c r="G30" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H30" s="8" t="s">
@@ -2729,19 +2721,19 @@
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A31" s="26"/>
+      <c r="A31" s="28"/>
       <c r="B31" s="7"/>
-      <c r="C31" s="18" t="s">
+      <c r="C31" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="D31" s="18" t="s">
+      <c r="D31" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="E31" s="32" t="s">
+      <c r="E31" s="34" t="s">
         <v>10</v>
       </c>
       <c r="F31" s="7"/>
-      <c r="G31" s="18" t="s">
+      <c r="G31" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H31" s="8" t="s">
@@ -2749,25 +2741,25 @@
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A32" s="23" t="s">
+      <c r="A32" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="22" t="s">
+      <c r="B32" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C32" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="D32" s="18" t="s">
+      <c r="D32" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="E32" s="19" t="s">
+      <c r="E32" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="F32" s="20" t="s">
+      <c r="F32" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="G32" s="18" t="s">
+      <c r="G32" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H32" s="8" t="s">
@@ -2775,9 +2767,9 @@
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A33" s="26"/>
+      <c r="A33" s="28"/>
       <c r="B33" s="7"/>
-      <c r="C33" s="18" t="s">
+      <c r="C33" s="20" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="7"/>
@@ -2787,23 +2779,23 @@
       <c r="H33" s="7"/>
     </row>
     <row r="34" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A34" s="23" t="s">
+      <c r="A34" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="B34" s="22" t="s">
+      <c r="B34" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="C34" s="18" t="s">
+      <c r="C34" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="D34" s="18"/>
-      <c r="E34" s="19" t="s">
+      <c r="D34" s="20"/>
+      <c r="E34" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="F34" s="20" t="s">
+      <c r="F34" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="G34" s="18" t="s">
+      <c r="G34" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H34" s="8" t="s">
@@ -2811,59 +2803,59 @@
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A35" s="25"/>
+      <c r="A35" s="27"/>
       <c r="B35" s="6"/>
-      <c r="C35" s="18" t="s">
+      <c r="C35" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="D35" s="18"/>
+      <c r="D35" s="20"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
     </row>
     <row r="36" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A36" s="25"/>
+      <c r="A36" s="27"/>
       <c r="B36" s="6"/>
-      <c r="C36" s="18" t="s">
+      <c r="C36" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="D36" s="18"/>
+      <c r="D36" s="20"/>
       <c r="E36" s="6"/>
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
     </row>
     <row r="37" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A37" s="26"/>
+      <c r="A37" s="28"/>
       <c r="B37" s="7"/>
-      <c r="C37" s="33" t="s">
+      <c r="C37" s="35" t="s">
         <v>90</v>
       </c>
-      <c r="D37" s="33"/>
+      <c r="D37" s="35"/>
       <c r="E37" s="7"/>
       <c r="F37" s="7"/>
       <c r="G37" s="7"/>
       <c r="H37" s="7"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A38" s="22" t="s">
+      <c r="A38" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="B38" s="22" t="s">
+      <c r="B38" s="24" t="s">
         <v>92</v>
       </c>
-      <c r="C38" s="34" t="s">
+      <c r="C38" s="36" t="s">
         <v>93</v>
       </c>
-      <c r="D38" s="34"/>
-      <c r="E38" s="32" t="s">
+      <c r="D38" s="36"/>
+      <c r="E38" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="F38" s="35" t="s">
+      <c r="F38" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="G38" s="18" t="s">
+      <c r="G38" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H38" s="8" t="s">
@@ -2872,14 +2864,14 @@
     </row>
     <row r="39" ht="15.75" customHeight="1" spans="1:8">
       <c r="A39" s="6"/>
-      <c r="B39" s="22" t="s">
+      <c r="B39" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="C39" s="34" t="s">
+      <c r="C39" s="36" t="s">
         <v>95</v>
       </c>
-      <c r="D39" s="34"/>
-      <c r="E39" s="32" t="s">
+      <c r="D39" s="36"/>
+      <c r="E39" s="34" t="s">
         <v>60</v>
       </c>
       <c r="F39" s="7"/>
@@ -2888,22 +2880,22 @@
     </row>
     <row r="40" ht="28.5" customHeight="1" spans="1:8">
       <c r="A40" s="6"/>
-      <c r="B40" s="22" t="s">
+      <c r="B40" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="C40" s="34" t="s">
+      <c r="C40" s="36" t="s">
         <v>97</v>
       </c>
-      <c r="D40" s="36" t="s">
+      <c r="D40" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="E40" s="32" t="s">
+      <c r="E40" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="F40" s="31" t="s">
+      <c r="F40" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="G40" s="18" t="s">
+      <c r="G40" s="20" t="s">
         <v>35</v>
       </c>
       <c r="H40" s="8" t="s">
@@ -2912,22 +2904,22 @@
     </row>
     <row r="41" ht="15.75" customHeight="1" spans="1:8">
       <c r="A41" s="6"/>
-      <c r="B41" s="22" t="s">
+      <c r="B41" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="C41" s="18" t="s">
+      <c r="C41" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="D41" s="34" t="s">
+      <c r="D41" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="E41" s="32" t="s">
+      <c r="E41" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="F41" s="31" t="s">
+      <c r="F41" s="33" t="s">
         <v>102</v>
       </c>
-      <c r="G41" s="18" t="s">
+      <c r="G41" s="20" t="s">
         <v>103</v>
       </c>
       <c r="H41" s="8" t="s">
@@ -2936,34 +2928,34 @@
     </row>
     <row r="42" ht="15.75" customHeight="1" spans="1:8">
       <c r="A42" s="6"/>
-      <c r="B42" s="22" t="s">
+      <c r="B42" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="C42" s="18" t="s">
+      <c r="C42" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="D42" s="34"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="31"/>
-      <c r="G42" s="18"/>
+      <c r="D42" s="36"/>
+      <c r="E42" s="34"/>
+      <c r="F42" s="33"/>
+      <c r="G42" s="20"/>
       <c r="H42" s="8"/>
     </row>
     <row r="43" ht="15.75" customHeight="1" spans="1:8">
       <c r="A43" s="7"/>
-      <c r="B43" s="22" t="s">
+      <c r="B43" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="C43" s="34" t="s">
+      <c r="C43" s="36" t="s">
         <v>107</v>
       </c>
-      <c r="D43" s="34"/>
-      <c r="E43" s="32" t="s">
+      <c r="D43" s="36"/>
+      <c r="E43" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="F43" s="31" t="s">
+      <c r="F43" s="33" t="s">
         <v>108</v>
       </c>
-      <c r="G43" s="18" t="s">
+      <c r="G43" s="20" t="s">
         <v>109</v>
       </c>
       <c r="H43" s="8" t="s">
@@ -2971,25 +2963,25 @@
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A44" s="37" t="s">
+      <c r="A44" s="39" t="s">
         <v>110</v>
       </c>
-      <c r="B44" s="38" t="s">
+      <c r="B44" s="40" t="s">
         <v>111</v>
       </c>
-      <c r="C44" s="39" t="s">
+      <c r="C44" s="41" t="s">
         <v>112</v>
       </c>
-      <c r="D44" s="39" t="s">
+      <c r="D44" s="41" t="s">
         <v>113</v>
       </c>
-      <c r="E44" s="40" t="s">
+      <c r="E44" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="F44" s="41" t="s">
+      <c r="F44" s="43" t="s">
         <v>114</v>
       </c>
-      <c r="G44" s="42" t="s">
+      <c r="G44" s="44" t="s">
         <v>35</v>
       </c>
       <c r="H44" s="9" t="s">
@@ -2997,19 +2989,19 @@
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A45" s="25"/>
+      <c r="A45" s="27"/>
       <c r="B45" s="6"/>
-      <c r="C45" s="34" t="s">
+      <c r="C45" s="36" t="s">
         <v>115</v>
       </c>
-      <c r="D45" s="34" t="s">
+      <c r="D45" s="36" t="s">
         <v>116</v>
       </c>
       <c r="E45" s="6"/>
-      <c r="F45" s="43" t="s">
+      <c r="F45" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="G45" s="18" t="s">
+      <c r="G45" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H45" s="8" t="s">
@@ -3017,29 +3009,29 @@
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A46" s="25"/>
+      <c r="A46" s="27"/>
       <c r="B46" s="6"/>
-      <c r="C46" s="34" t="s">
+      <c r="C46" s="36" t="s">
         <v>117</v>
       </c>
-      <c r="D46" s="34"/>
+      <c r="D46" s="36"/>
       <c r="E46" s="6"/>
       <c r="F46" s="7"/>
       <c r="G46" s="7"/>
       <c r="H46" s="7"/>
     </row>
     <row r="47" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A47" s="25"/>
+      <c r="A47" s="27"/>
       <c r="B47" s="6"/>
-      <c r="C47" s="34" t="s">
+      <c r="C47" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="D47" s="34"/>
+      <c r="D47" s="36"/>
       <c r="E47" s="6"/>
-      <c r="F47" s="43" t="s">
+      <c r="F47" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="G47" s="18" t="s">
+      <c r="G47" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H47" s="8" t="s">
@@ -3047,121 +3039,121 @@
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A48" s="26"/>
+      <c r="A48" s="28"/>
       <c r="B48" s="7"/>
-      <c r="C48" s="44" t="s">
+      <c r="C48" s="46" t="s">
         <v>119</v>
       </c>
-      <c r="D48" s="44"/>
+      <c r="D48" s="46"/>
       <c r="E48" s="7"/>
-      <c r="F48" s="27" t="s">
+      <c r="F48" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="G48" s="33" t="s">
+      <c r="G48" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="H48" s="45" t="s">
+      <c r="H48" s="47" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="49" ht="42.75" customHeight="1" spans="1:8">
-      <c r="A49" s="46" t="s">
+      <c r="A49" s="48" t="s">
         <v>120</v>
       </c>
-      <c r="B49" s="46" t="s">
+      <c r="B49" s="48" t="s">
         <v>120</v>
       </c>
-      <c r="C49" s="47" t="s">
+      <c r="C49" s="49" t="s">
         <v>121</v>
       </c>
-      <c r="D49" s="48" t="s">
+      <c r="D49" s="50" t="s">
         <v>122</v>
       </c>
-      <c r="E49" s="49" t="s">
+      <c r="E49" s="51" t="s">
         <v>40</v>
       </c>
-      <c r="F49" s="50"/>
-      <c r="G49" s="51" t="s">
+      <c r="F49" s="52"/>
+      <c r="G49" s="53" t="s">
         <v>103</v>
       </c>
-      <c r="H49" s="52"/>
+      <c r="H49" s="54"/>
     </row>
     <row r="50" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A50" s="53"/>
-      <c r="B50" s="53"/>
-      <c r="C50" s="47" t="s">
+      <c r="A50" s="55"/>
+      <c r="B50" s="55"/>
+      <c r="C50" s="49" t="s">
         <v>123</v>
       </c>
-      <c r="D50" s="54" t="s">
+      <c r="D50" s="56" t="s">
         <v>124</v>
       </c>
-      <c r="E50" s="55" t="s">
+      <c r="E50" s="57" t="s">
         <v>60</v>
       </c>
-      <c r="F50" s="56"/>
-      <c r="G50" s="51" t="s">
+      <c r="F50" s="58"/>
+      <c r="G50" s="53" t="s">
         <v>103</v>
       </c>
-      <c r="H50" s="57"/>
+      <c r="H50" s="59"/>
     </row>
     <row r="51" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A51" s="53"/>
-      <c r="B51" s="53"/>
-      <c r="C51" s="47" t="s">
+      <c r="A51" s="55"/>
+      <c r="B51" s="55"/>
+      <c r="C51" s="49" t="s">
         <v>125</v>
       </c>
-      <c r="D51" s="58" t="s">
+      <c r="D51" s="60" t="s">
         <v>126</v>
       </c>
-      <c r="E51" s="55" t="s">
+      <c r="E51" s="57" t="s">
         <v>60</v>
       </c>
-      <c r="F51" s="50"/>
-      <c r="G51" s="51" t="s">
+      <c r="F51" s="52"/>
+      <c r="G51" s="53" t="s">
         <v>103</v>
       </c>
-      <c r="H51" s="52"/>
+      <c r="H51" s="54"/>
     </row>
     <row r="52" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A52" s="59"/>
-      <c r="B52" s="59"/>
-      <c r="C52" s="58" t="s">
+      <c r="A52" s="61"/>
+      <c r="B52" s="61"/>
+      <c r="C52" s="60" t="s">
         <v>127</v>
       </c>
-      <c r="D52" s="48" t="s">
+      <c r="D52" s="50" t="s">
         <v>128</v>
       </c>
-      <c r="E52" s="60" t="s">
+      <c r="E52" s="62" t="s">
         <v>10</v>
       </c>
-      <c r="F52" s="50" t="s">
+      <c r="F52" s="52" t="s">
         <v>129</v>
       </c>
-      <c r="G52" s="51" t="s">
+      <c r="G52" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="H52" s="52" t="s">
+      <c r="H52" s="54" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A53" s="38" t="s">
+      <c r="A53" s="40" t="s">
         <v>130</v>
       </c>
-      <c r="B53" s="38" t="s">
+      <c r="B53" s="40" t="s">
         <v>131</v>
       </c>
-      <c r="C53" s="39" t="s">
+      <c r="C53" s="41" t="s">
         <v>132</v>
       </c>
-      <c r="D53" s="39"/>
-      <c r="E53" s="40" t="s">
+      <c r="D53" s="41"/>
+      <c r="E53" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="F53" s="41" t="s">
+      <c r="F53" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="G53" s="42" t="s">
+      <c r="G53" s="44" t="s">
         <v>12</v>
       </c>
       <c r="H53" s="9" t="s">
@@ -3170,22 +3162,22 @@
     </row>
     <row r="54" ht="28.5" customHeight="1" spans="1:8">
       <c r="A54" s="7"/>
-      <c r="B54" s="22" t="s">
+      <c r="B54" s="24" t="s">
         <v>133</v>
       </c>
       <c r="C54" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="D54" s="36" t="s">
+      <c r="D54" s="38" t="s">
         <v>135</v>
       </c>
-      <c r="E54" s="32" t="s">
+      <c r="E54" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="F54" s="31" t="s">
+      <c r="F54" s="33" t="s">
         <v>136</v>
       </c>
-      <c r="G54" s="18" t="s">
+      <c r="G54" s="20" t="s">
         <v>103</v>
       </c>
       <c r="H54" s="8" t="s">
@@ -3193,21 +3185,21 @@
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A55" s="23" t="s">
+      <c r="A55" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="B55" s="22" t="s">
+      <c r="B55" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="C55" s="34" t="s">
+      <c r="C55" s="36" t="s">
         <v>139</v>
       </c>
-      <c r="D55" s="34"/>
-      <c r="E55" s="32" t="s">
+      <c r="D55" s="36"/>
+      <c r="E55" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="F55" s="31"/>
-      <c r="G55" s="18" t="s">
+      <c r="F55" s="33"/>
+      <c r="G55" s="20" t="s">
         <v>140</v>
       </c>
       <c r="H55" s="8" t="s">
@@ -3215,49 +3207,49 @@
       </c>
     </row>
     <row r="56" ht="42.75" customHeight="1" spans="1:8">
-      <c r="A56" s="23" t="s">
+      <c r="A56" s="25" t="s">
         <v>141</v>
       </c>
-      <c r="B56" s="22" t="s">
+      <c r="B56" s="24" t="s">
         <v>142</v>
       </c>
-      <c r="C56" s="34" t="s">
+      <c r="C56" s="36" t="s">
         <v>143</v>
       </c>
-      <c r="D56" s="36" t="s">
+      <c r="D56" s="38" t="s">
         <v>144</v>
       </c>
-      <c r="E56" s="32" t="s">
+      <c r="E56" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="F56" s="43" t="s">
+      <c r="F56" s="45" t="s">
         <v>145</v>
       </c>
-      <c r="G56" s="18"/>
+      <c r="G56" s="20"/>
       <c r="H56" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="57" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A57" s="22" t="s">
+      <c r="A57" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="B57" s="22" t="s">
+      <c r="B57" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="C57" s="34" t="s">
+      <c r="C57" s="36" t="s">
         <v>147</v>
       </c>
-      <c r="D57" s="34" t="s">
+      <c r="D57" s="36" t="s">
         <v>148</v>
       </c>
-      <c r="E57" s="32" t="s">
+      <c r="E57" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="F57" s="43" t="s">
+      <c r="F57" s="45" t="s">
         <v>149</v>
       </c>
-      <c r="G57" s="18" t="s">
+      <c r="G57" s="20" t="s">
         <v>103</v>
       </c>
       <c r="H57" s="8" t="s">
@@ -3265,50 +3257,50 @@
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A58" s="61" t="s">
+      <c r="A58" s="63" t="s">
         <v>150</v>
       </c>
-      <c r="B58" s="61" t="s">
+      <c r="B58" s="63" t="s">
         <v>150</v>
       </c>
-      <c r="C58" s="33" t="s">
+      <c r="C58" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="D58" s="44" t="s">
+      <c r="D58" s="46" t="s">
         <v>152</v>
       </c>
-      <c r="E58" s="62" t="s">
+      <c r="E58" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="F58" s="63" t="s">
+      <c r="F58" s="65" t="s">
         <v>153</v>
       </c>
-      <c r="G58" s="33" t="s">
+      <c r="G58" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="H58" s="45" t="s">
+      <c r="H58" s="47" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="59" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A59" s="46" t="s">
+      <c r="A59" s="48" t="s">
         <v>154</v>
       </c>
-      <c r="B59" s="46" t="s">
+      <c r="B59" s="48" t="s">
         <v>154</v>
       </c>
-      <c r="C59" s="64" t="s">
+      <c r="C59" s="66" t="s">
         <v>155</v>
       </c>
-      <c r="D59" s="56"/>
-      <c r="E59" s="60" t="s">
+      <c r="D59" s="58"/>
+      <c r="E59" s="62" t="s">
         <v>10</v>
       </c>
-      <c r="F59" s="56"/>
-      <c r="G59" s="33" t="s">
+      <c r="F59" s="58"/>
+      <c r="G59" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="H59" s="57" t="s">
+      <c r="H59" s="59" t="s">
         <v>13</v>
       </c>
     </row>
@@ -3379,16 +3371,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H31"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.2" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="11.7" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7019230769231" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7019230769231" style="1" customWidth="1"/>
     <col min="3" max="3" width="40" style="1" customWidth="1"/>
-    <col min="4" max="4" width="41.4545454545455" style="1" customWidth="1"/>
+    <col min="4" max="4" width="41.4519230769231" style="1" customWidth="1"/>
     <col min="5" max="5" width="62" style="1" customWidth="1"/>
-    <col min="6" max="6" width="7.7" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.70192307692308" style="1" customWidth="1"/>
     <col min="7" max="7" width="10" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.7" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.70192307692308" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:8">
@@ -3625,9 +3617,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" ht="126" customHeight="1" spans="1:8">
+    <row r="12" ht="81" customHeight="1" spans="1:8">
       <c r="A12" s="6"/>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="11" t="s">
         <v>191</v>
       </c>
       <c r="C12" s="5" t="s">
@@ -3640,10 +3632,10 @@
         <v>194</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>162</v>
@@ -3651,39 +3643,29 @@
     </row>
     <row r="13" ht="81" customHeight="1" spans="1:8">
       <c r="A13" s="6"/>
-      <c r="B13" s="7"/>
+      <c r="B13" s="12"/>
       <c r="C13" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>162</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
     </row>
     <row r="14" ht="96" customHeight="1" spans="1:8">
       <c r="A14" s="6"/>
       <c r="B14" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>198</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>201</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>60</v>
@@ -3698,16 +3680,16 @@
     <row r="15" ht="111" customHeight="1" spans="1:8">
       <c r="A15" s="6"/>
       <c r="B15" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>202</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>205</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>40</v>
@@ -3722,16 +3704,16 @@
     <row r="16" ht="51" customHeight="1" spans="1:8">
       <c r="A16" s="6"/>
       <c r="B16" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="E16" s="5" t="s">
         <v>206</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>209</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>10</v>
@@ -3747,13 +3729,13 @@
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="5" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>40</v>
@@ -3769,13 +3751,13 @@
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="5" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>10</v>
@@ -3789,13 +3771,13 @@
       <c r="A19" s="6"/>
       <c r="B19" s="7"/>
       <c r="C19" s="5" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
@@ -3804,16 +3786,16 @@
     <row r="20" ht="111" customHeight="1" spans="1:8">
       <c r="A20" s="6"/>
       <c r="B20" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="E20" s="5" t="s">
         <v>219</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>222</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>40</v>
@@ -3829,13 +3811,13 @@
       <c r="A21" s="6"/>
       <c r="B21" s="7"/>
       <c r="C21" s="5" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>10</v>
@@ -3850,16 +3832,16 @@
     <row r="22" ht="96" customHeight="1" spans="1:8">
       <c r="A22" s="6"/>
       <c r="B22" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>226</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>229</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>40</v>
@@ -3875,13 +3857,13 @@
       <c r="A23" s="6"/>
       <c r="B23" s="7"/>
       <c r="C23" s="5" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>10</v>
@@ -3896,16 +3878,16 @@
     <row r="24" ht="96" customHeight="1" spans="1:8">
       <c r="A24" s="6"/>
       <c r="B24" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="E24" s="5" t="s">
         <v>233</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>235</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>236</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>40</v>
@@ -3920,16 +3902,16 @@
     <row r="25" ht="81" customHeight="1" spans="1:8">
       <c r="A25" s="6"/>
       <c r="B25" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E25" s="5" t="s">
         <v>237</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>240</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>10</v>
@@ -3945,13 +3927,13 @@
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="C26" s="5" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>10</v>
@@ -3967,13 +3949,13 @@
       <c r="A27" s="6"/>
       <c r="B27" s="7"/>
       <c r="C27" s="5" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="F27" s="7"/>
       <c r="G27" s="4" t="s">
@@ -3984,16 +3966,16 @@
     <row r="28" ht="171" customHeight="1" spans="1:8">
       <c r="A28" s="6"/>
       <c r="B28" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="E28" s="5" t="s">
         <v>247</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>249</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>250</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>10</v>
@@ -4009,13 +3991,13 @@
       <c r="A29" s="6"/>
       <c r="B29" s="7"/>
       <c r="C29" s="5" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>10</v>
@@ -4030,16 +4012,16 @@
     <row r="30" ht="81" customHeight="1" spans="1:8">
       <c r="A30" s="6"/>
       <c r="B30" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="E30" s="5" t="s">
         <v>254</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>257</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>40</v>
@@ -4055,13 +4037,13 @@
       <c r="A31" s="7"/>
       <c r="B31" s="7"/>
       <c r="C31" s="5" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>10</v>
@@ -4074,11 +4056,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="19">
     <mergeCell ref="A2:A31"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="B5:B11"/>
-    <mergeCell ref="B12:B13"/>
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="B22:B23"/>

</xml_diff>

<commit_message>
docs: update PA project progress excel file
binary file changes for the PA progress tracking spreadsheet
</commit_message>
<xml_diff>
--- a/PA替代需求列表.xlsx
+++ b/PA替代需求列表.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
-    <sheet name="策略需求差异" sheetId="3" r:id="rId2"/>
+    <sheet name="策略需求差异" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="259">
   <si>
     <t>一级需求</t>
   </si>
@@ -619,13 +619,16 @@
     <t>NAT策略</t>
   </si>
   <si>
-    <t>支持NAT规则主动/主动HA绑定（Active/Active HA Binding）</t>
-  </si>
-  <si>
-    <t>主动/主动HA下NAT规则绑定会话所有者</t>
-  </si>
-  <si>
-    <t>PA主动/主动HA配置下NAT规则可绑定会话所有者/会话设置，控制NAT会话的设备绑定，仅A/A模式可见（PA Web帮助p150）；天融信HA为主备双机热备模式（天融信手册《配置双机热备功能》页），无主动/主动模式及NAT规则绑定机制</t>
+    <t>支持双活HA下的NAT规则会话绑定</t>
+  </si>
+  <si>
+    <t>双活HA模式下，NAT规则可绑定会话所有者并指定会话设置，控制NAT会话归属设备</t>
+  </si>
+  <si>
+    <t>PA双活（Active/Active）HA配置下NAT规则可绑定会话所有者/会话设置，控制NAT会话的设备绑定，仅A/A模式可见（PA Web帮助p150）；天融信HA为主备双机热备模式（天融信手册《配置双机热备功能》页），无双活模式及NAT规则绑定机制</t>
+  </si>
+  <si>
+    <t>平台</t>
   </si>
   <si>
     <t>QoS策略</t>
@@ -1615,7 +1618,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1643,10 +1646,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1867,13 +1867,13 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>784010</xdr:colOff>
+      <xdr:colOff>1111670</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>18250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>2984010</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>320820</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>187275</xdr:rowOff>
     </xdr:to>
@@ -1884,7 +1884,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6471920" y="6399530"/>
+          <a:off x="6799580" y="6399530"/>
           <a:ext cx="2200275" cy="349885"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1908,7 +1908,7 @@
                 </a:srgbClr>
               </a:solidFill>
               <a:latin typeface="Arial" panose="020B0604020202090204"/>
-              <a:ea typeface="宋体" panose="02010600030101010101" pitchFamily="7" charset="-122"/>
+              <a:ea typeface="宋体"/>
             </a:rPr>
             <a:t>AI 生成</a:t>
           </a:r>
@@ -1919,7 +1919,74 @@
               </a:srgbClr>
             </a:solidFill>
             <a:latin typeface="Arial" panose="020B0604020202090204"/>
-            <a:ea typeface="宋体" panose="02010600030101010101" pitchFamily="7" charset="-122"/>
+            <a:ea typeface="宋体"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2084490</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>469100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1547005</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>819100</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Watermark"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6799580" y="6399530"/>
+          <a:ext cx="2200275" cy="349885"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="b"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="r"/>
+          <a:r>
+            <a:rPr lang="zh-CN" sz="1600" dirty="0">
+              <a:solidFill>
+                <a:srgbClr val="808080">
+                  <a:alpha val="19999"/>
+                </a:srgbClr>
+              </a:solidFill>
+              <a:latin typeface="Arial" panose="020B0604020202090204"/>
+              <a:ea typeface="宋体"/>
+            </a:rPr>
+            <a:t>AI 生成</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" sz="1600" dirty="0">
+            <a:solidFill>
+              <a:srgbClr val="808080">
+                <a:alpha val="19999"/>
+              </a:srgbClr>
+            </a:solidFill>
+            <a:latin typeface="Arial" panose="020B0604020202090204"/>
+            <a:ea typeface="宋体"/>
           </a:endParaRPr>
         </a:p>
       </xdr:txBody>
@@ -2197,51 +2264,51 @@
     <col min="5" max="5" width="7.71153846153846" style="1" customWidth="1"/>
     <col min="6" max="6" width="37.8557692307692" style="1" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="9.71153846153846" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.71153846153846" style="14" customWidth="1"/>
+    <col min="8" max="8" width="9.71153846153846" style="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="17"/>
-      <c r="G1" s="16" t="s">
+      <c r="F1" s="16"/>
+      <c r="G1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="H1" s="15" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="C2" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="20"/>
-      <c r="E2" s="21" t="s">
+      <c r="D2" s="19"/>
+      <c r="E2" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="G2" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H2" s="8" t="s">
@@ -2250,22 +2317,22 @@
     </row>
     <row r="3" ht="36" customHeight="1" spans="1:8">
       <c r="A3" s="6"/>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="E3" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="19" t="s">
         <v>18</v>
       </c>
       <c r="H3" s="8" t="s">
@@ -2275,10 +2342,10 @@
     <row r="4" ht="36" customHeight="1" spans="1:8">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="19" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="6"/>
@@ -2289,10 +2356,10 @@
     <row r="5" ht="36" customHeight="1" spans="1:8">
       <c r="A5" s="6"/>
       <c r="B5" s="7"/>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="19" t="s">
         <v>21</v>
       </c>
       <c r="E5" s="7"/>
@@ -2302,22 +2369,22 @@
     </row>
     <row r="6" ht="14.25" customHeight="1" spans="1:8">
       <c r="A6" s="6"/>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H6" s="8" t="s">
@@ -2327,10 +2394,10 @@
     <row r="7" ht="14.25" customHeight="1" spans="1:8">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="19" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="6"/>
@@ -2341,10 +2408,10 @@
     <row r="8" ht="14.25" customHeight="1" spans="1:8">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="19" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="6"/>
@@ -2355,10 +2422,10 @@
     <row r="9" ht="14.25" customHeight="1" spans="1:8">
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="19" t="s">
         <v>24</v>
       </c>
       <c r="E9" s="6"/>
@@ -2369,10 +2436,10 @@
     <row r="10" ht="14.25" customHeight="1" spans="1:8">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="20"/>
+      <c r="D10" s="19"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
@@ -2381,10 +2448,10 @@
     <row r="11" ht="14.25" customHeight="1" spans="1:8">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="20"/>
+      <c r="D11" s="19"/>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
@@ -2393,10 +2460,10 @@
     <row r="12" ht="14.25" customHeight="1" spans="1:8">
       <c r="A12" s="6"/>
       <c r="B12" s="7"/>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="20"/>
+      <c r="D12" s="19"/>
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
@@ -2404,22 +2471,22 @@
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:8">
       <c r="A13" s="7"/>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="21" t="s">
+      <c r="E13" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="22" t="s">
+      <c r="F13" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="G13" s="19" t="s">
         <v>35</v>
       </c>
       <c r="H13" s="8" t="s">
@@ -2427,25 +2494,25 @@
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A14" s="25" t="s">
+      <c r="A14" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="19" t="s">
         <v>38</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="E14" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="F14" s="22" t="s">
+      <c r="F14" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="20" t="s">
+      <c r="G14" s="19" t="s">
         <v>42</v>
       </c>
       <c r="H14" s="8" t="s">
@@ -2453,9 +2520,9 @@
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A15" s="27"/>
+      <c r="A15" s="26"/>
       <c r="B15" s="6"/>
-      <c r="C15" s="20" t="s">
+      <c r="C15" s="19" t="s">
         <v>43</v>
       </c>
       <c r="D15" s="6"/>
@@ -2465,9 +2532,9 @@
       <c r="H15" s="6"/>
     </row>
     <row r="16" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A16" s="27"/>
+      <c r="A16" s="26"/>
       <c r="B16" s="6"/>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="19" t="s">
         <v>44</v>
       </c>
       <c r="D16" s="6"/>
@@ -2477,9 +2544,9 @@
       <c r="H16" s="6"/>
     </row>
     <row r="17" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A17" s="27"/>
+      <c r="A17" s="26"/>
       <c r="B17" s="6"/>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="19" t="s">
         <v>45</v>
       </c>
       <c r="D17" s="6"/>
@@ -2489,9 +2556,9 @@
       <c r="H17" s="6"/>
     </row>
     <row r="18" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A18" s="27"/>
+      <c r="A18" s="26"/>
       <c r="B18" s="6"/>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="19" t="s">
         <v>46</v>
       </c>
       <c r="D18" s="6"/>
@@ -2501,9 +2568,9 @@
       <c r="H18" s="6"/>
     </row>
     <row r="19" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A19" s="27"/>
+      <c r="A19" s="26"/>
       <c r="B19" s="6"/>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="19" t="s">
         <v>47</v>
       </c>
       <c r="D19" s="6"/>
@@ -2513,9 +2580,9 @@
       <c r="H19" s="6"/>
     </row>
     <row r="20" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A20" s="27"/>
+      <c r="A20" s="26"/>
       <c r="B20" s="6"/>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="19" t="s">
         <v>48</v>
       </c>
       <c r="D20" s="6"/>
@@ -2525,9 +2592,9 @@
       <c r="H20" s="6"/>
     </row>
     <row r="21" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A21" s="27"/>
+      <c r="A21" s="26"/>
       <c r="B21" s="6"/>
-      <c r="C21" s="20" t="s">
+      <c r="C21" s="19" t="s">
         <v>49</v>
       </c>
       <c r="D21" s="6"/>
@@ -2537,9 +2604,9 @@
       <c r="H21" s="6"/>
     </row>
     <row r="22" ht="32.25" customHeight="1" spans="1:8">
-      <c r="A22" s="28"/>
+      <c r="A22" s="27"/>
       <c r="B22" s="7"/>
-      <c r="C22" s="20" t="s">
+      <c r="C22" s="19" t="s">
         <v>50</v>
       </c>
       <c r="D22" s="7"/>
@@ -2549,25 +2616,25 @@
       <c r="H22" s="7"/>
     </row>
     <row r="23" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="24" t="s">
+      <c r="B23" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="20" t="s">
+      <c r="C23" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="20" t="s">
+      <c r="D23" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E23" s="21" t="s">
+      <c r="E23" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="29" t="s">
+      <c r="F23" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="G23" s="20" t="s">
+      <c r="G23" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H23" s="8" t="s">
@@ -2575,25 +2642,25 @@
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A24" s="25" t="s">
+      <c r="A24" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="20" t="s">
+      <c r="C24" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="20" t="s">
+      <c r="D24" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="E24" s="21" t="s">
+      <c r="E24" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="F24" s="30" t="s">
+      <c r="F24" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="G24" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H24" s="8" t="s">
@@ -2601,63 +2668,63 @@
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A25" s="25" t="s">
+      <c r="A25" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="20" t="s">
+      <c r="C25" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="31" t="s">
+      <c r="D25" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="E25" s="21" t="s">
+      <c r="E25" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="F25" s="22" t="s">
+      <c r="F25" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="G25" s="20" t="s">
+      <c r="G25" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H25" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="26" s="13" customFormat="1" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A26" s="27"/>
-      <c r="B26" s="24" t="s">
+    <row r="26" s="12" customFormat="1" ht="28.5" customHeight="1" spans="1:8">
+      <c r="A26" s="26"/>
+      <c r="B26" s="23" t="s">
         <v>66</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="31"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="20"/>
+      <c r="D26" s="30"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="19"/>
       <c r="H26" s="8"/>
     </row>
     <row r="27" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A27" s="27"/>
-      <c r="B27" s="24" t="s">
+      <c r="A27" s="26"/>
+      <c r="B27" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="20" t="s">
+      <c r="C27" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="D27" s="20" t="s">
+      <c r="D27" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="E27" s="21" t="s">
+      <c r="E27" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="F27" s="22" t="s">
+      <c r="F27" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="G27" s="20" t="s">
+      <c r="G27" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H27" s="8" t="s">
@@ -2665,9 +2732,9 @@
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A28" s="27"/>
+      <c r="A28" s="26"/>
       <c r="B28" s="7"/>
-      <c r="C28" s="20" t="s">
+      <c r="C28" s="19" t="s">
         <v>71</v>
       </c>
       <c r="D28" s="7"/>
@@ -2677,23 +2744,23 @@
       <c r="H28" s="7"/>
     </row>
     <row r="29" ht="60" customHeight="1" spans="1:8">
-      <c r="A29" s="27"/>
-      <c r="B29" s="24" t="s">
+      <c r="A29" s="26"/>
+      <c r="B29" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="C29" s="19" t="s">
         <v>73</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E29" s="21" t="s">
+      <c r="E29" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="F29" s="33" t="s">
+      <c r="F29" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="G29" s="20" t="s">
+      <c r="G29" s="19" t="s">
         <v>35</v>
       </c>
       <c r="H29" s="8" t="s">
@@ -2701,19 +2768,19 @@
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A30" s="27"/>
+      <c r="A30" s="26"/>
       <c r="B30" s="6"/>
-      <c r="C30" s="20" t="s">
+      <c r="C30" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="D30" s="20" t="s">
+      <c r="D30" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="E30" s="21" t="s">
+      <c r="E30" s="20" t="s">
         <v>10</v>
       </c>
       <c r="F30" s="6"/>
-      <c r="G30" s="20" t="s">
+      <c r="G30" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H30" s="8" t="s">
@@ -2721,19 +2788,19 @@
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A31" s="28"/>
+      <c r="A31" s="27"/>
       <c r="B31" s="7"/>
-      <c r="C31" s="20" t="s">
+      <c r="C31" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="D31" s="20" t="s">
+      <c r="D31" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="E31" s="34" t="s">
+      <c r="E31" s="33" t="s">
         <v>10</v>
       </c>
       <c r="F31" s="7"/>
-      <c r="G31" s="20" t="s">
+      <c r="G31" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H31" s="8" t="s">
@@ -2741,25 +2808,25 @@
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A32" s="25" t="s">
+      <c r="A32" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="24" t="s">
+      <c r="B32" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="C32" s="20" t="s">
+      <c r="C32" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="D32" s="20" t="s">
+      <c r="D32" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="E32" s="21" t="s">
+      <c r="E32" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="F32" s="22" t="s">
+      <c r="F32" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="G32" s="20" t="s">
+      <c r="G32" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H32" s="8" t="s">
@@ -2767,9 +2834,9 @@
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A33" s="28"/>
+      <c r="A33" s="27"/>
       <c r="B33" s="7"/>
-      <c r="C33" s="20" t="s">
+      <c r="C33" s="19" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="7"/>
@@ -2779,23 +2846,23 @@
       <c r="H33" s="7"/>
     </row>
     <row r="34" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A34" s="25" t="s">
+      <c r="A34" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="B34" s="24" t="s">
+      <c r="B34" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="C34" s="20" t="s">
+      <c r="C34" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="D34" s="20"/>
-      <c r="E34" s="21" t="s">
+      <c r="D34" s="19"/>
+      <c r="E34" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="F34" s="22" t="s">
+      <c r="F34" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="G34" s="20" t="s">
+      <c r="G34" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H34" s="8" t="s">
@@ -2803,59 +2870,59 @@
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A35" s="27"/>
+      <c r="A35" s="26"/>
       <c r="B35" s="6"/>
-      <c r="C35" s="20" t="s">
+      <c r="C35" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="D35" s="20"/>
+      <c r="D35" s="19"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
     </row>
     <row r="36" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A36" s="27"/>
+      <c r="A36" s="26"/>
       <c r="B36" s="6"/>
-      <c r="C36" s="20" t="s">
+      <c r="C36" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="D36" s="20"/>
+      <c r="D36" s="19"/>
       <c r="E36" s="6"/>
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
     </row>
     <row r="37" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A37" s="28"/>
+      <c r="A37" s="27"/>
       <c r="B37" s="7"/>
-      <c r="C37" s="35" t="s">
+      <c r="C37" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="D37" s="35"/>
+      <c r="D37" s="34"/>
       <c r="E37" s="7"/>
       <c r="F37" s="7"/>
       <c r="G37" s="7"/>
       <c r="H37" s="7"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A38" s="24" t="s">
+      <c r="A38" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B38" s="24" t="s">
+      <c r="B38" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="C38" s="36" t="s">
+      <c r="C38" s="35" t="s">
         <v>93</v>
       </c>
-      <c r="D38" s="36"/>
-      <c r="E38" s="34" t="s">
+      <c r="D38" s="35"/>
+      <c r="E38" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="F38" s="37" t="s">
+      <c r="F38" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="G38" s="20" t="s">
+      <c r="G38" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H38" s="8" t="s">
@@ -2864,14 +2931,14 @@
     </row>
     <row r="39" ht="15.75" customHeight="1" spans="1:8">
       <c r="A39" s="6"/>
-      <c r="B39" s="24" t="s">
+      <c r="B39" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="C39" s="36" t="s">
+      <c r="C39" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="D39" s="36"/>
-      <c r="E39" s="34" t="s">
+      <c r="D39" s="35"/>
+      <c r="E39" s="33" t="s">
         <v>60</v>
       </c>
       <c r="F39" s="7"/>
@@ -2880,22 +2947,22 @@
     </row>
     <row r="40" ht="28.5" customHeight="1" spans="1:8">
       <c r="A40" s="6"/>
-      <c r="B40" s="24" t="s">
+      <c r="B40" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="C40" s="36" t="s">
+      <c r="C40" s="35" t="s">
         <v>97</v>
       </c>
-      <c r="D40" s="38" t="s">
+      <c r="D40" s="37" t="s">
         <v>98</v>
       </c>
-      <c r="E40" s="34" t="s">
+      <c r="E40" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="F40" s="33" t="s">
+      <c r="F40" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="G40" s="20" t="s">
+      <c r="G40" s="19" t="s">
         <v>35</v>
       </c>
       <c r="H40" s="8" t="s">
@@ -2904,22 +2971,22 @@
     </row>
     <row r="41" ht="15.75" customHeight="1" spans="1:8">
       <c r="A41" s="6"/>
-      <c r="B41" s="24" t="s">
+      <c r="B41" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="C41" s="20" t="s">
+      <c r="C41" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="D41" s="36" t="s">
+      <c r="D41" s="35" t="s">
         <v>101</v>
       </c>
-      <c r="E41" s="34" t="s">
+      <c r="E41" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="F41" s="33" t="s">
+      <c r="F41" s="32" t="s">
         <v>102</v>
       </c>
-      <c r="G41" s="20" t="s">
+      <c r="G41" s="19" t="s">
         <v>103</v>
       </c>
       <c r="H41" s="8" t="s">
@@ -2928,34 +2995,34 @@
     </row>
     <row r="42" ht="15.75" customHeight="1" spans="1:8">
       <c r="A42" s="6"/>
-      <c r="B42" s="24" t="s">
+      <c r="B42" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="C42" s="20" t="s">
+      <c r="C42" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="D42" s="36"/>
-      <c r="E42" s="34"/>
-      <c r="F42" s="33"/>
-      <c r="G42" s="20"/>
+      <c r="D42" s="35"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="19"/>
       <c r="H42" s="8"/>
     </row>
     <row r="43" ht="15.75" customHeight="1" spans="1:8">
       <c r="A43" s="7"/>
-      <c r="B43" s="24" t="s">
+      <c r="B43" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="C43" s="36" t="s">
+      <c r="C43" s="35" t="s">
         <v>107</v>
       </c>
-      <c r="D43" s="36"/>
-      <c r="E43" s="34" t="s">
+      <c r="D43" s="35"/>
+      <c r="E43" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="F43" s="33" t="s">
+      <c r="F43" s="32" t="s">
         <v>108</v>
       </c>
-      <c r="G43" s="20" t="s">
+      <c r="G43" s="19" t="s">
         <v>109</v>
       </c>
       <c r="H43" s="8" t="s">
@@ -2963,25 +3030,25 @@
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A44" s="39" t="s">
+      <c r="A44" s="38" t="s">
         <v>110</v>
       </c>
-      <c r="B44" s="40" t="s">
+      <c r="B44" s="39" t="s">
         <v>111</v>
       </c>
-      <c r="C44" s="41" t="s">
+      <c r="C44" s="40" t="s">
         <v>112</v>
       </c>
-      <c r="D44" s="41" t="s">
+      <c r="D44" s="40" t="s">
         <v>113</v>
       </c>
-      <c r="E44" s="42" t="s">
+      <c r="E44" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="F44" s="43" t="s">
+      <c r="F44" s="42" t="s">
         <v>114</v>
       </c>
-      <c r="G44" s="44" t="s">
+      <c r="G44" s="43" t="s">
         <v>35</v>
       </c>
       <c r="H44" s="9" t="s">
@@ -2989,19 +3056,19 @@
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A45" s="27"/>
+      <c r="A45" s="26"/>
       <c r="B45" s="6"/>
-      <c r="C45" s="36" t="s">
+      <c r="C45" s="35" t="s">
         <v>115</v>
       </c>
-      <c r="D45" s="36" t="s">
+      <c r="D45" s="35" t="s">
         <v>116</v>
       </c>
       <c r="E45" s="6"/>
-      <c r="F45" s="45" t="s">
+      <c r="F45" s="44" t="s">
         <v>61</v>
       </c>
-      <c r="G45" s="20" t="s">
+      <c r="G45" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H45" s="8" t="s">
@@ -3009,29 +3076,29 @@
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A46" s="27"/>
+      <c r="A46" s="26"/>
       <c r="B46" s="6"/>
-      <c r="C46" s="36" t="s">
+      <c r="C46" s="35" t="s">
         <v>117</v>
       </c>
-      <c r="D46" s="36"/>
+      <c r="D46" s="35"/>
       <c r="E46" s="6"/>
       <c r="F46" s="7"/>
       <c r="G46" s="7"/>
       <c r="H46" s="7"/>
     </row>
     <row r="47" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A47" s="27"/>
+      <c r="A47" s="26"/>
       <c r="B47" s="6"/>
-      <c r="C47" s="36" t="s">
+      <c r="C47" s="35" t="s">
         <v>118</v>
       </c>
-      <c r="D47" s="36"/>
+      <c r="D47" s="35"/>
       <c r="E47" s="6"/>
-      <c r="F47" s="45" t="s">
+      <c r="F47" s="44" t="s">
         <v>61</v>
       </c>
-      <c r="G47" s="20" t="s">
+      <c r="G47" s="19" t="s">
         <v>12</v>
       </c>
       <c r="H47" s="8" t="s">
@@ -3039,121 +3106,121 @@
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A48" s="28"/>
+      <c r="A48" s="27"/>
       <c r="B48" s="7"/>
-      <c r="C48" s="46" t="s">
+      <c r="C48" s="45" t="s">
         <v>119</v>
       </c>
-      <c r="D48" s="46"/>
+      <c r="D48" s="45"/>
       <c r="E48" s="7"/>
-      <c r="F48" s="29" t="s">
+      <c r="F48" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="G48" s="35" t="s">
+      <c r="G48" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="H48" s="47" t="s">
+      <c r="H48" s="46" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="49" ht="42.75" customHeight="1" spans="1:8">
-      <c r="A49" s="48" t="s">
+      <c r="A49" s="47" t="s">
         <v>120</v>
       </c>
-      <c r="B49" s="48" t="s">
+      <c r="B49" s="47" t="s">
         <v>120</v>
       </c>
-      <c r="C49" s="49" t="s">
+      <c r="C49" s="48" t="s">
         <v>121</v>
       </c>
-      <c r="D49" s="50" t="s">
+      <c r="D49" s="49" t="s">
         <v>122</v>
       </c>
-      <c r="E49" s="51" t="s">
+      <c r="E49" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="F49" s="52"/>
-      <c r="G49" s="53" t="s">
+      <c r="F49" s="51"/>
+      <c r="G49" s="52" t="s">
         <v>103</v>
       </c>
-      <c r="H49" s="54"/>
+      <c r="H49" s="53"/>
     </row>
     <row r="50" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A50" s="55"/>
-      <c r="B50" s="55"/>
-      <c r="C50" s="49" t="s">
+      <c r="A50" s="54"/>
+      <c r="B50" s="54"/>
+      <c r="C50" s="48" t="s">
         <v>123</v>
       </c>
-      <c r="D50" s="56" t="s">
+      <c r="D50" s="55" t="s">
         <v>124</v>
       </c>
-      <c r="E50" s="57" t="s">
+      <c r="E50" s="56" t="s">
         <v>60</v>
       </c>
-      <c r="F50" s="58"/>
-      <c r="G50" s="53" t="s">
+      <c r="F50" s="57"/>
+      <c r="G50" s="52" t="s">
         <v>103</v>
       </c>
-      <c r="H50" s="59"/>
+      <c r="H50" s="58"/>
     </row>
     <row r="51" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A51" s="55"/>
-      <c r="B51" s="55"/>
-      <c r="C51" s="49" t="s">
+      <c r="A51" s="54"/>
+      <c r="B51" s="54"/>
+      <c r="C51" s="48" t="s">
         <v>125</v>
       </c>
-      <c r="D51" s="60" t="s">
+      <c r="D51" s="59" t="s">
         <v>126</v>
       </c>
-      <c r="E51" s="57" t="s">
+      <c r="E51" s="56" t="s">
         <v>60</v>
       </c>
-      <c r="F51" s="52"/>
-      <c r="G51" s="53" t="s">
+      <c r="F51" s="51"/>
+      <c r="G51" s="52" t="s">
         <v>103</v>
       </c>
-      <c r="H51" s="54"/>
+      <c r="H51" s="53"/>
     </row>
     <row r="52" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A52" s="61"/>
-      <c r="B52" s="61"/>
-      <c r="C52" s="60" t="s">
+      <c r="A52" s="60"/>
+      <c r="B52" s="60"/>
+      <c r="C52" s="59" t="s">
         <v>127</v>
       </c>
-      <c r="D52" s="50" t="s">
+      <c r="D52" s="49" t="s">
         <v>128</v>
       </c>
-      <c r="E52" s="62" t="s">
+      <c r="E52" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="F52" s="52" t="s">
+      <c r="F52" s="51" t="s">
         <v>129</v>
       </c>
-      <c r="G52" s="53" t="s">
+      <c r="G52" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="H52" s="54" t="s">
+      <c r="H52" s="53" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A53" s="40" t="s">
+      <c r="A53" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="B53" s="40" t="s">
+      <c r="B53" s="39" t="s">
         <v>131</v>
       </c>
-      <c r="C53" s="41" t="s">
+      <c r="C53" s="40" t="s">
         <v>132</v>
       </c>
-      <c r="D53" s="41"/>
-      <c r="E53" s="42" t="s">
+      <c r="D53" s="40"/>
+      <c r="E53" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="F53" s="43" t="s">
+      <c r="F53" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="G53" s="44" t="s">
+      <c r="G53" s="43" t="s">
         <v>12</v>
       </c>
       <c r="H53" s="9" t="s">
@@ -3162,22 +3229,22 @@
     </row>
     <row r="54" ht="28.5" customHeight="1" spans="1:8">
       <c r="A54" s="7"/>
-      <c r="B54" s="24" t="s">
+      <c r="B54" s="23" t="s">
         <v>133</v>
       </c>
       <c r="C54" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="D54" s="38" t="s">
+      <c r="D54" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="E54" s="34" t="s">
+      <c r="E54" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="F54" s="33" t="s">
+      <c r="F54" s="32" t="s">
         <v>136</v>
       </c>
-      <c r="G54" s="20" t="s">
+      <c r="G54" s="19" t="s">
         <v>103</v>
       </c>
       <c r="H54" s="8" t="s">
@@ -3185,21 +3252,21 @@
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A55" s="25" t="s">
+      <c r="A55" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="B55" s="24" t="s">
+      <c r="B55" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="C55" s="36" t="s">
+      <c r="C55" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="D55" s="36"/>
-      <c r="E55" s="34" t="s">
+      <c r="D55" s="35"/>
+      <c r="E55" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="F55" s="33"/>
-      <c r="G55" s="20" t="s">
+      <c r="F55" s="32"/>
+      <c r="G55" s="19" t="s">
         <v>140</v>
       </c>
       <c r="H55" s="8" t="s">
@@ -3207,49 +3274,49 @@
       </c>
     </row>
     <row r="56" ht="42.75" customHeight="1" spans="1:8">
-      <c r="A56" s="25" t="s">
+      <c r="A56" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="B56" s="24" t="s">
+      <c r="B56" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="C56" s="36" t="s">
+      <c r="C56" s="35" t="s">
         <v>143</v>
       </c>
-      <c r="D56" s="38" t="s">
+      <c r="D56" s="37" t="s">
         <v>144</v>
       </c>
-      <c r="E56" s="34" t="s">
+      <c r="E56" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="F56" s="45" t="s">
+      <c r="F56" s="44" t="s">
         <v>145</v>
       </c>
-      <c r="G56" s="20"/>
+      <c r="G56" s="19"/>
       <c r="H56" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="57" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A57" s="24" t="s">
+      <c r="A57" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="B57" s="24" t="s">
+      <c r="B57" s="23" t="s">
         <v>146</v>
       </c>
-      <c r="C57" s="36" t="s">
+      <c r="C57" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="D57" s="36" t="s">
+      <c r="D57" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="E57" s="34" t="s">
+      <c r="E57" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="F57" s="45" t="s">
+      <c r="F57" s="44" t="s">
         <v>149</v>
       </c>
-      <c r="G57" s="20" t="s">
+      <c r="G57" s="19" t="s">
         <v>103</v>
       </c>
       <c r="H57" s="8" t="s">
@@ -3257,50 +3324,50 @@
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A58" s="63" t="s">
+      <c r="A58" s="62" t="s">
         <v>150</v>
       </c>
-      <c r="B58" s="63" t="s">
+      <c r="B58" s="62" t="s">
         <v>150</v>
       </c>
-      <c r="C58" s="35" t="s">
+      <c r="C58" s="34" t="s">
         <v>151</v>
       </c>
-      <c r="D58" s="46" t="s">
+      <c r="D58" s="45" t="s">
         <v>152</v>
       </c>
-      <c r="E58" s="64" t="s">
+      <c r="E58" s="63" t="s">
         <v>40</v>
       </c>
-      <c r="F58" s="65" t="s">
+      <c r="F58" s="64" t="s">
         <v>153</v>
       </c>
-      <c r="G58" s="35" t="s">
+      <c r="G58" s="34" t="s">
         <v>103</v>
       </c>
-      <c r="H58" s="47" t="s">
+      <c r="H58" s="46" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="59" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A59" s="48" t="s">
+      <c r="A59" s="47" t="s">
         <v>154</v>
       </c>
-      <c r="B59" s="48" t="s">
+      <c r="B59" s="47" t="s">
         <v>154</v>
       </c>
-      <c r="C59" s="66" t="s">
+      <c r="C59" s="65" t="s">
         <v>155</v>
       </c>
-      <c r="D59" s="58"/>
-      <c r="E59" s="62" t="s">
+      <c r="D59" s="57"/>
+      <c r="E59" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="F59" s="58"/>
-      <c r="G59" s="35" t="s">
+      <c r="F59" s="57"/>
+      <c r="G59" s="34" t="s">
         <v>103</v>
       </c>
-      <c r="H59" s="59" t="s">
+      <c r="H59" s="58" t="s">
         <v>13</v>
       </c>
     </row>
@@ -3370,7 +3437,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.2" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="11.7019230769231" style="1" customWidth="1"/>
@@ -3632,195 +3699,207 @@
         <v>194</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>109</v>
       </c>
       <c r="H12" s="4" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="13" ht="96" customHeight="1" spans="1:8">
+      <c r="A13" s="6"/>
+      <c r="B13" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="13" ht="81" customHeight="1" spans="1:8">
-      <c r="A13" s="6"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" ht="96" customHeight="1" spans="1:8">
+    <row r="14" ht="111" customHeight="1" spans="1:8">
       <c r="A14" s="6"/>
       <c r="B14" s="4" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>188</v>
+        <v>103</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="15" ht="111" customHeight="1" spans="1:8">
+    <row r="15" ht="51" customHeight="1" spans="1:8">
       <c r="A15" s="6"/>
       <c r="B15" s="4" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="16" ht="51" customHeight="1" spans="1:8">
+    <row r="16" ht="126" customHeight="1" spans="1:8">
       <c r="A16" s="6"/>
-      <c r="B16" s="4" t="s">
-        <v>203</v>
-      </c>
+      <c r="B16" s="6"/>
       <c r="C16" s="5" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="17" ht="126" customHeight="1" spans="1:8">
+    <row r="17" ht="66" customHeight="1" spans="1:8">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="5" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="F17" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" ht="96" customHeight="1" spans="1:8">
+      <c r="A18" s="6"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+    </row>
+    <row r="19" ht="111" customHeight="1" spans="1:8">
+      <c r="A19" s="6"/>
+      <c r="B19" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="F19" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="G17" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="18" ht="66" customHeight="1" spans="1:8">
-      <c r="A18" s="6"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="F18" s="4" t="s">
+      <c r="G19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" ht="66" customHeight="1" spans="1:8">
+      <c r="A20" s="6"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H18" s="6"/>
-    </row>
-    <row r="19" ht="96" customHeight="1" spans="1:8">
-      <c r="A19" s="6"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-    </row>
-    <row r="20" ht="111" customHeight="1" spans="1:8">
-      <c r="A20" s="6"/>
-      <c r="B20" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>109</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" ht="66" customHeight="1" spans="1:8">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="21" ht="96" customHeight="1" spans="1:8">
       <c r="A21" s="6"/>
-      <c r="B21" s="7"/>
+      <c r="B21" s="4" t="s">
+        <v>224</v>
+      </c>
       <c r="C21" s="5" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>109</v>
@@ -3829,22 +3908,20 @@
         <v>162</v>
       </c>
     </row>
-    <row r="22" ht="96" customHeight="1" spans="1:8">
+    <row r="22" ht="51" customHeight="1" spans="1:8">
       <c r="A22" s="6"/>
-      <c r="B22" s="4" t="s">
-        <v>223</v>
-      </c>
+      <c r="B22" s="7"/>
       <c r="C22" s="5" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>109</v>
@@ -3853,44 +3930,46 @@
         <v>162</v>
       </c>
     </row>
-    <row r="23" ht="51" customHeight="1" spans="1:8">
+    <row r="23" ht="96" customHeight="1" spans="1:8">
       <c r="A23" s="6"/>
-      <c r="B23" s="7"/>
+      <c r="B23" s="4" t="s">
+        <v>231</v>
+      </c>
       <c r="C23" s="5" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="24" ht="96" customHeight="1" spans="1:8">
+    <row r="24" ht="81" customHeight="1" spans="1:8">
       <c r="A24" s="6"/>
       <c r="B24" s="4" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G24" s="4" t="s">
         <v>103</v>
@@ -3899,83 +3978,81 @@
         <v>162</v>
       </c>
     </row>
-    <row r="25" ht="81" customHeight="1" spans="1:8">
+    <row r="25" ht="126" customHeight="1" spans="1:8">
       <c r="A25" s="6"/>
-      <c r="B25" s="4" t="s">
-        <v>234</v>
-      </c>
+      <c r="B25" s="6"/>
       <c r="C25" s="5" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="26" ht="126" customHeight="1" spans="1:8">
+    <row r="26" ht="96" customHeight="1" spans="1:8">
       <c r="A26" s="6"/>
-      <c r="B26" s="6"/>
+      <c r="B26" s="7"/>
       <c r="C26" s="5" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="F26" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="F26" s="7"/>
+      <c r="G26" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="H26" s="7"/>
+    </row>
+    <row r="27" ht="171" customHeight="1" spans="1:8">
+      <c r="A27" s="6"/>
+      <c r="B27" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="F27" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G27" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="H27" s="4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="27" ht="96" customHeight="1" spans="1:8">
-      <c r="A27" s="6"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="F27" s="7"/>
-      <c r="G27" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="H27" s="7"/>
-    </row>
-    <row r="28" ht="171" customHeight="1" spans="1:8">
+    <row r="28" ht="126" customHeight="1" spans="1:8">
       <c r="A28" s="6"/>
-      <c r="B28" s="4" t="s">
-        <v>244</v>
-      </c>
+      <c r="B28" s="7"/>
       <c r="C28" s="5" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>10</v>
@@ -3987,97 +4064,76 @@
         <v>162</v>
       </c>
     </row>
-    <row r="29" ht="126" customHeight="1" spans="1:8">
+    <row r="29" ht="81" customHeight="1" spans="1:8">
       <c r="A29" s="6"/>
-      <c r="B29" s="7"/>
+      <c r="B29" s="3" t="s">
+        <v>252</v>
+      </c>
       <c r="C29" s="5" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="F29" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" ht="81" customHeight="1" spans="1:8">
+      <c r="A30" s="7"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="F30" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H29" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="30" ht="81" customHeight="1" spans="1:8">
-      <c r="A30" s="6"/>
-      <c r="B30" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>252</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="G30" s="4" t="s">
         <v>188</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" ht="81" customHeight="1" spans="1:8">
-      <c r="A31" s="7"/>
-      <c r="B31" s="7"/>
-      <c r="C31" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G31" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="H31" s="4" t="s">
         <v>162</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A2:A31"/>
+    <mergeCell ref="A2:A30"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="B5:B11"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="B15:B18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="B29:B30"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F25:F26"/>
     <mergeCell ref="G3:G4"/>
     <mergeCell ref="G8:G9"/>
-    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="G17:G18"/>
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="H6:H9"/>
-    <mergeCell ref="H17:H19"/>
-    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="H16:H18"/>
+    <mergeCell ref="H25:H26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: update PA产品方案Excel file
update the PA product plan excel document with latest changes
</commit_message>
<xml_diff>
--- a/PA替代需求列表.xlsx
+++ b/PA替代需求列表.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="256">
   <si>
     <t>一级需求</t>
   </si>
@@ -550,7 +550,7 @@
     <t>PA除全局TCP/UDP会话超时外，可在应用程序对象上定义专用超时，匹配该应用的流量覆盖全局值（PA Web帮助p215、p695）；天融信手册未见应用级超时覆盖（仅SSLVPN会话超时设置与黑名单老化）；迁移评估项：需排查现网PA为数据库/长连接业务单独配置的应用超时并逐条转换，否则长连接业务频繁中断</t>
   </si>
   <si>
-    <t>安全策略(Security)</t>
+    <t>安全策略</t>
   </si>
   <si>
     <t>支持配置HIP主机信息配置文件</t>
@@ -643,7 +643,7 @@
     <t>PA QoS规则可直接按DSCP值或IP优先级/ToS匹配调度（PA Web帮助p155）；天融信支持DSCP/802.1p(CoS)识别与重标记，但需在独立流量管理模块配置（虚拟通道+限制/保证带宽+通道优先级，天融信手册《流量管理》页），未直接耦合在基础访问控制策略表内（联网核实厂商流控资料，手册未详载）</t>
   </si>
   <si>
-    <t>基于策略转发(PBF)</t>
+    <t>基于策略转发</t>
   </si>
   <si>
     <t>支持PBF强制对称返回</t>
@@ -655,10 +655,10 @@
     <t>PA对称返回：虚拟路由器替代返回流量的路由查找，将流量引导回接收SYN数据包的MAC地址（ARP表确定下一跳），双ISP双活/非对称路由核心机制（PA管理指南p1294）；天融信手册检索无对称返回/回程机制命中，策略路由与LLB的回程保障能力待验证；迁移评估项：多ISP双活环境需实测天融信回包路由对称性，否则现网业务中断</t>
   </si>
   <si>
-    <t>解密策略(Decryption)</t>
-  </si>
-  <si>
-    <t>支持解密流量镜像到专用接口（Decryption Port Mirroring）</t>
+    <t>解密策略</t>
+  </si>
+  <si>
+    <t>支持解密流量镜像到专用接口</t>
   </si>
   <si>
     <t>解密后明文流量镜像至专用接口供第三方分析</t>
@@ -667,7 +667,7 @@
     <t>PA解密后将明文流量镜像到专用接口供IDS/抓包，需激活免费许可证（PA管理指南p1059）；天融信无解密流量镜像专用功能（仅SSL卸载+WAF镜像联动）</t>
   </si>
   <si>
-    <t>支持解密不受信证书分离处理（Forward Untrust Certificate）</t>
+    <t>支持解密不受信证书分离处理</t>
   </si>
   <si>
     <t>外部无效证书以不受信转发证书重签，保留浏览器告警</t>
@@ -676,7 +676,7 @@
     <t>PA转发代理遇外部过期/不受信证书时，不用内部信任CA重签，而是专用Forward Untrust Certificate重签名，让浏览器保留不受信告警（PA管理指南p994、p1030）；天融信SSL解密（透明代理/服务器SSL解密，天融信手册《代理策略》页）未见受信/不受信双证书体系；迁移评估项：需验证天融信对外部无效证书的处理方式，避免直接阻断（白屏）或信任重签（掩盖风险）</t>
   </si>
   <si>
-    <t>支持解密规则按URL类别选择性解密（URL Category）</t>
+    <t>支持解密规则按URL类别选择性解密</t>
   </si>
   <si>
     <t>按URL类别圈定解密范围，排除银行/医疗等敏感类</t>
@@ -685,7 +685,7 @@
     <t>PA解密规则可按URL类别（含自定义类别）选择解密范围，可排除银行/医疗等敏感类别不解密（PA Web帮助p164）；天融信SSL解密（代理策略/代理模板）无按URL类别选择解密机制（检索无命中）</t>
   </si>
   <si>
-    <t>支持SSH代理解密与SSH隧道控制（SSH Proxy）</t>
+    <t>支持SSH代理解密与SSH隧道控制</t>
   </si>
   <si>
     <t>SSH代理解密+SSH隧道(ssh-tunnel)识别控制</t>
@@ -697,22 +697,13 @@
     <t>网络数据包代理(NPBroker)</t>
   </si>
   <si>
-    <t>支持内联数据包代理策略将流量转发第三方安全链（NPBroker）</t>
-  </si>
-  <si>
-    <t>已解密/未解密流量内联转发第三方安全链，L3路由转发</t>
+    <t>支持内联数据包代理策略将流量转发第三方安全链</t>
+  </si>
+  <si>
+    <t>已解密/未解密/非TLS流量内联转发第三方安全链，L3路由转发，支持转发流量类型选择</t>
   </si>
   <si>
     <t>PA网络数据包代理策略将已解密/未解密TLS/非TLS流量内联转发至第三方安全工具，路径选择选项卡应用数据包代理配置文件定义经路由L3安全链的转发方式（PA Web帮助p167-170）；天融信无网络数据包代理模块，最接近手段为WAF旁路联动（经交换机镜像引流，天融信手册《与WAF联动》页），非内联且无回注路径；对应矩阵#122</t>
-  </si>
-  <si>
-    <t>支持NPBroker转发流量类型选择（TLS解密/未解密/非TLS）</t>
-  </si>
-  <si>
-    <t>TLS解密/未解密/非TLS流量类型选择</t>
-  </si>
-  <si>
-    <t>PA规则可选Forward TLS(Decrypted)/未解密/非TLS多种流量类型；需免费许可证（PA Web帮助p167）；天融信无网络数据包代理模块（矩阵#122）</t>
   </si>
   <si>
     <t>隧道检测(Tunnel Inspection)</t>
@@ -1618,11 +1609,19 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1637,11 +1636,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1652,6 +1651,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1677,6 +1677,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1740,6 +1743,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1860,140 +1866,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="absolute">
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1111670</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>18250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>320820</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>187275</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Watermark"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6799580" y="6399530"/>
-          <a:ext cx="2200275" cy="349885"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="b"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="zh-CN" sz="1600" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="808080">
-                  <a:alpha val="19999"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202090204"/>
-              <a:ea typeface="宋体"/>
-            </a:rPr>
-            <a:t>AI 生成</a:t>
-          </a:r>
-          <a:endParaRPr lang="zh-CN" sz="1600" dirty="0">
-            <a:solidFill>
-              <a:srgbClr val="808080">
-                <a:alpha val="19999"/>
-              </a:srgbClr>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202090204"/>
-            <a:ea typeface="宋体"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="absolute">
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>2084490</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>469100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>1547005</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>819100</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Watermark"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6799580" y="6399530"/>
-          <a:ext cx="2200275" cy="349885"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="b"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="zh-CN" sz="1600" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="808080">
-                  <a:alpha val="19999"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202090204"/>
-              <a:ea typeface="宋体"/>
-            </a:rPr>
-            <a:t>AI 生成</a:t>
-          </a:r>
-          <a:endParaRPr lang="zh-CN" sz="1600" dirty="0">
-            <a:solidFill>
-              <a:srgbClr val="808080">
-                <a:alpha val="19999"/>
-              </a:srgbClr>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202090204"/>
-            <a:ea typeface="宋体"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2257,1117 +2129,1117 @@
   <dimension ref="A1:H59"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.2" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="11.7115384615385" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7115384615385" style="1" customWidth="1"/>
-    <col min="3" max="3" width="54.7115384615385" style="1" customWidth="1"/>
-    <col min="4" max="4" width="45.2884615384615" style="1" customWidth="1"/>
-    <col min="5" max="5" width="7.71153846153846" style="1" customWidth="1"/>
-    <col min="6" max="6" width="37.8557692307692" style="1" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="9.71153846153846" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.71153846153846" style="13" customWidth="1"/>
+    <col min="1" max="1" width="11.7115384615385" style="15" customWidth="1"/>
+    <col min="2" max="2" width="19.7115384615385" style="15" customWidth="1"/>
+    <col min="3" max="3" width="54.7115384615385" style="15" customWidth="1"/>
+    <col min="4" max="4" width="45.2884615384615" style="15" customWidth="1"/>
+    <col min="5" max="5" width="7.71153846153846" style="15" customWidth="1"/>
+    <col min="6" max="6" width="37.8557692307692" style="15" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="9.71153846153846" style="15" customWidth="1"/>
+    <col min="8" max="8" width="9.71153846153846" style="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="16"/>
-      <c r="G1" s="15" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="18" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="19"/>
-      <c r="E2" s="20" t="s">
+      <c r="D2" s="22"/>
+      <c r="E2" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="19" t="s">
+      <c r="G2" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1" spans="1:8">
-      <c r="A3" s="6"/>
-      <c r="B3" s="18" t="s">
+      <c r="A3" s="8"/>
+      <c r="B3" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1" spans="1:8">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="19" t="s">
+      <c r="A4" s="8"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
     </row>
     <row r="5" ht="36" customHeight="1" spans="1:8">
-      <c r="A5" s="6"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="19" t="s">
+      <c r="A5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
     </row>
     <row r="6" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A6" s="6"/>
-      <c r="B6" s="23" t="s">
+      <c r="A6" s="8"/>
+      <c r="B6" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="19" t="s">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
     </row>
     <row r="8" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="19" t="s">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
     </row>
     <row r="9" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="19" t="s">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
     </row>
     <row r="10" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="19" t="s">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="19"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
     </row>
     <row r="11" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="19" t="s">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="19"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
     </row>
     <row r="12" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A12" s="6"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="19" t="s">
+      <c r="A12" s="8"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="19"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A13" s="7"/>
-      <c r="B13" s="23" t="s">
+      <c r="A13" s="9"/>
+      <c r="B13" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="20" t="s">
+      <c r="E13" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="21" t="s">
+      <c r="F13" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="H13" s="8" t="s">
+      <c r="H13" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="E14" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="F14" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="H14" s="8" t="s">
+      <c r="H14" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A15" s="26"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="19" t="s">
+      <c r="A15" s="30"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
     </row>
     <row r="16" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A16" s="26"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="19" t="s">
+      <c r="A16" s="30"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
     </row>
     <row r="17" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A17" s="26"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="19" t="s">
+      <c r="A17" s="30"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
     </row>
     <row r="18" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A18" s="26"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="19" t="s">
+      <c r="A18" s="30"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
     </row>
     <row r="19" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A19" s="26"/>
-      <c r="B19" s="6"/>
-      <c r="C19" s="19" t="s">
+      <c r="A19" s="30"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
     </row>
     <row r="20" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A20" s="26"/>
-      <c r="B20" s="6"/>
-      <c r="C20" s="19" t="s">
+      <c r="A20" s="30"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
     </row>
     <row r="21" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A21" s="26"/>
-      <c r="B21" s="6"/>
-      <c r="C21" s="19" t="s">
+      <c r="A21" s="30"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
     </row>
     <row r="22" ht="32.25" customHeight="1" spans="1:8">
-      <c r="A22" s="27"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="19" t="s">
+      <c r="A22" s="31"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
     </row>
     <row r="23" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A23" s="24" t="s">
+      <c r="A23" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="C23" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="D23" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="E23" s="20" t="s">
+      <c r="E23" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="28" t="s">
+      <c r="F23" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="G23" s="19" t="s">
+      <c r="G23" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H23" s="8" t="s">
+      <c r="H23" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A24" s="24" t="s">
+      <c r="A24" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="23" t="s">
+      <c r="B24" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="19" t="s">
+      <c r="C24" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="19" t="s">
+      <c r="D24" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="E24" s="20" t="s">
+      <c r="E24" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="F24" s="29" t="s">
+      <c r="F24" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="G24" s="19" t="s">
+      <c r="G24" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H24" s="8" t="s">
+      <c r="H24" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A25" s="24" t="s">
+      <c r="A25" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="C25" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="30" t="s">
+      <c r="D25" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="E25" s="20" t="s">
+      <c r="E25" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="F25" s="21" t="s">
+      <c r="F25" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="G25" s="19" t="s">
+      <c r="G25" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H25" s="8" t="s">
+      <c r="H25" s="25" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="26" s="12" customFormat="1" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A26" s="26"/>
-      <c r="B26" s="23" t="s">
+    <row r="26" s="14" customFormat="1" ht="28.5" customHeight="1" spans="1:8">
+      <c r="A26" s="30"/>
+      <c r="B26" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="30"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="8"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="35"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="25"/>
     </row>
     <row r="27" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A27" s="26"/>
-      <c r="B27" s="23" t="s">
+      <c r="A27" s="30"/>
+      <c r="B27" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="19" t="s">
+      <c r="C27" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="D27" s="19" t="s">
+      <c r="D27" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="E27" s="20" t="s">
+      <c r="E27" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="F27" s="21" t="s">
+      <c r="F27" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="G27" s="19" t="s">
+      <c r="G27" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H27" s="8" t="s">
+      <c r="H27" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A28" s="26"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="19" t="s">
+      <c r="A28" s="30"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
     </row>
     <row r="29" ht="60" customHeight="1" spans="1:8">
-      <c r="A29" s="26"/>
-      <c r="B29" s="23" t="s">
+      <c r="A29" s="30"/>
+      <c r="B29" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="C29" s="19" t="s">
+      <c r="C29" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="E29" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="F29" s="32" t="s">
+      <c r="F29" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="G29" s="19" t="s">
+      <c r="G29" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="H29" s="8" t="s">
+      <c r="H29" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A30" s="26"/>
-      <c r="B30" s="6"/>
-      <c r="C30" s="19" t="s">
+      <c r="A30" s="30"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="D30" s="19" t="s">
+      <c r="D30" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="E30" s="20" t="s">
+      <c r="E30" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="F30" s="6"/>
-      <c r="G30" s="19" t="s">
+      <c r="F30" s="8"/>
+      <c r="G30" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H30" s="8" t="s">
+      <c r="H30" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A31" s="27"/>
-      <c r="B31" s="7"/>
-      <c r="C31" s="19" t="s">
+      <c r="A31" s="31"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="D31" s="19" t="s">
+      <c r="D31" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="E31" s="33" t="s">
+      <c r="E31" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="F31" s="7"/>
-      <c r="G31" s="19" t="s">
+      <c r="F31" s="9"/>
+      <c r="G31" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H31" s="8" t="s">
+      <c r="H31" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A32" s="24" t="s">
+      <c r="A32" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="23" t="s">
+      <c r="B32" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="C32" s="19" t="s">
+      <c r="C32" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="D32" s="19" t="s">
+      <c r="D32" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="E32" s="20" t="s">
+      <c r="E32" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="F32" s="21" t="s">
+      <c r="F32" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="G32" s="19" t="s">
+      <c r="G32" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H32" s="8" t="s">
+      <c r="H32" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A33" s="27"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="19" t="s">
+      <c r="A33" s="31"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="7"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
     </row>
     <row r="34" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A34" s="24" t="s">
+      <c r="A34" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="B34" s="23" t="s">
+      <c r="B34" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="C34" s="19" t="s">
+      <c r="C34" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="D34" s="19"/>
-      <c r="E34" s="20" t="s">
+      <c r="D34" s="22"/>
+      <c r="E34" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="F34" s="21" t="s">
+      <c r="F34" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="G34" s="19" t="s">
+      <c r="G34" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H34" s="8" t="s">
+      <c r="H34" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A35" s="26"/>
-      <c r="B35" s="6"/>
-      <c r="C35" s="19" t="s">
+      <c r="A35" s="30"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="D35" s="19"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
-      <c r="H35" s="6"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
     </row>
     <row r="36" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A36" s="26"/>
-      <c r="B36" s="6"/>
-      <c r="C36" s="19" t="s">
+      <c r="A36" s="30"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="D36" s="19"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
+      <c r="D36" s="22"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
     </row>
     <row r="37" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A37" s="27"/>
-      <c r="B37" s="7"/>
-      <c r="C37" s="34" t="s">
+      <c r="A37" s="31"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="D37" s="34"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A38" s="23" t="s">
+      <c r="A38" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="B38" s="23" t="s">
+      <c r="B38" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="C38" s="35" t="s">
+      <c r="C38" s="39" t="s">
         <v>93</v>
       </c>
-      <c r="D38" s="35"/>
-      <c r="E38" s="33" t="s">
+      <c r="D38" s="39"/>
+      <c r="E38" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="F38" s="36" t="s">
+      <c r="F38" s="40" t="s">
         <v>61</v>
       </c>
-      <c r="G38" s="19" t="s">
+      <c r="G38" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H38" s="8" t="s">
+      <c r="H38" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A39" s="6"/>
-      <c r="B39" s="23" t="s">
+      <c r="A39" s="8"/>
+      <c r="B39" s="27" t="s">
         <v>94</v>
       </c>
-      <c r="C39" s="35" t="s">
+      <c r="C39" s="39" t="s">
         <v>95</v>
       </c>
-      <c r="D39" s="35"/>
-      <c r="E39" s="33" t="s">
+      <c r="D39" s="39"/>
+      <c r="E39" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="F39" s="7"/>
-      <c r="G39" s="7"/>
-      <c r="H39" s="7"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
     </row>
     <row r="40" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A40" s="6"/>
-      <c r="B40" s="23" t="s">
+      <c r="A40" s="8"/>
+      <c r="B40" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="C40" s="35" t="s">
+      <c r="C40" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="D40" s="37" t="s">
+      <c r="D40" s="41" t="s">
         <v>98</v>
       </c>
-      <c r="E40" s="33" t="s">
+      <c r="E40" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="F40" s="32" t="s">
+      <c r="F40" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="G40" s="19" t="s">
+      <c r="G40" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="H40" s="8" t="s">
+      <c r="H40" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A41" s="6"/>
-      <c r="B41" s="23" t="s">
+      <c r="A41" s="8"/>
+      <c r="B41" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="C41" s="19" t="s">
+      <c r="C41" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="D41" s="35" t="s">
+      <c r="D41" s="39" t="s">
         <v>101</v>
       </c>
-      <c r="E41" s="33" t="s">
+      <c r="E41" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="F41" s="32" t="s">
+      <c r="F41" s="36" t="s">
         <v>102</v>
       </c>
-      <c r="G41" s="19" t="s">
+      <c r="G41" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="H41" s="8" t="s">
+      <c r="H41" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A42" s="6"/>
-      <c r="B42" s="23" t="s">
+      <c r="A42" s="8"/>
+      <c r="B42" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="C42" s="19" t="s">
+      <c r="C42" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="D42" s="35"/>
-      <c r="E42" s="33"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="19"/>
-      <c r="H42" s="8"/>
+      <c r="D42" s="39"/>
+      <c r="E42" s="37"/>
+      <c r="F42" s="36"/>
+      <c r="G42" s="22"/>
+      <c r="H42" s="25"/>
     </row>
     <row r="43" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A43" s="7"/>
-      <c r="B43" s="23" t="s">
+      <c r="A43" s="9"/>
+      <c r="B43" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="C43" s="35" t="s">
+      <c r="C43" s="39" t="s">
         <v>107</v>
       </c>
-      <c r="D43" s="35"/>
-      <c r="E43" s="33" t="s">
+      <c r="D43" s="39"/>
+      <c r="E43" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="F43" s="32" t="s">
+      <c r="F43" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="G43" s="19" t="s">
+      <c r="G43" s="22" t="s">
         <v>109</v>
       </c>
-      <c r="H43" s="8" t="s">
+      <c r="H43" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A44" s="38" t="s">
+      <c r="A44" s="42" t="s">
         <v>110</v>
       </c>
-      <c r="B44" s="39" t="s">
+      <c r="B44" s="43" t="s">
         <v>111</v>
       </c>
-      <c r="C44" s="40" t="s">
+      <c r="C44" s="44" t="s">
         <v>112</v>
       </c>
-      <c r="D44" s="40" t="s">
+      <c r="D44" s="44" t="s">
         <v>113</v>
       </c>
-      <c r="E44" s="41" t="s">
+      <c r="E44" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="F44" s="42" t="s">
+      <c r="F44" s="46" t="s">
         <v>114</v>
       </c>
-      <c r="G44" s="43" t="s">
+      <c r="G44" s="47" t="s">
         <v>35</v>
       </c>
-      <c r="H44" s="9" t="s">
+      <c r="H44" s="48" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A45" s="26"/>
-      <c r="B45" s="6"/>
-      <c r="C45" s="35" t="s">
+      <c r="A45" s="30"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="39" t="s">
         <v>115</v>
       </c>
-      <c r="D45" s="35" t="s">
+      <c r="D45" s="39" t="s">
         <v>116</v>
       </c>
-      <c r="E45" s="6"/>
-      <c r="F45" s="44" t="s">
+      <c r="E45" s="8"/>
+      <c r="F45" s="49" t="s">
         <v>61</v>
       </c>
-      <c r="G45" s="19" t="s">
+      <c r="G45" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H45" s="8" t="s">
+      <c r="H45" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A46" s="26"/>
-      <c r="B46" s="6"/>
-      <c r="C46" s="35" t="s">
+      <c r="A46" s="30"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="39" t="s">
         <v>117</v>
       </c>
-      <c r="D46" s="35"/>
-      <c r="E46" s="6"/>
-      <c r="F46" s="7"/>
-      <c r="G46" s="7"/>
-      <c r="H46" s="7"/>
+      <c r="D46" s="39"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
     </row>
     <row r="47" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A47" s="26"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="35" t="s">
+      <c r="A47" s="30"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="39" t="s">
         <v>118</v>
       </c>
-      <c r="D47" s="35"/>
-      <c r="E47" s="6"/>
-      <c r="F47" s="44" t="s">
+      <c r="D47" s="39"/>
+      <c r="E47" s="8"/>
+      <c r="F47" s="49" t="s">
         <v>61</v>
       </c>
-      <c r="G47" s="19" t="s">
+      <c r="G47" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H47" s="8" t="s">
+      <c r="H47" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A48" s="27"/>
-      <c r="B48" s="7"/>
-      <c r="C48" s="45" t="s">
+      <c r="A48" s="31"/>
+      <c r="B48" s="9"/>
+      <c r="C48" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="D48" s="45"/>
-      <c r="E48" s="7"/>
-      <c r="F48" s="28" t="s">
+      <c r="D48" s="50"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="G48" s="34" t="s">
+      <c r="G48" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="H48" s="46" t="s">
+      <c r="H48" s="51" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="49" ht="42.75" customHeight="1" spans="1:8">
-      <c r="A49" s="47" t="s">
+      <c r="A49" s="52" t="s">
         <v>120</v>
       </c>
-      <c r="B49" s="47" t="s">
+      <c r="B49" s="52" t="s">
         <v>120</v>
       </c>
-      <c r="C49" s="48" t="s">
+      <c r="C49" s="53" t="s">
         <v>121</v>
       </c>
-      <c r="D49" s="49" t="s">
+      <c r="D49" s="54" t="s">
         <v>122</v>
       </c>
-      <c r="E49" s="50" t="s">
+      <c r="E49" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="F49" s="51"/>
-      <c r="G49" s="52" t="s">
+      <c r="F49" s="56"/>
+      <c r="G49" s="57" t="s">
         <v>103</v>
       </c>
-      <c r="H49" s="53"/>
+      <c r="H49" s="58"/>
     </row>
     <row r="50" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A50" s="54"/>
-      <c r="B50" s="54"/>
-      <c r="C50" s="48" t="s">
+      <c r="A50" s="59"/>
+      <c r="B50" s="59"/>
+      <c r="C50" s="53" t="s">
         <v>123</v>
       </c>
-      <c r="D50" s="55" t="s">
+      <c r="D50" s="60" t="s">
         <v>124</v>
       </c>
-      <c r="E50" s="56" t="s">
+      <c r="E50" s="61" t="s">
         <v>60</v>
       </c>
-      <c r="F50" s="57"/>
-      <c r="G50" s="52" t="s">
+      <c r="F50" s="62"/>
+      <c r="G50" s="57" t="s">
         <v>103</v>
       </c>
-      <c r="H50" s="58"/>
+      <c r="H50" s="63"/>
     </row>
     <row r="51" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A51" s="54"/>
-      <c r="B51" s="54"/>
-      <c r="C51" s="48" t="s">
+      <c r="A51" s="59"/>
+      <c r="B51" s="59"/>
+      <c r="C51" s="53" t="s">
         <v>125</v>
       </c>
-      <c r="D51" s="59" t="s">
+      <c r="D51" s="64" t="s">
         <v>126</v>
       </c>
-      <c r="E51" s="56" t="s">
+      <c r="E51" s="61" t="s">
         <v>60</v>
       </c>
-      <c r="F51" s="51"/>
-      <c r="G51" s="52" t="s">
+      <c r="F51" s="56"/>
+      <c r="G51" s="57" t="s">
         <v>103</v>
       </c>
-      <c r="H51" s="53"/>
+      <c r="H51" s="58"/>
     </row>
     <row r="52" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A52" s="60"/>
-      <c r="B52" s="60"/>
-      <c r="C52" s="59" t="s">
+      <c r="A52" s="65"/>
+      <c r="B52" s="65"/>
+      <c r="C52" s="64" t="s">
         <v>127</v>
       </c>
-      <c r="D52" s="49" t="s">
+      <c r="D52" s="54" t="s">
         <v>128</v>
       </c>
-      <c r="E52" s="61" t="s">
+      <c r="E52" s="66" t="s">
         <v>10</v>
       </c>
-      <c r="F52" s="51" t="s">
+      <c r="F52" s="56" t="s">
         <v>129</v>
       </c>
-      <c r="G52" s="52" t="s">
+      <c r="G52" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="H52" s="53" t="s">
+      <c r="H52" s="58" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A53" s="39" t="s">
+      <c r="A53" s="43" t="s">
         <v>130</v>
       </c>
-      <c r="B53" s="39" t="s">
+      <c r="B53" s="43" t="s">
         <v>131</v>
       </c>
-      <c r="C53" s="40" t="s">
+      <c r="C53" s="44" t="s">
         <v>132</v>
       </c>
-      <c r="D53" s="40"/>
-      <c r="E53" s="41" t="s">
+      <c r="D53" s="44"/>
+      <c r="E53" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="F53" s="42" t="s">
+      <c r="F53" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="G53" s="43" t="s">
+      <c r="G53" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="H53" s="9" t="s">
+      <c r="H53" s="48" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="54" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A54" s="7"/>
-      <c r="B54" s="23" t="s">
+      <c r="A54" s="9"/>
+      <c r="B54" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="C54" s="8" t="s">
+      <c r="C54" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="D54" s="37" t="s">
+      <c r="D54" s="41" t="s">
         <v>135</v>
       </c>
-      <c r="E54" s="33" t="s">
+      <c r="E54" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="F54" s="32" t="s">
+      <c r="F54" s="36" t="s">
         <v>136</v>
       </c>
-      <c r="G54" s="19" t="s">
+      <c r="G54" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="H54" s="8" t="s">
+      <c r="H54" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A55" s="24" t="s">
+      <c r="A55" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="B55" s="23" t="s">
+      <c r="B55" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="C55" s="35" t="s">
+      <c r="C55" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="D55" s="35"/>
-      <c r="E55" s="33" t="s">
+      <c r="D55" s="39"/>
+      <c r="E55" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="F55" s="32"/>
-      <c r="G55" s="19" t="s">
+      <c r="F55" s="36"/>
+      <c r="G55" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="H55" s="8" t="s">
+      <c r="H55" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="56" ht="42.75" customHeight="1" spans="1:8">
-      <c r="A56" s="24" t="s">
+      <c r="A56" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="B56" s="23" t="s">
+      <c r="B56" s="27" t="s">
         <v>142</v>
       </c>
-      <c r="C56" s="35" t="s">
+      <c r="C56" s="39" t="s">
         <v>143</v>
       </c>
-      <c r="D56" s="37" t="s">
+      <c r="D56" s="41" t="s">
         <v>144</v>
       </c>
-      <c r="E56" s="33" t="s">
+      <c r="E56" s="37" t="s">
         <v>40</v>
       </c>
-      <c r="F56" s="44" t="s">
+      <c r="F56" s="49" t="s">
         <v>145</v>
       </c>
-      <c r="G56" s="19"/>
-      <c r="H56" s="8" t="s">
+      <c r="G56" s="22"/>
+      <c r="H56" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="57" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A57" s="23" t="s">
+      <c r="A57" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="B57" s="23" t="s">
+      <c r="B57" s="27" t="s">
         <v>146</v>
       </c>
-      <c r="C57" s="35" t="s">
+      <c r="C57" s="39" t="s">
         <v>147</v>
       </c>
-      <c r="D57" s="35" t="s">
+      <c r="D57" s="39" t="s">
         <v>148</v>
       </c>
-      <c r="E57" s="33" t="s">
+      <c r="E57" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="F57" s="44" t="s">
+      <c r="F57" s="49" t="s">
         <v>149</v>
       </c>
-      <c r="G57" s="19" t="s">
+      <c r="G57" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="H57" s="8" t="s">
+      <c r="H57" s="25" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A58" s="62" t="s">
+      <c r="A58" s="67" t="s">
         <v>150</v>
       </c>
-      <c r="B58" s="62" t="s">
+      <c r="B58" s="67" t="s">
         <v>150</v>
       </c>
-      <c r="C58" s="34" t="s">
+      <c r="C58" s="38" t="s">
         <v>151</v>
       </c>
-      <c r="D58" s="45" t="s">
+      <c r="D58" s="50" t="s">
         <v>152</v>
       </c>
-      <c r="E58" s="63" t="s">
+      <c r="E58" s="68" t="s">
         <v>40</v>
       </c>
-      <c r="F58" s="64" t="s">
+      <c r="F58" s="69" t="s">
         <v>153</v>
       </c>
-      <c r="G58" s="34" t="s">
+      <c r="G58" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="H58" s="46" t="s">
+      <c r="H58" s="51" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="59" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A59" s="47" t="s">
+      <c r="A59" s="52" t="s">
         <v>154</v>
       </c>
-      <c r="B59" s="47" t="s">
+      <c r="B59" s="52" t="s">
         <v>154</v>
       </c>
-      <c r="C59" s="65" t="s">
+      <c r="C59" s="70" t="s">
         <v>155</v>
       </c>
-      <c r="D59" s="57"/>
-      <c r="E59" s="61" t="s">
+      <c r="D59" s="62"/>
+      <c r="E59" s="66" t="s">
         <v>10</v>
       </c>
-      <c r="F59" s="57"/>
-      <c r="G59" s="34" t="s">
+      <c r="F59" s="62"/>
+      <c r="G59" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="H59" s="58" t="s">
+      <c r="H59" s="63" t="s">
         <v>13</v>
       </c>
     </row>
@@ -3430,710 +3302,690 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.2" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="11.7019230769231" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7019230769231" style="1" customWidth="1"/>
-    <col min="3" max="3" width="40" style="1" customWidth="1"/>
-    <col min="4" max="4" width="41.4519230769231" style="1" customWidth="1"/>
-    <col min="5" max="5" width="62" style="1" customWidth="1"/>
+    <col min="1" max="2" width="19.3942307692308" style="1" customWidth="1"/>
+    <col min="3" max="3" width="40" style="2" customWidth="1"/>
+    <col min="4" max="4" width="41.4519230769231" style="2" customWidth="1"/>
+    <col min="5" max="5" width="62" style="2" customWidth="1"/>
     <col min="6" max="6" width="7.70192307692308" style="1" customWidth="1"/>
     <col min="7" max="7" width="10" style="1" customWidth="1"/>
     <col min="8" max="8" width="9.70192307692308" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="9" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:8">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" ht="51" customHeight="1" spans="1:8">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="6" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="3" ht="84" customHeight="1" spans="1:8">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="5" t="s">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="6" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1" spans="1:8">
-      <c r="A4" s="6"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="5" t="s">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
     </row>
     <row r="5" ht="51" customHeight="1" spans="1:8">
-      <c r="A5" s="6"/>
-      <c r="B5" s="3" t="s">
+      <c r="A5" s="8"/>
+      <c r="B5" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="6" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="6" ht="51" customHeight="1" spans="1:8">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="5" t="s">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="6" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="7" ht="56" customHeight="1" spans="1:8">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="5" t="s">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="H7" s="6"/>
+      <c r="H7" s="8"/>
     </row>
     <row r="8" ht="84" customHeight="1" spans="1:8">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="5" t="s">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="G8" s="7"/>
-      <c r="H8" s="6"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="8"/>
     </row>
     <row r="9" ht="112" customHeight="1" spans="1:8">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="5" t="s">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
     </row>
     <row r="10" ht="171" customHeight="1" spans="1:8">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="5" t="s">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" ht="56" customHeight="1" spans="1:8">
-      <c r="A11" s="6"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="10" t="s">
+      <c r="A11" s="8"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10" t="s">
+      <c r="D11" s="12"/>
+      <c r="E11" s="12" t="s">
         <v>190</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H11" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="12" ht="81" customHeight="1" spans="1:8">
-      <c r="A12" s="6"/>
-      <c r="B12" s="11" t="s">
+      <c r="A12" s="8"/>
+      <c r="B12" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="6" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="13" ht="96" customHeight="1" spans="1:8">
-      <c r="A13" s="6"/>
-      <c r="B13" s="4" t="s">
+      <c r="A13" s="8"/>
+      <c r="B13" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="H13" s="6" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="14" ht="111" customHeight="1" spans="1:8">
-      <c r="A14" s="6"/>
-      <c r="B14" s="4" t="s">
+      <c r="A14" s="8"/>
+      <c r="B14" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H14" s="6" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="15" ht="51" customHeight="1" spans="1:8">
-      <c r="A15" s="6"/>
-      <c r="B15" s="4" t="s">
+      <c r="A15" s="8"/>
+      <c r="B15" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="H15" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" ht="126" customHeight="1" spans="1:8">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" ht="66" customHeight="1" spans="1:8">
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" ht="96" customHeight="1" spans="1:8">
+      <c r="A18" s="8"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" ht="111" customHeight="1" spans="1:8">
+      <c r="A19" s="8"/>
+      <c r="B19" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" ht="96" customHeight="1" spans="1:8">
+      <c r="A20" s="8"/>
+      <c r="B20" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H20" s="6" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="16" ht="126" customHeight="1" spans="1:8">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="F16" s="4" t="s">
+    <row r="21" ht="51" customHeight="1" spans="1:8">
+      <c r="A21" s="8"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="22" ht="96" customHeight="1" spans="1:8">
+      <c r="A22" s="8"/>
+      <c r="B22" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="F22" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G22" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H22" s="6" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="17" ht="66" customHeight="1" spans="1:8">
-      <c r="A17" s="6"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="F17" s="4" t="s">
+    <row r="23" ht="81" customHeight="1" spans="1:8">
+      <c r="A23" s="8"/>
+      <c r="B23" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="F23" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G23" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="24" ht="126" customHeight="1" spans="1:8">
+      <c r="A24" s="8"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G24" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="H17" s="6"/>
-    </row>
-    <row r="18" ht="96" customHeight="1" spans="1:8">
-      <c r="A18" s="6"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-    </row>
-    <row r="19" ht="111" customHeight="1" spans="1:8">
-      <c r="A19" s="6"/>
-      <c r="B19" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="F19" s="4" t="s">
+      <c r="H24" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="25" ht="96" customHeight="1" spans="1:8">
+      <c r="A25" s="8"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="F25" s="9"/>
+      <c r="G25" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H25" s="9"/>
+    </row>
+    <row r="26" ht="171" customHeight="1" spans="1:8">
+      <c r="A26" s="8"/>
+      <c r="B26" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="27" ht="126" customHeight="1" spans="1:8">
+      <c r="A27" s="8"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="28" ht="81" customHeight="1" spans="1:8">
+      <c r="A28" s="8"/>
+      <c r="B28" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="F28" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="G19" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H19" s="4" t="s">
+      <c r="G28" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" ht="66" customHeight="1" spans="1:8">
-      <c r="A20" s="6"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="F20" s="4" t="s">
+    <row r="29" ht="81" customHeight="1" spans="1:8">
+      <c r="A29" s="9"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="F29" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G20" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H20" s="4" t="s">
+      <c r="G29" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="H29" s="6" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="21" ht="96" customHeight="1" spans="1:8">
-      <c r="A21" s="6"/>
-      <c r="B21" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="22" ht="51" customHeight="1" spans="1:8">
-      <c r="A22" s="6"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="23" ht="96" customHeight="1" spans="1:8">
-      <c r="A23" s="6"/>
-      <c r="B23" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="24" ht="81" customHeight="1" spans="1:8">
-      <c r="A24" s="6"/>
-      <c r="B24" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="25" ht="126" customHeight="1" spans="1:8">
-      <c r="A25" s="6"/>
-      <c r="B25" s="6"/>
-      <c r="C25" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H25" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="26" ht="96" customHeight="1" spans="1:8">
-      <c r="A26" s="6"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="F26" s="7"/>
-      <c r="G26" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="H26" s="7"/>
-    </row>
-    <row r="27" ht="171" customHeight="1" spans="1:8">
-      <c r="A27" s="6"/>
-      <c r="B27" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H27" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="28" ht="126" customHeight="1" spans="1:8">
-      <c r="A28" s="6"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="5" t="s">
-        <v>249</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H28" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="29" ht="81" customHeight="1" spans="1:8">
-      <c r="A29" s="6"/>
-      <c r="B29" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="H29" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="30" ht="81" customHeight="1" spans="1:8">
-      <c r="A30" s="7"/>
-      <c r="B30" s="7"/>
-      <c r="C30" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>258</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="H30" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="A2:A30"/>
+  <mergeCells count="15">
+    <mergeCell ref="A2:A29"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="B5:B11"/>
     <mergeCell ref="B15:B18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B28:B29"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F24:F25"/>
     <mergeCell ref="G3:G4"/>
     <mergeCell ref="G8:G9"/>
-    <mergeCell ref="G17:G18"/>
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="H6:H9"/>
-    <mergeCell ref="H16:H18"/>
-    <mergeCell ref="H25:H26"/>
+    <mergeCell ref="H24:H25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: update PA project detail excel file
update the project details excel spreadsheet with latest changes
</commit_message>
<xml_diff>
--- a/PA替代需求列表.xlsx
+++ b/PA替代需求列表.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="300">
   <si>
     <t>一级需求</t>
   </si>
@@ -736,7 +736,7 @@
     <t>PA隧道检测策略可选启用：超过最大隧道检测级别的封装数据包丢弃（PA Web帮助p174）；天融信手册无对应选项（检索无命中）</t>
   </si>
   <si>
-    <t>支持解封装内层流量的独立安全区域映射与策略匹配</t>
+    <t>支持解配置内层流量的独立安全区域映射与策略匹配</t>
   </si>
   <si>
     <t>内层流量独立分配至指定的隧道源安全区域与隧道目的安全区域，实现隧道内层流量与原始外层流量的安全策略解耦与独立匹配</t>
@@ -754,7 +754,7 @@
     <t>经安全检测引擎处理完毕后，将响应流量自动重新封装并原路送回初始 VTEP 端点</t>
   </si>
   <si>
-    <t>应用覆盖(App Override)</t>
+    <t>应用覆盖</t>
   </si>
   <si>
     <t>支持应用替代流量跳过七层检测等效配置</t>
@@ -766,24 +766,6 @@
     <t>PA应用替代策略明确绕过第7层处理与威胁检查，改用第4层状态检查以加速（PA管理指南p1307）；天融信自定义应用加入规则库后仍默认经安全引擎检测（天融信手册《自定义应用》页）；迁移评估项：PA应用替代多为私有大流量业务加速，转换时需同步关闭对应策略的IPS/七层检测，否则性能被拖垮或误阻断</t>
   </si>
   <si>
-    <t>支持基于源/目的区域、地址、协议/端口的应用替代策略匹配</t>
-  </si>
-  <si>
-    <t>在源/目标选项卡配置区域和地址，在协议/应用程序选项卡配置 TCP/UDP 端口范围及替代后的应用名称</t>
-  </si>
-  <si>
-    <t>支持强制识别为指定应用并绕过 App-ID 深度检测</t>
-  </si>
-  <si>
-    <t>匹配流量不再经过常规 App-ID 七层解码，直接按指定应用名处理</t>
-  </si>
-  <si>
-    <t>支持应用替代流量仅执行四层状态检测（跳过七层威胁检测）</t>
-  </si>
-  <si>
-    <t>应用替代后的流量仅做 L4 状态转发，不触发 IPS/Threat/URL 等七层安全配置文件检测</t>
-  </si>
-  <si>
     <t>身份验证(Authentication)</t>
   </si>
   <si>
@@ -796,24 +778,15 @@
     <t>PA支持认证超时减少重复质询、Kerberos/SAML/RADIUS等对接（PA Web帮助p186）；天融信手册检索认证超时/单点登录/SSO无命中（仅在线用户在线时长查看与强制下线）；迁移评估项：需核实天融信认证会话有效期配置与SSO对接能力</t>
   </si>
   <si>
-    <t>支持流量策略触发多因素认证质询（MFA Enforcement）</t>
-  </si>
-  <si>
-    <t>流量策略匹配触发MFA质询（非登录场景，MFA供应商API/RADIUS）</t>
+    <t>支持基于应用与流量策略触发的业务级MF 质询</t>
+  </si>
+  <si>
+    <t>根据安全策略直接对高敏感业务流量触发 MFA 质询</t>
   </si>
   <si>
     <t>PA身份验证策略通过Authentication Enforcement对象对匹配流量强制质询，支持多因素身份验证（每因素独立超时，防火墙记录时间戳），MFA供应商API/RADIUS对接（PA Web帮助p185-186、p310、p735-742）；天融信双因子认证（密码+短信/证书/Ukey）仅限管理员/用户登录场景（天融信手册《登录安全策略》页），无流量策略触发MFA质询</t>
   </si>
   <si>
-    <t>支持User-ID动态映射时效性等效（AD日志毫秒级更新）</t>
-  </si>
-  <si>
-    <t>AD域事件日志毫秒级IP-用户映射更新</t>
-  </si>
-  <si>
-    <t>PA无代理架构通过读取域控事件日志实现IP-用户毫秒级动态映射，大规模部署有专项规划（PA管理指南p866-867）；天融信AD对接的轮询间隔与并发认证能力手册未量化；迁移评估项：数万AD用户且移动频繁场景需实测天融信映射更新时延，避免基于用户的策略出现间歇性未授权拦截</t>
-  </si>
-  <si>
     <t>支持身份验证策略规则的多维匹配与 Enforcement 对象</t>
   </si>
   <si>
@@ -823,34 +796,16 @@
     <t>PA身份验证策略支持源/目的区域、地址、用户、HIP等多维匹配，并绑定Authentication Enforcement对象指定认证方式与MFA供应商（PA Web帮助p182-186）；天融信无独立认证策略库，认证绑定于用户访问策略与门户认证（天融信手册《管理用户》页）；对应矩阵#35</t>
   </si>
   <si>
-    <t>支持多种身份验证协议与级联认证</t>
-  </si>
-  <si>
-    <t>Authentication Profile 支持 LDAP、RADIUS、TACACS+、Kerberos、SAML、Local DB、MFA；Authentication Sequence 支持多源级联</t>
-  </si>
-  <si>
-    <t>PA Authentication Profile支持LDAP/RADIUS/TACACS+/Kerberos/SAML/本地/MFA，Authentication Sequence支持多源级联认证（PA Web帮助p182-186）；天融信联动外部认证服务器支持RADIUS/LDAP/TACACS（天融信手册《用户管理》页），SAML对接与多源级联认证手册未见；部分支持</t>
-  </si>
-  <si>
-    <t>支持 User-ID IP-用户映射多源采集</t>
-  </si>
-  <si>
-    <t>支持 AD 安全日志、Syslog、XML API、WMI、DHCP 日志、TS Agent、VM 信息源等多渠道映射</t>
-  </si>
-  <si>
-    <t>PA User-ID支持AD安全日志/Syslog/XML API/WMI/DHCP日志/TS Agent等多源IP-用户映射采集（PA管理指南p866起）；天融信用户认证经AD/LDAP/RADIUS联动实现（天融信手册《用户管理》《添加Radius服务器》页），XML API/WMI/TS Agent等多源采集机制手册未见；部分支持</t>
-  </si>
-  <si>
-    <t>支持认证门户与超时控制</t>
-  </si>
-  <si>
-    <t>未认证流量重定向至 Captive Portal；支持 Authentication Timeout 与 Idle Timeout</t>
-  </si>
-  <si>
-    <t>支持 User-ID 动态映射时效性与可信源过滤</t>
-  </si>
-  <si>
-    <t>支持 IP-用户映射老化时间配置；支持 Trusted Source Address 过滤无效映射（p884）</t>
+    <t>支持 IP-用户映射的可信源地址过滤</t>
+  </si>
+  <si>
+    <t>配置可信源地址（Trusted Source Address）白名单，仅允许指定的域控、日志服务器或 Agent 提交 IP-用户映射关系，自动识别并过滤来自代理设备（Proxy/NAT）或非授权日志源的无效映射</t>
+  </si>
+  <si>
+    <t>支持 IP-用户映射关系的独立老化控制</t>
+  </si>
+  <si>
+    <t>对动态采集的 IP-用户映射关系配置独立的老化超时时间（Mapping Timeout），支持根据用户离线或超时事件自动清空映射表项，防止 IP 重用导致的身份误判。</t>
   </si>
   <si>
     <t>DoS防护(DoS Protection)</t>
@@ -1884,7 +1839,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1959,9 +1914,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1974,30 +1926,30 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -2633,95 +2585,95 @@
   <dimension ref="A1:H59"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.2" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="11.7115384615385" style="54" customWidth="1"/>
-    <col min="2" max="2" width="19.7115384615385" style="54" customWidth="1"/>
-    <col min="3" max="3" width="54.7115384615385" style="54" customWidth="1"/>
-    <col min="4" max="4" width="45.2884615384615" style="54" customWidth="1"/>
-    <col min="5" max="5" width="7.71153846153846" style="54" customWidth="1"/>
-    <col min="6" max="6" width="37.8557692307692" style="54" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="9.71153846153846" style="54" customWidth="1"/>
-    <col min="8" max="8" width="9.71153846153846" style="55" customWidth="1"/>
+    <col min="1" max="1" width="11.7115384615385" style="53" customWidth="1"/>
+    <col min="2" max="2" width="19.7115384615385" style="53" customWidth="1"/>
+    <col min="3" max="3" width="54.7115384615385" style="53" customWidth="1"/>
+    <col min="4" max="4" width="45.2884615384615" style="53" customWidth="1"/>
+    <col min="5" max="5" width="7.71153846153846" style="53" customWidth="1"/>
+    <col min="6" max="6" width="37.8557692307692" style="53" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="9.71153846153846" style="53" customWidth="1"/>
+    <col min="8" max="8" width="9.71153846153846" style="54" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="57" t="s">
+      <c r="C1" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="57" t="s">
+      <c r="D1" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="58" t="s">
+      <c r="E1" s="57" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="58"/>
-      <c r="G1" s="57" t="s">
+      <c r="F1" s="57"/>
+      <c r="G1" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="57" t="s">
+      <c r="H1" s="56" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="60" t="s">
+      <c r="B2" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="61" t="s">
+      <c r="C2" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="61"/>
-      <c r="E2" s="62" t="s">
+      <c r="D2" s="60"/>
+      <c r="E2" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="63" t="s">
+      <c r="F2" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="61" t="s">
+      <c r="G2" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="37" t="s">
+      <c r="H2" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1" spans="1:8">
       <c r="A3" s="11"/>
-      <c r="B3" s="60" t="s">
+      <c r="B3" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="61" t="s">
+      <c r="C3" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="61" t="s">
+      <c r="D3" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="62" t="s">
+      <c r="E3" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="64" t="s">
+      <c r="F3" s="63" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="61" t="s">
+      <c r="G3" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="37" t="s">
+      <c r="H3" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1" spans="1:8">
       <c r="A4" s="11"/>
       <c r="B4" s="11"/>
-      <c r="C4" s="61" t="s">
+      <c r="C4" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="61" t="s">
+      <c r="D4" s="60" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="11"/>
@@ -2732,10 +2684,10 @@
     <row r="5" ht="36" customHeight="1" spans="1:8">
       <c r="A5" s="11"/>
       <c r="B5" s="12"/>
-      <c r="C5" s="61" t="s">
+      <c r="C5" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="61" t="s">
+      <c r="D5" s="60" t="s">
         <v>21</v>
       </c>
       <c r="E5" s="12"/>
@@ -2745,35 +2697,35 @@
     </row>
     <row r="6" ht="14.25" customHeight="1" spans="1:8">
       <c r="A6" s="11"/>
-      <c r="B6" s="65" t="s">
+      <c r="B6" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="61" t="s">
+      <c r="C6" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="61" t="s">
+      <c r="D6" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="62" t="s">
+      <c r="E6" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="63" t="s">
+      <c r="F6" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="61" t="s">
+      <c r="G6" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="37" t="s">
+      <c r="H6" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1" spans="1:8">
       <c r="A7" s="11"/>
       <c r="B7" s="11"/>
-      <c r="C7" s="61" t="s">
+      <c r="C7" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="61" t="s">
+      <c r="D7" s="60" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="11"/>
@@ -2784,10 +2736,10 @@
     <row r="8" ht="14.25" customHeight="1" spans="1:8">
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
-      <c r="C8" s="61" t="s">
+      <c r="C8" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="61" t="s">
+      <c r="D8" s="60" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="11"/>
@@ -2798,10 +2750,10 @@
     <row r="9" ht="14.25" customHeight="1" spans="1:8">
       <c r="A9" s="11"/>
       <c r="B9" s="11"/>
-      <c r="C9" s="61" t="s">
+      <c r="C9" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="61" t="s">
+      <c r="D9" s="60" t="s">
         <v>24</v>
       </c>
       <c r="E9" s="11"/>
@@ -2812,10 +2764,10 @@
     <row r="10" ht="14.25" customHeight="1" spans="1:8">
       <c r="A10" s="11"/>
       <c r="B10" s="11"/>
-      <c r="C10" s="61" t="s">
+      <c r="C10" s="60" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="61"/>
+      <c r="D10" s="60"/>
       <c r="E10" s="11"/>
       <c r="F10" s="11"/>
       <c r="G10" s="11"/>
@@ -2824,10 +2776,10 @@
     <row r="11" ht="14.25" customHeight="1" spans="1:8">
       <c r="A11" s="11"/>
       <c r="B11" s="11"/>
-      <c r="C11" s="61" t="s">
+      <c r="C11" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="61"/>
+      <c r="D11" s="60"/>
       <c r="E11" s="11"/>
       <c r="F11" s="11"/>
       <c r="G11" s="11"/>
@@ -2836,10 +2788,10 @@
     <row r="12" ht="14.25" customHeight="1" spans="1:8">
       <c r="A12" s="11"/>
       <c r="B12" s="12"/>
-      <c r="C12" s="61" t="s">
+      <c r="C12" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="61"/>
+      <c r="D12" s="60"/>
       <c r="E12" s="12"/>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
@@ -2847,58 +2799,58 @@
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:8">
       <c r="A13" s="12"/>
-      <c r="B13" s="65" t="s">
+      <c r="B13" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="61" t="s">
+      <c r="C13" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="61" t="s">
+      <c r="D13" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="62" t="s">
+      <c r="E13" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="63" t="s">
+      <c r="F13" s="62" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="61" t="s">
+      <c r="G13" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="H13" s="37" t="s">
+      <c r="H13" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A14" s="66" t="s">
+      <c r="A14" s="65" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="67" t="s">
+      <c r="B14" s="66" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="61" t="s">
+      <c r="C14" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="37" t="s">
+      <c r="D14" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="62" t="s">
+      <c r="E14" s="61" t="s">
         <v>40</v>
       </c>
-      <c r="F14" s="63" t="s">
+      <c r="F14" s="62" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="61" t="s">
+      <c r="G14" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="H14" s="37" t="s">
+      <c r="H14" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1" spans="1:8">
       <c r="A15" s="14"/>
       <c r="B15" s="11"/>
-      <c r="C15" s="61" t="s">
+      <c r="C15" s="60" t="s">
         <v>43</v>
       </c>
       <c r="D15" s="11"/>
@@ -2910,7 +2862,7 @@
     <row r="16" ht="14.25" customHeight="1" spans="1:8">
       <c r="A16" s="14"/>
       <c r="B16" s="11"/>
-      <c r="C16" s="61" t="s">
+      <c r="C16" s="60" t="s">
         <v>44</v>
       </c>
       <c r="D16" s="11"/>
@@ -2922,7 +2874,7 @@
     <row r="17" ht="14.25" customHeight="1" spans="1:8">
       <c r="A17" s="14"/>
       <c r="B17" s="11"/>
-      <c r="C17" s="61" t="s">
+      <c r="C17" s="60" t="s">
         <v>45</v>
       </c>
       <c r="D17" s="11"/>
@@ -2934,7 +2886,7 @@
     <row r="18" ht="14.25" customHeight="1" spans="1:8">
       <c r="A18" s="14"/>
       <c r="B18" s="11"/>
-      <c r="C18" s="61" t="s">
+      <c r="C18" s="60" t="s">
         <v>46</v>
       </c>
       <c r="D18" s="11"/>
@@ -2946,7 +2898,7 @@
     <row r="19" ht="14.25" customHeight="1" spans="1:8">
       <c r="A19" s="14"/>
       <c r="B19" s="11"/>
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="60" t="s">
         <v>47</v>
       </c>
       <c r="D19" s="11"/>
@@ -2958,7 +2910,7 @@
     <row r="20" ht="14.25" customHeight="1" spans="1:8">
       <c r="A20" s="14"/>
       <c r="B20" s="11"/>
-      <c r="C20" s="61" t="s">
+      <c r="C20" s="60" t="s">
         <v>48</v>
       </c>
       <c r="D20" s="11"/>
@@ -2970,7 +2922,7 @@
     <row r="21" ht="14.25" customHeight="1" spans="1:8">
       <c r="A21" s="14"/>
       <c r="B21" s="11"/>
-      <c r="C21" s="61" t="s">
+      <c r="C21" s="60" t="s">
         <v>49</v>
       </c>
       <c r="D21" s="11"/>
@@ -2982,7 +2934,7 @@
     <row r="22" ht="32.25" customHeight="1" spans="1:8">
       <c r="A22" s="13"/>
       <c r="B22" s="12"/>
-      <c r="C22" s="61" t="s">
+      <c r="C22" s="60" t="s">
         <v>50</v>
       </c>
       <c r="D22" s="12"/>
@@ -2992,125 +2944,125 @@
       <c r="H22" s="12"/>
     </row>
     <row r="23" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A23" s="66" t="s">
+      <c r="A23" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="65" t="s">
+      <c r="B23" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="61" t="s">
+      <c r="C23" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="61" t="s">
+      <c r="D23" s="60" t="s">
         <v>54</v>
       </c>
-      <c r="E23" s="62" t="s">
+      <c r="E23" s="61" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="68" t="s">
+      <c r="F23" s="67" t="s">
         <v>55</v>
       </c>
-      <c r="G23" s="61" t="s">
+      <c r="G23" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H23" s="37" t="s">
+      <c r="H23" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A24" s="66" t="s">
+      <c r="A24" s="65" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="65" t="s">
+      <c r="B24" s="64" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="61" t="s">
+      <c r="C24" s="60" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="61" t="s">
+      <c r="D24" s="60" t="s">
         <v>59</v>
       </c>
-      <c r="E24" s="62" t="s">
+      <c r="E24" s="61" t="s">
         <v>60</v>
       </c>
-      <c r="F24" s="69" t="s">
+      <c r="F24" s="68" t="s">
         <v>61</v>
       </c>
-      <c r="G24" s="61" t="s">
+      <c r="G24" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H24" s="37" t="s">
+      <c r="H24" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A25" s="66" t="s">
+      <c r="A25" s="65" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="65" t="s">
+      <c r="B25" s="64" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="61" t="s">
+      <c r="C25" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="70" t="s">
+      <c r="D25" s="69" t="s">
         <v>65</v>
       </c>
-      <c r="E25" s="62" t="s">
+      <c r="E25" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="F25" s="63" t="s">
+      <c r="F25" s="62" t="s">
         <v>61</v>
       </c>
-      <c r="G25" s="61" t="s">
+      <c r="G25" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H25" s="37" t="s">
+      <c r="H25" s="35" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="26" s="53" customFormat="1" ht="28.5" customHeight="1" spans="1:8">
+    <row r="26" s="52" customFormat="1" ht="28.5" customHeight="1" spans="1:8">
       <c r="A26" s="14"/>
-      <c r="B26" s="65" t="s">
+      <c r="B26" s="64" t="s">
         <v>66</v>
       </c>
-      <c r="C26" s="37" t="s">
+      <c r="C26" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="70"/>
-      <c r="E26" s="71"/>
-      <c r="F26" s="63"/>
-      <c r="G26" s="61"/>
-      <c r="H26" s="37"/>
+      <c r="D26" s="69"/>
+      <c r="E26" s="70"/>
+      <c r="F26" s="62"/>
+      <c r="G26" s="60"/>
+      <c r="H26" s="35"/>
     </row>
     <row r="27" ht="14.25" customHeight="1" spans="1:8">
       <c r="A27" s="14"/>
-      <c r="B27" s="65" t="s">
+      <c r="B27" s="64" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="61" t="s">
+      <c r="C27" s="60" t="s">
         <v>69</v>
       </c>
-      <c r="D27" s="61" t="s">
+      <c r="D27" s="60" t="s">
         <v>70</v>
       </c>
-      <c r="E27" s="62" t="s">
+      <c r="E27" s="61" t="s">
         <v>60</v>
       </c>
-      <c r="F27" s="63" t="s">
+      <c r="F27" s="62" t="s">
         <v>61</v>
       </c>
-      <c r="G27" s="61" t="s">
+      <c r="G27" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H27" s="37" t="s">
+      <c r="H27" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" spans="1:8">
       <c r="A28" s="14"/>
       <c r="B28" s="12"/>
-      <c r="C28" s="61" t="s">
+      <c r="C28" s="60" t="s">
         <v>71</v>
       </c>
       <c r="D28" s="12"/>
@@ -3121,98 +3073,98 @@
     </row>
     <row r="29" ht="60" customHeight="1" spans="1:8">
       <c r="A29" s="14"/>
-      <c r="B29" s="65" t="s">
+      <c r="B29" s="64" t="s">
         <v>72</v>
       </c>
-      <c r="C29" s="61" t="s">
+      <c r="C29" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="D29" s="37" t="s">
+      <c r="D29" s="35" t="s">
         <v>74</v>
       </c>
-      <c r="E29" s="62" t="s">
+      <c r="E29" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="F29" s="72" t="s">
+      <c r="F29" s="71" t="s">
         <v>75</v>
       </c>
-      <c r="G29" s="61" t="s">
+      <c r="G29" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="H29" s="37" t="s">
+      <c r="H29" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" spans="1:8">
       <c r="A30" s="14"/>
       <c r="B30" s="11"/>
-      <c r="C30" s="61" t="s">
+      <c r="C30" s="60" t="s">
         <v>76</v>
       </c>
-      <c r="D30" s="61" t="s">
+      <c r="D30" s="60" t="s">
         <v>77</v>
       </c>
-      <c r="E30" s="62" t="s">
+      <c r="E30" s="61" t="s">
         <v>10</v>
       </c>
       <c r="F30" s="11"/>
-      <c r="G30" s="61" t="s">
+      <c r="G30" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H30" s="37" t="s">
+      <c r="H30" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" spans="1:8">
       <c r="A31" s="13"/>
       <c r="B31" s="12"/>
-      <c r="C31" s="61" t="s">
+      <c r="C31" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="D31" s="61" t="s">
+      <c r="D31" s="60" t="s">
         <v>77</v>
       </c>
-      <c r="E31" s="73" t="s">
+      <c r="E31" s="72" t="s">
         <v>10</v>
       </c>
       <c r="F31" s="12"/>
-      <c r="G31" s="61" t="s">
+      <c r="G31" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H31" s="37" t="s">
+      <c r="H31" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A32" s="66" t="s">
+      <c r="A32" s="65" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="65" t="s">
+      <c r="B32" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="C32" s="61" t="s">
+      <c r="C32" s="60" t="s">
         <v>81</v>
       </c>
-      <c r="D32" s="61" t="s">
+      <c r="D32" s="60" t="s">
         <v>82</v>
       </c>
-      <c r="E32" s="62" t="s">
+      <c r="E32" s="61" t="s">
         <v>60</v>
       </c>
-      <c r="F32" s="63" t="s">
+      <c r="F32" s="62" t="s">
         <v>83</v>
       </c>
-      <c r="G32" s="61" t="s">
+      <c r="G32" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H32" s="37" t="s">
+      <c r="H32" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1" spans="1:8">
       <c r="A33" s="13"/>
       <c r="B33" s="12"/>
-      <c r="C33" s="61" t="s">
+      <c r="C33" s="60" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="12"/>
@@ -3222,36 +3174,36 @@
       <c r="H33" s="12"/>
     </row>
     <row r="34" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A34" s="66" t="s">
+      <c r="A34" s="65" t="s">
         <v>85</v>
       </c>
-      <c r="B34" s="65" t="s">
+      <c r="B34" s="64" t="s">
         <v>86</v>
       </c>
-      <c r="C34" s="61" t="s">
+      <c r="C34" s="60" t="s">
         <v>87</v>
       </c>
-      <c r="D34" s="61"/>
-      <c r="E34" s="62" t="s">
+      <c r="D34" s="60"/>
+      <c r="E34" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="F34" s="63" t="s">
+      <c r="F34" s="62" t="s">
         <v>61</v>
       </c>
-      <c r="G34" s="61" t="s">
+      <c r="G34" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H34" s="37" t="s">
+      <c r="H34" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1" spans="1:8">
       <c r="A35" s="14"/>
       <c r="B35" s="11"/>
-      <c r="C35" s="61" t="s">
+      <c r="C35" s="60" t="s">
         <v>88</v>
       </c>
-      <c r="D35" s="61"/>
+      <c r="D35" s="60"/>
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
       <c r="G35" s="11"/>
@@ -3260,10 +3212,10 @@
     <row r="36" ht="14.25" customHeight="1" spans="1:8">
       <c r="A36" s="14"/>
       <c r="B36" s="11"/>
-      <c r="C36" s="61" t="s">
+      <c r="C36" s="60" t="s">
         <v>89</v>
       </c>
-      <c r="D36" s="61"/>
+      <c r="D36" s="60"/>
       <c r="E36" s="11"/>
       <c r="F36" s="11"/>
       <c r="G36" s="11"/>
@@ -3272,49 +3224,49 @@
     <row r="37" ht="14.25" customHeight="1" spans="1:8">
       <c r="A37" s="13"/>
       <c r="B37" s="12"/>
-      <c r="C37" s="74" t="s">
+      <c r="C37" s="73" t="s">
         <v>90</v>
       </c>
-      <c r="D37" s="74"/>
+      <c r="D37" s="73"/>
       <c r="E37" s="12"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
       <c r="H37" s="12"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A38" s="65" t="s">
+      <c r="A38" s="64" t="s">
         <v>91</v>
       </c>
-      <c r="B38" s="65" t="s">
+      <c r="B38" s="64" t="s">
         <v>92</v>
       </c>
-      <c r="C38" s="75" t="s">
+      <c r="C38" s="74" t="s">
         <v>93</v>
       </c>
-      <c r="D38" s="75"/>
-      <c r="E38" s="73" t="s">
+      <c r="D38" s="74"/>
+      <c r="E38" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="F38" s="76" t="s">
+      <c r="F38" s="75" t="s">
         <v>61</v>
       </c>
-      <c r="G38" s="61" t="s">
+      <c r="G38" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H38" s="37" t="s">
+      <c r="H38" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" spans="1:8">
       <c r="A39" s="11"/>
-      <c r="B39" s="65" t="s">
+      <c r="B39" s="64" t="s">
         <v>94</v>
       </c>
-      <c r="C39" s="75" t="s">
+      <c r="C39" s="74" t="s">
         <v>95</v>
       </c>
-      <c r="D39" s="75"/>
-      <c r="E39" s="73" t="s">
+      <c r="D39" s="74"/>
+      <c r="E39" s="72" t="s">
         <v>60</v>
       </c>
       <c r="F39" s="12"/>
@@ -3323,141 +3275,141 @@
     </row>
     <row r="40" ht="28.5" customHeight="1" spans="1:8">
       <c r="A40" s="11"/>
-      <c r="B40" s="65" t="s">
+      <c r="B40" s="64" t="s">
         <v>96</v>
       </c>
-      <c r="C40" s="75" t="s">
+      <c r="C40" s="74" t="s">
         <v>97</v>
       </c>
-      <c r="D40" s="77" t="s">
+      <c r="D40" s="76" t="s">
         <v>98</v>
       </c>
-      <c r="E40" s="73" t="s">
+      <c r="E40" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="F40" s="72" t="s">
+      <c r="F40" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="G40" s="61" t="s">
+      <c r="G40" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="H40" s="37" t="s">
+      <c r="H40" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" spans="1:8">
       <c r="A41" s="11"/>
-      <c r="B41" s="65" t="s">
+      <c r="B41" s="64" t="s">
         <v>99</v>
       </c>
-      <c r="C41" s="61" t="s">
+      <c r="C41" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="D41" s="75" t="s">
+      <c r="D41" s="74" t="s">
         <v>101</v>
       </c>
-      <c r="E41" s="73" t="s">
+      <c r="E41" s="72" t="s">
         <v>60</v>
       </c>
-      <c r="F41" s="72" t="s">
+      <c r="F41" s="71" t="s">
         <v>102</v>
       </c>
-      <c r="G41" s="61" t="s">
+      <c r="G41" s="60" t="s">
         <v>103</v>
       </c>
-      <c r="H41" s="37" t="s">
+      <c r="H41" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" spans="1:8">
       <c r="A42" s="11"/>
-      <c r="B42" s="65" t="s">
+      <c r="B42" s="64" t="s">
         <v>104</v>
       </c>
-      <c r="C42" s="61" t="s">
+      <c r="C42" s="60" t="s">
         <v>105</v>
       </c>
-      <c r="D42" s="75"/>
-      <c r="E42" s="73"/>
-      <c r="F42" s="72"/>
-      <c r="G42" s="61"/>
-      <c r="H42" s="37"/>
+      <c r="D42" s="74"/>
+      <c r="E42" s="72"/>
+      <c r="F42" s="71"/>
+      <c r="G42" s="60"/>
+      <c r="H42" s="35"/>
     </row>
     <row r="43" ht="15.75" customHeight="1" spans="1:8">
       <c r="A43" s="12"/>
-      <c r="B43" s="65" t="s">
+      <c r="B43" s="64" t="s">
         <v>106</v>
       </c>
-      <c r="C43" s="75" t="s">
+      <c r="C43" s="74" t="s">
         <v>107</v>
       </c>
-      <c r="D43" s="75"/>
-      <c r="E43" s="73" t="s">
+      <c r="D43" s="74"/>
+      <c r="E43" s="72" t="s">
         <v>60</v>
       </c>
-      <c r="F43" s="72" t="s">
+      <c r="F43" s="71" t="s">
         <v>108</v>
       </c>
-      <c r="G43" s="61" t="s">
+      <c r="G43" s="60" t="s">
         <v>109</v>
       </c>
-      <c r="H43" s="37" t="s">
+      <c r="H43" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A44" s="78" t="s">
+      <c r="A44" s="77" t="s">
         <v>110</v>
       </c>
-      <c r="B44" s="79" t="s">
+      <c r="B44" s="78" t="s">
         <v>111</v>
       </c>
-      <c r="C44" s="80" t="s">
+      <c r="C44" s="79" t="s">
         <v>112</v>
       </c>
-      <c r="D44" s="80" t="s">
+      <c r="D44" s="79" t="s">
         <v>113</v>
       </c>
-      <c r="E44" s="81" t="s">
+      <c r="E44" s="80" t="s">
         <v>40</v>
       </c>
-      <c r="F44" s="82" t="s">
+      <c r="F44" s="81" t="s">
         <v>114</v>
       </c>
-      <c r="G44" s="83" t="s">
+      <c r="G44" s="82" t="s">
         <v>35</v>
       </c>
-      <c r="H44" s="39" t="s">
+      <c r="H44" s="38" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1" spans="1:8">
       <c r="A45" s="14"/>
       <c r="B45" s="11"/>
-      <c r="C45" s="75" t="s">
+      <c r="C45" s="74" t="s">
         <v>115</v>
       </c>
-      <c r="D45" s="75" t="s">
+      <c r="D45" s="74" t="s">
         <v>116</v>
       </c>
       <c r="E45" s="11"/>
-      <c r="F45" s="84" t="s">
+      <c r="F45" s="83" t="s">
         <v>61</v>
       </c>
-      <c r="G45" s="61" t="s">
+      <c r="G45" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H45" s="37" t="s">
+      <c r="H45" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" spans="1:8">
       <c r="A46" s="14"/>
       <c r="B46" s="11"/>
-      <c r="C46" s="75" t="s">
+      <c r="C46" s="74" t="s">
         <v>117</v>
       </c>
-      <c r="D46" s="75"/>
+      <c r="D46" s="74"/>
       <c r="E46" s="11"/>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
@@ -3466,284 +3418,284 @@
     <row r="47" ht="14.25" customHeight="1" spans="1:8">
       <c r="A47" s="14"/>
       <c r="B47" s="11"/>
-      <c r="C47" s="75" t="s">
+      <c r="C47" s="74" t="s">
         <v>118</v>
       </c>
-      <c r="D47" s="75"/>
+      <c r="D47" s="74"/>
       <c r="E47" s="11"/>
-      <c r="F47" s="84" t="s">
+      <c r="F47" s="83" t="s">
         <v>61</v>
       </c>
-      <c r="G47" s="61" t="s">
+      <c r="G47" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="H47" s="37" t="s">
+      <c r="H47" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" spans="1:8">
       <c r="A48" s="13"/>
       <c r="B48" s="12"/>
-      <c r="C48" s="85" t="s">
+      <c r="C48" s="84" t="s">
         <v>119</v>
       </c>
-      <c r="D48" s="85"/>
+      <c r="D48" s="84"/>
       <c r="E48" s="12"/>
-      <c r="F48" s="68" t="s">
+      <c r="F48" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="G48" s="74" t="s">
+      <c r="G48" s="73" t="s">
         <v>12</v>
       </c>
-      <c r="H48" s="86" t="s">
+      <c r="H48" s="85" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="49" ht="42.75" customHeight="1" spans="1:8">
-      <c r="A49" s="87" t="s">
+      <c r="A49" s="86" t="s">
         <v>120</v>
       </c>
-      <c r="B49" s="87" t="s">
+      <c r="B49" s="86" t="s">
         <v>120</v>
       </c>
-      <c r="C49" s="88" t="s">
+      <c r="C49" s="87" t="s">
         <v>121</v>
       </c>
-      <c r="D49" s="89" t="s">
+      <c r="D49" s="88" t="s">
         <v>122</v>
       </c>
-      <c r="E49" s="90" t="s">
+      <c r="E49" s="89" t="s">
         <v>40</v>
       </c>
-      <c r="F49" s="91"/>
-      <c r="G49" s="92" t="s">
+      <c r="F49" s="90"/>
+      <c r="G49" s="91" t="s">
         <v>103</v>
       </c>
-      <c r="H49" s="93"/>
+      <c r="H49" s="92"/>
     </row>
     <row r="50" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A50" s="94"/>
-      <c r="B50" s="94"/>
-      <c r="C50" s="88" t="s">
+      <c r="A50" s="93"/>
+      <c r="B50" s="93"/>
+      <c r="C50" s="87" t="s">
         <v>123</v>
       </c>
-      <c r="D50" s="95" t="s">
+      <c r="D50" s="94" t="s">
         <v>124</v>
       </c>
-      <c r="E50" s="96" t="s">
+      <c r="E50" s="95" t="s">
         <v>60</v>
       </c>
-      <c r="F50" s="97"/>
-      <c r="G50" s="92" t="s">
+      <c r="F50" s="96"/>
+      <c r="G50" s="91" t="s">
         <v>103</v>
       </c>
-      <c r="H50" s="98"/>
+      <c r="H50" s="97"/>
     </row>
     <row r="51" ht="14.25" customHeight="1" spans="1:8">
-      <c r="A51" s="94"/>
-      <c r="B51" s="94"/>
-      <c r="C51" s="88" t="s">
+      <c r="A51" s="93"/>
+      <c r="B51" s="93"/>
+      <c r="C51" s="87" t="s">
         <v>125</v>
       </c>
-      <c r="D51" s="99" t="s">
+      <c r="D51" s="98" t="s">
         <v>126</v>
       </c>
-      <c r="E51" s="96" t="s">
+      <c r="E51" s="95" t="s">
         <v>60</v>
       </c>
-      <c r="F51" s="91"/>
-      <c r="G51" s="92" t="s">
+      <c r="F51" s="90"/>
+      <c r="G51" s="91" t="s">
         <v>103</v>
       </c>
-      <c r="H51" s="93"/>
+      <c r="H51" s="92"/>
     </row>
     <row r="52" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A52" s="100"/>
-      <c r="B52" s="100"/>
-      <c r="C52" s="99" t="s">
+      <c r="A52" s="99"/>
+      <c r="B52" s="99"/>
+      <c r="C52" s="98" t="s">
         <v>127</v>
       </c>
-      <c r="D52" s="89" t="s">
+      <c r="D52" s="88" t="s">
         <v>128</v>
       </c>
-      <c r="E52" s="101" t="s">
+      <c r="E52" s="100" t="s">
         <v>10</v>
       </c>
-      <c r="F52" s="91" t="s">
+      <c r="F52" s="90" t="s">
         <v>129</v>
       </c>
-      <c r="G52" s="92" t="s">
+      <c r="G52" s="91" t="s">
         <v>12</v>
       </c>
-      <c r="H52" s="93" t="s">
+      <c r="H52" s="92" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A53" s="79" t="s">
+      <c r="A53" s="78" t="s">
         <v>130</v>
       </c>
-      <c r="B53" s="79" t="s">
+      <c r="B53" s="78" t="s">
         <v>131</v>
       </c>
-      <c r="C53" s="80" t="s">
+      <c r="C53" s="79" t="s">
         <v>132</v>
       </c>
-      <c r="D53" s="80"/>
-      <c r="E53" s="81" t="s">
+      <c r="D53" s="79"/>
+      <c r="E53" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="F53" s="82" t="s">
+      <c r="F53" s="81" t="s">
         <v>61</v>
       </c>
-      <c r="G53" s="83" t="s">
+      <c r="G53" s="82" t="s">
         <v>12</v>
       </c>
-      <c r="H53" s="39" t="s">
+      <c r="H53" s="38" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="54" ht="28.5" customHeight="1" spans="1:8">
       <c r="A54" s="12"/>
-      <c r="B54" s="65" t="s">
+      <c r="B54" s="64" t="s">
         <v>133</v>
       </c>
-      <c r="C54" s="37" t="s">
+      <c r="C54" s="35" t="s">
         <v>134</v>
       </c>
-      <c r="D54" s="77" t="s">
+      <c r="D54" s="76" t="s">
         <v>135</v>
       </c>
-      <c r="E54" s="73" t="s">
+      <c r="E54" s="72" t="s">
         <v>60</v>
       </c>
-      <c r="F54" s="72" t="s">
+      <c r="F54" s="71" t="s">
         <v>136</v>
       </c>
-      <c r="G54" s="61" t="s">
+      <c r="G54" s="60" t="s">
         <v>103</v>
       </c>
-      <c r="H54" s="37" t="s">
+      <c r="H54" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A55" s="66" t="s">
+      <c r="A55" s="65" t="s">
         <v>137</v>
       </c>
-      <c r="B55" s="65" t="s">
+      <c r="B55" s="64" t="s">
         <v>138</v>
       </c>
-      <c r="C55" s="75" t="s">
+      <c r="C55" s="74" t="s">
         <v>139</v>
       </c>
-      <c r="D55" s="75"/>
-      <c r="E55" s="73" t="s">
+      <c r="D55" s="74"/>
+      <c r="E55" s="72" t="s">
         <v>60</v>
       </c>
-      <c r="F55" s="72"/>
-      <c r="G55" s="61" t="s">
+      <c r="F55" s="71"/>
+      <c r="G55" s="60" t="s">
         <v>140</v>
       </c>
-      <c r="H55" s="37" t="s">
+      <c r="H55" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="56" ht="42.75" customHeight="1" spans="1:8">
-      <c r="A56" s="66" t="s">
+      <c r="A56" s="65" t="s">
         <v>141</v>
       </c>
-      <c r="B56" s="65" t="s">
+      <c r="B56" s="64" t="s">
         <v>142</v>
       </c>
-      <c r="C56" s="75" t="s">
+      <c r="C56" s="74" t="s">
         <v>143</v>
       </c>
-      <c r="D56" s="77" t="s">
+      <c r="D56" s="76" t="s">
         <v>144</v>
       </c>
-      <c r="E56" s="73" t="s">
+      <c r="E56" s="72" t="s">
         <v>40</v>
       </c>
-      <c r="F56" s="84" t="s">
+      <c r="F56" s="83" t="s">
         <v>145</v>
       </c>
-      <c r="G56" s="61"/>
-      <c r="H56" s="37" t="s">
+      <c r="G56" s="60"/>
+      <c r="H56" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="57" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A57" s="65" t="s">
+      <c r="A57" s="64" t="s">
         <v>141</v>
       </c>
-      <c r="B57" s="65" t="s">
+      <c r="B57" s="64" t="s">
         <v>146</v>
       </c>
-      <c r="C57" s="75" t="s">
+      <c r="C57" s="74" t="s">
         <v>147</v>
       </c>
-      <c r="D57" s="75" t="s">
+      <c r="D57" s="74" t="s">
         <v>148</v>
       </c>
-      <c r="E57" s="73" t="s">
+      <c r="E57" s="72" t="s">
         <v>60</v>
       </c>
-      <c r="F57" s="84" t="s">
+      <c r="F57" s="83" t="s">
         <v>149</v>
       </c>
-      <c r="G57" s="61" t="s">
+      <c r="G57" s="60" t="s">
         <v>103</v>
       </c>
-      <c r="H57" s="37" t="s">
+      <c r="H57" s="35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1" spans="1:8">
-      <c r="A58" s="102" t="s">
+      <c r="A58" s="101" t="s">
         <v>150</v>
       </c>
-      <c r="B58" s="102" t="s">
+      <c r="B58" s="101" t="s">
         <v>150</v>
       </c>
-      <c r="C58" s="74" t="s">
+      <c r="C58" s="73" t="s">
         <v>151</v>
       </c>
-      <c r="D58" s="85" t="s">
+      <c r="D58" s="84" t="s">
         <v>152</v>
       </c>
-      <c r="E58" s="103" t="s">
+      <c r="E58" s="102" t="s">
         <v>40</v>
       </c>
-      <c r="F58" s="104" t="s">
+      <c r="F58" s="103" t="s">
         <v>153</v>
       </c>
-      <c r="G58" s="74" t="s">
+      <c r="G58" s="73" t="s">
         <v>103</v>
       </c>
-      <c r="H58" s="86" t="s">
+      <c r="H58" s="85" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="59" ht="28.5" customHeight="1" spans="1:8">
-      <c r="A59" s="87" t="s">
+      <c r="A59" s="86" t="s">
         <v>154</v>
       </c>
-      <c r="B59" s="87" t="s">
+      <c r="B59" s="86" t="s">
         <v>154</v>
       </c>
-      <c r="C59" s="105" t="s">
+      <c r="C59" s="104" t="s">
         <v>155</v>
       </c>
-      <c r="D59" s="97"/>
-      <c r="E59" s="101" t="s">
+      <c r="D59" s="96"/>
+      <c r="E59" s="100" t="s">
         <v>10</v>
       </c>
-      <c r="F59" s="97"/>
-      <c r="G59" s="74" t="s">
+      <c r="F59" s="96"/>
+      <c r="G59" s="73" t="s">
         <v>103</v>
       </c>
-      <c r="H59" s="98" t="s">
+      <c r="H59" s="97" t="s">
         <v>13</v>
       </c>
     </row>
@@ -3813,7 +3765,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.2" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="2" width="19.3942307692308" style="2" customWidth="1"/>
@@ -4283,7 +4235,7 @@
         <v>227</v>
       </c>
       <c r="F21" s="21" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>109</v>
@@ -4303,7 +4255,7 @@
         <v>230</v>
       </c>
       <c r="F22" s="21" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="G22" s="8" t="s">
         <v>109</v>
@@ -4320,7 +4272,7 @@
       </c>
       <c r="E23" s="24"/>
       <c r="F23" s="25" t="s">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="G23" s="26" t="s">
         <v>109</v>
@@ -4362,17 +4314,17 @@
     <row r="26" ht="51" customHeight="1" spans="1:8">
       <c r="A26" s="11"/>
       <c r="B26" s="12"/>
-      <c r="C26" s="28" t="s">
+      <c r="C26" s="23" t="s">
         <v>235</v>
       </c>
-      <c r="D26" s="28" t="s">
+      <c r="D26" s="23" t="s">
         <v>236</v>
       </c>
-      <c r="E26" s="29"/>
-      <c r="F26" s="30" t="s">
+      <c r="E26" s="28"/>
+      <c r="F26" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="G26" s="31" t="s">
+      <c r="G26" s="30" t="s">
         <v>109</v>
       </c>
       <c r="H26" s="10" t="s">
@@ -4384,13 +4336,13 @@
       <c r="B27" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="C27" s="32" t="s">
+      <c r="C27" s="31" t="s">
         <v>238</v>
       </c>
-      <c r="D27" s="32" t="s">
+      <c r="D27" s="31" t="s">
         <v>239</v>
       </c>
-      <c r="E27" s="32" t="s">
+      <c r="E27" s="31" t="s">
         <v>240</v>
       </c>
       <c r="F27" s="16" t="s">
@@ -4401,514 +4353,413 @@
       </c>
       <c r="H27" s="10"/>
     </row>
-    <row r="28" ht="51" customHeight="1" spans="1:8">
+    <row r="28" ht="126" customHeight="1" spans="1:8">
       <c r="A28" s="11"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="33" t="s">
+      <c r="B28" s="32" t="s">
         <v>241</v>
       </c>
-      <c r="D28" s="33" t="s">
+      <c r="C28" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="E28" s="9"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="10"/>
-    </row>
-    <row r="29" ht="51" customHeight="1" spans="1:8">
+      <c r="D28" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="H28" s="33" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="29" ht="126" customHeight="1" spans="1:8">
       <c r="A29" s="11"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="33" t="s">
-        <v>243</v>
-      </c>
-      <c r="D29" s="33" t="s">
-        <v>244</v>
-      </c>
-      <c r="E29" s="9"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="10"/>
-    </row>
-    <row r="30" ht="81" customHeight="1" spans="1:8">
+      <c r="B29" s="34"/>
+      <c r="C29" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="F29" s="35" t="s">
+        <v>10</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="H29" s="36"/>
+    </row>
+    <row r="30" ht="74" customHeight="1" spans="1:8">
       <c r="A30" s="11"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="33" t="s">
-        <v>245</v>
-      </c>
-      <c r="D30" s="33" t="s">
-        <v>246</v>
-      </c>
-      <c r="E30" s="9"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="10"/>
-    </row>
-    <row r="31" ht="126" customHeight="1" spans="1:8">
+      <c r="B30" s="34"/>
+      <c r="C30" s="37" t="s">
+        <v>248</v>
+      </c>
+      <c r="D30" s="37" t="s">
+        <v>249</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="F30" s="38" t="s">
+        <v>10</v>
+      </c>
+      <c r="G30" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="H30" s="39"/>
+    </row>
+    <row r="31" ht="96" customHeight="1" spans="1:8">
       <c r="A31" s="11"/>
-      <c r="B31" s="34" t="s">
-        <v>247</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>248</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>249</v>
-      </c>
-      <c r="E31" s="9" t="s">
-        <v>250</v>
-      </c>
-      <c r="F31" s="8" t="s">
+      <c r="B31" s="34"/>
+      <c r="C31" s="37" t="s">
+        <v>251</v>
+      </c>
+      <c r="D31" s="37" t="s">
+        <v>252</v>
+      </c>
+      <c r="E31" s="9"/>
+      <c r="F31" s="38"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="36"/>
+    </row>
+    <row r="32" ht="96" customHeight="1" spans="1:8">
+      <c r="A32" s="11"/>
+      <c r="B32" s="34"/>
+      <c r="C32" s="40" t="s">
+        <v>253</v>
+      </c>
+      <c r="D32" s="37" t="s">
+        <v>254</v>
+      </c>
+      <c r="E32" s="9"/>
+      <c r="F32" s="38"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="36"/>
+    </row>
+    <row r="33" ht="117" customHeight="1" spans="1:8">
+      <c r="A33" s="11"/>
+      <c r="B33" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="C33" s="41" t="s">
+        <v>256</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="H33" s="16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34" ht="96" customHeight="1" spans="1:8">
+      <c r="A34" s="11"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="41" t="s">
+        <v>259</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="F34" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G31" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="H31" s="35" t="s">
+      <c r="G34" s="9" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="32" ht="126" customHeight="1" spans="1:8">
-      <c r="A32" s="11"/>
-      <c r="B32" s="36"/>
-      <c r="C32" s="9" t="s">
-        <v>251</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="E32" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="F32" s="37" t="s">
+      <c r="H34" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35" ht="96" customHeight="1" spans="1:8">
+      <c r="A35" s="11"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="40" t="s">
+        <v>262</v>
+      </c>
+      <c r="D35" s="37" t="s">
+        <v>263</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="H35" s="8"/>
+    </row>
+    <row r="36" ht="171" customHeight="1" spans="1:8">
+      <c r="A36" s="11"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="40" t="s">
+        <v>265</v>
+      </c>
+      <c r="D36" s="37" t="s">
+        <v>266</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G36" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="H36" s="21"/>
+    </row>
+    <row r="37" ht="126" customHeight="1" spans="1:8">
+      <c r="A37" s="11"/>
+      <c r="B37" s="42" t="s">
+        <v>268</v>
+      </c>
+      <c r="C37" s="43" t="s">
+        <v>269</v>
+      </c>
+      <c r="D37" s="43" t="s">
+        <v>270</v>
+      </c>
+      <c r="E37" s="43" t="s">
+        <v>271</v>
+      </c>
+      <c r="F37" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="G32" s="10" t="s">
+      <c r="G37" s="45" t="s">
         <v>109</v>
       </c>
-      <c r="H32" s="38"/>
-    </row>
-    <row r="33" ht="69" customHeight="1" spans="1:8">
-      <c r="A33" s="11"/>
-      <c r="B33" s="36"/>
-      <c r="C33" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="E33" s="9" t="s">
-        <v>256</v>
-      </c>
-      <c r="F33" s="39"/>
-      <c r="G33" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="H33" s="40"/>
-    </row>
-    <row r="34" ht="74" customHeight="1" spans="1:8">
-      <c r="A34" s="11"/>
-      <c r="B34" s="36"/>
-      <c r="C34" s="33" t="s">
-        <v>257</v>
-      </c>
-      <c r="D34" s="33" t="s">
-        <v>258</v>
-      </c>
-      <c r="E34" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="F34" s="39" t="s">
+      <c r="H37" s="46" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="38" ht="81" customHeight="1" spans="1:8">
+      <c r="A38" s="11"/>
+      <c r="B38" s="42"/>
+      <c r="C38" s="43" t="s">
+        <v>272</v>
+      </c>
+      <c r="D38" s="43" t="s">
+        <v>273</v>
+      </c>
+      <c r="E38" s="43" t="s">
+        <v>274</v>
+      </c>
+      <c r="F38" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="G34" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="H34" s="40"/>
-    </row>
-    <row r="35" ht="54" customHeight="1" spans="1:8">
-      <c r="A35" s="11"/>
-      <c r="B35" s="36"/>
-      <c r="C35" s="33" t="s">
-        <v>260</v>
-      </c>
-      <c r="D35" s="33" t="s">
-        <v>261</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>262</v>
-      </c>
-      <c r="F35" s="39" t="s">
-        <v>10</v>
-      </c>
-      <c r="G35" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="H35" s="40"/>
-    </row>
-    <row r="36" ht="47" customHeight="1" spans="1:8">
-      <c r="A36" s="11"/>
-      <c r="B36" s="36"/>
-      <c r="C36" s="33" t="s">
-        <v>263</v>
-      </c>
-      <c r="D36" s="33" t="s">
-        <v>264</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>265</v>
-      </c>
-      <c r="F36" s="39" t="s">
-        <v>10</v>
-      </c>
-      <c r="G36" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="H36" s="40"/>
-    </row>
-    <row r="37" ht="47" customHeight="1" spans="1:8">
-      <c r="A37" s="11"/>
-      <c r="B37" s="36"/>
-      <c r="C37" s="33" t="s">
-        <v>266</v>
-      </c>
-      <c r="D37" s="33" t="s">
-        <v>267</v>
-      </c>
-      <c r="E37" s="9"/>
-      <c r="F37" s="39"/>
-      <c r="G37" s="10"/>
-      <c r="H37" s="40"/>
-    </row>
-    <row r="38" ht="96" customHeight="1" spans="1:8">
-      <c r="A38" s="11"/>
-      <c r="B38" s="36"/>
-      <c r="C38" s="33" t="s">
-        <v>268</v>
-      </c>
-      <c r="D38" s="33" t="s">
-        <v>269</v>
-      </c>
-      <c r="E38" s="9"/>
-      <c r="F38" s="39"/>
-      <c r="G38" s="10"/>
-      <c r="H38" s="38"/>
-    </row>
-    <row r="39" ht="117" customHeight="1" spans="1:8">
+      <c r="G38" s="45" t="s">
+        <v>109</v>
+      </c>
+      <c r="H38" s="46" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="39" ht="81" customHeight="1" spans="1:8">
       <c r="A39" s="11"/>
-      <c r="B39" s="7" t="s">
-        <v>270</v>
+      <c r="B39" s="36" t="s">
+        <v>275</v>
       </c>
       <c r="C39" s="41" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="F39" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="G39" s="9" t="s">
+      <c r="G39" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="H39" s="29" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" ht="68" customHeight="1" spans="1:8">
+      <c r="A40" s="11"/>
+      <c r="B40" s="39"/>
+      <c r="C40" s="47" t="s">
+        <v>279</v>
+      </c>
+      <c r="D40" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="E40" s="20" t="s">
+        <v>281</v>
+      </c>
+      <c r="F40" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="G40" s="48" t="s">
+        <v>188</v>
+      </c>
+      <c r="H40" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="H39" s="16" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="40" ht="96" customHeight="1" spans="1:8">
-      <c r="A40" s="11"/>
-      <c r="B40" s="11"/>
-      <c r="C40" s="41" t="s">
-        <v>274</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>275</v>
-      </c>
-      <c r="E40" s="9" t="s">
-        <v>276</v>
-      </c>
-      <c r="F40" s="8" t="s">
+    </row>
+    <row r="41" ht="51" customHeight="1" spans="1:8">
+      <c r="A41" s="11"/>
+      <c r="B41" s="39"/>
+      <c r="C41" s="49" t="s">
+        <v>282</v>
+      </c>
+      <c r="D41" s="50" t="s">
+        <v>283</v>
+      </c>
+      <c r="E41" s="49" t="s">
+        <v>284</v>
+      </c>
+      <c r="F41" s="51" t="s">
         <v>10</v>
       </c>
-      <c r="G40" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="H40" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="41" ht="96" customHeight="1" spans="1:8">
-      <c r="A41" s="11"/>
-      <c r="B41" s="11"/>
-      <c r="C41" s="42" t="s">
-        <v>277</v>
-      </c>
-      <c r="D41" s="33" t="s">
-        <v>278</v>
-      </c>
-      <c r="E41" s="9" t="s">
-        <v>279</v>
-      </c>
-      <c r="F41" s="8" t="s">
+      <c r="G41" s="51" t="s">
+        <v>109</v>
+      </c>
+      <c r="H41" s="51"/>
+    </row>
+    <row r="42" ht="68" customHeight="1" spans="1:8">
+      <c r="A42" s="11"/>
+      <c r="B42" s="39"/>
+      <c r="C42" s="49" t="s">
+        <v>285</v>
+      </c>
+      <c r="D42" s="50" t="s">
+        <v>286</v>
+      </c>
+      <c r="E42" s="49" t="s">
+        <v>287</v>
+      </c>
+      <c r="F42" s="51" t="s">
+        <v>10</v>
+      </c>
+      <c r="G42" s="51" t="s">
+        <v>109</v>
+      </c>
+      <c r="H42" s="51"/>
+    </row>
+    <row r="43" ht="51" customHeight="1" spans="1:8">
+      <c r="A43" s="11"/>
+      <c r="B43" s="39"/>
+      <c r="C43" s="49" t="s">
+        <v>288</v>
+      </c>
+      <c r="D43" s="50" t="s">
+        <v>289</v>
+      </c>
+      <c r="E43" s="49" t="s">
+        <v>290</v>
+      </c>
+      <c r="F43" s="51" t="s">
+        <v>10</v>
+      </c>
+      <c r="G43" s="51" t="s">
+        <v>109</v>
+      </c>
+      <c r="H43" s="51"/>
+    </row>
+    <row r="44" ht="84" customHeight="1" spans="1:8">
+      <c r="A44" s="11"/>
+      <c r="B44" s="39"/>
+      <c r="C44" s="49" t="s">
+        <v>291</v>
+      </c>
+      <c r="D44" s="50" t="s">
+        <v>292</v>
+      </c>
+      <c r="E44" s="49" t="s">
+        <v>293</v>
+      </c>
+      <c r="F44" s="51" t="s">
         <v>60</v>
       </c>
-      <c r="G41" s="9" t="s">
+      <c r="G44" s="51" t="s">
         <v>188</v>
       </c>
-      <c r="H41" s="8"/>
-    </row>
-    <row r="42" ht="171" customHeight="1" spans="1:8">
-      <c r="A42" s="11"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="42" t="s">
-        <v>280</v>
-      </c>
-      <c r="D42" s="33" t="s">
-        <v>281</v>
-      </c>
-      <c r="E42" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="F42" s="8" t="s">
+      <c r="H44" s="51"/>
+    </row>
+    <row r="45" ht="51" customHeight="1" spans="1:8">
+      <c r="A45" s="11"/>
+      <c r="B45" s="39"/>
+      <c r="C45" s="49" t="s">
+        <v>294</v>
+      </c>
+      <c r="D45" s="50" t="s">
+        <v>295</v>
+      </c>
+      <c r="E45" s="50" t="s">
+        <v>296</v>
+      </c>
+      <c r="F45" s="51" t="s">
         <v>60</v>
       </c>
-      <c r="G42" s="9" t="s">
+      <c r="G45" s="51" t="s">
+        <v>109</v>
+      </c>
+      <c r="H45" s="51"/>
+    </row>
+    <row r="46" ht="51" spans="1:8">
+      <c r="A46" s="12"/>
+      <c r="B46" s="36"/>
+      <c r="C46" s="49" t="s">
+        <v>297</v>
+      </c>
+      <c r="D46" s="50" t="s">
+        <v>298</v>
+      </c>
+      <c r="E46" s="49" t="s">
+        <v>299</v>
+      </c>
+      <c r="F46" s="51" t="s">
+        <v>60</v>
+      </c>
+      <c r="G46" s="51" t="s">
         <v>188</v>
       </c>
-      <c r="H42" s="21"/>
-    </row>
-    <row r="43" ht="126" customHeight="1" spans="1:8">
-      <c r="A43" s="11"/>
-      <c r="B43" s="43" t="s">
-        <v>283</v>
-      </c>
-      <c r="C43" s="44" t="s">
-        <v>284</v>
-      </c>
-      <c r="D43" s="44" t="s">
-        <v>285</v>
-      </c>
-      <c r="E43" s="44" t="s">
-        <v>286</v>
-      </c>
-      <c r="F43" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="G43" s="46" t="s">
-        <v>109</v>
-      </c>
-      <c r="H43" s="47" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="44" ht="81" customHeight="1" spans="1:8">
-      <c r="A44" s="11"/>
-      <c r="B44" s="43"/>
-      <c r="C44" s="44" t="s">
-        <v>287</v>
-      </c>
-      <c r="D44" s="44" t="s">
-        <v>288</v>
-      </c>
-      <c r="E44" s="44" t="s">
-        <v>289</v>
-      </c>
-      <c r="F44" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="G44" s="46" t="s">
-        <v>109</v>
-      </c>
-      <c r="H44" s="47" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="45" ht="81" customHeight="1" spans="1:8">
-      <c r="A45" s="11"/>
-      <c r="B45" s="38" t="s">
-        <v>290</v>
-      </c>
-      <c r="C45" s="41" t="s">
-        <v>291</v>
-      </c>
-      <c r="D45" s="9" t="s">
-        <v>292</v>
-      </c>
-      <c r="E45" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="F45" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="G45" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="H45" s="30" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="46" ht="68" customHeight="1" spans="1:8">
-      <c r="A46" s="11"/>
-      <c r="B46" s="40"/>
-      <c r="C46" s="48" t="s">
-        <v>294</v>
-      </c>
-      <c r="D46" s="20" t="s">
-        <v>295</v>
-      </c>
-      <c r="E46" s="20" t="s">
-        <v>296</v>
-      </c>
-      <c r="F46" s="21" t="s">
-        <v>10</v>
-      </c>
-      <c r="G46" s="49" t="s">
-        <v>188</v>
-      </c>
-      <c r="H46" s="30" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="47" ht="51" customHeight="1" spans="1:8">
-      <c r="A47" s="11"/>
-      <c r="B47" s="40"/>
-      <c r="C47" s="50" t="s">
-        <v>297</v>
-      </c>
-      <c r="D47" s="51" t="s">
-        <v>298</v>
-      </c>
-      <c r="E47" s="50" t="s">
-        <v>299</v>
-      </c>
-      <c r="F47" s="52" t="s">
-        <v>10</v>
-      </c>
-      <c r="G47" s="52" t="s">
-        <v>109</v>
-      </c>
-      <c r="H47" s="52"/>
-    </row>
-    <row r="48" ht="68" customHeight="1" spans="1:8">
-      <c r="A48" s="11"/>
-      <c r="B48" s="40"/>
-      <c r="C48" s="50" t="s">
-        <v>300</v>
-      </c>
-      <c r="D48" s="51" t="s">
-        <v>301</v>
-      </c>
-      <c r="E48" s="50" t="s">
-        <v>302</v>
-      </c>
-      <c r="F48" s="52" t="s">
-        <v>10</v>
-      </c>
-      <c r="G48" s="52" t="s">
-        <v>109</v>
-      </c>
-      <c r="H48" s="52"/>
-    </row>
-    <row r="49" ht="51" customHeight="1" spans="1:8">
-      <c r="A49" s="11"/>
-      <c r="B49" s="40"/>
-      <c r="C49" s="50" t="s">
-        <v>303</v>
-      </c>
-      <c r="D49" s="51" t="s">
-        <v>304</v>
-      </c>
-      <c r="E49" s="50" t="s">
-        <v>305</v>
-      </c>
-      <c r="F49" s="52" t="s">
-        <v>10</v>
-      </c>
-      <c r="G49" s="52" t="s">
-        <v>109</v>
-      </c>
-      <c r="H49" s="52"/>
-    </row>
-    <row r="50" ht="84" customHeight="1" spans="1:8">
-      <c r="A50" s="11"/>
-      <c r="B50" s="40"/>
-      <c r="C50" s="50" t="s">
-        <v>306</v>
-      </c>
-      <c r="D50" s="51" t="s">
-        <v>307</v>
-      </c>
-      <c r="E50" s="50" t="s">
-        <v>308</v>
-      </c>
-      <c r="F50" s="52" t="s">
-        <v>60</v>
-      </c>
-      <c r="G50" s="52" t="s">
-        <v>188</v>
-      </c>
-      <c r="H50" s="52"/>
-    </row>
-    <row r="51" ht="51" customHeight="1" spans="1:8">
-      <c r="A51" s="11"/>
-      <c r="B51" s="40"/>
-      <c r="C51" s="50" t="s">
-        <v>309</v>
-      </c>
-      <c r="D51" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="E51" s="51" t="s">
-        <v>311</v>
-      </c>
-      <c r="F51" s="52" t="s">
-        <v>60</v>
-      </c>
-      <c r="G51" s="52" t="s">
-        <v>109</v>
-      </c>
-      <c r="H51" s="52"/>
-    </row>
-    <row r="52" ht="51" spans="1:8">
-      <c r="A52" s="12"/>
-      <c r="B52" s="38"/>
-      <c r="C52" s="50" t="s">
-        <v>312</v>
-      </c>
-      <c r="D52" s="51" t="s">
-        <v>313</v>
-      </c>
-      <c r="E52" s="50" t="s">
-        <v>314</v>
-      </c>
-      <c r="F52" s="52" t="s">
-        <v>60</v>
-      </c>
-      <c r="G52" s="52" t="s">
-        <v>188</v>
-      </c>
-      <c r="H52" s="52"/>
+      <c r="H46" s="51"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="A2:A52"/>
+  <mergeCells count="15">
+    <mergeCell ref="A2:A46"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="B5:B11"/>
     <mergeCell ref="B15:B18"/>
     <mergeCell ref="B20:B26"/>
-    <mergeCell ref="B27:B30"/>
-    <mergeCell ref="B31:B38"/>
-    <mergeCell ref="B39:B42"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="B45:B52"/>
+    <mergeCell ref="B28:B31"/>
+    <mergeCell ref="B33:B36"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B39:B46"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="G3:G4"/>
     <mergeCell ref="G8:G9"/>
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="H6:H9"/>
-    <mergeCell ref="H32:H38"/>
+    <mergeCell ref="H29:H31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>